<commit_message>
Update benchmark: 2026-03-01 06:55:38 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -1395,7 +1395,11 @@
           <t>600 TL</t>
         </is>
       </c>
-      <c r="D24" s="14" t="inlineStr"/>
+      <c r="D24" s="14" t="inlineStr">
+        <is>
+          <t>476,2 TL</t>
+        </is>
+      </c>
       <c r="E24" s="14" t="inlineStr">
         <is>
           <t>780 TL</t>
@@ -1443,7 +1447,11 @@
           <t>495,24 TL</t>
         </is>
       </c>
-      <c r="D25" s="14" t="inlineStr"/>
+      <c r="D25" s="14" t="inlineStr">
+        <is>
+          <t>428,58 TL</t>
+        </is>
+      </c>
       <c r="E25" s="14" t="inlineStr">
         <is>
           <t>780 TL</t>

</xml_diff>

<commit_message>
Update benchmark: 2026-03-02 07:07:15 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -601,11 +601,7 @@
         </is>
       </c>
       <c r="B2" s="13" t="inlineStr"/>
-      <c r="C2" s="14" t="inlineStr">
-        <is>
-          <t>30 TL - 30 TL</t>
-        </is>
-      </c>
+      <c r="C2" s="14" t="inlineStr"/>
       <c r="D2" s="14" t="inlineStr">
         <is>
           <t>33,33 TL - 33,33 TL</t>
@@ -728,11 +724,7 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="E6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 199,41 TL</t>
-        </is>
-      </c>
+      <c r="E6" s="14" t="inlineStr"/>
       <c r="F6" s="14" t="inlineStr"/>
       <c r="G6" s="14" t="inlineStr">
         <is>
@@ -898,7 +890,7 @@
       </c>
       <c r="C12" s="14" t="inlineStr">
         <is>
-          <t>WU: 1.000,01 USD–9,51 USD</t>
+          <t>WU: 1.000,01 USD–</t>
         </is>
       </c>
       <c r="D12" s="14" t="inlineStr">
@@ -930,24 +922,16 @@
       </c>
       <c r="C13" s="14" t="inlineStr">
         <is>
-          <t>Hesaba: Asgari 0 TL | Azami 0,94 TL</t>
+          <t>Hesaba: Asgari 0 TL | Azami 3.295,24 TL</t>
         </is>
       </c>
       <c r="D13" s="14" t="inlineStr">
         <is>
-          <t>Hesaba: Asgari 1 TL | Azami 909,5 TL</t>
-        </is>
-      </c>
-      <c r="E13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
-        </is>
-      </c>
-      <c r="F13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 795 TL | Azami 4.005 TL</t>
-        </is>
-      </c>
+          <t>Hesaba: Asgari 1 TL | Azami 8.937,14 TL</t>
+        </is>
+      </c>
+      <c r="E13" s="14" t="inlineStr"/>
+      <c r="F13" s="14" t="inlineStr"/>
       <c r="G13" s="14" t="inlineStr"/>
       <c r="H13" s="14" t="inlineStr">
         <is>
@@ -986,16 +970,8 @@
           <t>3.500 TL - 13.500 TL</t>
         </is>
       </c>
-      <c r="E14" s="14" t="inlineStr">
-        <is>
-          <t>2.170 TL - 2.170 TL</t>
-        </is>
-      </c>
-      <c r="F14" s="14" t="inlineStr">
-        <is>
-          <t>2.785,72 TL - 12.380,95 TL</t>
-        </is>
-      </c>
+      <c r="E14" s="14" t="inlineStr"/>
+      <c r="F14" s="14" t="inlineStr"/>
       <c r="G14" s="14" t="inlineStr">
         <is>
           <t>8.300 TL - 7,97 TL</t>

</xml_diff>

<commit_message>
Update benchmark: 2026-03-03 07:00:33 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -601,7 +601,11 @@
         </is>
       </c>
       <c r="B2" s="13" t="inlineStr"/>
-      <c r="C2" s="14" t="inlineStr"/>
+      <c r="C2" s="14" t="inlineStr">
+        <is>
+          <t>30 TL - 30 TL</t>
+        </is>
+      </c>
       <c r="D2" s="14" t="inlineStr">
         <is>
           <t>33,33 TL - 33,33 TL</t>
@@ -719,11 +723,7 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="D6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 199,41 TL</t>
-        </is>
-      </c>
+      <c r="D6" s="14" t="inlineStr"/>
       <c r="E6" s="14" t="inlineStr"/>
       <c r="F6" s="14" t="inlineStr"/>
       <c r="G6" s="14" t="inlineStr">
@@ -746,11 +746,7 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="K6" s="14" t="inlineStr">
-        <is>
-          <t>7,97 TL - 15,96 TL - 199,41 TL</t>
-        </is>
-      </c>
+      <c r="K6" s="14" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="B7" s="13" t="inlineStr">
@@ -890,14 +886,10 @@
       </c>
       <c r="C12" s="14" t="inlineStr">
         <is>
-          <t>WU: 1.000,01 USD–</t>
-        </is>
-      </c>
-      <c r="D12" s="14" t="inlineStr">
-        <is>
-          <t>WU: 0,75 USD–12 USD; Diğer: 700 TL–4.000 TL</t>
-        </is>
-      </c>
+          <t>WU: 1.000,01 USD–9,51 USD</t>
+        </is>
+      </c>
+      <c r="D12" s="14" t="inlineStr"/>
       <c r="E12" s="14" t="inlineStr"/>
       <c r="F12" s="14" t="inlineStr"/>
       <c r="G12" s="14" t="inlineStr">
@@ -908,11 +900,7 @@
       <c r="H12" s="14" t="inlineStr"/>
       <c r="I12" s="14" t="inlineStr"/>
       <c r="J12" s="14" t="inlineStr"/>
-      <c r="K12" s="14" t="inlineStr">
-        <is>
-          <t>WU: ,USD–; Diğer: 529 TL–4.454,74 TL</t>
-        </is>
-      </c>
+      <c r="K12" s="14" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="B13" s="13" t="inlineStr">
@@ -922,16 +910,16 @@
       </c>
       <c r="C13" s="14" t="inlineStr">
         <is>
-          <t>Hesaba: Asgari 0 TL | Azami 3.295,24 TL</t>
-        </is>
-      </c>
-      <c r="D13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 8.937,14 TL</t>
-        </is>
-      </c>
+          <t>Hesaba: Asgari 0 TL | Azami 0,94 TL</t>
+        </is>
+      </c>
+      <c r="D13" s="14" t="inlineStr"/>
       <c r="E13" s="14" t="inlineStr"/>
-      <c r="F13" s="14" t="inlineStr"/>
+      <c r="F13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 795 TL | Azami 4.005 TL</t>
+        </is>
+      </c>
       <c r="G13" s="14" t="inlineStr"/>
       <c r="H13" s="14" t="inlineStr">
         <is>
@@ -948,11 +936,7 @@
           <t>Hesaba: Asgari 1 TL | Azami 995,5 TL</t>
         </is>
       </c>
-      <c r="K13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 865,75 TL</t>
-        </is>
-      </c>
+      <c r="K13" s="14" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="B14" s="13" t="inlineStr">
@@ -965,13 +949,13 @@
           <t>40.000 TL - 2.485,72 TL</t>
         </is>
       </c>
-      <c r="D14" s="14" t="inlineStr">
-        <is>
-          <t>3.500 TL - 13.500 TL</t>
-        </is>
-      </c>
+      <c r="D14" s="14" t="inlineStr"/>
       <c r="E14" s="14" t="inlineStr"/>
-      <c r="F14" s="14" t="inlineStr"/>
+      <c r="F14" s="14" t="inlineStr">
+        <is>
+          <t>2.785,72 TL - 12.380,95 TL</t>
+        </is>
+      </c>
       <c r="G14" s="14" t="inlineStr">
         <is>
           <t>8.300 TL - 7,97 TL</t>
@@ -988,11 +972,7 @@
           <t>1.554,97 TL - 7.784 TL</t>
         </is>
       </c>
-      <c r="K14" s="14" t="inlineStr">
-        <is>
-          <t>1.196,51 TL - 5.583,74 TL</t>
-        </is>
-      </c>
+      <c r="K14" s="14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="12" t="inlineStr">

</xml_diff>

<commit_message>
Update benchmark: 2026-03-04 06:56:47 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -723,7 +723,11 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="D6" s="14" t="inlineStr"/>
+      <c r="D6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 199,41 TL</t>
+        </is>
+      </c>
       <c r="E6" s="14" t="inlineStr"/>
       <c r="F6" s="14" t="inlineStr"/>
       <c r="G6" s="14" t="inlineStr">
@@ -746,7 +750,11 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="K6" s="14" t="inlineStr"/>
+      <c r="K6" s="14" t="inlineStr">
+        <is>
+          <t>7,97 TL - 15,96 TL - 199,41 TL</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="B7" s="13" t="inlineStr">
@@ -889,7 +897,11 @@
           <t>WU: 1.000,01 USD–9,51 USD</t>
         </is>
       </c>
-      <c r="D12" s="14" t="inlineStr"/>
+      <c r="D12" s="14" t="inlineStr">
+        <is>
+          <t>WU: 0,75 USD–12 USD; Diğer: 700 TL–4.000 TL</t>
+        </is>
+      </c>
       <c r="E12" s="14" t="inlineStr"/>
       <c r="F12" s="14" t="inlineStr"/>
       <c r="G12" s="14" t="inlineStr">
@@ -900,7 +912,11 @@
       <c r="H12" s="14" t="inlineStr"/>
       <c r="I12" s="14" t="inlineStr"/>
       <c r="J12" s="14" t="inlineStr"/>
-      <c r="K12" s="14" t="inlineStr"/>
+      <c r="K12" s="14" t="inlineStr">
+        <is>
+          <t>WU: ,USD–; Diğer: 529 TL–4.454,74 TL</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="B13" s="13" t="inlineStr">
@@ -913,13 +929,13 @@
           <t>Hesaba: Asgari 0 TL | Azami 0,94 TL</t>
         </is>
       </c>
-      <c r="D13" s="14" t="inlineStr"/>
+      <c r="D13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
+        </is>
+      </c>
       <c r="E13" s="14" t="inlineStr"/>
-      <c r="F13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 795 TL | Azami 4.005 TL</t>
-        </is>
-      </c>
+      <c r="F13" s="14" t="inlineStr"/>
       <c r="G13" s="14" t="inlineStr"/>
       <c r="H13" s="14" t="inlineStr">
         <is>
@@ -936,7 +952,11 @@
           <t>Hesaba: Asgari 1 TL | Azami 995,5 TL</t>
         </is>
       </c>
-      <c r="K13" s="14" t="inlineStr"/>
+      <c r="K13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 865,75 TL</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="B14" s="13" t="inlineStr">
@@ -949,13 +969,13 @@
           <t>40.000 TL - 2.485,72 TL</t>
         </is>
       </c>
-      <c r="D14" s="14" t="inlineStr"/>
+      <c r="D14" s="14" t="inlineStr">
+        <is>
+          <t>3.500 TL - 13.500 TL</t>
+        </is>
+      </c>
       <c r="E14" s="14" t="inlineStr"/>
-      <c r="F14" s="14" t="inlineStr">
-        <is>
-          <t>2.785,72 TL - 12.380,95 TL</t>
-        </is>
-      </c>
+      <c r="F14" s="14" t="inlineStr"/>
       <c r="G14" s="14" t="inlineStr">
         <is>
           <t>8.300 TL - 7,97 TL</t>
@@ -972,7 +992,11 @@
           <t>1.554,97 TL - 7.784 TL</t>
         </is>
       </c>
-      <c r="K14" s="14" t="inlineStr"/>
+      <c r="K14" s="14" t="inlineStr">
+        <is>
+          <t>1.196,51 TL - 5.583,74 TL</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="12" t="inlineStr">
@@ -1002,7 +1026,7 @@
       </c>
       <c r="F15" s="14" t="inlineStr">
         <is>
-          <t>%0,5 Asgari Tutar: 361,9 TL Azami Tutar: 361,9 TL / 361,9 TL</t>
+          <t xml:space="preserve"> Asgari Tutar:  Azami Tutar: </t>
         </is>
       </c>
       <c r="G15" s="14" t="inlineStr">
@@ -1070,7 +1094,7 @@
       </c>
       <c r="F17" s="14" t="inlineStr">
         <is>
-          <t>%0,5 Asgari Tutar: 361,9 TL Azami Tutar: 361,9 TL / 361,9 TL</t>
+          <t xml:space="preserve"> Asgari Tutar:  Azami Tutar: </t>
         </is>
       </c>
       <c r="G17" s="14" t="inlineStr">
@@ -1152,11 +1176,7 @@
           <t>390 TL</t>
         </is>
       </c>
-      <c r="F20" s="14" t="inlineStr">
-        <is>
-          <t>123,81 TL</t>
-        </is>
-      </c>
+      <c r="F20" s="14" t="inlineStr"/>
       <c r="G20" s="14" t="inlineStr"/>
       <c r="H20" s="14" t="inlineStr">
         <is>
@@ -1202,7 +1222,7 @@
       </c>
       <c r="F21" s="14" t="inlineStr">
         <is>
-          <t>%0,5 Asgari Tutar: 544,76 TL Azami Tutar: 544,76 TL / 3.157,14 TL</t>
+          <t xml:space="preserve"> Asgari Tutar:  Azami Tutar: </t>
         </is>
       </c>
       <c r="G21" s="14" t="inlineStr">
@@ -1254,7 +1274,7 @@
       </c>
       <c r="F22" s="14" t="inlineStr">
         <is>
-          <t>%0,5 Asgari Tutar: 427,62 TL Azami Tutar: 427,62 TL / 1.669,52 TL</t>
+          <t xml:space="preserve"> Asgari Tutar:  Azami Tutar: </t>
         </is>
       </c>
       <c r="G22" s="14" t="inlineStr">
@@ -1304,11 +1324,7 @@
           <t>75 TL</t>
         </is>
       </c>
-      <c r="F23" s="14" t="inlineStr">
-        <is>
-          <t>86,67 TL</t>
-        </is>
-      </c>
+      <c r="F23" s="14" t="inlineStr"/>
       <c r="G23" s="14" t="inlineStr">
         <is>
           <t>600 TL</t>
@@ -1361,11 +1377,7 @@
           <t>780 TL</t>
         </is>
       </c>
-      <c r="F24" s="14" t="inlineStr">
-        <is>
-          <t>600 TL</t>
-        </is>
-      </c>
+      <c r="F24" s="14" t="inlineStr"/>
       <c r="G24" s="14" t="inlineStr">
         <is>
           <t>160 TL</t>
@@ -1413,11 +1425,7 @@
           <t>780 TL</t>
         </is>
       </c>
-      <c r="F25" s="14" t="inlineStr">
-        <is>
-          <t>600 TL</t>
-        </is>
-      </c>
+      <c r="F25" s="14" t="inlineStr"/>
       <c r="G25" s="14" t="inlineStr"/>
       <c r="H25" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update benchmark: 2026-03-05 07:01:43 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -750,11 +750,7 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="K6" s="14" t="inlineStr">
-        <is>
-          <t>7,97 TL - 15,96 TL - 199,41 TL</t>
-        </is>
-      </c>
+      <c r="K6" s="14" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="B7" s="13" t="inlineStr">
@@ -912,11 +908,7 @@
       <c r="H12" s="14" t="inlineStr"/>
       <c r="I12" s="14" t="inlineStr"/>
       <c r="J12" s="14" t="inlineStr"/>
-      <c r="K12" s="14" t="inlineStr">
-        <is>
-          <t>WU: ,USD–; Diğer: 529 TL–4.454,74 TL</t>
-        </is>
-      </c>
+      <c r="K12" s="14" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="B13" s="13" t="inlineStr">
@@ -935,7 +927,11 @@
         </is>
       </c>
       <c r="E13" s="14" t="inlineStr"/>
-      <c r="F13" s="14" t="inlineStr"/>
+      <c r="F13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 795 TL | Azami 4.005 TL</t>
+        </is>
+      </c>
       <c r="G13" s="14" t="inlineStr"/>
       <c r="H13" s="14" t="inlineStr">
         <is>
@@ -952,11 +948,7 @@
           <t>Hesaba: Asgari 1 TL | Azami 995,5 TL</t>
         </is>
       </c>
-      <c r="K13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 865,75 TL</t>
-        </is>
-      </c>
+      <c r="K13" s="14" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="B14" s="13" t="inlineStr">
@@ -975,7 +967,11 @@
         </is>
       </c>
       <c r="E14" s="14" t="inlineStr"/>
-      <c r="F14" s="14" t="inlineStr"/>
+      <c r="F14" s="14" t="inlineStr">
+        <is>
+          <t>2.785,72 TL - 12.380,95 TL</t>
+        </is>
+      </c>
       <c r="G14" s="14" t="inlineStr">
         <is>
           <t>8.300 TL - 7,97 TL</t>
@@ -992,11 +988,7 @@
           <t>1.554,97 TL - 7.784 TL</t>
         </is>
       </c>
-      <c r="K14" s="14" t="inlineStr">
-        <is>
-          <t>1.196,51 TL - 5.583,74 TL</t>
-        </is>
-      </c>
+      <c r="K14" s="14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="12" t="inlineStr">
@@ -1026,7 +1018,7 @@
       </c>
       <c r="F15" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Asgari Tutar:  Azami Tutar: </t>
+          <t>%0,5 Asgari Tutar: 361,9 TL Azami Tutar: 361,9 TL / 361,9 TL</t>
         </is>
       </c>
       <c r="G15" s="14" t="inlineStr">
@@ -1094,7 +1086,7 @@
       </c>
       <c r="F17" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Asgari Tutar:  Azami Tutar: </t>
+          <t>%0,5 Asgari Tutar: 361,9 TL Azami Tutar: 361,9 TL / 361,9 TL</t>
         </is>
       </c>
       <c r="G17" s="14" t="inlineStr">
@@ -1176,7 +1168,11 @@
           <t>390 TL</t>
         </is>
       </c>
-      <c r="F20" s="14" t="inlineStr"/>
+      <c r="F20" s="14" t="inlineStr">
+        <is>
+          <t>123,81 TL</t>
+        </is>
+      </c>
       <c r="G20" s="14" t="inlineStr"/>
       <c r="H20" s="14" t="inlineStr">
         <is>
@@ -1222,7 +1218,7 @@
       </c>
       <c r="F21" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Asgari Tutar:  Azami Tutar: </t>
+          <t>%0,5 Asgari Tutar: 544,76 TL Azami Tutar: 544,76 TL / 3.157,14 TL</t>
         </is>
       </c>
       <c r="G21" s="14" t="inlineStr">
@@ -1274,7 +1270,7 @@
       </c>
       <c r="F22" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Asgari Tutar:  Azami Tutar: </t>
+          <t>%0,5 Asgari Tutar: 427,62 TL Azami Tutar: 427,62 TL / 1.669,52 TL</t>
         </is>
       </c>
       <c r="G22" s="14" t="inlineStr">
@@ -1324,7 +1320,11 @@
           <t>75 TL</t>
         </is>
       </c>
-      <c r="F23" s="14" t="inlineStr"/>
+      <c r="F23" s="14" t="inlineStr">
+        <is>
+          <t>86,67 TL</t>
+        </is>
+      </c>
       <c r="G23" s="14" t="inlineStr">
         <is>
           <t>600 TL</t>
@@ -1377,7 +1377,11 @@
           <t>780 TL</t>
         </is>
       </c>
-      <c r="F24" s="14" t="inlineStr"/>
+      <c r="F24" s="14" t="inlineStr">
+        <is>
+          <t>600 TL</t>
+        </is>
+      </c>
       <c r="G24" s="14" t="inlineStr">
         <is>
           <t>160 TL</t>
@@ -1425,7 +1429,11 @@
           <t>780 TL</t>
         </is>
       </c>
-      <c r="F25" s="14" t="inlineStr"/>
+      <c r="F25" s="14" t="inlineStr">
+        <is>
+          <t>600 TL</t>
+        </is>
+      </c>
       <c r="G25" s="14" t="inlineStr"/>
       <c r="H25" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update benchmark: 2026-03-06 06:59:07 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -662,11 +662,7 @@
       <c r="D3" s="14" t="inlineStr"/>
       <c r="E3" s="14" t="inlineStr"/>
       <c r="F3" s="14" t="inlineStr"/>
-      <c r="G3" s="14" t="inlineStr">
-        <is>
-          <t>39,87 TRY - 79,76 TRY - 797,68 TRY</t>
-        </is>
-      </c>
+      <c r="G3" s="14" t="inlineStr"/>
       <c r="H3" s="14" t="inlineStr"/>
       <c r="I3" s="14" t="inlineStr"/>
       <c r="J3" s="14" t="inlineStr"/>
@@ -682,11 +678,7 @@
       <c r="D4" s="14" t="inlineStr"/>
       <c r="E4" s="14" t="inlineStr"/>
       <c r="F4" s="14" t="inlineStr"/>
-      <c r="G4" s="14" t="inlineStr">
-        <is>
-          <t>27,84 TRY - 55,69 TRY - 398,83 TRY</t>
-        </is>
-      </c>
+      <c r="G4" s="14" t="inlineStr"/>
       <c r="H4" s="14" t="inlineStr"/>
       <c r="I4" s="14" t="inlineStr"/>
       <c r="J4" s="14" t="inlineStr"/>
@@ -702,11 +694,7 @@
       <c r="D5" s="14" t="inlineStr"/>
       <c r="E5" s="14" t="inlineStr"/>
       <c r="F5" s="14" t="inlineStr"/>
-      <c r="G5" s="14" t="inlineStr">
-        <is>
-          <t>7,97 TRY - 15,96 TRY - 199,41 TRY</t>
-        </is>
-      </c>
+      <c r="G5" s="14" t="inlineStr"/>
       <c r="H5" s="14" t="inlineStr"/>
       <c r="I5" s="14" t="inlineStr"/>
       <c r="J5" s="14" t="inlineStr"/>
@@ -728,13 +716,13 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="E6" s="14" t="inlineStr"/>
+      <c r="E6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 199,41 TL</t>
+        </is>
+      </c>
       <c r="F6" s="14" t="inlineStr"/>
-      <c r="G6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 99,71 TL</t>
-        </is>
-      </c>
+      <c r="G6" s="14" t="inlineStr"/>
       <c r="H6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
@@ -750,7 +738,11 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="K6" s="14" t="inlineStr"/>
+      <c r="K6" s="14" t="inlineStr">
+        <is>
+          <t>7,97 TL - 15,96 TL - 199,41 TL</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="B7" s="13" t="inlineStr">
@@ -807,11 +799,7 @@
       <c r="D8" s="14" t="inlineStr"/>
       <c r="E8" s="14" t="inlineStr"/>
       <c r="F8" s="14" t="inlineStr"/>
-      <c r="G8" s="14" t="inlineStr">
-        <is>
-          <t>19,94 TRY - 39,88 TRY - 398,84 TRY</t>
-        </is>
-      </c>
+      <c r="G8" s="14" t="inlineStr"/>
       <c r="H8" s="14" t="inlineStr"/>
       <c r="I8" s="14" t="inlineStr"/>
       <c r="J8" s="14" t="inlineStr"/>
@@ -827,11 +815,7 @@
       <c r="D9" s="14" t="inlineStr"/>
       <c r="E9" s="14" t="inlineStr"/>
       <c r="F9" s="14" t="inlineStr"/>
-      <c r="G9" s="14" t="inlineStr">
-        <is>
-          <t>13,92 TRY - 27,85 TRY - 199,42 TRY</t>
-        </is>
-      </c>
+      <c r="G9" s="14" t="inlineStr"/>
       <c r="H9" s="14" t="inlineStr"/>
       <c r="I9" s="14" t="inlineStr"/>
       <c r="J9" s="14" t="inlineStr"/>
@@ -847,11 +831,7 @@
       <c r="D10" s="14" t="inlineStr"/>
       <c r="E10" s="14" t="inlineStr"/>
       <c r="F10" s="14" t="inlineStr"/>
-      <c r="G10" s="14" t="inlineStr">
-        <is>
-          <t>3,99 TRY - 7,98 TRY - 99,71 TRY</t>
-        </is>
-      </c>
+      <c r="G10" s="14" t="inlineStr"/>
       <c r="H10" s="14" t="inlineStr"/>
       <c r="I10" s="14" t="inlineStr"/>
       <c r="J10" s="14" t="inlineStr"/>
@@ -867,11 +847,7 @@
       <c r="D11" s="14" t="inlineStr"/>
       <c r="E11" s="14" t="inlineStr"/>
       <c r="F11" s="14" t="inlineStr"/>
-      <c r="G11" s="14" t="inlineStr">
-        <is>
-          <t>3,99 TRY - 7,98 TRY - 99,71 TRY</t>
-        </is>
-      </c>
+      <c r="G11" s="14" t="inlineStr"/>
       <c r="H11" s="14" t="inlineStr"/>
       <c r="I11" s="14" t="inlineStr"/>
       <c r="J11" s="14" t="inlineStr"/>
@@ -900,15 +876,15 @@
       </c>
       <c r="E12" s="14" t="inlineStr"/>
       <c r="F12" s="14" t="inlineStr"/>
-      <c r="G12" s="14" t="inlineStr">
-        <is>
-          <t>Şube (Kasadan): %0,5; Şube (Hesaptan): %0,75; İnternet: 15 USD</t>
-        </is>
-      </c>
+      <c r="G12" s="14" t="inlineStr"/>
       <c r="H12" s="14" t="inlineStr"/>
       <c r="I12" s="14" t="inlineStr"/>
       <c r="J12" s="14" t="inlineStr"/>
-      <c r="K12" s="14" t="inlineStr"/>
+      <c r="K12" s="14" t="inlineStr">
+        <is>
+          <t>WU: ,USD–; Diğer: 529 TL–4.454,74 TL</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="B13" s="13" t="inlineStr">
@@ -926,7 +902,11 @@
           <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
         </is>
       </c>
-      <c r="E13" s="14" t="inlineStr"/>
+      <c r="E13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
+        </is>
+      </c>
       <c r="F13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 795 TL | Azami 4.005 TL</t>
@@ -948,7 +928,11 @@
           <t>Hesaba: Asgari 1 TL | Azami 995,5 TL</t>
         </is>
       </c>
-      <c r="K13" s="14" t="inlineStr"/>
+      <c r="K13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 865,75 TL</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="B14" s="13" t="inlineStr">
@@ -966,17 +950,17 @@
           <t>3.500 TL - 13.500 TL</t>
         </is>
       </c>
-      <c r="E14" s="14" t="inlineStr"/>
+      <c r="E14" s="14" t="inlineStr">
+        <is>
+          <t>2.170 TL - 2.170 TL</t>
+        </is>
+      </c>
       <c r="F14" s="14" t="inlineStr">
         <is>
           <t>2.785,72 TL - 12.380,95 TL</t>
         </is>
       </c>
-      <c r="G14" s="14" t="inlineStr">
-        <is>
-          <t>8.300 TL - 7,97 TL</t>
-        </is>
-      </c>
+      <c r="G14" s="14" t="inlineStr"/>
       <c r="H14" s="14" t="inlineStr">
         <is>
           <t>3.000 TL - 6.000 TL</t>
@@ -988,7 +972,11 @@
           <t>1.554,97 TL - 7.784 TL</t>
         </is>
       </c>
-      <c r="K14" s="14" t="inlineStr"/>
+      <c r="K14" s="14" t="inlineStr">
+        <is>
+          <t>1.196,51 TL - 5.583,74 TL</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="12" t="inlineStr">

</xml_diff>

<commit_message>
Update benchmark: 2026-03-07 06:51:43 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -662,7 +662,11 @@
       <c r="D3" s="14" t="inlineStr"/>
       <c r="E3" s="14" t="inlineStr"/>
       <c r="F3" s="14" t="inlineStr"/>
-      <c r="G3" s="14" t="inlineStr"/>
+      <c r="G3" s="14" t="inlineStr">
+        <is>
+          <t>39,87 TRY - 79,76 TRY - 797,68 TRY</t>
+        </is>
+      </c>
       <c r="H3" s="14" t="inlineStr"/>
       <c r="I3" s="14" t="inlineStr"/>
       <c r="J3" s="14" t="inlineStr"/>
@@ -678,7 +682,11 @@
       <c r="D4" s="14" t="inlineStr"/>
       <c r="E4" s="14" t="inlineStr"/>
       <c r="F4" s="14" t="inlineStr"/>
-      <c r="G4" s="14" t="inlineStr"/>
+      <c r="G4" s="14" t="inlineStr">
+        <is>
+          <t>27,84 TRY - 55,69 TRY - 398,83 TRY</t>
+        </is>
+      </c>
       <c r="H4" s="14" t="inlineStr"/>
       <c r="I4" s="14" t="inlineStr"/>
       <c r="J4" s="14" t="inlineStr"/>
@@ -694,7 +702,11 @@
       <c r="D5" s="14" t="inlineStr"/>
       <c r="E5" s="14" t="inlineStr"/>
       <c r="F5" s="14" t="inlineStr"/>
-      <c r="G5" s="14" t="inlineStr"/>
+      <c r="G5" s="14" t="inlineStr">
+        <is>
+          <t>7,97 TRY - 15,96 TRY - 199,41 TRY</t>
+        </is>
+      </c>
       <c r="H5" s="14" t="inlineStr"/>
       <c r="I5" s="14" t="inlineStr"/>
       <c r="J5" s="14" t="inlineStr"/>
@@ -722,7 +734,11 @@
         </is>
       </c>
       <c r="F6" s="14" t="inlineStr"/>
-      <c r="G6" s="14" t="inlineStr"/>
+      <c r="G6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 99,71 TL</t>
+        </is>
+      </c>
       <c r="H6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
@@ -799,7 +815,11 @@
       <c r="D8" s="14" t="inlineStr"/>
       <c r="E8" s="14" t="inlineStr"/>
       <c r="F8" s="14" t="inlineStr"/>
-      <c r="G8" s="14" t="inlineStr"/>
+      <c r="G8" s="14" t="inlineStr">
+        <is>
+          <t>19,94 TRY - 39,88 TRY - 398,84 TRY</t>
+        </is>
+      </c>
       <c r="H8" s="14" t="inlineStr"/>
       <c r="I8" s="14" t="inlineStr"/>
       <c r="J8" s="14" t="inlineStr"/>
@@ -815,7 +835,11 @@
       <c r="D9" s="14" t="inlineStr"/>
       <c r="E9" s="14" t="inlineStr"/>
       <c r="F9" s="14" t="inlineStr"/>
-      <c r="G9" s="14" t="inlineStr"/>
+      <c r="G9" s="14" t="inlineStr">
+        <is>
+          <t>13,92 TRY - 27,85 TRY - 199,42 TRY</t>
+        </is>
+      </c>
       <c r="H9" s="14" t="inlineStr"/>
       <c r="I9" s="14" t="inlineStr"/>
       <c r="J9" s="14" t="inlineStr"/>
@@ -831,7 +855,11 @@
       <c r="D10" s="14" t="inlineStr"/>
       <c r="E10" s="14" t="inlineStr"/>
       <c r="F10" s="14" t="inlineStr"/>
-      <c r="G10" s="14" t="inlineStr"/>
+      <c r="G10" s="14" t="inlineStr">
+        <is>
+          <t>3,99 TRY - 7,98 TRY - 99,71 TRY</t>
+        </is>
+      </c>
       <c r="H10" s="14" t="inlineStr"/>
       <c r="I10" s="14" t="inlineStr"/>
       <c r="J10" s="14" t="inlineStr"/>
@@ -847,7 +875,11 @@
       <c r="D11" s="14" t="inlineStr"/>
       <c r="E11" s="14" t="inlineStr"/>
       <c r="F11" s="14" t="inlineStr"/>
-      <c r="G11" s="14" t="inlineStr"/>
+      <c r="G11" s="14" t="inlineStr">
+        <is>
+          <t>3,99 TRY - 7,98 TRY - 99,71 TRY</t>
+        </is>
+      </c>
       <c r="H11" s="14" t="inlineStr"/>
       <c r="I11" s="14" t="inlineStr"/>
       <c r="J11" s="14" t="inlineStr"/>
@@ -876,7 +908,11 @@
       </c>
       <c r="E12" s="14" t="inlineStr"/>
       <c r="F12" s="14" t="inlineStr"/>
-      <c r="G12" s="14" t="inlineStr"/>
+      <c r="G12" s="14" t="inlineStr">
+        <is>
+          <t>Şube (Kasadan): %0,5; Şube (Hesaptan): %0,75; İnternet: 15 USD</t>
+        </is>
+      </c>
       <c r="H12" s="14" t="inlineStr"/>
       <c r="I12" s="14" t="inlineStr"/>
       <c r="J12" s="14" t="inlineStr"/>
@@ -960,7 +996,11 @@
           <t>2.785,72 TL - 12.380,95 TL</t>
         </is>
       </c>
-      <c r="G14" s="14" t="inlineStr"/>
+      <c r="G14" s="14" t="inlineStr">
+        <is>
+          <t>8.300 TL - 7,97 TL</t>
+        </is>
+      </c>
       <c r="H14" s="14" t="inlineStr">
         <is>
           <t>3.000 TL - 6.000 TL</t>

</xml_diff>

<commit_message>
Update benchmark: 2026-03-09 07:10:10 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -728,11 +728,7 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="E6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 199,41 TL</t>
-        </is>
-      </c>
+      <c r="E6" s="14" t="inlineStr"/>
       <c r="F6" s="14" t="inlineStr"/>
       <c r="G6" s="14" t="inlineStr">
         <is>
@@ -754,11 +750,7 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="K6" s="14" t="inlineStr">
-        <is>
-          <t>7,97 TL - 15,96 TL - 199,41 TL</t>
-        </is>
-      </c>
+      <c r="K6" s="14" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="B7" s="13" t="inlineStr">
@@ -916,11 +908,7 @@
       <c r="H12" s="14" t="inlineStr"/>
       <c r="I12" s="14" t="inlineStr"/>
       <c r="J12" s="14" t="inlineStr"/>
-      <c r="K12" s="14" t="inlineStr">
-        <is>
-          <t>WU: ,USD–; Diğer: 529 TL–4.454,74 TL</t>
-        </is>
-      </c>
+      <c r="K12" s="14" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="B13" s="13" t="inlineStr">
@@ -938,16 +926,8 @@
           <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
         </is>
       </c>
-      <c r="E13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
-        </is>
-      </c>
-      <c r="F13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 795 TL | Azami 4.005 TL</t>
-        </is>
-      </c>
+      <c r="E13" s="14" t="inlineStr"/>
+      <c r="F13" s="14" t="inlineStr"/>
       <c r="G13" s="14" t="inlineStr"/>
       <c r="H13" s="14" t="inlineStr">
         <is>
@@ -964,11 +944,7 @@
           <t>Hesaba: Asgari 1 TL | Azami 995,5 TL</t>
         </is>
       </c>
-      <c r="K13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 865,75 TL</t>
-        </is>
-      </c>
+      <c r="K13" s="14" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="B14" s="13" t="inlineStr">
@@ -986,16 +962,8 @@
           <t>3.500 TL - 13.500 TL</t>
         </is>
       </c>
-      <c r="E14" s="14" t="inlineStr">
-        <is>
-          <t>2.170 TL - 2.170 TL</t>
-        </is>
-      </c>
-      <c r="F14" s="14" t="inlineStr">
-        <is>
-          <t>2.785,72 TL - 12.380,95 TL</t>
-        </is>
-      </c>
+      <c r="E14" s="14" t="inlineStr"/>
+      <c r="F14" s="14" t="inlineStr"/>
       <c r="G14" s="14" t="inlineStr">
         <is>
           <t>8.300 TL - 7,97 TL</t>
@@ -1012,11 +980,7 @@
           <t>1.554,97 TL - 7.784 TL</t>
         </is>
       </c>
-      <c r="K14" s="14" t="inlineStr">
-        <is>
-          <t>1.196,51 TL - 5.583,74 TL</t>
-        </is>
-      </c>
+      <c r="K14" s="14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="12" t="inlineStr">

</xml_diff>

<commit_message>
Update benchmark: 2026-03-10 06:59:11 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -636,11 +636,7 @@
           <t>18 TL - 18 TL</t>
         </is>
       </c>
-      <c r="J2" s="14" t="inlineStr">
-        <is>
-          <t>65 TL - 65 TL</t>
-        </is>
-      </c>
+      <c r="J2" s="14" t="inlineStr"/>
       <c r="K2" s="14" t="inlineStr">
         <is>
           <t>32,62 TL - 32,62 TL</t>
@@ -723,11 +719,7 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="D6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 199,41 TL</t>
-        </is>
-      </c>
+      <c r="D6" s="14" t="inlineStr"/>
       <c r="E6" s="14" t="inlineStr"/>
       <c r="F6" s="14" t="inlineStr"/>
       <c r="G6" s="14" t="inlineStr">
@@ -745,12 +737,12 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="J6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 199,41 TL</t>
-        </is>
-      </c>
-      <c r="K6" s="14" t="inlineStr"/>
+      <c r="J6" s="14" t="inlineStr"/>
+      <c r="K6" s="14" t="inlineStr">
+        <is>
+          <t>7,97 TL - 15,96 TL - 199,41 TL</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="B7" s="13" t="inlineStr">
@@ -781,11 +773,7 @@
         </is>
       </c>
       <c r="I7" s="14" t="inlineStr"/>
-      <c r="J7" s="14" t="inlineStr">
-        <is>
-          <t>%2,5</t>
-        </is>
-      </c>
+      <c r="J7" s="14" t="inlineStr"/>
       <c r="K7" s="14" t="inlineStr">
         <is>
           <t>%3,1</t>
@@ -893,11 +881,7 @@
           <t>WU: 1.000,01 USD–9,51 USD</t>
         </is>
       </c>
-      <c r="D12" s="14" t="inlineStr">
-        <is>
-          <t>WU: 0,75 USD–12 USD; Diğer: 700 TL–4.000 TL</t>
-        </is>
-      </c>
+      <c r="D12" s="14" t="inlineStr"/>
       <c r="E12" s="14" t="inlineStr"/>
       <c r="F12" s="14" t="inlineStr"/>
       <c r="G12" s="14" t="inlineStr">
@@ -908,7 +892,11 @@
       <c r="H12" s="14" t="inlineStr"/>
       <c r="I12" s="14" t="inlineStr"/>
       <c r="J12" s="14" t="inlineStr"/>
-      <c r="K12" s="14" t="inlineStr"/>
+      <c r="K12" s="14" t="inlineStr">
+        <is>
+          <t>WU: ,USD–; Diğer: 529 TL–4.454,74 TL</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="B13" s="13" t="inlineStr">
@@ -921,11 +909,7 @@
           <t>Hesaba: Asgari 0 TL | Azami 0,94 TL</t>
         </is>
       </c>
-      <c r="D13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
-        </is>
-      </c>
+      <c r="D13" s="14" t="inlineStr"/>
       <c r="E13" s="14" t="inlineStr"/>
       <c r="F13" s="14" t="inlineStr"/>
       <c r="G13" s="14" t="inlineStr"/>
@@ -939,12 +923,12 @@
           <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
         </is>
       </c>
-      <c r="J13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 995,5 TL</t>
-        </is>
-      </c>
-      <c r="K13" s="14" t="inlineStr"/>
+      <c r="J13" s="14" t="inlineStr"/>
+      <c r="K13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 865,75 TL</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="B14" s="13" t="inlineStr">
@@ -957,11 +941,7 @@
           <t>40.000 TL - 2.485,72 TL</t>
         </is>
       </c>
-      <c r="D14" s="14" t="inlineStr">
-        <is>
-          <t>3.500 TL - 13.500 TL</t>
-        </is>
-      </c>
+      <c r="D14" s="14" t="inlineStr"/>
       <c r="E14" s="14" t="inlineStr"/>
       <c r="F14" s="14" t="inlineStr"/>
       <c r="G14" s="14" t="inlineStr">
@@ -975,12 +955,12 @@
         </is>
       </c>
       <c r="I14" s="14" t="inlineStr"/>
-      <c r="J14" s="14" t="inlineStr">
-        <is>
-          <t>1.554,97 TL - 7.784 TL</t>
-        </is>
-      </c>
-      <c r="K14" s="14" t="inlineStr"/>
+      <c r="J14" s="14" t="inlineStr"/>
+      <c r="K14" s="14" t="inlineStr">
+        <is>
+          <t>1.196,51 TL - 5.583,74 TL</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="12" t="inlineStr">

</xml_diff>

<commit_message>
Update benchmark: 2026-03-11 07:02:56 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -636,7 +636,11 @@
           <t>18 TL - 18 TL</t>
         </is>
       </c>
-      <c r="J2" s="14" t="inlineStr"/>
+      <c r="J2" s="14" t="inlineStr">
+        <is>
+          <t>65 TL - 65 TL</t>
+        </is>
+      </c>
       <c r="K2" s="14" t="inlineStr">
         <is>
           <t>32,62 TL - 32,62 TL</t>
@@ -714,13 +718,17 @@
           <t>DÜZENLİ EFT</t>
         </is>
       </c>
-      <c r="C6" s="14" t="inlineStr">
+      <c r="C6" s="14" t="inlineStr"/>
+      <c r="D6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="D6" s="14" t="inlineStr"/>
-      <c r="E6" s="14" t="inlineStr"/>
+      <c r="E6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 199,41 TL</t>
+        </is>
+      </c>
       <c r="F6" s="14" t="inlineStr"/>
       <c r="G6" s="14" t="inlineStr">
         <is>
@@ -737,7 +745,11 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="J6" s="14" t="inlineStr"/>
+      <c r="J6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 199,41 TL</t>
+        </is>
+      </c>
       <c r="K6" s="14" t="inlineStr">
         <is>
           <t>7,97 TL - 15,96 TL - 199,41 TL</t>
@@ -773,7 +785,11 @@
         </is>
       </c>
       <c r="I7" s="14" t="inlineStr"/>
-      <c r="J7" s="14" t="inlineStr"/>
+      <c r="J7" s="14" t="inlineStr">
+        <is>
+          <t>%3,5</t>
+        </is>
+      </c>
       <c r="K7" s="14" t="inlineStr">
         <is>
           <t>%3,1</t>
@@ -876,12 +892,12 @@
           <t>GİDEN SWIFT</t>
         </is>
       </c>
-      <c r="C12" s="14" t="inlineStr">
-        <is>
-          <t>WU: 1.000,01 USD–9,51 USD</t>
-        </is>
-      </c>
-      <c r="D12" s="14" t="inlineStr"/>
+      <c r="C12" s="14" t="inlineStr"/>
+      <c r="D12" s="14" t="inlineStr">
+        <is>
+          <t>WU: 0,75 USD–12 USD; Diğer: 700 TL–4.000 TL</t>
+        </is>
+      </c>
       <c r="E12" s="14" t="inlineStr"/>
       <c r="F12" s="14" t="inlineStr"/>
       <c r="G12" s="14" t="inlineStr">
@@ -904,14 +920,22 @@
           <t>GELEN SWIFT</t>
         </is>
       </c>
-      <c r="C13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 0 TL | Azami 0,94 TL</t>
-        </is>
-      </c>
-      <c r="D13" s="14" t="inlineStr"/>
-      <c r="E13" s="14" t="inlineStr"/>
-      <c r="F13" s="14" t="inlineStr"/>
+      <c r="C13" s="14" t="inlineStr"/>
+      <c r="D13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
+        </is>
+      </c>
+      <c r="E13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
+        </is>
+      </c>
+      <c r="F13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 795 TL | Azami 4.005 TL</t>
+        </is>
+      </c>
       <c r="G13" s="14" t="inlineStr"/>
       <c r="H13" s="14" t="inlineStr">
         <is>
@@ -923,7 +947,11 @@
           <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
         </is>
       </c>
-      <c r="J13" s="14" t="inlineStr"/>
+      <c r="J13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 1.303 TL</t>
+        </is>
+      </c>
       <c r="K13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 865,75 TL</t>
@@ -936,14 +964,22 @@
           <t>GİDEN SWIFT - Mobil</t>
         </is>
       </c>
-      <c r="C14" s="14" t="inlineStr">
-        <is>
-          <t>40.000 TL - 2.485,72 TL</t>
-        </is>
-      </c>
-      <c r="D14" s="14" t="inlineStr"/>
-      <c r="E14" s="14" t="inlineStr"/>
-      <c r="F14" s="14" t="inlineStr"/>
+      <c r="C14" s="14" t="inlineStr"/>
+      <c r="D14" s="14" t="inlineStr">
+        <is>
+          <t>3.500 TL - 13.500 TL</t>
+        </is>
+      </c>
+      <c r="E14" s="14" t="inlineStr">
+        <is>
+          <t>2.170 TL - 2.170 TL</t>
+        </is>
+      </c>
+      <c r="F14" s="14" t="inlineStr">
+        <is>
+          <t>2.785,72 TL - 12.380,95 TL</t>
+        </is>
+      </c>
       <c r="G14" s="14" t="inlineStr">
         <is>
           <t>8.300 TL - 7,97 TL</t>
@@ -955,7 +991,11 @@
         </is>
       </c>
       <c r="I14" s="14" t="inlineStr"/>
-      <c r="J14" s="14" t="inlineStr"/>
+      <c r="J14" s="14" t="inlineStr">
+        <is>
+          <t>1.554,97 TL - 7.784 TL</t>
+        </is>
+      </c>
       <c r="K14" s="14" t="inlineStr">
         <is>
           <t>1.196,51 TL - 5.583,74 TL</t>

</xml_diff>

<commit_message>
Update benchmark: 2026-03-12 07:05:01 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -718,28 +718,24 @@
           <t>DÜZENLİ EFT</t>
         </is>
       </c>
-      <c r="C6" s="14" t="inlineStr"/>
+      <c r="C6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 199,41 TL</t>
+        </is>
+      </c>
       <c r="D6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="E6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 199,41 TL</t>
-        </is>
-      </c>
+      <c r="E6" s="14" t="inlineStr"/>
       <c r="F6" s="14" t="inlineStr"/>
       <c r="G6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 99,71 TL</t>
         </is>
       </c>
-      <c r="H6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 199,41 TL</t>
-        </is>
-      </c>
+      <c r="H6" s="14" t="inlineStr"/>
       <c r="I6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
@@ -892,7 +888,11 @@
           <t>GİDEN SWIFT</t>
         </is>
       </c>
-      <c r="C12" s="14" t="inlineStr"/>
+      <c r="C12" s="14" t="inlineStr">
+        <is>
+          <t>WU: 1.000,01 USD–9,51 USD</t>
+        </is>
+      </c>
       <c r="D12" s="14" t="inlineStr">
         <is>
           <t>WU: 0,75 USD–12 USD; Diğer: 700 TL–4.000 TL</t>
@@ -920,28 +920,24 @@
           <t>GELEN SWIFT</t>
         </is>
       </c>
-      <c r="C13" s="14" t="inlineStr"/>
+      <c r="C13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 0 TL | Azami 0,94 TL</t>
+        </is>
+      </c>
       <c r="D13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
         </is>
       </c>
-      <c r="E13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
-        </is>
-      </c>
+      <c r="E13" s="14" t="inlineStr"/>
       <c r="F13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 795 TL | Azami 4.005 TL</t>
         </is>
       </c>
       <c r="G13" s="14" t="inlineStr"/>
-      <c r="H13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
-        </is>
-      </c>
+      <c r="H13" s="14" t="inlineStr"/>
       <c r="I13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
@@ -964,17 +960,17 @@
           <t>GİDEN SWIFT - Mobil</t>
         </is>
       </c>
-      <c r="C14" s="14" t="inlineStr"/>
+      <c r="C14" s="14" t="inlineStr">
+        <is>
+          <t>40.000 TL - 2.485,72 TL</t>
+        </is>
+      </c>
       <c r="D14" s="14" t="inlineStr">
         <is>
           <t>3.500 TL - 13.500 TL</t>
         </is>
       </c>
-      <c r="E14" s="14" t="inlineStr">
-        <is>
-          <t>2.170 TL - 2.170 TL</t>
-        </is>
-      </c>
+      <c r="E14" s="14" t="inlineStr"/>
       <c r="F14" s="14" t="inlineStr">
         <is>
           <t>2.785,72 TL - 12.380,95 TL</t>
@@ -985,11 +981,7 @@
           <t>8.300 TL - 7,97 TL</t>
         </is>
       </c>
-      <c r="H14" s="14" t="inlineStr">
-        <is>
-          <t>3.000 TL - 6.000 TL</t>
-        </is>
-      </c>
+      <c r="H14" s="14" t="inlineStr"/>
       <c r="I14" s="14" t="inlineStr"/>
       <c r="J14" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update benchmark: 2026-03-13 07:02:12 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -718,34 +718,30 @@
           <t>DÜZENLİ EFT</t>
         </is>
       </c>
-      <c r="C6" s="14" t="inlineStr">
+      <c r="C6" s="14" t="inlineStr"/>
+      <c r="D6" s="14" t="inlineStr"/>
+      <c r="E6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="D6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 199,41 TL</t>
-        </is>
-      </c>
-      <c r="E6" s="14" t="inlineStr"/>
       <c r="F6" s="14" t="inlineStr"/>
       <c r="G6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 99,71 TL</t>
         </is>
       </c>
-      <c r="H6" s="14" t="inlineStr"/>
+      <c r="H6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 199,41 TL</t>
+        </is>
+      </c>
       <c r="I6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="J6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 199,41 TL</t>
-        </is>
-      </c>
+      <c r="J6" s="14" t="inlineStr"/>
       <c r="K6" s="14" t="inlineStr">
         <is>
           <t>7,97 TL - 15,96 TL - 199,41 TL</t>
@@ -888,16 +884,8 @@
           <t>GİDEN SWIFT</t>
         </is>
       </c>
-      <c r="C12" s="14" t="inlineStr">
-        <is>
-          <t>WU: 1.000,01 USD–9,51 USD</t>
-        </is>
-      </c>
-      <c r="D12" s="14" t="inlineStr">
-        <is>
-          <t>WU: 0,75 USD–12 USD; Diğer: 700 TL–4.000 TL</t>
-        </is>
-      </c>
+      <c r="C12" s="14" t="inlineStr"/>
+      <c r="D12" s="14" t="inlineStr"/>
       <c r="E12" s="14" t="inlineStr"/>
       <c r="F12" s="14" t="inlineStr"/>
       <c r="G12" s="14" t="inlineStr">
@@ -920,34 +908,30 @@
           <t>GELEN SWIFT</t>
         </is>
       </c>
-      <c r="C13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 0 TL | Azami 0,94 TL</t>
-        </is>
-      </c>
-      <c r="D13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
-        </is>
-      </c>
-      <c r="E13" s="14" t="inlineStr"/>
+      <c r="C13" s="14" t="inlineStr"/>
+      <c r="D13" s="14" t="inlineStr"/>
+      <c r="E13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
+        </is>
+      </c>
       <c r="F13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 795 TL | Azami 4.005 TL</t>
         </is>
       </c>
       <c r="G13" s="14" t="inlineStr"/>
-      <c r="H13" s="14" t="inlineStr"/>
+      <c r="H13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
+        </is>
+      </c>
       <c r="I13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
         </is>
       </c>
-      <c r="J13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 1.303 TL</t>
-        </is>
-      </c>
+      <c r="J13" s="14" t="inlineStr"/>
       <c r="K13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 865,75 TL</t>
@@ -960,17 +944,13 @@
           <t>GİDEN SWIFT - Mobil</t>
         </is>
       </c>
-      <c r="C14" s="14" t="inlineStr">
-        <is>
-          <t>40.000 TL - 2.485,72 TL</t>
-        </is>
-      </c>
-      <c r="D14" s="14" t="inlineStr">
-        <is>
-          <t>3.500 TL - 13.500 TL</t>
-        </is>
-      </c>
-      <c r="E14" s="14" t="inlineStr"/>
+      <c r="C14" s="14" t="inlineStr"/>
+      <c r="D14" s="14" t="inlineStr"/>
+      <c r="E14" s="14" t="inlineStr">
+        <is>
+          <t>2.170 TL - 2.170 TL</t>
+        </is>
+      </c>
       <c r="F14" s="14" t="inlineStr">
         <is>
           <t>2.785,72 TL - 12.380,95 TL</t>
@@ -981,13 +961,13 @@
           <t>8.300 TL - 7,97 TL</t>
         </is>
       </c>
-      <c r="H14" s="14" t="inlineStr"/>
+      <c r="H14" s="14" t="inlineStr">
+        <is>
+          <t>3.000 TL - 6.000 TL</t>
+        </is>
+      </c>
       <c r="I14" s="14" t="inlineStr"/>
-      <c r="J14" s="14" t="inlineStr">
-        <is>
-          <t>1.554,97 TL - 7.784 TL</t>
-        </is>
-      </c>
+      <c r="J14" s="14" t="inlineStr"/>
       <c r="K14" s="14" t="inlineStr">
         <is>
           <t>1.196,51 TL - 5.583,74 TL</t>

</xml_diff>

<commit_message>
Update benchmark: 2026-03-14 06:53:50 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -718,7 +718,11 @@
           <t>DÜZENLİ EFT</t>
         </is>
       </c>
-      <c r="C6" s="14" t="inlineStr"/>
+      <c r="C6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 199,41 TL</t>
+        </is>
+      </c>
       <c r="D6" s="14" t="inlineStr"/>
       <c r="E6" s="14" t="inlineStr">
         <is>
@@ -741,7 +745,11 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="J6" s="14" t="inlineStr"/>
+      <c r="J6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 199,41 TL</t>
+        </is>
+      </c>
       <c r="K6" s="14" t="inlineStr">
         <is>
           <t>7,97 TL - 15,96 TL - 199,41 TL</t>
@@ -884,7 +892,11 @@
           <t>GİDEN SWIFT</t>
         </is>
       </c>
-      <c r="C12" s="14" t="inlineStr"/>
+      <c r="C12" s="14" t="inlineStr">
+        <is>
+          <t>WU: 1.000,01 USD–9,51 USD</t>
+        </is>
+      </c>
       <c r="D12" s="14" t="inlineStr"/>
       <c r="E12" s="14" t="inlineStr"/>
       <c r="F12" s="14" t="inlineStr"/>
@@ -908,7 +920,11 @@
           <t>GELEN SWIFT</t>
         </is>
       </c>
-      <c r="C13" s="14" t="inlineStr"/>
+      <c r="C13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 0 TL | Azami 0,94 TL</t>
+        </is>
+      </c>
       <c r="D13" s="14" t="inlineStr"/>
       <c r="E13" s="14" t="inlineStr">
         <is>
@@ -931,7 +947,11 @@
           <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
         </is>
       </c>
-      <c r="J13" s="14" t="inlineStr"/>
+      <c r="J13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 1.303 TL</t>
+        </is>
+      </c>
       <c r="K13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 865,75 TL</t>
@@ -944,7 +964,11 @@
           <t>GİDEN SWIFT - Mobil</t>
         </is>
       </c>
-      <c r="C14" s="14" t="inlineStr"/>
+      <c r="C14" s="14" t="inlineStr">
+        <is>
+          <t>40.000 TL - 2.485,72 TL</t>
+        </is>
+      </c>
       <c r="D14" s="14" t="inlineStr"/>
       <c r="E14" s="14" t="inlineStr">
         <is>
@@ -967,7 +991,11 @@
         </is>
       </c>
       <c r="I14" s="14" t="inlineStr"/>
-      <c r="J14" s="14" t="inlineStr"/>
+      <c r="J14" s="14" t="inlineStr">
+        <is>
+          <t>1.554,97 TL - 7.784 TL</t>
+        </is>
+      </c>
       <c r="K14" s="14" t="inlineStr">
         <is>
           <t>1.196,51 TL - 5.583,74 TL</t>

</xml_diff>

<commit_message>
Update benchmark: 2026-03-15 07:05:59 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -723,7 +723,11 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="D6" s="14" t="inlineStr"/>
+      <c r="D6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 199,41 TL</t>
+        </is>
+      </c>
       <c r="E6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
@@ -735,11 +739,7 @@
           <t>8.300,01 TL - 99,71 TL</t>
         </is>
       </c>
-      <c r="H6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 199,41 TL</t>
-        </is>
-      </c>
+      <c r="H6" s="14" t="inlineStr"/>
       <c r="I6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
@@ -897,7 +897,11 @@
           <t>WU: 1.000,01 USD–9,51 USD</t>
         </is>
       </c>
-      <c r="D12" s="14" t="inlineStr"/>
+      <c r="D12" s="14" t="inlineStr">
+        <is>
+          <t>WU: 0,75 USD–12 USD; Diğer: 700 TL–4.000 TL</t>
+        </is>
+      </c>
       <c r="E12" s="14" t="inlineStr"/>
       <c r="F12" s="14" t="inlineStr"/>
       <c r="G12" s="14" t="inlineStr">
@@ -925,23 +929,19 @@
           <t>Hesaba: Asgari 0 TL | Azami 0,94 TL</t>
         </is>
       </c>
-      <c r="D13" s="14" t="inlineStr"/>
+      <c r="D13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
+        </is>
+      </c>
       <c r="E13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
         </is>
       </c>
-      <c r="F13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 795 TL | Azami 4.005 TL</t>
-        </is>
-      </c>
+      <c r="F13" s="14" t="inlineStr"/>
       <c r="G13" s="14" t="inlineStr"/>
-      <c r="H13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
-        </is>
-      </c>
+      <c r="H13" s="14" t="inlineStr"/>
       <c r="I13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
@@ -969,27 +969,23 @@
           <t>40.000 TL - 2.485,72 TL</t>
         </is>
       </c>
-      <c r="D14" s="14" t="inlineStr"/>
+      <c r="D14" s="14" t="inlineStr">
+        <is>
+          <t>3.500 TL - 13.500 TL</t>
+        </is>
+      </c>
       <c r="E14" s="14" t="inlineStr">
         <is>
           <t>2.170 TL - 2.170 TL</t>
         </is>
       </c>
-      <c r="F14" s="14" t="inlineStr">
-        <is>
-          <t>2.785,72 TL - 12.380,95 TL</t>
-        </is>
-      </c>
+      <c r="F14" s="14" t="inlineStr"/>
       <c r="G14" s="14" t="inlineStr">
         <is>
           <t>8.300 TL - 7,97 TL</t>
         </is>
       </c>
-      <c r="H14" s="14" t="inlineStr">
-        <is>
-          <t>3.000 TL - 6.000 TL</t>
-        </is>
-      </c>
+      <c r="H14" s="14" t="inlineStr"/>
       <c r="I14" s="14" t="inlineStr"/>
       <c r="J14" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update benchmark: 2026-03-16 07:26:10 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -718,16 +718,8 @@
           <t>DÜZENLİ EFT</t>
         </is>
       </c>
-      <c r="C6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 199,41 TL</t>
-        </is>
-      </c>
-      <c r="D6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 199,41 TL</t>
-        </is>
-      </c>
+      <c r="C6" s="14" t="inlineStr"/>
+      <c r="D6" s="14" t="inlineStr"/>
       <c r="E6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
@@ -739,7 +731,11 @@
           <t>8.300,01 TL - 99,71 TL</t>
         </is>
       </c>
-      <c r="H6" s="14" t="inlineStr"/>
+      <c r="H6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 199,41 TL</t>
+        </is>
+      </c>
       <c r="I6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
@@ -892,16 +888,8 @@
           <t>GİDEN SWIFT</t>
         </is>
       </c>
-      <c r="C12" s="14" t="inlineStr">
-        <is>
-          <t>WU: 1.000,01 USD–9,51 USD</t>
-        </is>
-      </c>
-      <c r="D12" s="14" t="inlineStr">
-        <is>
-          <t>WU: 0,75 USD–12 USD; Diğer: 700 TL–4.000 TL</t>
-        </is>
-      </c>
+      <c r="C12" s="14" t="inlineStr"/>
+      <c r="D12" s="14" t="inlineStr"/>
       <c r="E12" s="14" t="inlineStr"/>
       <c r="F12" s="14" t="inlineStr"/>
       <c r="G12" s="14" t="inlineStr">
@@ -924,24 +912,24 @@
           <t>GELEN SWIFT</t>
         </is>
       </c>
-      <c r="C13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 0 TL | Azami 0,94 TL</t>
-        </is>
-      </c>
-      <c r="D13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
-        </is>
-      </c>
+      <c r="C13" s="14" t="inlineStr"/>
+      <c r="D13" s="14" t="inlineStr"/>
       <c r="E13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
         </is>
       </c>
-      <c r="F13" s="14" t="inlineStr"/>
+      <c r="F13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 795 TL | Azami 4.005 TL</t>
+        </is>
+      </c>
       <c r="G13" s="14" t="inlineStr"/>
-      <c r="H13" s="14" t="inlineStr"/>
+      <c r="H13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
+        </is>
+      </c>
       <c r="I13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
@@ -964,28 +952,28 @@
           <t>GİDEN SWIFT - Mobil</t>
         </is>
       </c>
-      <c r="C14" s="14" t="inlineStr">
-        <is>
-          <t>40.000 TL - 2.485,72 TL</t>
-        </is>
-      </c>
-      <c r="D14" s="14" t="inlineStr">
-        <is>
-          <t>3.500 TL - 13.500 TL</t>
-        </is>
-      </c>
+      <c r="C14" s="14" t="inlineStr"/>
+      <c r="D14" s="14" t="inlineStr"/>
       <c r="E14" s="14" t="inlineStr">
         <is>
           <t>2.170 TL - 2.170 TL</t>
         </is>
       </c>
-      <c r="F14" s="14" t="inlineStr"/>
+      <c r="F14" s="14" t="inlineStr">
+        <is>
+          <t>2.785,72 TL - 12.380,95 TL</t>
+        </is>
+      </c>
       <c r="G14" s="14" t="inlineStr">
         <is>
           <t>8.300 TL - 7,97 TL</t>
         </is>
       </c>
-      <c r="H14" s="14" t="inlineStr"/>
+      <c r="H14" s="14" t="inlineStr">
+        <is>
+          <t>3.000 TL - 6.000 TL</t>
+        </is>
+      </c>
       <c r="I14" s="14" t="inlineStr"/>
       <c r="J14" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update benchmark: 2026-03-17 07:13:11 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -718,8 +718,16 @@
           <t>DÜZENLİ EFT</t>
         </is>
       </c>
-      <c r="C6" s="14" t="inlineStr"/>
-      <c r="D6" s="14" t="inlineStr"/>
+      <c r="C6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 199,41 TL</t>
+        </is>
+      </c>
+      <c r="D6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 199,41 TL</t>
+        </is>
+      </c>
       <c r="E6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
@@ -888,8 +896,16 @@
           <t>GİDEN SWIFT</t>
         </is>
       </c>
-      <c r="C12" s="14" t="inlineStr"/>
-      <c r="D12" s="14" t="inlineStr"/>
+      <c r="C12" s="14" t="inlineStr">
+        <is>
+          <t>WU: 1.000,01 USD–9,51 USD</t>
+        </is>
+      </c>
+      <c r="D12" s="14" t="inlineStr">
+        <is>
+          <t>WU: 0,75 USD–12 USD; Diğer: 700 TL–4.000 TL</t>
+        </is>
+      </c>
       <c r="E12" s="14" t="inlineStr"/>
       <c r="F12" s="14" t="inlineStr"/>
       <c r="G12" s="14" t="inlineStr">
@@ -912,18 +928,22 @@
           <t>GELEN SWIFT</t>
         </is>
       </c>
-      <c r="C13" s="14" t="inlineStr"/>
-      <c r="D13" s="14" t="inlineStr"/>
+      <c r="C13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 0 TL | Azami 0,94 TL</t>
+        </is>
+      </c>
+      <c r="D13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
+        </is>
+      </c>
       <c r="E13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
         </is>
       </c>
-      <c r="F13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 795 TL | Azami 4.005 TL</t>
-        </is>
-      </c>
+      <c r="F13" s="14" t="inlineStr"/>
       <c r="G13" s="14" t="inlineStr"/>
       <c r="H13" s="14" t="inlineStr">
         <is>
@@ -952,8 +972,16 @@
           <t>GİDEN SWIFT - Mobil</t>
         </is>
       </c>
-      <c r="C14" s="14" t="inlineStr"/>
-      <c r="D14" s="14" t="inlineStr"/>
+      <c r="C14" s="14" t="inlineStr">
+        <is>
+          <t>40.000 TL - 2.485,72 TL</t>
+        </is>
+      </c>
+      <c r="D14" s="14" t="inlineStr">
+        <is>
+          <t>3.500 TL - 13.500 TL</t>
+        </is>
+      </c>
       <c r="E14" s="14" t="inlineStr">
         <is>
           <t>2.170 TL - 2.170 TL</t>

</xml_diff>

<commit_message>
Update benchmark: 2026-03-18 07:10:10 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -662,11 +662,7 @@
       <c r="D3" s="14" t="inlineStr"/>
       <c r="E3" s="14" t="inlineStr"/>
       <c r="F3" s="14" t="inlineStr"/>
-      <c r="G3" s="14" t="inlineStr">
-        <is>
-          <t>39,87 TRY - 79,76 TRY - 797,68 TRY</t>
-        </is>
-      </c>
+      <c r="G3" s="14" t="inlineStr"/>
       <c r="H3" s="14" t="inlineStr"/>
       <c r="I3" s="14" t="inlineStr"/>
       <c r="J3" s="14" t="inlineStr"/>
@@ -682,11 +678,7 @@
       <c r="D4" s="14" t="inlineStr"/>
       <c r="E4" s="14" t="inlineStr"/>
       <c r="F4" s="14" t="inlineStr"/>
-      <c r="G4" s="14" t="inlineStr">
-        <is>
-          <t>27,84 TRY - 55,69 TRY - 398,83 TRY</t>
-        </is>
-      </c>
+      <c r="G4" s="14" t="inlineStr"/>
       <c r="H4" s="14" t="inlineStr"/>
       <c r="I4" s="14" t="inlineStr"/>
       <c r="J4" s="14" t="inlineStr"/>
@@ -702,11 +694,7 @@
       <c r="D5" s="14" t="inlineStr"/>
       <c r="E5" s="14" t="inlineStr"/>
       <c r="F5" s="14" t="inlineStr"/>
-      <c r="G5" s="14" t="inlineStr">
-        <is>
-          <t>7,97 TRY - 15,96 TRY - 199,41 TRY</t>
-        </is>
-      </c>
+      <c r="G5" s="14" t="inlineStr"/>
       <c r="H5" s="14" t="inlineStr"/>
       <c r="I5" s="14" t="inlineStr"/>
       <c r="J5" s="14" t="inlineStr"/>
@@ -734,31 +722,19 @@
         </is>
       </c>
       <c r="F6" s="14" t="inlineStr"/>
-      <c r="G6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 99,71 TL</t>
-        </is>
-      </c>
+      <c r="G6" s="14" t="inlineStr"/>
       <c r="H6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="I6" s="14" t="inlineStr">
+      <c r="I6" s="14" t="inlineStr"/>
+      <c r="J6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="J6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 199,41 TL</t>
-        </is>
-      </c>
-      <c r="K6" s="14" t="inlineStr">
-        <is>
-          <t>7,97 TL - 15,96 TL - 199,41 TL</t>
-        </is>
-      </c>
+      <c r="K6" s="14" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="B7" s="13" t="inlineStr">
@@ -815,11 +791,7 @@
       <c r="D8" s="14" t="inlineStr"/>
       <c r="E8" s="14" t="inlineStr"/>
       <c r="F8" s="14" t="inlineStr"/>
-      <c r="G8" s="14" t="inlineStr">
-        <is>
-          <t>19,94 TRY - 39,88 TRY - 398,84 TRY</t>
-        </is>
-      </c>
+      <c r="G8" s="14" t="inlineStr"/>
       <c r="H8" s="14" t="inlineStr"/>
       <c r="I8" s="14" t="inlineStr"/>
       <c r="J8" s="14" t="inlineStr"/>
@@ -835,11 +807,7 @@
       <c r="D9" s="14" t="inlineStr"/>
       <c r="E9" s="14" t="inlineStr"/>
       <c r="F9" s="14" t="inlineStr"/>
-      <c r="G9" s="14" t="inlineStr">
-        <is>
-          <t>13,92 TRY - 27,85 TRY - 199,42 TRY</t>
-        </is>
-      </c>
+      <c r="G9" s="14" t="inlineStr"/>
       <c r="H9" s="14" t="inlineStr"/>
       <c r="I9" s="14" t="inlineStr"/>
       <c r="J9" s="14" t="inlineStr"/>
@@ -855,11 +823,7 @@
       <c r="D10" s="14" t="inlineStr"/>
       <c r="E10" s="14" t="inlineStr"/>
       <c r="F10" s="14" t="inlineStr"/>
-      <c r="G10" s="14" t="inlineStr">
-        <is>
-          <t>3,99 TRY - 7,98 TRY - 99,71 TRY</t>
-        </is>
-      </c>
+      <c r="G10" s="14" t="inlineStr"/>
       <c r="H10" s="14" t="inlineStr"/>
       <c r="I10" s="14" t="inlineStr"/>
       <c r="J10" s="14" t="inlineStr"/>
@@ -875,11 +839,7 @@
       <c r="D11" s="14" t="inlineStr"/>
       <c r="E11" s="14" t="inlineStr"/>
       <c r="F11" s="14" t="inlineStr"/>
-      <c r="G11" s="14" t="inlineStr">
-        <is>
-          <t>3,99 TRY - 7,98 TRY - 99,71 TRY</t>
-        </is>
-      </c>
+      <c r="G11" s="14" t="inlineStr"/>
       <c r="H11" s="14" t="inlineStr"/>
       <c r="I11" s="14" t="inlineStr"/>
       <c r="J11" s="14" t="inlineStr"/>
@@ -908,19 +868,11 @@
       </c>
       <c r="E12" s="14" t="inlineStr"/>
       <c r="F12" s="14" t="inlineStr"/>
-      <c r="G12" s="14" t="inlineStr">
-        <is>
-          <t>Şube (Kasadan): %0,5; Şube (Hesaptan): %0,75; İnternet: 15 USD</t>
-        </is>
-      </c>
+      <c r="G12" s="14" t="inlineStr"/>
       <c r="H12" s="14" t="inlineStr"/>
       <c r="I12" s="14" t="inlineStr"/>
       <c r="J12" s="14" t="inlineStr"/>
-      <c r="K12" s="14" t="inlineStr">
-        <is>
-          <t>WU: ,USD–; Diğer: 529 TL–4.454,74 TL</t>
-        </is>
-      </c>
+      <c r="K12" s="14" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="B13" s="13" t="inlineStr">
@@ -950,21 +902,13 @@
           <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
         </is>
       </c>
-      <c r="I13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
-        </is>
-      </c>
+      <c r="I13" s="14" t="inlineStr"/>
       <c r="J13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.303 TL</t>
         </is>
       </c>
-      <c r="K13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 865,75 TL</t>
-        </is>
-      </c>
+      <c r="K13" s="14" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="B14" s="13" t="inlineStr">
@@ -992,11 +936,7 @@
           <t>2.785,72 TL - 12.380,95 TL</t>
         </is>
       </c>
-      <c r="G14" s="14" t="inlineStr">
-        <is>
-          <t>8.300 TL - 7,97 TL</t>
-        </is>
-      </c>
+      <c r="G14" s="14" t="inlineStr"/>
       <c r="H14" s="14" t="inlineStr">
         <is>
           <t>3.000 TL - 6.000 TL</t>
@@ -1008,11 +948,7 @@
           <t>1.554,97 TL - 7.784 TL</t>
         </is>
       </c>
-      <c r="K14" s="14" t="inlineStr">
-        <is>
-          <t>1.196,51 TL - 5.583,74 TL</t>
-        </is>
-      </c>
+      <c r="K14" s="14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="12" t="inlineStr">

</xml_diff>

<commit_message>
Update benchmark: 2026-03-19 07:07:20 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -662,7 +662,11 @@
       <c r="D3" s="14" t="inlineStr"/>
       <c r="E3" s="14" t="inlineStr"/>
       <c r="F3" s="14" t="inlineStr"/>
-      <c r="G3" s="14" t="inlineStr"/>
+      <c r="G3" s="14" t="inlineStr">
+        <is>
+          <t>39,87 TRY - 79,76 TRY - 797,68 TRY</t>
+        </is>
+      </c>
       <c r="H3" s="14" t="inlineStr"/>
       <c r="I3" s="14" t="inlineStr"/>
       <c r="J3" s="14" t="inlineStr"/>
@@ -678,7 +682,11 @@
       <c r="D4" s="14" t="inlineStr"/>
       <c r="E4" s="14" t="inlineStr"/>
       <c r="F4" s="14" t="inlineStr"/>
-      <c r="G4" s="14" t="inlineStr"/>
+      <c r="G4" s="14" t="inlineStr">
+        <is>
+          <t>27,84 TRY - 55,69 TRY - 398,83 TRY</t>
+        </is>
+      </c>
       <c r="H4" s="14" t="inlineStr"/>
       <c r="I4" s="14" t="inlineStr"/>
       <c r="J4" s="14" t="inlineStr"/>
@@ -694,7 +702,11 @@
       <c r="D5" s="14" t="inlineStr"/>
       <c r="E5" s="14" t="inlineStr"/>
       <c r="F5" s="14" t="inlineStr"/>
-      <c r="G5" s="14" t="inlineStr"/>
+      <c r="G5" s="14" t="inlineStr">
+        <is>
+          <t>7,97 TRY - 15,96 TRY - 199,41 TRY</t>
+        </is>
+      </c>
       <c r="H5" s="14" t="inlineStr"/>
       <c r="I5" s="14" t="inlineStr"/>
       <c r="J5" s="14" t="inlineStr"/>
@@ -716,13 +728,13 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="E6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 199,41 TL</t>
-        </is>
-      </c>
+      <c r="E6" s="14" t="inlineStr"/>
       <c r="F6" s="14" t="inlineStr"/>
-      <c r="G6" s="14" t="inlineStr"/>
+      <c r="G6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 99,71 TL</t>
+        </is>
+      </c>
       <c r="H6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
@@ -734,7 +746,11 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="K6" s="14" t="inlineStr"/>
+      <c r="K6" s="14" t="inlineStr">
+        <is>
+          <t>7,97 TL - 15,96 TL - 199,41 TL</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="B7" s="13" t="inlineStr">
@@ -791,7 +807,11 @@
       <c r="D8" s="14" t="inlineStr"/>
       <c r="E8" s="14" t="inlineStr"/>
       <c r="F8" s="14" t="inlineStr"/>
-      <c r="G8" s="14" t="inlineStr"/>
+      <c r="G8" s="14" t="inlineStr">
+        <is>
+          <t>19,94 TRY - 39,88 TRY - 398,84 TRY</t>
+        </is>
+      </c>
       <c r="H8" s="14" t="inlineStr"/>
       <c r="I8" s="14" t="inlineStr"/>
       <c r="J8" s="14" t="inlineStr"/>
@@ -807,7 +827,11 @@
       <c r="D9" s="14" t="inlineStr"/>
       <c r="E9" s="14" t="inlineStr"/>
       <c r="F9" s="14" t="inlineStr"/>
-      <c r="G9" s="14" t="inlineStr"/>
+      <c r="G9" s="14" t="inlineStr">
+        <is>
+          <t>13,92 TRY - 27,85 TRY - 199,42 TRY</t>
+        </is>
+      </c>
       <c r="H9" s="14" t="inlineStr"/>
       <c r="I9" s="14" t="inlineStr"/>
       <c r="J9" s="14" t="inlineStr"/>
@@ -823,7 +847,11 @@
       <c r="D10" s="14" t="inlineStr"/>
       <c r="E10" s="14" t="inlineStr"/>
       <c r="F10" s="14" t="inlineStr"/>
-      <c r="G10" s="14" t="inlineStr"/>
+      <c r="G10" s="14" t="inlineStr">
+        <is>
+          <t>3,99 TRY - 7,98 TRY - 99,71 TRY</t>
+        </is>
+      </c>
       <c r="H10" s="14" t="inlineStr"/>
       <c r="I10" s="14" t="inlineStr"/>
       <c r="J10" s="14" t="inlineStr"/>
@@ -839,7 +867,11 @@
       <c r="D11" s="14" t="inlineStr"/>
       <c r="E11" s="14" t="inlineStr"/>
       <c r="F11" s="14" t="inlineStr"/>
-      <c r="G11" s="14" t="inlineStr"/>
+      <c r="G11" s="14" t="inlineStr">
+        <is>
+          <t>3,99 TRY - 7,98 TRY - 99,71 TRY</t>
+        </is>
+      </c>
       <c r="H11" s="14" t="inlineStr"/>
       <c r="I11" s="14" t="inlineStr"/>
       <c r="J11" s="14" t="inlineStr"/>
@@ -863,16 +895,24 @@
       </c>
       <c r="D12" s="14" t="inlineStr">
         <is>
-          <t>WU: 0,75 USD–12 USD; Diğer: 700 TL–4.000 TL</t>
+          <t>Diğer: 700 TL–4.000 TL</t>
         </is>
       </c>
       <c r="E12" s="14" t="inlineStr"/>
       <c r="F12" s="14" t="inlineStr"/>
-      <c r="G12" s="14" t="inlineStr"/>
+      <c r="G12" s="14" t="inlineStr">
+        <is>
+          <t>Şube (Kasadan): %0,5; Şube (Hesaptan): %0,75; İnternet: 15 USD</t>
+        </is>
+      </c>
       <c r="H12" s="14" t="inlineStr"/>
       <c r="I12" s="14" t="inlineStr"/>
       <c r="J12" s="14" t="inlineStr"/>
-      <c r="K12" s="14" t="inlineStr"/>
+      <c r="K12" s="14" t="inlineStr">
+        <is>
+          <t>WU: ,USD–; Diğer: 529 TL–4.454,74 TL</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="B13" s="13" t="inlineStr">
@@ -890,11 +930,7 @@
           <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
         </is>
       </c>
-      <c r="E13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
-        </is>
-      </c>
+      <c r="E13" s="14" t="inlineStr"/>
       <c r="F13" s="14" t="inlineStr"/>
       <c r="G13" s="14" t="inlineStr"/>
       <c r="H13" s="14" t="inlineStr">
@@ -908,7 +944,11 @@
           <t>Hesaba: Asgari 1 TL | Azami 1.303 TL</t>
         </is>
       </c>
-      <c r="K13" s="14" t="inlineStr"/>
+      <c r="K13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 865,75 TL</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="B14" s="13" t="inlineStr">
@@ -926,17 +966,17 @@
           <t>3.500 TL - 13.500 TL</t>
         </is>
       </c>
-      <c r="E14" s="14" t="inlineStr">
-        <is>
-          <t>2.170 TL - 2.170 TL</t>
-        </is>
-      </c>
+      <c r="E14" s="14" t="inlineStr"/>
       <c r="F14" s="14" t="inlineStr">
         <is>
           <t>2.785,72 TL - 12.380,95 TL</t>
         </is>
       </c>
-      <c r="G14" s="14" t="inlineStr"/>
+      <c r="G14" s="14" t="inlineStr">
+        <is>
+          <t>8.300 TL - 7,97 TL</t>
+        </is>
+      </c>
       <c r="H14" s="14" t="inlineStr">
         <is>
           <t>3.000 TL - 6.000 TL</t>
@@ -948,7 +988,11 @@
           <t>1.554,97 TL - 7.784 TL</t>
         </is>
       </c>
-      <c r="K14" s="14" t="inlineStr"/>
+      <c r="K14" s="14" t="inlineStr">
+        <is>
+          <t>1.196,51 TL - 5.583,74 TL</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="12" t="inlineStr">

</xml_diff>

<commit_message>
Update benchmark: 2026-03-20 07:04:30 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -728,7 +728,11 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="E6" s="14" t="inlineStr"/>
+      <c r="E6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 199,41 TL</t>
+        </is>
+      </c>
       <c r="F6" s="14" t="inlineStr"/>
       <c r="G6" s="14" t="inlineStr">
         <is>
@@ -740,7 +744,11 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="I6" s="14" t="inlineStr"/>
+      <c r="I6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 199,41 TL</t>
+        </is>
+      </c>
       <c r="J6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
@@ -895,7 +903,7 @@
       </c>
       <c r="D12" s="14" t="inlineStr">
         <is>
-          <t>Diğer: 700 TL–4.000 TL</t>
+          <t>WU: 0,75 USD–12 USD; Diğer: 700 TL–4.000 TL</t>
         </is>
       </c>
       <c r="E12" s="14" t="inlineStr"/>
@@ -930,7 +938,11 @@
           <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
         </is>
       </c>
-      <c r="E13" s="14" t="inlineStr"/>
+      <c r="E13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
+        </is>
+      </c>
       <c r="F13" s="14" t="inlineStr"/>
       <c r="G13" s="14" t="inlineStr"/>
       <c r="H13" s="14" t="inlineStr">
@@ -938,7 +950,11 @@
           <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
         </is>
       </c>
-      <c r="I13" s="14" t="inlineStr"/>
+      <c r="I13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
+        </is>
+      </c>
       <c r="J13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.303 TL</t>
@@ -966,7 +982,11 @@
           <t>3.500 TL - 13.500 TL</t>
         </is>
       </c>
-      <c r="E14" s="14" t="inlineStr"/>
+      <c r="E14" s="14" t="inlineStr">
+        <is>
+          <t>2.170 TL - 2.170 TL</t>
+        </is>
+      </c>
       <c r="F14" s="14" t="inlineStr">
         <is>
           <t>2.785,72 TL - 12.380,95 TL</t>

</xml_diff>

<commit_message>
Update benchmark: 2026-03-21 06:50:36 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -601,11 +601,7 @@
         </is>
       </c>
       <c r="B2" s="13" t="inlineStr"/>
-      <c r="C2" s="14" t="inlineStr">
-        <is>
-          <t>30 TL - 30 TL</t>
-        </is>
-      </c>
+      <c r="C2" s="14" t="inlineStr"/>
       <c r="D2" s="14" t="inlineStr">
         <is>
           <t>33,33 TL - 33,33 TL</t>
@@ -749,11 +745,7 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="J6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 199,41 TL</t>
-        </is>
-      </c>
+      <c r="J6" s="14" t="inlineStr"/>
       <c r="K6" s="14" t="inlineStr">
         <is>
           <t>7,97 TL - 15,96 TL - 199,41 TL</t>
@@ -898,12 +890,12 @@
       </c>
       <c r="C12" s="14" t="inlineStr">
         <is>
-          <t>WU: 1.000,01 USD–9,51 USD</t>
+          <t>WU: 1.000,01 USD–</t>
         </is>
       </c>
       <c r="D12" s="14" t="inlineStr">
         <is>
-          <t>WU: 0,75 USD–12 USD; Diğer: 700 TL–4.000 TL</t>
+          <t>Diğer: 700 TL–4.000 TL</t>
         </is>
       </c>
       <c r="E12" s="14" t="inlineStr"/>
@@ -930,7 +922,7 @@
       </c>
       <c r="C13" s="14" t="inlineStr">
         <is>
-          <t>Hesaba: Asgari 0 TL | Azami 0,94 TL</t>
+          <t>Hesaba: Asgari 0 TL | Azami 3.295,24 TL</t>
         </is>
       </c>
       <c r="D13" s="14" t="inlineStr">
@@ -955,11 +947,7 @@
           <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
         </is>
       </c>
-      <c r="J13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 1.303 TL</t>
-        </is>
-      </c>
+      <c r="J13" s="14" t="inlineStr"/>
       <c r="K13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 865,75 TL</t>
@@ -1003,11 +991,7 @@
         </is>
       </c>
       <c r="I14" s="14" t="inlineStr"/>
-      <c r="J14" s="14" t="inlineStr">
-        <is>
-          <t>1.554,97 TL - 7.784 TL</t>
-        </is>
-      </c>
+      <c r="J14" s="14" t="inlineStr"/>
       <c r="K14" s="14" t="inlineStr">
         <is>
           <t>1.196,51 TL - 5.583,74 TL</t>

</xml_diff>

<commit_message>
Update benchmark: 2026-03-22 07:03:25 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -601,7 +601,11 @@
         </is>
       </c>
       <c r="B2" s="13" t="inlineStr"/>
-      <c r="C2" s="14" t="inlineStr"/>
+      <c r="C2" s="14" t="inlineStr">
+        <is>
+          <t>30 TL - 30 TL</t>
+        </is>
+      </c>
       <c r="D2" s="14" t="inlineStr">
         <is>
           <t>33,33 TL - 33,33 TL</t>
@@ -745,7 +749,11 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="J6" s="14" t="inlineStr"/>
+      <c r="J6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 199,41 TL</t>
+        </is>
+      </c>
       <c r="K6" s="14" t="inlineStr">
         <is>
           <t>7,97 TL - 15,96 TL - 199,41 TL</t>
@@ -890,12 +898,12 @@
       </c>
       <c r="C12" s="14" t="inlineStr">
         <is>
-          <t>WU: 1.000,01 USD–</t>
+          <t>WU: 1.000,01 USD–9,51 USD</t>
         </is>
       </c>
       <c r="D12" s="14" t="inlineStr">
         <is>
-          <t>Diğer: 700 TL–4.000 TL</t>
+          <t>WU: 0,75 USD–12 USD; Diğer: 700 TL–4.000 TL</t>
         </is>
       </c>
       <c r="E12" s="14" t="inlineStr"/>
@@ -922,7 +930,7 @@
       </c>
       <c r="C13" s="14" t="inlineStr">
         <is>
-          <t>Hesaba: Asgari 0 TL | Azami 3.295,24 TL</t>
+          <t>Hesaba: Asgari 0 TL | Azami 0,94 TL</t>
         </is>
       </c>
       <c r="D13" s="14" t="inlineStr">
@@ -947,7 +955,11 @@
           <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
         </is>
       </c>
-      <c r="J13" s="14" t="inlineStr"/>
+      <c r="J13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 1.303 TL</t>
+        </is>
+      </c>
       <c r="K13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 865,75 TL</t>
@@ -991,7 +1003,11 @@
         </is>
       </c>
       <c r="I14" s="14" t="inlineStr"/>
-      <c r="J14" s="14" t="inlineStr"/>
+      <c r="J14" s="14" t="inlineStr">
+        <is>
+          <t>1.554,97 TL - 7.784 TL</t>
+        </is>
+      </c>
       <c r="K14" s="14" t="inlineStr">
         <is>
           <t>1.196,51 TL - 5.583,74 TL</t>

</xml_diff>

<commit_message>
Update benchmark: 2026-03-27 07:15:36 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -903,7 +903,7 @@
       </c>
       <c r="D12" s="14" t="inlineStr">
         <is>
-          <t>Diğer: 700 TL–4.000 TL</t>
+          <t>WU: 0,75 USD–12 USD; Diğer: 700 TL–4.000 TL</t>
         </is>
       </c>
       <c r="E12" s="14" t="inlineStr"/>
@@ -987,11 +987,7 @@
           <t>2.170 TL - 2.170 TL</t>
         </is>
       </c>
-      <c r="F14" s="14" t="inlineStr">
-        <is>
-          <t>2.785,72 TL - 12.380,95 TL</t>
-        </is>
-      </c>
+      <c r="F14" s="14" t="inlineStr"/>
       <c r="G14" s="14" t="inlineStr">
         <is>
           <t>8.300 TL - 7,97 TL</t>

</xml_diff>

<commit_message>
Update benchmark: 2026-03-28 07:07:47 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -987,7 +987,11 @@
           <t>2.170 TL - 2.170 TL</t>
         </is>
       </c>
-      <c r="F14" s="14" t="inlineStr"/>
+      <c r="F14" s="14" t="inlineStr">
+        <is>
+          <t>2.785,72 TL - 12.380,95 TL</t>
+        </is>
+      </c>
       <c r="G14" s="14" t="inlineStr">
         <is>
           <t>8.300 TL - 7,97 TL</t>

</xml_diff>

<commit_message>
Update benchmark: 2026-03-30 07:36:13 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -662,11 +662,7 @@
       <c r="D3" s="14" t="inlineStr"/>
       <c r="E3" s="14" t="inlineStr"/>
       <c r="F3" s="14" t="inlineStr"/>
-      <c r="G3" s="14" t="inlineStr">
-        <is>
-          <t>39,87 TRY - 79,76 TRY - 797,68 TRY</t>
-        </is>
-      </c>
+      <c r="G3" s="14" t="inlineStr"/>
       <c r="H3" s="14" t="inlineStr"/>
       <c r="I3" s="14" t="inlineStr"/>
       <c r="J3" s="14" t="inlineStr"/>
@@ -682,11 +678,7 @@
       <c r="D4" s="14" t="inlineStr"/>
       <c r="E4" s="14" t="inlineStr"/>
       <c r="F4" s="14" t="inlineStr"/>
-      <c r="G4" s="14" t="inlineStr">
-        <is>
-          <t>27,84 TRY - 55,69 TRY - 398,83 TRY</t>
-        </is>
-      </c>
+      <c r="G4" s="14" t="inlineStr"/>
       <c r="H4" s="14" t="inlineStr"/>
       <c r="I4" s="14" t="inlineStr"/>
       <c r="J4" s="14" t="inlineStr"/>
@@ -702,11 +694,7 @@
       <c r="D5" s="14" t="inlineStr"/>
       <c r="E5" s="14" t="inlineStr"/>
       <c r="F5" s="14" t="inlineStr"/>
-      <c r="G5" s="14" t="inlineStr">
-        <is>
-          <t>7,97 TRY - 15,96 TRY - 199,41 TRY</t>
-        </is>
-      </c>
+      <c r="G5" s="14" t="inlineStr"/>
       <c r="H5" s="14" t="inlineStr"/>
       <c r="I5" s="14" t="inlineStr"/>
       <c r="J5" s="14" t="inlineStr"/>
@@ -734,11 +722,7 @@
         </is>
       </c>
       <c r="F6" s="14" t="inlineStr"/>
-      <c r="G6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 99,71 TL</t>
-        </is>
-      </c>
+      <c r="G6" s="14" t="inlineStr"/>
       <c r="H6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
@@ -815,11 +799,7 @@
       <c r="D8" s="14" t="inlineStr"/>
       <c r="E8" s="14" t="inlineStr"/>
       <c r="F8" s="14" t="inlineStr"/>
-      <c r="G8" s="14" t="inlineStr">
-        <is>
-          <t>19,94 TRY - 39,88 TRY - 398,84 TRY</t>
-        </is>
-      </c>
+      <c r="G8" s="14" t="inlineStr"/>
       <c r="H8" s="14" t="inlineStr"/>
       <c r="I8" s="14" t="inlineStr"/>
       <c r="J8" s="14" t="inlineStr"/>
@@ -835,11 +815,7 @@
       <c r="D9" s="14" t="inlineStr"/>
       <c r="E9" s="14" t="inlineStr"/>
       <c r="F9" s="14" t="inlineStr"/>
-      <c r="G9" s="14" t="inlineStr">
-        <is>
-          <t>13,92 TRY - 27,85 TRY - 199,42 TRY</t>
-        </is>
-      </c>
+      <c r="G9" s="14" t="inlineStr"/>
       <c r="H9" s="14" t="inlineStr"/>
       <c r="I9" s="14" t="inlineStr"/>
       <c r="J9" s="14" t="inlineStr"/>
@@ -855,11 +831,7 @@
       <c r="D10" s="14" t="inlineStr"/>
       <c r="E10" s="14" t="inlineStr"/>
       <c r="F10" s="14" t="inlineStr"/>
-      <c r="G10" s="14" t="inlineStr">
-        <is>
-          <t>3,99 TRY - 7,98 TRY - 99,71 TRY</t>
-        </is>
-      </c>
+      <c r="G10" s="14" t="inlineStr"/>
       <c r="H10" s="14" t="inlineStr"/>
       <c r="I10" s="14" t="inlineStr"/>
       <c r="J10" s="14" t="inlineStr"/>
@@ -875,11 +847,7 @@
       <c r="D11" s="14" t="inlineStr"/>
       <c r="E11" s="14" t="inlineStr"/>
       <c r="F11" s="14" t="inlineStr"/>
-      <c r="G11" s="14" t="inlineStr">
-        <is>
-          <t>3,99 TRY - 7,98 TRY - 99,71 TRY</t>
-        </is>
-      </c>
+      <c r="G11" s="14" t="inlineStr"/>
       <c r="H11" s="14" t="inlineStr"/>
       <c r="I11" s="14" t="inlineStr"/>
       <c r="J11" s="14" t="inlineStr"/>
@@ -908,11 +876,7 @@
       </c>
       <c r="E12" s="14" t="inlineStr"/>
       <c r="F12" s="14" t="inlineStr"/>
-      <c r="G12" s="14" t="inlineStr">
-        <is>
-          <t>Şube (Kasadan): %0,5; Şube (Hesaptan): %0,75; İnternet: 15 USD</t>
-        </is>
-      </c>
+      <c r="G12" s="14" t="inlineStr"/>
       <c r="H12" s="14" t="inlineStr"/>
       <c r="I12" s="14" t="inlineStr"/>
       <c r="J12" s="14" t="inlineStr"/>
@@ -992,11 +956,7 @@
           <t>2.785,72 TL - 12.380,95 TL</t>
         </is>
       </c>
-      <c r="G14" s="14" t="inlineStr">
-        <is>
-          <t>8.300 TL - 7,97 TL</t>
-        </is>
-      </c>
+      <c r="G14" s="14" t="inlineStr"/>
       <c r="H14" s="14" t="inlineStr">
         <is>
           <t>3.000 TL - 6.000 TL</t>

</xml_diff>

<commit_message>
Update benchmark: 2026-03-31 07:24:01 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -662,7 +662,11 @@
       <c r="D3" s="14" t="inlineStr"/>
       <c r="E3" s="14" t="inlineStr"/>
       <c r="F3" s="14" t="inlineStr"/>
-      <c r="G3" s="14" t="inlineStr"/>
+      <c r="G3" s="14" t="inlineStr">
+        <is>
+          <t>39,87 TRY - 79,76 TRY - 797,68 TRY</t>
+        </is>
+      </c>
       <c r="H3" s="14" t="inlineStr"/>
       <c r="I3" s="14" t="inlineStr"/>
       <c r="J3" s="14" t="inlineStr"/>
@@ -678,7 +682,11 @@
       <c r="D4" s="14" t="inlineStr"/>
       <c r="E4" s="14" t="inlineStr"/>
       <c r="F4" s="14" t="inlineStr"/>
-      <c r="G4" s="14" t="inlineStr"/>
+      <c r="G4" s="14" t="inlineStr">
+        <is>
+          <t>27,84 TRY - 55,69 TRY - 398,83 TRY</t>
+        </is>
+      </c>
       <c r="H4" s="14" t="inlineStr"/>
       <c r="I4" s="14" t="inlineStr"/>
       <c r="J4" s="14" t="inlineStr"/>
@@ -694,7 +702,11 @@
       <c r="D5" s="14" t="inlineStr"/>
       <c r="E5" s="14" t="inlineStr"/>
       <c r="F5" s="14" t="inlineStr"/>
-      <c r="G5" s="14" t="inlineStr"/>
+      <c r="G5" s="14" t="inlineStr">
+        <is>
+          <t>7,97 TRY - 15,96 TRY - 199,41 TRY</t>
+        </is>
+      </c>
       <c r="H5" s="14" t="inlineStr"/>
       <c r="I5" s="14" t="inlineStr"/>
       <c r="J5" s="14" t="inlineStr"/>
@@ -711,18 +723,18 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="D6" s="14" t="inlineStr">
+      <c r="D6" s="14" t="inlineStr"/>
+      <c r="E6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="E6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 199,41 TL</t>
-        </is>
-      </c>
       <c r="F6" s="14" t="inlineStr"/>
-      <c r="G6" s="14" t="inlineStr"/>
+      <c r="G6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 99,71 TL</t>
+        </is>
+      </c>
       <c r="H6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
@@ -799,7 +811,11 @@
       <c r="D8" s="14" t="inlineStr"/>
       <c r="E8" s="14" t="inlineStr"/>
       <c r="F8" s="14" t="inlineStr"/>
-      <c r="G8" s="14" t="inlineStr"/>
+      <c r="G8" s="14" t="inlineStr">
+        <is>
+          <t>19,94 TRY - 39,88 TRY - 398,84 TRY</t>
+        </is>
+      </c>
       <c r="H8" s="14" t="inlineStr"/>
       <c r="I8" s="14" t="inlineStr"/>
       <c r="J8" s="14" t="inlineStr"/>
@@ -815,7 +831,11 @@
       <c r="D9" s="14" t="inlineStr"/>
       <c r="E9" s="14" t="inlineStr"/>
       <c r="F9" s="14" t="inlineStr"/>
-      <c r="G9" s="14" t="inlineStr"/>
+      <c r="G9" s="14" t="inlineStr">
+        <is>
+          <t>13,92 TRY - 27,85 TRY - 199,42 TRY</t>
+        </is>
+      </c>
       <c r="H9" s="14" t="inlineStr"/>
       <c r="I9" s="14" t="inlineStr"/>
       <c r="J9" s="14" t="inlineStr"/>
@@ -831,7 +851,11 @@
       <c r="D10" s="14" t="inlineStr"/>
       <c r="E10" s="14" t="inlineStr"/>
       <c r="F10" s="14" t="inlineStr"/>
-      <c r="G10" s="14" t="inlineStr"/>
+      <c r="G10" s="14" t="inlineStr">
+        <is>
+          <t>3,99 TRY - 7,98 TRY - 99,71 TRY</t>
+        </is>
+      </c>
       <c r="H10" s="14" t="inlineStr"/>
       <c r="I10" s="14" t="inlineStr"/>
       <c r="J10" s="14" t="inlineStr"/>
@@ -847,7 +871,11 @@
       <c r="D11" s="14" t="inlineStr"/>
       <c r="E11" s="14" t="inlineStr"/>
       <c r="F11" s="14" t="inlineStr"/>
-      <c r="G11" s="14" t="inlineStr"/>
+      <c r="G11" s="14" t="inlineStr">
+        <is>
+          <t>3,99 TRY - 7,98 TRY - 99,71 TRY</t>
+        </is>
+      </c>
       <c r="H11" s="14" t="inlineStr"/>
       <c r="I11" s="14" t="inlineStr"/>
       <c r="J11" s="14" t="inlineStr"/>
@@ -869,14 +897,14 @@
           <t>WU: 1.000,01 USD–9,51 USD</t>
         </is>
       </c>
-      <c r="D12" s="14" t="inlineStr">
-        <is>
-          <t>WU: 0,75 USD–12 USD; Diğer: 700 TL–4.000 TL</t>
-        </is>
-      </c>
+      <c r="D12" s="14" t="inlineStr"/>
       <c r="E12" s="14" t="inlineStr"/>
       <c r="F12" s="14" t="inlineStr"/>
-      <c r="G12" s="14" t="inlineStr"/>
+      <c r="G12" s="14" t="inlineStr">
+        <is>
+          <t>Şube (Kasadan): %0,5; Şube (Hesaptan): %0,75; İnternet: 15 USD</t>
+        </is>
+      </c>
       <c r="H12" s="14" t="inlineStr"/>
       <c r="I12" s="14" t="inlineStr"/>
       <c r="J12" s="14" t="inlineStr"/>
@@ -897,11 +925,7 @@
           <t>Hesaba: Asgari 0 TL | Azami 0,94 TL</t>
         </is>
       </c>
-      <c r="D13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
-        </is>
-      </c>
+      <c r="D13" s="14" t="inlineStr"/>
       <c r="E13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
@@ -941,11 +965,7 @@
           <t>40.000 TL - 2.485,72 TL</t>
         </is>
       </c>
-      <c r="D14" s="14" t="inlineStr">
-        <is>
-          <t>3.500 TL - 13.500 TL</t>
-        </is>
-      </c>
+      <c r="D14" s="14" t="inlineStr"/>
       <c r="E14" s="14" t="inlineStr">
         <is>
           <t>2.170 TL - 2.170 TL</t>
@@ -956,7 +976,11 @@
           <t>2.785,72 TL - 12.380,95 TL</t>
         </is>
       </c>
-      <c r="G14" s="14" t="inlineStr"/>
+      <c r="G14" s="14" t="inlineStr">
+        <is>
+          <t>8.300 TL - 7,97 TL</t>
+        </is>
+      </c>
       <c r="H14" s="14" t="inlineStr">
         <is>
           <t>3.000 TL - 6.000 TL</t>

</xml_diff>

<commit_message>
Update benchmark: 2026-04-01 07:29:03 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -718,11 +718,7 @@
           <t>DÜZENLİ EFT</t>
         </is>
       </c>
-      <c r="C6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 199,41 TL</t>
-        </is>
-      </c>
+      <c r="C6" s="14" t="inlineStr"/>
       <c r="D6" s="14" t="inlineStr"/>
       <c r="E6" s="14" t="inlineStr">
         <is>
@@ -735,11 +731,7 @@
           <t>8.300,01 TL - 99,71 TL</t>
         </is>
       </c>
-      <c r="H6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 199,41 TL</t>
-        </is>
-      </c>
+      <c r="H6" s="14" t="inlineStr"/>
       <c r="I6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
@@ -892,11 +884,7 @@
           <t>GİDEN SWIFT</t>
         </is>
       </c>
-      <c r="C12" s="14" t="inlineStr">
-        <is>
-          <t>WU: 1.000,01 USD–9,51 USD</t>
-        </is>
-      </c>
+      <c r="C12" s="14" t="inlineStr"/>
       <c r="D12" s="14" t="inlineStr"/>
       <c r="E12" s="14" t="inlineStr"/>
       <c r="F12" s="14" t="inlineStr"/>
@@ -920,11 +908,7 @@
           <t>GELEN SWIFT</t>
         </is>
       </c>
-      <c r="C13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 0 TL | Azami 0,94 TL</t>
-        </is>
-      </c>
+      <c r="C13" s="14" t="inlineStr"/>
       <c r="D13" s="14" t="inlineStr"/>
       <c r="E13" s="14" t="inlineStr">
         <is>
@@ -933,11 +917,7 @@
       </c>
       <c r="F13" s="14" t="inlineStr"/>
       <c r="G13" s="14" t="inlineStr"/>
-      <c r="H13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
-        </is>
-      </c>
+      <c r="H13" s="14" t="inlineStr"/>
       <c r="I13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
@@ -960,11 +940,7 @@
           <t>GİDEN SWIFT - Mobil</t>
         </is>
       </c>
-      <c r="C14" s="14" t="inlineStr">
-        <is>
-          <t>40.000 TL - 2.485,72 TL</t>
-        </is>
-      </c>
+      <c r="C14" s="14" t="inlineStr"/>
       <c r="D14" s="14" t="inlineStr"/>
       <c r="E14" s="14" t="inlineStr">
         <is>
@@ -981,11 +957,7 @@
           <t>8.300 TL - 7,97 TL</t>
         </is>
       </c>
-      <c r="H14" s="14" t="inlineStr">
-        <is>
-          <t>3.000 TL - 6.000 TL</t>
-        </is>
-      </c>
+      <c r="H14" s="14" t="inlineStr"/>
       <c r="I14" s="14" t="inlineStr"/>
       <c r="J14" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update benchmark: 2026-04-02 07:22:41 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -616,11 +616,7 @@
           <t>26 TL - 26 TL</t>
         </is>
       </c>
-      <c r="F2" s="14" t="inlineStr">
-        <is>
-          <t>33,33 TL - 33,33 TL</t>
-        </is>
-      </c>
+      <c r="F2" s="14" t="inlineStr"/>
       <c r="G2" s="14" t="inlineStr">
         <is>
           <t>15 TL - 15 TL</t>
@@ -718,8 +714,16 @@
           <t>DÜZENLİ EFT</t>
         </is>
       </c>
-      <c r="C6" s="14" t="inlineStr"/>
-      <c r="D6" s="14" t="inlineStr"/>
+      <c r="C6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 199,41 TL</t>
+        </is>
+      </c>
+      <c r="D6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 199,41 TL</t>
+        </is>
+      </c>
       <c r="E6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
@@ -731,7 +735,11 @@
           <t>8.300,01 TL - 99,71 TL</t>
         </is>
       </c>
-      <c r="H6" s="14" t="inlineStr"/>
+      <c r="H6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 199,41 TL</t>
+        </is>
+      </c>
       <c r="I6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
@@ -761,11 +769,7 @@
         </is>
       </c>
       <c r="E7" s="14" t="inlineStr"/>
-      <c r="F7" s="14" t="inlineStr">
-        <is>
-          <t>%3</t>
-        </is>
-      </c>
+      <c r="F7" s="14" t="inlineStr"/>
       <c r="G7" s="14" t="inlineStr">
         <is>
           <t>1 TRY (Kredi kartı ile ödemelerde ek olarak nakit avans faizi uygulanır.)</t>
@@ -884,8 +888,16 @@
           <t>GİDEN SWIFT</t>
         </is>
       </c>
-      <c r="C12" s="14" t="inlineStr"/>
-      <c r="D12" s="14" t="inlineStr"/>
+      <c r="C12" s="14" t="inlineStr">
+        <is>
+          <t>WU: 1.000,01 USD–9,51 USD</t>
+        </is>
+      </c>
+      <c r="D12" s="14" t="inlineStr">
+        <is>
+          <t>WU: 0,75 USD–12 USD; Diğer: 700 TL–4.000 TL</t>
+        </is>
+      </c>
       <c r="E12" s="14" t="inlineStr"/>
       <c r="F12" s="14" t="inlineStr"/>
       <c r="G12" s="14" t="inlineStr">
@@ -908,8 +920,16 @@
           <t>GELEN SWIFT</t>
         </is>
       </c>
-      <c r="C13" s="14" t="inlineStr"/>
-      <c r="D13" s="14" t="inlineStr"/>
+      <c r="C13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 0 TL | Azami 0,94 TL</t>
+        </is>
+      </c>
+      <c r="D13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
+        </is>
+      </c>
       <c r="E13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
@@ -917,7 +937,11 @@
       </c>
       <c r="F13" s="14" t="inlineStr"/>
       <c r="G13" s="14" t="inlineStr"/>
-      <c r="H13" s="14" t="inlineStr"/>
+      <c r="H13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
+        </is>
+      </c>
       <c r="I13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
@@ -940,8 +964,16 @@
           <t>GİDEN SWIFT - Mobil</t>
         </is>
       </c>
-      <c r="C14" s="14" t="inlineStr"/>
-      <c r="D14" s="14" t="inlineStr"/>
+      <c r="C14" s="14" t="inlineStr">
+        <is>
+          <t>40.000 TL - 2.485,72 TL</t>
+        </is>
+      </c>
+      <c r="D14" s="14" t="inlineStr">
+        <is>
+          <t>3.500 TL - 13.500 TL</t>
+        </is>
+      </c>
       <c r="E14" s="14" t="inlineStr">
         <is>
           <t>2.170 TL - 2.170 TL</t>
@@ -957,7 +989,11 @@
           <t>8.300 TL - 7,97 TL</t>
         </is>
       </c>
-      <c r="H14" s="14" t="inlineStr"/>
+      <c r="H14" s="14" t="inlineStr">
+        <is>
+          <t>3.000 TL - 6.000 TL</t>
+        </is>
+      </c>
       <c r="I14" s="14" t="inlineStr"/>
       <c r="J14" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update benchmark: 2026-04-03 07:21:23 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -616,7 +616,11 @@
           <t>26 TL - 26 TL</t>
         </is>
       </c>
-      <c r="F2" s="14" t="inlineStr"/>
+      <c r="F2" s="14" t="inlineStr">
+        <is>
+          <t>33,33 TL - 33,33 TL</t>
+        </is>
+      </c>
       <c r="G2" s="14" t="inlineStr">
         <is>
           <t>15 TL - 15 TL</t>
@@ -769,7 +773,11 @@
         </is>
       </c>
       <c r="E7" s="14" t="inlineStr"/>
-      <c r="F7" s="14" t="inlineStr"/>
+      <c r="F7" s="14" t="inlineStr">
+        <is>
+          <t>%3</t>
+        </is>
+      </c>
       <c r="G7" s="14" t="inlineStr">
         <is>
           <t>1 TRY (Kredi kartı ile ödemelerde ek olarak nakit avans faizi uygulanır.)</t>

</xml_diff>

<commit_message>
Update benchmark: 2026-04-04 07:09:30 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -754,11 +754,7 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="K6" s="14" t="inlineStr">
-        <is>
-          <t>7,97 TL - 15,96 TL - 199,41 TL</t>
-        </is>
-      </c>
+      <c r="K6" s="14" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="B7" s="13" t="inlineStr">
@@ -916,11 +912,7 @@
       <c r="H12" s="14" t="inlineStr"/>
       <c r="I12" s="14" t="inlineStr"/>
       <c r="J12" s="14" t="inlineStr"/>
-      <c r="K12" s="14" t="inlineStr">
-        <is>
-          <t>WU: ,USD–; Diğer: 529 TL–4.454,74 TL</t>
-        </is>
-      </c>
+      <c r="K12" s="14" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="B13" s="13" t="inlineStr">
@@ -960,11 +952,7 @@
           <t>Hesaba: Asgari 1 TL | Azami 1.303 TL</t>
         </is>
       </c>
-      <c r="K13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 865,75 TL</t>
-        </is>
-      </c>
+      <c r="K13" s="14" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="B14" s="13" t="inlineStr">
@@ -1008,11 +996,7 @@
           <t>1.554,97 TL - 7.784 TL</t>
         </is>
       </c>
-      <c r="K14" s="14" t="inlineStr">
-        <is>
-          <t>1.196,51 TL - 5.583,74 TL</t>
-        </is>
-      </c>
+      <c r="K14" s="14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="12" t="inlineStr">

</xml_diff>

<commit_message>
Update benchmark: 2026-04-05 07:16:14 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -723,11 +723,7 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="D6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 199,41 TL</t>
-        </is>
-      </c>
+      <c r="D6" s="14" t="inlineStr"/>
       <c r="E6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
@@ -754,7 +750,11 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="K6" s="14" t="inlineStr"/>
+      <c r="K6" s="14" t="inlineStr">
+        <is>
+          <t>7,97 TL - 15,96 TL - 199,41 TL</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="B7" s="13" t="inlineStr">
@@ -897,11 +897,7 @@
           <t>WU: 1.000,01 USD–9,51 USD</t>
         </is>
       </c>
-      <c r="D12" s="14" t="inlineStr">
-        <is>
-          <t>WU: 0,75 USD–12 USD; Diğer: 700 TL–4.000 TL</t>
-        </is>
-      </c>
+      <c r="D12" s="14" t="inlineStr"/>
       <c r="E12" s="14" t="inlineStr"/>
       <c r="F12" s="14" t="inlineStr"/>
       <c r="G12" s="14" t="inlineStr">
@@ -912,7 +908,11 @@
       <c r="H12" s="14" t="inlineStr"/>
       <c r="I12" s="14" t="inlineStr"/>
       <c r="J12" s="14" t="inlineStr"/>
-      <c r="K12" s="14" t="inlineStr"/>
+      <c r="K12" s="14" t="inlineStr">
+        <is>
+          <t>WU: ,USD–; Diğer: 529 TL–4.454,74 TL</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="B13" s="13" t="inlineStr">
@@ -925,11 +925,7 @@
           <t>Hesaba: Asgari 0 TL | Azami 0,94 TL</t>
         </is>
       </c>
-      <c r="D13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
-        </is>
-      </c>
+      <c r="D13" s="14" t="inlineStr"/>
       <c r="E13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
@@ -952,7 +948,11 @@
           <t>Hesaba: Asgari 1 TL | Azami 1.303 TL</t>
         </is>
       </c>
-      <c r="K13" s="14" t="inlineStr"/>
+      <c r="K13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 865,75 TL</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="B14" s="13" t="inlineStr">
@@ -965,11 +965,7 @@
           <t>40.000 TL - 2.485,72 TL</t>
         </is>
       </c>
-      <c r="D14" s="14" t="inlineStr">
-        <is>
-          <t>3.500 TL - 13.500 TL</t>
-        </is>
-      </c>
+      <c r="D14" s="14" t="inlineStr"/>
       <c r="E14" s="14" t="inlineStr">
         <is>
           <t>2.170 TL - 2.170 TL</t>
@@ -996,7 +992,11 @@
           <t>1.554,97 TL - 7.784 TL</t>
         </is>
       </c>
-      <c r="K14" s="14" t="inlineStr"/>
+      <c r="K14" s="14" t="inlineStr">
+        <is>
+          <t>1.196,51 TL - 5.583,74 TL</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="12" t="inlineStr">

</xml_diff>

<commit_message>
Update benchmark: 2026-04-06 07:51:32 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -740,11 +740,7 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="I6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 199,41 TL</t>
-        </is>
-      </c>
+      <c r="I6" s="14" t="inlineStr"/>
       <c r="J6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
@@ -938,11 +934,7 @@
           <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
         </is>
       </c>
-      <c r="I13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
-        </is>
-      </c>
+      <c r="I13" s="14" t="inlineStr"/>
       <c r="J13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.303 TL</t>
@@ -971,11 +963,7 @@
           <t>2.170 TL - 2.170 TL</t>
         </is>
       </c>
-      <c r="F14" s="14" t="inlineStr">
-        <is>
-          <t>2.785,72 TL - 12.380,95 TL</t>
-        </is>
-      </c>
+      <c r="F14" s="14" t="inlineStr"/>
       <c r="G14" s="14" t="inlineStr">
         <is>
           <t>8.300 TL - 7,97 TL</t>

</xml_diff>

<commit_message>
Update benchmark: 2026-04-07 07:25:56 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -662,11 +662,7 @@
       <c r="D3" s="14" t="inlineStr"/>
       <c r="E3" s="14" t="inlineStr"/>
       <c r="F3" s="14" t="inlineStr"/>
-      <c r="G3" s="14" t="inlineStr">
-        <is>
-          <t>39,87 TRY - 79,76 TRY - 797,68 TRY</t>
-        </is>
-      </c>
+      <c r="G3" s="14" t="inlineStr"/>
       <c r="H3" s="14" t="inlineStr"/>
       <c r="I3" s="14" t="inlineStr"/>
       <c r="J3" s="14" t="inlineStr"/>
@@ -682,11 +678,7 @@
       <c r="D4" s="14" t="inlineStr"/>
       <c r="E4" s="14" t="inlineStr"/>
       <c r="F4" s="14" t="inlineStr"/>
-      <c r="G4" s="14" t="inlineStr">
-        <is>
-          <t>27,84 TRY - 55,69 TRY - 398,83 TRY</t>
-        </is>
-      </c>
+      <c r="G4" s="14" t="inlineStr"/>
       <c r="H4" s="14" t="inlineStr"/>
       <c r="I4" s="14" t="inlineStr"/>
       <c r="J4" s="14" t="inlineStr"/>
@@ -702,11 +694,7 @@
       <c r="D5" s="14" t="inlineStr"/>
       <c r="E5" s="14" t="inlineStr"/>
       <c r="F5" s="14" t="inlineStr"/>
-      <c r="G5" s="14" t="inlineStr">
-        <is>
-          <t>7,97 TRY - 15,96 TRY - 199,41 TRY</t>
-        </is>
-      </c>
+      <c r="G5" s="14" t="inlineStr"/>
       <c r="H5" s="14" t="inlineStr"/>
       <c r="I5" s="14" t="inlineStr"/>
       <c r="J5" s="14" t="inlineStr"/>
@@ -718,39 +706,23 @@
           <t>DÜZENLİ EFT</t>
         </is>
       </c>
-      <c r="C6" s="14" t="inlineStr">
+      <c r="C6" s="14" t="inlineStr"/>
+      <c r="D6" s="14" t="inlineStr"/>
+      <c r="E6" s="14" t="inlineStr"/>
+      <c r="F6" s="14" t="inlineStr"/>
+      <c r="G6" s="14" t="inlineStr"/>
+      <c r="H6" s="14" t="inlineStr"/>
+      <c r="I6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="D6" s="14" t="inlineStr"/>
-      <c r="E6" s="14" t="inlineStr">
+      <c r="J6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="F6" s="14" t="inlineStr"/>
-      <c r="G6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 99,71 TL</t>
-        </is>
-      </c>
-      <c r="H6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 199,41 TL</t>
-        </is>
-      </c>
-      <c r="I6" s="14" t="inlineStr"/>
-      <c r="J6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 199,41 TL</t>
-        </is>
-      </c>
-      <c r="K6" s="14" t="inlineStr">
-        <is>
-          <t>7,97 TL - 15,96 TL - 199,41 TL</t>
-        </is>
-      </c>
+      <c r="K6" s="14" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="B7" s="13" t="inlineStr">
@@ -807,11 +779,7 @@
       <c r="D8" s="14" t="inlineStr"/>
       <c r="E8" s="14" t="inlineStr"/>
       <c r="F8" s="14" t="inlineStr"/>
-      <c r="G8" s="14" t="inlineStr">
-        <is>
-          <t>19,94 TRY - 39,88 TRY - 398,84 TRY</t>
-        </is>
-      </c>
+      <c r="G8" s="14" t="inlineStr"/>
       <c r="H8" s="14" t="inlineStr"/>
       <c r="I8" s="14" t="inlineStr"/>
       <c r="J8" s="14" t="inlineStr"/>
@@ -827,11 +795,7 @@
       <c r="D9" s="14" t="inlineStr"/>
       <c r="E9" s="14" t="inlineStr"/>
       <c r="F9" s="14" t="inlineStr"/>
-      <c r="G9" s="14" t="inlineStr">
-        <is>
-          <t>13,92 TRY - 27,85 TRY - 199,42 TRY</t>
-        </is>
-      </c>
+      <c r="G9" s="14" t="inlineStr"/>
       <c r="H9" s="14" t="inlineStr"/>
       <c r="I9" s="14" t="inlineStr"/>
       <c r="J9" s="14" t="inlineStr"/>
@@ -847,11 +811,7 @@
       <c r="D10" s="14" t="inlineStr"/>
       <c r="E10" s="14" t="inlineStr"/>
       <c r="F10" s="14" t="inlineStr"/>
-      <c r="G10" s="14" t="inlineStr">
-        <is>
-          <t>3,99 TRY - 7,98 TRY - 99,71 TRY</t>
-        </is>
-      </c>
+      <c r="G10" s="14" t="inlineStr"/>
       <c r="H10" s="14" t="inlineStr"/>
       <c r="I10" s="14" t="inlineStr"/>
       <c r="J10" s="14" t="inlineStr"/>
@@ -867,11 +827,7 @@
       <c r="D11" s="14" t="inlineStr"/>
       <c r="E11" s="14" t="inlineStr"/>
       <c r="F11" s="14" t="inlineStr"/>
-      <c r="G11" s="14" t="inlineStr">
-        <is>
-          <t>3,99 TRY - 7,98 TRY - 99,71 TRY</t>
-        </is>
-      </c>
+      <c r="G11" s="14" t="inlineStr"/>
       <c r="H11" s="14" t="inlineStr"/>
       <c r="I11" s="14" t="inlineStr"/>
       <c r="J11" s="14" t="inlineStr"/>
@@ -888,27 +844,15 @@
           <t>GİDEN SWIFT</t>
         </is>
       </c>
-      <c r="C12" s="14" t="inlineStr">
-        <is>
-          <t>WU: 1.000,01 USD–9,51 USD</t>
-        </is>
-      </c>
+      <c r="C12" s="14" t="inlineStr"/>
       <c r="D12" s="14" t="inlineStr"/>
       <c r="E12" s="14" t="inlineStr"/>
       <c r="F12" s="14" t="inlineStr"/>
-      <c r="G12" s="14" t="inlineStr">
-        <is>
-          <t>Şube (Kasadan): %0,5; Şube (Hesaptan): %0,75; İnternet: 15 USD</t>
-        </is>
-      </c>
+      <c r="G12" s="14" t="inlineStr"/>
       <c r="H12" s="14" t="inlineStr"/>
       <c r="I12" s="14" t="inlineStr"/>
       <c r="J12" s="14" t="inlineStr"/>
-      <c r="K12" s="14" t="inlineStr">
-        <is>
-          <t>WU: ,USD–; Diğer: 529 TL–4.454,74 TL</t>
-        </is>
-      </c>
+      <c r="K12" s="14" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="B13" s="13" t="inlineStr">
@@ -916,35 +860,23 @@
           <t>GELEN SWIFT</t>
         </is>
       </c>
-      <c r="C13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 0 TL | Azami 0,94 TL</t>
-        </is>
-      </c>
+      <c r="C13" s="14" t="inlineStr"/>
       <c r="D13" s="14" t="inlineStr"/>
-      <c r="E13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
-        </is>
-      </c>
+      <c r="E13" s="14" t="inlineStr"/>
       <c r="F13" s="14" t="inlineStr"/>
       <c r="G13" s="14" t="inlineStr"/>
-      <c r="H13" s="14" t="inlineStr">
+      <c r="H13" s="14" t="inlineStr"/>
+      <c r="I13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
         </is>
       </c>
-      <c r="I13" s="14" t="inlineStr"/>
       <c r="J13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.303 TL</t>
         </is>
       </c>
-      <c r="K13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 865,75 TL</t>
-        </is>
-      </c>
+      <c r="K13" s="14" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="B14" s="13" t="inlineStr">
@@ -952,39 +884,19 @@
           <t>GİDEN SWIFT - Mobil</t>
         </is>
       </c>
-      <c r="C14" s="14" t="inlineStr">
-        <is>
-          <t>40.000 TL - 2.485,72 TL</t>
-        </is>
-      </c>
+      <c r="C14" s="14" t="inlineStr"/>
       <c r="D14" s="14" t="inlineStr"/>
-      <c r="E14" s="14" t="inlineStr">
-        <is>
-          <t>2.170 TL - 2.170 TL</t>
-        </is>
-      </c>
+      <c r="E14" s="14" t="inlineStr"/>
       <c r="F14" s="14" t="inlineStr"/>
-      <c r="G14" s="14" t="inlineStr">
-        <is>
-          <t>8.300 TL - 7,97 TL</t>
-        </is>
-      </c>
-      <c r="H14" s="14" t="inlineStr">
-        <is>
-          <t>3.000 TL - 6.000 TL</t>
-        </is>
-      </c>
+      <c r="G14" s="14" t="inlineStr"/>
+      <c r="H14" s="14" t="inlineStr"/>
       <c r="I14" s="14" t="inlineStr"/>
       <c r="J14" s="14" t="inlineStr">
         <is>
           <t>1.554,97 TL - 7.784 TL</t>
         </is>
       </c>
-      <c r="K14" s="14" t="inlineStr">
-        <is>
-          <t>1.196,51 TL - 5.583,74 TL</t>
-        </is>
-      </c>
+      <c r="K14" s="14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="12" t="inlineStr">

</xml_diff>

<commit_message>
Update benchmark: 2026-04-08 07:26:46 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -662,7 +662,11 @@
       <c r="D3" s="14" t="inlineStr"/>
       <c r="E3" s="14" t="inlineStr"/>
       <c r="F3" s="14" t="inlineStr"/>
-      <c r="G3" s="14" t="inlineStr"/>
+      <c r="G3" s="14" t="inlineStr">
+        <is>
+          <t>39,87 TRY - 79,76 TRY - 797,68 TRY</t>
+        </is>
+      </c>
       <c r="H3" s="14" t="inlineStr"/>
       <c r="I3" s="14" t="inlineStr"/>
       <c r="J3" s="14" t="inlineStr"/>
@@ -678,7 +682,11 @@
       <c r="D4" s="14" t="inlineStr"/>
       <c r="E4" s="14" t="inlineStr"/>
       <c r="F4" s="14" t="inlineStr"/>
-      <c r="G4" s="14" t="inlineStr"/>
+      <c r="G4" s="14" t="inlineStr">
+        <is>
+          <t>27,84 TRY - 55,69 TRY - 398,83 TRY</t>
+        </is>
+      </c>
       <c r="H4" s="14" t="inlineStr"/>
       <c r="I4" s="14" t="inlineStr"/>
       <c r="J4" s="14" t="inlineStr"/>
@@ -694,7 +702,11 @@
       <c r="D5" s="14" t="inlineStr"/>
       <c r="E5" s="14" t="inlineStr"/>
       <c r="F5" s="14" t="inlineStr"/>
-      <c r="G5" s="14" t="inlineStr"/>
+      <c r="G5" s="14" t="inlineStr">
+        <is>
+          <t>7,97 TRY - 15,96 TRY - 199,41 TRY</t>
+        </is>
+      </c>
       <c r="H5" s="14" t="inlineStr"/>
       <c r="I5" s="14" t="inlineStr"/>
       <c r="J5" s="14" t="inlineStr"/>
@@ -706,22 +718,34 @@
           <t>DÜZENLİ EFT</t>
         </is>
       </c>
-      <c r="C6" s="14" t="inlineStr"/>
+      <c r="C6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 199,41 TL</t>
+        </is>
+      </c>
       <c r="D6" s="14" t="inlineStr"/>
-      <c r="E6" s="14" t="inlineStr"/>
+      <c r="E6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 199,41 TL</t>
+        </is>
+      </c>
       <c r="F6" s="14" t="inlineStr"/>
-      <c r="G6" s="14" t="inlineStr"/>
-      <c r="H6" s="14" t="inlineStr"/>
+      <c r="G6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 99,71 TL</t>
+        </is>
+      </c>
+      <c r="H6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 199,41 TL</t>
+        </is>
+      </c>
       <c r="I6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="J6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 199,41 TL</t>
-        </is>
-      </c>
+      <c r="J6" s="14" t="inlineStr"/>
       <c r="K6" s="14" t="inlineStr"/>
     </row>
     <row r="7">
@@ -779,7 +803,11 @@
       <c r="D8" s="14" t="inlineStr"/>
       <c r="E8" s="14" t="inlineStr"/>
       <c r="F8" s="14" t="inlineStr"/>
-      <c r="G8" s="14" t="inlineStr"/>
+      <c r="G8" s="14" t="inlineStr">
+        <is>
+          <t>19,94 TRY - 39,88 TRY - 398,84 TRY</t>
+        </is>
+      </c>
       <c r="H8" s="14" t="inlineStr"/>
       <c r="I8" s="14" t="inlineStr"/>
       <c r="J8" s="14" t="inlineStr"/>
@@ -795,7 +823,11 @@
       <c r="D9" s="14" t="inlineStr"/>
       <c r="E9" s="14" t="inlineStr"/>
       <c r="F9" s="14" t="inlineStr"/>
-      <c r="G9" s="14" t="inlineStr"/>
+      <c r="G9" s="14" t="inlineStr">
+        <is>
+          <t>13,92 TRY - 27,85 TRY - 199,42 TRY</t>
+        </is>
+      </c>
       <c r="H9" s="14" t="inlineStr"/>
       <c r="I9" s="14" t="inlineStr"/>
       <c r="J9" s="14" t="inlineStr"/>
@@ -811,7 +843,11 @@
       <c r="D10" s="14" t="inlineStr"/>
       <c r="E10" s="14" t="inlineStr"/>
       <c r="F10" s="14" t="inlineStr"/>
-      <c r="G10" s="14" t="inlineStr"/>
+      <c r="G10" s="14" t="inlineStr">
+        <is>
+          <t>3,99 TRY - 7,98 TRY - 99,71 TRY</t>
+        </is>
+      </c>
       <c r="H10" s="14" t="inlineStr"/>
       <c r="I10" s="14" t="inlineStr"/>
       <c r="J10" s="14" t="inlineStr"/>
@@ -827,7 +863,11 @@
       <c r="D11" s="14" t="inlineStr"/>
       <c r="E11" s="14" t="inlineStr"/>
       <c r="F11" s="14" t="inlineStr"/>
-      <c r="G11" s="14" t="inlineStr"/>
+      <c r="G11" s="14" t="inlineStr">
+        <is>
+          <t>3,99 TRY - 7,98 TRY - 99,71 TRY</t>
+        </is>
+      </c>
       <c r="H11" s="14" t="inlineStr"/>
       <c r="I11" s="14" t="inlineStr"/>
       <c r="J11" s="14" t="inlineStr"/>
@@ -844,11 +884,19 @@
           <t>GİDEN SWIFT</t>
         </is>
       </c>
-      <c r="C12" s="14" t="inlineStr"/>
+      <c r="C12" s="14" t="inlineStr">
+        <is>
+          <t>WU: 1.000,01 USD–9,51 USD</t>
+        </is>
+      </c>
       <c r="D12" s="14" t="inlineStr"/>
       <c r="E12" s="14" t="inlineStr"/>
       <c r="F12" s="14" t="inlineStr"/>
-      <c r="G12" s="14" t="inlineStr"/>
+      <c r="G12" s="14" t="inlineStr">
+        <is>
+          <t>Şube (Kasadan): %0,5; Şube (Hesaptan): %0,75; İnternet: 15 USD</t>
+        </is>
+      </c>
       <c r="H12" s="14" t="inlineStr"/>
       <c r="I12" s="14" t="inlineStr"/>
       <c r="J12" s="14" t="inlineStr"/>
@@ -860,22 +908,30 @@
           <t>GELEN SWIFT</t>
         </is>
       </c>
-      <c r="C13" s="14" t="inlineStr"/>
+      <c r="C13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 0 TL | Azami 0,94 TL</t>
+        </is>
+      </c>
       <c r="D13" s="14" t="inlineStr"/>
-      <c r="E13" s="14" t="inlineStr"/>
+      <c r="E13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
+        </is>
+      </c>
       <c r="F13" s="14" t="inlineStr"/>
       <c r="G13" s="14" t="inlineStr"/>
-      <c r="H13" s="14" t="inlineStr"/>
+      <c r="H13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
+        </is>
+      </c>
       <c r="I13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
         </is>
       </c>
-      <c r="J13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 1.303 TL</t>
-        </is>
-      </c>
+      <c r="J13" s="14" t="inlineStr"/>
       <c r="K13" s="14" t="inlineStr"/>
     </row>
     <row r="14">
@@ -884,18 +940,30 @@
           <t>GİDEN SWIFT - Mobil</t>
         </is>
       </c>
-      <c r="C14" s="14" t="inlineStr"/>
+      <c r="C14" s="14" t="inlineStr">
+        <is>
+          <t>40.000 TL - 2.485,72 TL</t>
+        </is>
+      </c>
       <c r="D14" s="14" t="inlineStr"/>
-      <c r="E14" s="14" t="inlineStr"/>
+      <c r="E14" s="14" t="inlineStr">
+        <is>
+          <t>2.170 TL - 2.170 TL</t>
+        </is>
+      </c>
       <c r="F14" s="14" t="inlineStr"/>
-      <c r="G14" s="14" t="inlineStr"/>
-      <c r="H14" s="14" t="inlineStr"/>
+      <c r="G14" s="14" t="inlineStr">
+        <is>
+          <t>8.300 TL - 7,97 TL</t>
+        </is>
+      </c>
+      <c r="H14" s="14" t="inlineStr">
+        <is>
+          <t>3.000 TL - 6.000 TL</t>
+        </is>
+      </c>
       <c r="I14" s="14" t="inlineStr"/>
-      <c r="J14" s="14" t="inlineStr">
-        <is>
-          <t>1.554,97 TL - 7.784 TL</t>
-        </is>
-      </c>
+      <c r="J14" s="14" t="inlineStr"/>
       <c r="K14" s="14" t="inlineStr"/>
     </row>
     <row r="15">

</xml_diff>

<commit_message>
Update benchmark: 2026-04-09 07:31:18 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -662,11 +662,7 @@
       <c r="D3" s="14" t="inlineStr"/>
       <c r="E3" s="14" t="inlineStr"/>
       <c r="F3" s="14" t="inlineStr"/>
-      <c r="G3" s="14" t="inlineStr">
-        <is>
-          <t>39,87 TRY - 79,76 TRY - 797,68 TRY</t>
-        </is>
-      </c>
+      <c r="G3" s="14" t="inlineStr"/>
       <c r="H3" s="14" t="inlineStr"/>
       <c r="I3" s="14" t="inlineStr"/>
       <c r="J3" s="14" t="inlineStr"/>
@@ -682,11 +678,7 @@
       <c r="D4" s="14" t="inlineStr"/>
       <c r="E4" s="14" t="inlineStr"/>
       <c r="F4" s="14" t="inlineStr"/>
-      <c r="G4" s="14" t="inlineStr">
-        <is>
-          <t>27,84 TRY - 55,69 TRY - 398,83 TRY</t>
-        </is>
-      </c>
+      <c r="G4" s="14" t="inlineStr"/>
       <c r="H4" s="14" t="inlineStr"/>
       <c r="I4" s="14" t="inlineStr"/>
       <c r="J4" s="14" t="inlineStr"/>
@@ -702,11 +694,7 @@
       <c r="D5" s="14" t="inlineStr"/>
       <c r="E5" s="14" t="inlineStr"/>
       <c r="F5" s="14" t="inlineStr"/>
-      <c r="G5" s="14" t="inlineStr">
-        <is>
-          <t>7,97 TRY - 15,96 TRY - 199,41 TRY</t>
-        </is>
-      </c>
+      <c r="G5" s="14" t="inlineStr"/>
       <c r="H5" s="14" t="inlineStr"/>
       <c r="I5" s="14" t="inlineStr"/>
       <c r="J5" s="14" t="inlineStr"/>
@@ -730,11 +718,7 @@
         </is>
       </c>
       <c r="F6" s="14" t="inlineStr"/>
-      <c r="G6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 99,71 TL</t>
-        </is>
-      </c>
+      <c r="G6" s="14" t="inlineStr"/>
       <c r="H6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
@@ -745,8 +729,16 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="J6" s="14" t="inlineStr"/>
-      <c r="K6" s="14" t="inlineStr"/>
+      <c r="J6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 199,41 TL</t>
+        </is>
+      </c>
+      <c r="K6" s="14" t="inlineStr">
+        <is>
+          <t>7,97 TL - 15,96 TL - 199,41 TL</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="B7" s="13" t="inlineStr">
@@ -803,11 +795,7 @@
       <c r="D8" s="14" t="inlineStr"/>
       <c r="E8" s="14" t="inlineStr"/>
       <c r="F8" s="14" t="inlineStr"/>
-      <c r="G8" s="14" t="inlineStr">
-        <is>
-          <t>19,94 TRY - 39,88 TRY - 398,84 TRY</t>
-        </is>
-      </c>
+      <c r="G8" s="14" t="inlineStr"/>
       <c r="H8" s="14" t="inlineStr"/>
       <c r="I8" s="14" t="inlineStr"/>
       <c r="J8" s="14" t="inlineStr"/>
@@ -823,11 +811,7 @@
       <c r="D9" s="14" t="inlineStr"/>
       <c r="E9" s="14" t="inlineStr"/>
       <c r="F9" s="14" t="inlineStr"/>
-      <c r="G9" s="14" t="inlineStr">
-        <is>
-          <t>13,92 TRY - 27,85 TRY - 199,42 TRY</t>
-        </is>
-      </c>
+      <c r="G9" s="14" t="inlineStr"/>
       <c r="H9" s="14" t="inlineStr"/>
       <c r="I9" s="14" t="inlineStr"/>
       <c r="J9" s="14" t="inlineStr"/>
@@ -843,11 +827,7 @@
       <c r="D10" s="14" t="inlineStr"/>
       <c r="E10" s="14" t="inlineStr"/>
       <c r="F10" s="14" t="inlineStr"/>
-      <c r="G10" s="14" t="inlineStr">
-        <is>
-          <t>3,99 TRY - 7,98 TRY - 99,71 TRY</t>
-        </is>
-      </c>
+      <c r="G10" s="14" t="inlineStr"/>
       <c r="H10" s="14" t="inlineStr"/>
       <c r="I10" s="14" t="inlineStr"/>
       <c r="J10" s="14" t="inlineStr"/>
@@ -863,11 +843,7 @@
       <c r="D11" s="14" t="inlineStr"/>
       <c r="E11" s="14" t="inlineStr"/>
       <c r="F11" s="14" t="inlineStr"/>
-      <c r="G11" s="14" t="inlineStr">
-        <is>
-          <t>3,99 TRY - 7,98 TRY - 99,71 TRY</t>
-        </is>
-      </c>
+      <c r="G11" s="14" t="inlineStr"/>
       <c r="H11" s="14" t="inlineStr"/>
       <c r="I11" s="14" t="inlineStr"/>
       <c r="J11" s="14" t="inlineStr"/>
@@ -886,21 +862,21 @@
       </c>
       <c r="C12" s="14" t="inlineStr">
         <is>
-          <t>WU: 1.000,01 USD–9,51 USD</t>
+          <t>WU: 3.000,01 USD–9,51 USD</t>
         </is>
       </c>
       <c r="D12" s="14" t="inlineStr"/>
       <c r="E12" s="14" t="inlineStr"/>
       <c r="F12" s="14" t="inlineStr"/>
-      <c r="G12" s="14" t="inlineStr">
-        <is>
-          <t>Şube (Kasadan): %0,5; Şube (Hesaptan): %0,75; İnternet: 15 USD</t>
-        </is>
-      </c>
+      <c r="G12" s="14" t="inlineStr"/>
       <c r="H12" s="14" t="inlineStr"/>
       <c r="I12" s="14" t="inlineStr"/>
       <c r="J12" s="14" t="inlineStr"/>
-      <c r="K12" s="14" t="inlineStr"/>
+      <c r="K12" s="14" t="inlineStr">
+        <is>
+          <t>WU: ,USD–; Diğer: 529 TL–4.454,74 TL</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="B13" s="13" t="inlineStr">
@@ -931,8 +907,16 @@
           <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
         </is>
       </c>
-      <c r="J13" s="14" t="inlineStr"/>
-      <c r="K13" s="14" t="inlineStr"/>
+      <c r="J13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 1.303 TL</t>
+        </is>
+      </c>
+      <c r="K13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 865,75 TL</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="B14" s="13" t="inlineStr">
@@ -951,20 +935,28 @@
           <t>2.170 TL - 2.170 TL</t>
         </is>
       </c>
-      <c r="F14" s="14" t="inlineStr"/>
-      <c r="G14" s="14" t="inlineStr">
-        <is>
-          <t>8.300 TL - 7,97 TL</t>
-        </is>
-      </c>
+      <c r="F14" s="14" t="inlineStr">
+        <is>
+          <t>2.785,72 TL - 12.380,95 TL</t>
+        </is>
+      </c>
+      <c r="G14" s="14" t="inlineStr"/>
       <c r="H14" s="14" t="inlineStr">
         <is>
           <t>3.000 TL - 6.000 TL</t>
         </is>
       </c>
       <c r="I14" s="14" t="inlineStr"/>
-      <c r="J14" s="14" t="inlineStr"/>
-      <c r="K14" s="14" t="inlineStr"/>
+      <c r="J14" s="14" t="inlineStr">
+        <is>
+          <t>1.554,97 TL - 7.784 TL</t>
+        </is>
+      </c>
+      <c r="K14" s="14" t="inlineStr">
+        <is>
+          <t>1.196,51 TL - 5.583,74 TL</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="12" t="inlineStr">

</xml_diff>

<commit_message>
Update benchmark: 2026-04-10 07:38:10 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -662,7 +662,11 @@
       <c r="D3" s="14" t="inlineStr"/>
       <c r="E3" s="14" t="inlineStr"/>
       <c r="F3" s="14" t="inlineStr"/>
-      <c r="G3" s="14" t="inlineStr"/>
+      <c r="G3" s="14" t="inlineStr">
+        <is>
+          <t>39,87 TRY - 79,76 TRY - 797,68 TRY</t>
+        </is>
+      </c>
       <c r="H3" s="14" t="inlineStr"/>
       <c r="I3" s="14" t="inlineStr"/>
       <c r="J3" s="14" t="inlineStr"/>
@@ -678,7 +682,11 @@
       <c r="D4" s="14" t="inlineStr"/>
       <c r="E4" s="14" t="inlineStr"/>
       <c r="F4" s="14" t="inlineStr"/>
-      <c r="G4" s="14" t="inlineStr"/>
+      <c r="G4" s="14" t="inlineStr">
+        <is>
+          <t>27,84 TRY - 55,69 TRY - 398,83 TRY</t>
+        </is>
+      </c>
       <c r="H4" s="14" t="inlineStr"/>
       <c r="I4" s="14" t="inlineStr"/>
       <c r="J4" s="14" t="inlineStr"/>
@@ -694,7 +702,11 @@
       <c r="D5" s="14" t="inlineStr"/>
       <c r="E5" s="14" t="inlineStr"/>
       <c r="F5" s="14" t="inlineStr"/>
-      <c r="G5" s="14" t="inlineStr"/>
+      <c r="G5" s="14" t="inlineStr">
+        <is>
+          <t>7,97 TRY - 15,96 TRY - 199,41 TRY</t>
+        </is>
+      </c>
       <c r="H5" s="14" t="inlineStr"/>
       <c r="I5" s="14" t="inlineStr"/>
       <c r="J5" s="14" t="inlineStr"/>
@@ -711,14 +723,22 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="D6" s="14" t="inlineStr"/>
+      <c r="D6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 199,41 TL</t>
+        </is>
+      </c>
       <c r="E6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
       <c r="F6" s="14" t="inlineStr"/>
-      <c r="G6" s="14" t="inlineStr"/>
+      <c r="G6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 99,71 TL</t>
+        </is>
+      </c>
       <c r="H6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
@@ -795,7 +815,11 @@
       <c r="D8" s="14" t="inlineStr"/>
       <c r="E8" s="14" t="inlineStr"/>
       <c r="F8" s="14" t="inlineStr"/>
-      <c r="G8" s="14" t="inlineStr"/>
+      <c r="G8" s="14" t="inlineStr">
+        <is>
+          <t>19,94 TRY - 39,88 TRY - 398,84 TRY</t>
+        </is>
+      </c>
       <c r="H8" s="14" t="inlineStr"/>
       <c r="I8" s="14" t="inlineStr"/>
       <c r="J8" s="14" t="inlineStr"/>
@@ -811,7 +835,11 @@
       <c r="D9" s="14" t="inlineStr"/>
       <c r="E9" s="14" t="inlineStr"/>
       <c r="F9" s="14" t="inlineStr"/>
-      <c r="G9" s="14" t="inlineStr"/>
+      <c r="G9" s="14" t="inlineStr">
+        <is>
+          <t>13,92 TRY - 27,85 TRY - 199,42 TRY</t>
+        </is>
+      </c>
       <c r="H9" s="14" t="inlineStr"/>
       <c r="I9" s="14" t="inlineStr"/>
       <c r="J9" s="14" t="inlineStr"/>
@@ -827,7 +855,11 @@
       <c r="D10" s="14" t="inlineStr"/>
       <c r="E10" s="14" t="inlineStr"/>
       <c r="F10" s="14" t="inlineStr"/>
-      <c r="G10" s="14" t="inlineStr"/>
+      <c r="G10" s="14" t="inlineStr">
+        <is>
+          <t>3,99 TRY - 7,98 TRY - 99,71 TRY</t>
+        </is>
+      </c>
       <c r="H10" s="14" t="inlineStr"/>
       <c r="I10" s="14" t="inlineStr"/>
       <c r="J10" s="14" t="inlineStr"/>
@@ -843,7 +875,11 @@
       <c r="D11" s="14" t="inlineStr"/>
       <c r="E11" s="14" t="inlineStr"/>
       <c r="F11" s="14" t="inlineStr"/>
-      <c r="G11" s="14" t="inlineStr"/>
+      <c r="G11" s="14" t="inlineStr">
+        <is>
+          <t>3,99 TRY - 7,98 TRY - 99,71 TRY</t>
+        </is>
+      </c>
       <c r="H11" s="14" t="inlineStr"/>
       <c r="I11" s="14" t="inlineStr"/>
       <c r="J11" s="14" t="inlineStr"/>
@@ -865,10 +901,18 @@
           <t>WU: 3.000,01 USD–9,51 USD</t>
         </is>
       </c>
-      <c r="D12" s="14" t="inlineStr"/>
+      <c r="D12" s="14" t="inlineStr">
+        <is>
+          <t>WU: 0,75 USD–12 USD; Diğer: 700 TL–4.000 TL</t>
+        </is>
+      </c>
       <c r="E12" s="14" t="inlineStr"/>
       <c r="F12" s="14" t="inlineStr"/>
-      <c r="G12" s="14" t="inlineStr"/>
+      <c r="G12" s="14" t="inlineStr">
+        <is>
+          <t>Şube (Kasadan): %0,5; Şube (Hesaptan): %0,75; İnternet: 15 USD</t>
+        </is>
+      </c>
       <c r="H12" s="14" t="inlineStr"/>
       <c r="I12" s="14" t="inlineStr"/>
       <c r="J12" s="14" t="inlineStr"/>
@@ -889,7 +933,11 @@
           <t>Hesaba: Asgari 0 TL | Azami 0,94 TL</t>
         </is>
       </c>
-      <c r="D13" s="14" t="inlineStr"/>
+      <c r="D13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
+        </is>
+      </c>
       <c r="E13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
@@ -914,7 +962,7 @@
       </c>
       <c r="K13" s="14" t="inlineStr">
         <is>
-          <t>Hesaba: Asgari 1 TL | Azami 865,75 TL</t>
+          <t>Hesaba: Asgari 1 TL | Azami 69,62 TL</t>
         </is>
       </c>
     </row>
@@ -929,18 +977,22 @@
           <t>40.000 TL - 2.485,72 TL</t>
         </is>
       </c>
-      <c r="D14" s="14" t="inlineStr"/>
+      <c r="D14" s="14" t="inlineStr">
+        <is>
+          <t>3.500 TL - 13.500 TL</t>
+        </is>
+      </c>
       <c r="E14" s="14" t="inlineStr">
         <is>
           <t>2.170 TL - 2.170 TL</t>
         </is>
       </c>
-      <c r="F14" s="14" t="inlineStr">
-        <is>
-          <t>2.785,72 TL - 12.380,95 TL</t>
-        </is>
-      </c>
-      <c r="G14" s="14" t="inlineStr"/>
+      <c r="F14" s="14" t="inlineStr"/>
+      <c r="G14" s="14" t="inlineStr">
+        <is>
+          <t>8.300 TL - 7,97 TL</t>
+        </is>
+      </c>
       <c r="H14" s="14" t="inlineStr">
         <is>
           <t>3.000 TL - 6.000 TL</t>

</xml_diff>

<commit_message>
Update benchmark: 2026-04-11 07:09:39 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -723,11 +723,7 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="D6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 199,41 TL</t>
-        </is>
-      </c>
+      <c r="D6" s="14" t="inlineStr"/>
       <c r="E6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
@@ -744,11 +740,7 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="I6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 199,41 TL</t>
-        </is>
-      </c>
+      <c r="I6" s="14" t="inlineStr"/>
       <c r="J6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
@@ -901,11 +893,7 @@
           <t>WU: 3.000,01 USD–9,51 USD</t>
         </is>
       </c>
-      <c r="D12" s="14" t="inlineStr">
-        <is>
-          <t>WU: 0,75 USD–12 USD; Diğer: 700 TL–4.000 TL</t>
-        </is>
-      </c>
+      <c r="D12" s="14" t="inlineStr"/>
       <c r="E12" s="14" t="inlineStr"/>
       <c r="F12" s="14" t="inlineStr"/>
       <c r="G12" s="14" t="inlineStr">
@@ -933,14 +921,10 @@
           <t>Hesaba: Asgari 0 TL | Azami 0,94 TL</t>
         </is>
       </c>
-      <c r="D13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
-        </is>
-      </c>
+      <c r="D13" s="14" t="inlineStr"/>
       <c r="E13" s="14" t="inlineStr">
         <is>
-          <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
+          <t>Hesaba: Asgari 1 TL | Azami 11.380 TL</t>
         </is>
       </c>
       <c r="F13" s="14" t="inlineStr"/>
@@ -950,11 +934,7 @@
           <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
         </is>
       </c>
-      <c r="I13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
-        </is>
-      </c>
+      <c r="I13" s="14" t="inlineStr"/>
       <c r="J13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.303 TL</t>
@@ -962,7 +942,7 @@
       </c>
       <c r="K13" s="14" t="inlineStr">
         <is>
-          <t>Hesaba: Asgari 1 TL | Azami 69,62 TL</t>
+          <t>Hesaba: Asgari 1 TL | Azami 865,75 TL</t>
         </is>
       </c>
     </row>
@@ -977,17 +957,17 @@
           <t>40.000 TL - 2.485,72 TL</t>
         </is>
       </c>
-      <c r="D14" s="14" t="inlineStr">
-        <is>
-          <t>3.500 TL - 13.500 TL</t>
-        </is>
-      </c>
+      <c r="D14" s="14" t="inlineStr"/>
       <c r="E14" s="14" t="inlineStr">
         <is>
           <t>2.170 TL - 2.170 TL</t>
         </is>
       </c>
-      <c r="F14" s="14" t="inlineStr"/>
+      <c r="F14" s="14" t="inlineStr">
+        <is>
+          <t>2.785,72 TL - 12.380,95 TL</t>
+        </is>
+      </c>
       <c r="G14" s="14" t="inlineStr">
         <is>
           <t>8.300 TL - 7,97 TL</t>

</xml_diff>

<commit_message>
Update benchmark: 2026-04-12 07:23:08 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -723,7 +723,11 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="D6" s="14" t="inlineStr"/>
+      <c r="D6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 199,41 TL</t>
+        </is>
+      </c>
       <c r="E6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
@@ -740,7 +744,11 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="I6" s="14" t="inlineStr"/>
+      <c r="I6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 199,41 TL</t>
+        </is>
+      </c>
       <c r="J6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
@@ -893,7 +901,11 @@
           <t>WU: 3.000,01 USD–9,51 USD</t>
         </is>
       </c>
-      <c r="D12" s="14" t="inlineStr"/>
+      <c r="D12" s="14" t="inlineStr">
+        <is>
+          <t>WU: 0,75 USD–12 USD; Diğer: 700 TL–4.000 TL</t>
+        </is>
+      </c>
       <c r="E12" s="14" t="inlineStr"/>
       <c r="F12" s="14" t="inlineStr"/>
       <c r="G12" s="14" t="inlineStr">
@@ -921,10 +933,14 @@
           <t>Hesaba: Asgari 0 TL | Azami 0,94 TL</t>
         </is>
       </c>
-      <c r="D13" s="14" t="inlineStr"/>
+      <c r="D13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
+        </is>
+      </c>
       <c r="E13" s="14" t="inlineStr">
         <is>
-          <t>Hesaba: Asgari 1 TL | Azami 11.380 TL</t>
+          <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
         </is>
       </c>
       <c r="F13" s="14" t="inlineStr"/>
@@ -934,7 +950,11 @@
           <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
         </is>
       </c>
-      <c r="I13" s="14" t="inlineStr"/>
+      <c r="I13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
+        </is>
+      </c>
       <c r="J13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.303 TL</t>
@@ -957,7 +977,11 @@
           <t>40.000 TL - 2.485,72 TL</t>
         </is>
       </c>
-      <c r="D14" s="14" t="inlineStr"/>
+      <c r="D14" s="14" t="inlineStr">
+        <is>
+          <t>3.500 TL - 13.500 TL</t>
+        </is>
+      </c>
       <c r="E14" s="14" t="inlineStr">
         <is>
           <t>2.170 TL - 2.170 TL</t>

</xml_diff>

<commit_message>
Update benchmark: 2026-04-13 08:11:27 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -718,16 +718,8 @@
           <t>DÜZENLİ EFT</t>
         </is>
       </c>
-      <c r="C6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 199,41 TL</t>
-        </is>
-      </c>
-      <c r="D6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 199,41 TL</t>
-        </is>
-      </c>
+      <c r="C6" s="14" t="inlineStr"/>
+      <c r="D6" s="14" t="inlineStr"/>
       <c r="E6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
@@ -739,11 +731,7 @@
           <t>8.300,01 TL - 99,71 TL</t>
         </is>
       </c>
-      <c r="H6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 199,41 TL</t>
-        </is>
-      </c>
+      <c r="H6" s="14" t="inlineStr"/>
       <c r="I6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
@@ -896,16 +884,8 @@
           <t>GİDEN SWIFT</t>
         </is>
       </c>
-      <c r="C12" s="14" t="inlineStr">
-        <is>
-          <t>WU: 3.000,01 USD–9,51 USD</t>
-        </is>
-      </c>
-      <c r="D12" s="14" t="inlineStr">
-        <is>
-          <t>WU: 0,75 USD–12 USD; Diğer: 700 TL–4.000 TL</t>
-        </is>
-      </c>
+      <c r="C12" s="14" t="inlineStr"/>
+      <c r="D12" s="14" t="inlineStr"/>
       <c r="E12" s="14" t="inlineStr"/>
       <c r="F12" s="14" t="inlineStr"/>
       <c r="G12" s="14" t="inlineStr">
@@ -928,16 +908,8 @@
           <t>GELEN SWIFT</t>
         </is>
       </c>
-      <c r="C13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 0 TL | Azami 0,94 TL</t>
-        </is>
-      </c>
-      <c r="D13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
-        </is>
-      </c>
+      <c r="C13" s="14" t="inlineStr"/>
+      <c r="D13" s="14" t="inlineStr"/>
       <c r="E13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
@@ -945,11 +917,7 @@
       </c>
       <c r="F13" s="14" t="inlineStr"/>
       <c r="G13" s="14" t="inlineStr"/>
-      <c r="H13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
-        </is>
-      </c>
+      <c r="H13" s="14" t="inlineStr"/>
       <c r="I13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
@@ -972,16 +940,8 @@
           <t>GİDEN SWIFT - Mobil</t>
         </is>
       </c>
-      <c r="C14" s="14" t="inlineStr">
-        <is>
-          <t>40.000 TL - 2.485,72 TL</t>
-        </is>
-      </c>
-      <c r="D14" s="14" t="inlineStr">
-        <is>
-          <t>3.500 TL - 13.500 TL</t>
-        </is>
-      </c>
+      <c r="C14" s="14" t="inlineStr"/>
+      <c r="D14" s="14" t="inlineStr"/>
       <c r="E14" s="14" t="inlineStr">
         <is>
           <t>2.170 TL - 2.170 TL</t>
@@ -997,11 +957,7 @@
           <t>8.300 TL - 7,97 TL</t>
         </is>
       </c>
-      <c r="H14" s="14" t="inlineStr">
-        <is>
-          <t>3.000 TL - 6.000 TL</t>
-        </is>
-      </c>
+      <c r="H14" s="14" t="inlineStr"/>
       <c r="I14" s="14" t="inlineStr"/>
       <c r="J14" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update benchmark: 2026-04-14 07:54:40 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -718,8 +718,16 @@
           <t>DÜZENLİ EFT</t>
         </is>
       </c>
-      <c r="C6" s="14" t="inlineStr"/>
-      <c r="D6" s="14" t="inlineStr"/>
+      <c r="C6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 199,41 TL</t>
+        </is>
+      </c>
+      <c r="D6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 199,41 TL</t>
+        </is>
+      </c>
       <c r="E6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
@@ -731,7 +739,11 @@
           <t>8.300,01 TL - 99,71 TL</t>
         </is>
       </c>
-      <c r="H6" s="14" t="inlineStr"/>
+      <c r="H6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 199,41 TL</t>
+        </is>
+      </c>
       <c r="I6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
@@ -884,8 +896,16 @@
           <t>GİDEN SWIFT</t>
         </is>
       </c>
-      <c r="C12" s="14" t="inlineStr"/>
-      <c r="D12" s="14" t="inlineStr"/>
+      <c r="C12" s="14" t="inlineStr">
+        <is>
+          <t>WU: 3.000,01 USD–9,51 USD</t>
+        </is>
+      </c>
+      <c r="D12" s="14" t="inlineStr">
+        <is>
+          <t>WU: 0,75 USD–12 USD; Diğer: 700 TL–4.000 TL</t>
+        </is>
+      </c>
       <c r="E12" s="14" t="inlineStr"/>
       <c r="F12" s="14" t="inlineStr"/>
       <c r="G12" s="14" t="inlineStr">
@@ -908,8 +928,16 @@
           <t>GELEN SWIFT</t>
         </is>
       </c>
-      <c r="C13" s="14" t="inlineStr"/>
-      <c r="D13" s="14" t="inlineStr"/>
+      <c r="C13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 0 TL | Azami 0,94 TL</t>
+        </is>
+      </c>
+      <c r="D13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
+        </is>
+      </c>
       <c r="E13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
@@ -917,7 +945,11 @@
       </c>
       <c r="F13" s="14" t="inlineStr"/>
       <c r="G13" s="14" t="inlineStr"/>
-      <c r="H13" s="14" t="inlineStr"/>
+      <c r="H13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
+        </is>
+      </c>
       <c r="I13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
@@ -940,24 +972,32 @@
           <t>GİDEN SWIFT - Mobil</t>
         </is>
       </c>
-      <c r="C14" s="14" t="inlineStr"/>
-      <c r="D14" s="14" t="inlineStr"/>
+      <c r="C14" s="14" t="inlineStr">
+        <is>
+          <t>40.000 TL - 2.485,72 TL</t>
+        </is>
+      </c>
+      <c r="D14" s="14" t="inlineStr">
+        <is>
+          <t>3.500 TL - 13.500 TL</t>
+        </is>
+      </c>
       <c r="E14" s="14" t="inlineStr">
         <is>
           <t>2.170 TL - 2.170 TL</t>
         </is>
       </c>
-      <c r="F14" s="14" t="inlineStr">
-        <is>
-          <t>2.785,72 TL - 12.380,95 TL</t>
-        </is>
-      </c>
+      <c r="F14" s="14" t="inlineStr"/>
       <c r="G14" s="14" t="inlineStr">
         <is>
           <t>8.300 TL - 7,97 TL</t>
         </is>
       </c>
-      <c r="H14" s="14" t="inlineStr"/>
+      <c r="H14" s="14" t="inlineStr">
+        <is>
+          <t>3.000 TL - 6.000 TL</t>
+        </is>
+      </c>
       <c r="I14" s="14" t="inlineStr"/>
       <c r="J14" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update benchmark: 2026-04-15 07:55:00 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -723,11 +723,7 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="D6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 199,41 TL</t>
-        </is>
-      </c>
+      <c r="D6" s="14" t="inlineStr"/>
       <c r="E6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
@@ -739,26 +735,18 @@
           <t>8.300,01 TL - 99,71 TL</t>
         </is>
       </c>
-      <c r="H6" s="14" t="inlineStr">
+      <c r="H6" s="14" t="inlineStr"/>
+      <c r="I6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="I6" s="14" t="inlineStr">
+      <c r="J6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="J6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 199,41 TL</t>
-        </is>
-      </c>
-      <c r="K6" s="14" t="inlineStr">
-        <is>
-          <t>7,97 TL - 15,96 TL - 199,41 TL</t>
-        </is>
-      </c>
+      <c r="K6" s="14" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="B7" s="13" t="inlineStr">
@@ -901,11 +889,7 @@
           <t>WU: 3.000,01 USD–9,51 USD</t>
         </is>
       </c>
-      <c r="D12" s="14" t="inlineStr">
-        <is>
-          <t>WU: 0,75 USD–12 USD; Diğer: 700 TL–4.000 TL</t>
-        </is>
-      </c>
+      <c r="D12" s="14" t="inlineStr"/>
       <c r="E12" s="14" t="inlineStr"/>
       <c r="F12" s="14" t="inlineStr"/>
       <c r="G12" s="14" t="inlineStr">
@@ -916,11 +900,7 @@
       <c r="H12" s="14" t="inlineStr"/>
       <c r="I12" s="14" t="inlineStr"/>
       <c r="J12" s="14" t="inlineStr"/>
-      <c r="K12" s="14" t="inlineStr">
-        <is>
-          <t>WU: ,USD–; Diğer: 529 TL–4.454,74 TL</t>
-        </is>
-      </c>
+      <c r="K12" s="14" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="B13" s="13" t="inlineStr">
@@ -933,11 +913,7 @@
           <t>Hesaba: Asgari 0 TL | Azami 0,94 TL</t>
         </is>
       </c>
-      <c r="D13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
-        </is>
-      </c>
+      <c r="D13" s="14" t="inlineStr"/>
       <c r="E13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
@@ -945,26 +921,18 @@
       </c>
       <c r="F13" s="14" t="inlineStr"/>
       <c r="G13" s="14" t="inlineStr"/>
-      <c r="H13" s="14" t="inlineStr">
+      <c r="H13" s="14" t="inlineStr"/>
+      <c r="I13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
         </is>
       </c>
-      <c r="I13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
-        </is>
-      </c>
       <c r="J13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.303 TL</t>
         </is>
       </c>
-      <c r="K13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 865,75 TL</t>
-        </is>
-      </c>
+      <c r="K13" s="14" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="B14" s="13" t="inlineStr">
@@ -977,11 +945,7 @@
           <t>40.000 TL - 2.485,72 TL</t>
         </is>
       </c>
-      <c r="D14" s="14" t="inlineStr">
-        <is>
-          <t>3.500 TL - 13.500 TL</t>
-        </is>
-      </c>
+      <c r="D14" s="14" t="inlineStr"/>
       <c r="E14" s="14" t="inlineStr">
         <is>
           <t>2.170 TL - 2.170 TL</t>
@@ -993,22 +957,14 @@
           <t>8.300 TL - 7,97 TL</t>
         </is>
       </c>
-      <c r="H14" s="14" t="inlineStr">
-        <is>
-          <t>3.000 TL - 6.000 TL</t>
-        </is>
-      </c>
+      <c r="H14" s="14" t="inlineStr"/>
       <c r="I14" s="14" t="inlineStr"/>
       <c r="J14" s="14" t="inlineStr">
         <is>
           <t>1.554,97 TL - 7.784 TL</t>
         </is>
       </c>
-      <c r="K14" s="14" t="inlineStr">
-        <is>
-          <t>1.196,51 TL - 5.583,74 TL</t>
-        </is>
-      </c>
+      <c r="K14" s="14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="12" t="inlineStr">

</xml_diff>

<commit_message>
Update benchmark: 2026-04-16 07:53:50 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -718,35 +718,31 @@
           <t>DÜZENLİ EFT</t>
         </is>
       </c>
-      <c r="C6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 199,41 TL</t>
-        </is>
-      </c>
+      <c r="C6" s="14" t="inlineStr"/>
       <c r="D6" s="14" t="inlineStr"/>
-      <c r="E6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 199,41 TL</t>
-        </is>
-      </c>
+      <c r="E6" s="14" t="inlineStr"/>
       <c r="F6" s="14" t="inlineStr"/>
       <c r="G6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 99,71 TL</t>
         </is>
       </c>
-      <c r="H6" s="14" t="inlineStr"/>
+      <c r="H6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 199,41 TL</t>
+        </is>
+      </c>
       <c r="I6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="J6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 199,41 TL</t>
-        </is>
-      </c>
-      <c r="K6" s="14" t="inlineStr"/>
+      <c r="J6" s="14" t="inlineStr"/>
+      <c r="K6" s="14" t="inlineStr">
+        <is>
+          <t>7,97 TL - 15,96 TL - 199,41 TL</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="B7" s="13" t="inlineStr">
@@ -884,11 +880,7 @@
           <t>GİDEN SWIFT</t>
         </is>
       </c>
-      <c r="C12" s="14" t="inlineStr">
-        <is>
-          <t>WU: 3.000,01 USD–9,51 USD</t>
-        </is>
-      </c>
+      <c r="C12" s="14" t="inlineStr"/>
       <c r="D12" s="14" t="inlineStr"/>
       <c r="E12" s="14" t="inlineStr"/>
       <c r="F12" s="14" t="inlineStr"/>
@@ -900,7 +892,11 @@
       <c r="H12" s="14" t="inlineStr"/>
       <c r="I12" s="14" t="inlineStr"/>
       <c r="J12" s="14" t="inlineStr"/>
-      <c r="K12" s="14" t="inlineStr"/>
+      <c r="K12" s="14" t="inlineStr">
+        <is>
+          <t>WU: ,USD–; Diğer: 529 TL–4.454,74 TL</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="B13" s="13" t="inlineStr">
@@ -908,31 +904,27 @@
           <t>GELEN SWIFT</t>
         </is>
       </c>
-      <c r="C13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 0 TL | Azami 0,94 TL</t>
-        </is>
-      </c>
+      <c r="C13" s="14" t="inlineStr"/>
       <c r="D13" s="14" t="inlineStr"/>
-      <c r="E13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
-        </is>
-      </c>
+      <c r="E13" s="14" t="inlineStr"/>
       <c r="F13" s="14" t="inlineStr"/>
       <c r="G13" s="14" t="inlineStr"/>
-      <c r="H13" s="14" t="inlineStr"/>
+      <c r="H13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
+        </is>
+      </c>
       <c r="I13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
         </is>
       </c>
-      <c r="J13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 1.303 TL</t>
-        </is>
-      </c>
-      <c r="K13" s="14" t="inlineStr"/>
+      <c r="J13" s="14" t="inlineStr"/>
+      <c r="K13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 865,75 TL</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="B14" s="13" t="inlineStr">
@@ -940,31 +932,27 @@
           <t>GİDEN SWIFT - Mobil</t>
         </is>
       </c>
-      <c r="C14" s="14" t="inlineStr">
-        <is>
-          <t>40.000 TL - 2.485,72 TL</t>
-        </is>
-      </c>
+      <c r="C14" s="14" t="inlineStr"/>
       <c r="D14" s="14" t="inlineStr"/>
-      <c r="E14" s="14" t="inlineStr">
-        <is>
-          <t>2.170 TL - 2.170 TL</t>
-        </is>
-      </c>
+      <c r="E14" s="14" t="inlineStr"/>
       <c r="F14" s="14" t="inlineStr"/>
       <c r="G14" s="14" t="inlineStr">
         <is>
           <t>8.300 TL - 7,97 TL</t>
         </is>
       </c>
-      <c r="H14" s="14" t="inlineStr"/>
+      <c r="H14" s="14" t="inlineStr">
+        <is>
+          <t>3.000 TL - 6.000 TL</t>
+        </is>
+      </c>
       <c r="I14" s="14" t="inlineStr"/>
-      <c r="J14" s="14" t="inlineStr">
-        <is>
-          <t>1.554,97 TL - 7.784 TL</t>
-        </is>
-      </c>
-      <c r="K14" s="14" t="inlineStr"/>
+      <c r="J14" s="14" t="inlineStr"/>
+      <c r="K14" s="14" t="inlineStr">
+        <is>
+          <t>1.196,51 TL - 5.583,74 TL</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="12" t="inlineStr">

</xml_diff>

<commit_message>
Update benchmark: 2026-04-17 07:55:31 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -662,11 +662,7 @@
       <c r="D3" s="14" t="inlineStr"/>
       <c r="E3" s="14" t="inlineStr"/>
       <c r="F3" s="14" t="inlineStr"/>
-      <c r="G3" s="14" t="inlineStr">
-        <is>
-          <t>39,87 TRY - 79,76 TRY - 797,68 TRY</t>
-        </is>
-      </c>
+      <c r="G3" s="14" t="inlineStr"/>
       <c r="H3" s="14" t="inlineStr"/>
       <c r="I3" s="14" t="inlineStr"/>
       <c r="J3" s="14" t="inlineStr"/>
@@ -682,11 +678,7 @@
       <c r="D4" s="14" t="inlineStr"/>
       <c r="E4" s="14" t="inlineStr"/>
       <c r="F4" s="14" t="inlineStr"/>
-      <c r="G4" s="14" t="inlineStr">
-        <is>
-          <t>27,84 TRY - 55,69 TRY - 398,83 TRY</t>
-        </is>
-      </c>
+      <c r="G4" s="14" t="inlineStr"/>
       <c r="H4" s="14" t="inlineStr"/>
       <c r="I4" s="14" t="inlineStr"/>
       <c r="J4" s="14" t="inlineStr"/>
@@ -702,11 +694,7 @@
       <c r="D5" s="14" t="inlineStr"/>
       <c r="E5" s="14" t="inlineStr"/>
       <c r="F5" s="14" t="inlineStr"/>
-      <c r="G5" s="14" t="inlineStr">
-        <is>
-          <t>7,97 TRY - 15,96 TRY - 199,41 TRY</t>
-        </is>
-      </c>
+      <c r="G5" s="14" t="inlineStr"/>
       <c r="H5" s="14" t="inlineStr"/>
       <c r="I5" s="14" t="inlineStr"/>
       <c r="J5" s="14" t="inlineStr"/>
@@ -718,15 +706,23 @@
           <t>DÜZENLİ EFT</t>
         </is>
       </c>
-      <c r="C6" s="14" t="inlineStr"/>
-      <c r="D6" s="14" t="inlineStr"/>
-      <c r="E6" s="14" t="inlineStr"/>
+      <c r="C6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 199,41 TL</t>
+        </is>
+      </c>
+      <c r="D6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 199,41 TL</t>
+        </is>
+      </c>
+      <c r="E6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 199,41 TL</t>
+        </is>
+      </c>
       <c r="F6" s="14" t="inlineStr"/>
-      <c r="G6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 99,71 TL</t>
-        </is>
-      </c>
+      <c r="G6" s="14" t="inlineStr"/>
       <c r="H6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
@@ -737,7 +733,11 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="J6" s="14" t="inlineStr"/>
+      <c r="J6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 199,41 TL</t>
+        </is>
+      </c>
       <c r="K6" s="14" t="inlineStr">
         <is>
           <t>7,97 TL - 15,96 TL - 199,41 TL</t>
@@ -799,11 +799,7 @@
       <c r="D8" s="14" t="inlineStr"/>
       <c r="E8" s="14" t="inlineStr"/>
       <c r="F8" s="14" t="inlineStr"/>
-      <c r="G8" s="14" t="inlineStr">
-        <is>
-          <t>19,94 TRY - 39,88 TRY - 398,84 TRY</t>
-        </is>
-      </c>
+      <c r="G8" s="14" t="inlineStr"/>
       <c r="H8" s="14" t="inlineStr"/>
       <c r="I8" s="14" t="inlineStr"/>
       <c r="J8" s="14" t="inlineStr"/>
@@ -819,11 +815,7 @@
       <c r="D9" s="14" t="inlineStr"/>
       <c r="E9" s="14" t="inlineStr"/>
       <c r="F9" s="14" t="inlineStr"/>
-      <c r="G9" s="14" t="inlineStr">
-        <is>
-          <t>13,92 TRY - 27,85 TRY - 199,42 TRY</t>
-        </is>
-      </c>
+      <c r="G9" s="14" t="inlineStr"/>
       <c r="H9" s="14" t="inlineStr"/>
       <c r="I9" s="14" t="inlineStr"/>
       <c r="J9" s="14" t="inlineStr"/>
@@ -839,11 +831,7 @@
       <c r="D10" s="14" t="inlineStr"/>
       <c r="E10" s="14" t="inlineStr"/>
       <c r="F10" s="14" t="inlineStr"/>
-      <c r="G10" s="14" t="inlineStr">
-        <is>
-          <t>3,99 TRY - 7,98 TRY - 99,71 TRY</t>
-        </is>
-      </c>
+      <c r="G10" s="14" t="inlineStr"/>
       <c r="H10" s="14" t="inlineStr"/>
       <c r="I10" s="14" t="inlineStr"/>
       <c r="J10" s="14" t="inlineStr"/>
@@ -859,11 +847,7 @@
       <c r="D11" s="14" t="inlineStr"/>
       <c r="E11" s="14" t="inlineStr"/>
       <c r="F11" s="14" t="inlineStr"/>
-      <c r="G11" s="14" t="inlineStr">
-        <is>
-          <t>3,99 TRY - 7,98 TRY - 99,71 TRY</t>
-        </is>
-      </c>
+      <c r="G11" s="14" t="inlineStr"/>
       <c r="H11" s="14" t="inlineStr"/>
       <c r="I11" s="14" t="inlineStr"/>
       <c r="J11" s="14" t="inlineStr"/>
@@ -880,15 +864,19 @@
           <t>GİDEN SWIFT</t>
         </is>
       </c>
-      <c r="C12" s="14" t="inlineStr"/>
-      <c r="D12" s="14" t="inlineStr"/>
+      <c r="C12" s="14" t="inlineStr">
+        <is>
+          <t>WU: 1.000,01 USD–9,51 USD</t>
+        </is>
+      </c>
+      <c r="D12" s="14" t="inlineStr">
+        <is>
+          <t>WU: 0,75 USD–12 USD; Diğer: 700 TL–4.000 TL</t>
+        </is>
+      </c>
       <c r="E12" s="14" t="inlineStr"/>
       <c r="F12" s="14" t="inlineStr"/>
-      <c r="G12" s="14" t="inlineStr">
-        <is>
-          <t>Şube (Kasadan): %0,5; Şube (Hesaptan): %0,75; İnternet: 15 USD</t>
-        </is>
-      </c>
+      <c r="G12" s="14" t="inlineStr"/>
       <c r="H12" s="14" t="inlineStr"/>
       <c r="I12" s="14" t="inlineStr"/>
       <c r="J12" s="14" t="inlineStr"/>
@@ -904,9 +892,21 @@
           <t>GELEN SWIFT</t>
         </is>
       </c>
-      <c r="C13" s="14" t="inlineStr"/>
-      <c r="D13" s="14" t="inlineStr"/>
-      <c r="E13" s="14" t="inlineStr"/>
+      <c r="C13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 0 TL | Azami 0,94 TL</t>
+        </is>
+      </c>
+      <c r="D13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
+        </is>
+      </c>
+      <c r="E13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
+        </is>
+      </c>
       <c r="F13" s="14" t="inlineStr"/>
       <c r="G13" s="14" t="inlineStr"/>
       <c r="H13" s="14" t="inlineStr">
@@ -919,7 +919,11 @@
           <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
         </is>
       </c>
-      <c r="J13" s="14" t="inlineStr"/>
+      <c r="J13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 1.303 TL</t>
+        </is>
+      </c>
       <c r="K13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 865,75 TL</t>
@@ -932,22 +936,38 @@
           <t>GİDEN SWIFT - Mobil</t>
         </is>
       </c>
-      <c r="C14" s="14" t="inlineStr"/>
-      <c r="D14" s="14" t="inlineStr"/>
-      <c r="E14" s="14" t="inlineStr"/>
-      <c r="F14" s="14" t="inlineStr"/>
-      <c r="G14" s="14" t="inlineStr">
-        <is>
-          <t>8.300 TL - 7,97 TL</t>
-        </is>
-      </c>
+      <c r="C14" s="14" t="inlineStr">
+        <is>
+          <t>40.000 TL - 2.485,72 TL</t>
+        </is>
+      </c>
+      <c r="D14" s="14" t="inlineStr">
+        <is>
+          <t>3.500 TL - 13.500 TL</t>
+        </is>
+      </c>
+      <c r="E14" s="14" t="inlineStr">
+        <is>
+          <t>2.170 TL - 2.170 TL</t>
+        </is>
+      </c>
+      <c r="F14" s="14" t="inlineStr">
+        <is>
+          <t>2.785,72 TL - 12.380,95 TL</t>
+        </is>
+      </c>
+      <c r="G14" s="14" t="inlineStr"/>
       <c r="H14" s="14" t="inlineStr">
         <is>
           <t>3.000 TL - 6.000 TL</t>
         </is>
       </c>
       <c r="I14" s="14" t="inlineStr"/>
-      <c r="J14" s="14" t="inlineStr"/>
+      <c r="J14" s="14" t="inlineStr">
+        <is>
+          <t>1.554,97 TL - 7.784 TL</t>
+        </is>
+      </c>
       <c r="K14" s="14" t="inlineStr">
         <is>
           <t>1.196,51 TL - 5.583,74 TL</t>

</xml_diff>

<commit_message>
Update benchmark: 2026-04-18 07:16:54 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -662,7 +662,11 @@
       <c r="D3" s="14" t="inlineStr"/>
       <c r="E3" s="14" t="inlineStr"/>
       <c r="F3" s="14" t="inlineStr"/>
-      <c r="G3" s="14" t="inlineStr"/>
+      <c r="G3" s="14" t="inlineStr">
+        <is>
+          <t>39,87 TRY - 79,76 TRY - 797,68 TRY</t>
+        </is>
+      </c>
       <c r="H3" s="14" t="inlineStr"/>
       <c r="I3" s="14" t="inlineStr"/>
       <c r="J3" s="14" t="inlineStr"/>
@@ -678,7 +682,11 @@
       <c r="D4" s="14" t="inlineStr"/>
       <c r="E4" s="14" t="inlineStr"/>
       <c r="F4" s="14" t="inlineStr"/>
-      <c r="G4" s="14" t="inlineStr"/>
+      <c r="G4" s="14" t="inlineStr">
+        <is>
+          <t>27,84 TRY - 55,69 TRY - 398,83 TRY</t>
+        </is>
+      </c>
       <c r="H4" s="14" t="inlineStr"/>
       <c r="I4" s="14" t="inlineStr"/>
       <c r="J4" s="14" t="inlineStr"/>
@@ -694,7 +702,11 @@
       <c r="D5" s="14" t="inlineStr"/>
       <c r="E5" s="14" t="inlineStr"/>
       <c r="F5" s="14" t="inlineStr"/>
-      <c r="G5" s="14" t="inlineStr"/>
+      <c r="G5" s="14" t="inlineStr">
+        <is>
+          <t>7,97 TRY - 15,96 TRY - 199,41 TRY</t>
+        </is>
+      </c>
       <c r="H5" s="14" t="inlineStr"/>
       <c r="I5" s="14" t="inlineStr"/>
       <c r="J5" s="14" t="inlineStr"/>
@@ -716,13 +728,13 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="E6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 199,41 TL</t>
-        </is>
-      </c>
+      <c r="E6" s="14" t="inlineStr"/>
       <c r="F6" s="14" t="inlineStr"/>
-      <c r="G6" s="14" t="inlineStr"/>
+      <c r="G6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 99,71 TL</t>
+        </is>
+      </c>
       <c r="H6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
@@ -799,7 +811,11 @@
       <c r="D8" s="14" t="inlineStr"/>
       <c r="E8" s="14" t="inlineStr"/>
       <c r="F8" s="14" t="inlineStr"/>
-      <c r="G8" s="14" t="inlineStr"/>
+      <c r="G8" s="14" t="inlineStr">
+        <is>
+          <t>19,94 TRY - 39,88 TRY - 398,84 TRY</t>
+        </is>
+      </c>
       <c r="H8" s="14" t="inlineStr"/>
       <c r="I8" s="14" t="inlineStr"/>
       <c r="J8" s="14" t="inlineStr"/>
@@ -815,7 +831,11 @@
       <c r="D9" s="14" t="inlineStr"/>
       <c r="E9" s="14" t="inlineStr"/>
       <c r="F9" s="14" t="inlineStr"/>
-      <c r="G9" s="14" t="inlineStr"/>
+      <c r="G9" s="14" t="inlineStr">
+        <is>
+          <t>13,92 TRY - 27,85 TRY - 199,42 TRY</t>
+        </is>
+      </c>
       <c r="H9" s="14" t="inlineStr"/>
       <c r="I9" s="14" t="inlineStr"/>
       <c r="J9" s="14" t="inlineStr"/>
@@ -831,7 +851,11 @@
       <c r="D10" s="14" t="inlineStr"/>
       <c r="E10" s="14" t="inlineStr"/>
       <c r="F10" s="14" t="inlineStr"/>
-      <c r="G10" s="14" t="inlineStr"/>
+      <c r="G10" s="14" t="inlineStr">
+        <is>
+          <t>3,99 TRY - 7,98 TRY - 99,71 TRY</t>
+        </is>
+      </c>
       <c r="H10" s="14" t="inlineStr"/>
       <c r="I10" s="14" t="inlineStr"/>
       <c r="J10" s="14" t="inlineStr"/>
@@ -847,7 +871,11 @@
       <c r="D11" s="14" t="inlineStr"/>
       <c r="E11" s="14" t="inlineStr"/>
       <c r="F11" s="14" t="inlineStr"/>
-      <c r="G11" s="14" t="inlineStr"/>
+      <c r="G11" s="14" t="inlineStr">
+        <is>
+          <t>3,99 TRY - 7,98 TRY - 99,71 TRY</t>
+        </is>
+      </c>
       <c r="H11" s="14" t="inlineStr"/>
       <c r="I11" s="14" t="inlineStr"/>
       <c r="J11" s="14" t="inlineStr"/>
@@ -876,7 +904,11 @@
       </c>
       <c r="E12" s="14" t="inlineStr"/>
       <c r="F12" s="14" t="inlineStr"/>
-      <c r="G12" s="14" t="inlineStr"/>
+      <c r="G12" s="14" t="inlineStr">
+        <is>
+          <t>Şube (Kasadan): %0,5; Şube (Hesaptan): %0,75; İnternet: 15 USD</t>
+        </is>
+      </c>
       <c r="H12" s="14" t="inlineStr"/>
       <c r="I12" s="14" t="inlineStr"/>
       <c r="J12" s="14" t="inlineStr"/>
@@ -902,11 +934,7 @@
           <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
         </is>
       </c>
-      <c r="E13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
-        </is>
-      </c>
+      <c r="E13" s="14" t="inlineStr"/>
       <c r="F13" s="14" t="inlineStr"/>
       <c r="G13" s="14" t="inlineStr"/>
       <c r="H13" s="14" t="inlineStr">
@@ -946,17 +974,17 @@
           <t>3.500 TL - 13.500 TL</t>
         </is>
       </c>
-      <c r="E14" s="14" t="inlineStr">
-        <is>
-          <t>2.170 TL - 2.170 TL</t>
-        </is>
-      </c>
+      <c r="E14" s="14" t="inlineStr"/>
       <c r="F14" s="14" t="inlineStr">
         <is>
           <t>2.785,72 TL - 12.380,95 TL</t>
         </is>
       </c>
-      <c r="G14" s="14" t="inlineStr"/>
+      <c r="G14" s="14" t="inlineStr">
+        <is>
+          <t>8.300 TL - 7,97 TL</t>
+        </is>
+      </c>
       <c r="H14" s="14" t="inlineStr">
         <is>
           <t>3.000 TL - 6.000 TL</t>

</xml_diff>

<commit_message>
Update benchmark: 2026-04-19 07:28:29 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -728,7 +728,11 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="E6" s="14" t="inlineStr"/>
+      <c r="E6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 199,41 TL</t>
+        </is>
+      </c>
       <c r="F6" s="14" t="inlineStr"/>
       <c r="G6" s="14" t="inlineStr">
         <is>
@@ -934,7 +938,11 @@
           <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
         </is>
       </c>
-      <c r="E13" s="14" t="inlineStr"/>
+      <c r="E13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
+        </is>
+      </c>
       <c r="F13" s="14" t="inlineStr"/>
       <c r="G13" s="14" t="inlineStr"/>
       <c r="H13" s="14" t="inlineStr">
@@ -974,7 +982,11 @@
           <t>3.500 TL - 13.500 TL</t>
         </is>
       </c>
-      <c r="E14" s="14" t="inlineStr"/>
+      <c r="E14" s="14" t="inlineStr">
+        <is>
+          <t>2.170 TL - 2.170 TL</t>
+        </is>
+      </c>
       <c r="F14" s="14" t="inlineStr">
         <is>
           <t>2.785,72 TL - 12.380,95 TL</t>

</xml_diff>

<commit_message>
Update benchmark: 2026-04-20 08:16:12 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -723,11 +723,7 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="D6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 199,41 TL</t>
-        </is>
-      </c>
+      <c r="D6" s="14" t="inlineStr"/>
       <c r="E6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
@@ -901,11 +897,7 @@
           <t>WU: 1.000,01 USD–9,51 USD</t>
         </is>
       </c>
-      <c r="D12" s="14" t="inlineStr">
-        <is>
-          <t>WU: 0,75 USD–12 USD; Diğer: 700 TL–4.000 TL</t>
-        </is>
-      </c>
+      <c r="D12" s="14" t="inlineStr"/>
       <c r="E12" s="14" t="inlineStr"/>
       <c r="F12" s="14" t="inlineStr"/>
       <c r="G12" s="14" t="inlineStr">
@@ -933,11 +925,7 @@
           <t>Hesaba: Asgari 0 TL | Azami 0,94 TL</t>
         </is>
       </c>
-      <c r="D13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
-        </is>
-      </c>
+      <c r="D13" s="14" t="inlineStr"/>
       <c r="E13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
@@ -977,11 +965,7 @@
           <t>40.000 TL - 2.485,72 TL</t>
         </is>
       </c>
-      <c r="D14" s="14" t="inlineStr">
-        <is>
-          <t>3.500 TL - 13.500 TL</t>
-        </is>
-      </c>
+      <c r="D14" s="14" t="inlineStr"/>
       <c r="E14" s="14" t="inlineStr">
         <is>
           <t>2.170 TL - 2.170 TL</t>

</xml_diff>

<commit_message>
Update benchmark: 2026-04-21 07:58:18 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -971,11 +971,7 @@
           <t>2.170 TL - 2.170 TL</t>
         </is>
       </c>
-      <c r="F14" s="14" t="inlineStr">
-        <is>
-          <t>2.785,72 TL - 12.380,95 TL</t>
-        </is>
-      </c>
+      <c r="F14" s="14" t="inlineStr"/>
       <c r="G14" s="14" t="inlineStr">
         <is>
           <t>8.300 TL - 7,97 TL</t>

</xml_diff>

<commit_message>
Update benchmark: 2026-04-22 07:54:55 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -662,11 +662,7 @@
       <c r="D3" s="14" t="inlineStr"/>
       <c r="E3" s="14" t="inlineStr"/>
       <c r="F3" s="14" t="inlineStr"/>
-      <c r="G3" s="14" t="inlineStr">
-        <is>
-          <t>39,87 TRY - 79,76 TRY - 797,68 TRY</t>
-        </is>
-      </c>
+      <c r="G3" s="14" t="inlineStr"/>
       <c r="H3" s="14" t="inlineStr"/>
       <c r="I3" s="14" t="inlineStr"/>
       <c r="J3" s="14" t="inlineStr"/>
@@ -682,11 +678,7 @@
       <c r="D4" s="14" t="inlineStr"/>
       <c r="E4" s="14" t="inlineStr"/>
       <c r="F4" s="14" t="inlineStr"/>
-      <c r="G4" s="14" t="inlineStr">
-        <is>
-          <t>27,84 TRY - 55,69 TRY - 398,83 TRY</t>
-        </is>
-      </c>
+      <c r="G4" s="14" t="inlineStr"/>
       <c r="H4" s="14" t="inlineStr"/>
       <c r="I4" s="14" t="inlineStr"/>
       <c r="J4" s="14" t="inlineStr"/>
@@ -702,11 +694,7 @@
       <c r="D5" s="14" t="inlineStr"/>
       <c r="E5" s="14" t="inlineStr"/>
       <c r="F5" s="14" t="inlineStr"/>
-      <c r="G5" s="14" t="inlineStr">
-        <is>
-          <t>7,97 TRY - 15,96 TRY - 199,41 TRY</t>
-        </is>
-      </c>
+      <c r="G5" s="14" t="inlineStr"/>
       <c r="H5" s="14" t="inlineStr"/>
       <c r="I5" s="14" t="inlineStr"/>
       <c r="J5" s="14" t="inlineStr"/>
@@ -718,11 +706,7 @@
           <t>DÜZENLİ EFT</t>
         </is>
       </c>
-      <c r="C6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 199,41 TL</t>
-        </is>
-      </c>
+      <c r="C6" s="14" t="inlineStr"/>
       <c r="D6" s="14" t="inlineStr"/>
       <c r="E6" s="14" t="inlineStr">
         <is>
@@ -730,11 +714,7 @@
         </is>
       </c>
       <c r="F6" s="14" t="inlineStr"/>
-      <c r="G6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 99,71 TL</t>
-        </is>
-      </c>
+      <c r="G6" s="14" t="inlineStr"/>
       <c r="H6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
@@ -811,11 +791,7 @@
       <c r="D8" s="14" t="inlineStr"/>
       <c r="E8" s="14" t="inlineStr"/>
       <c r="F8" s="14" t="inlineStr"/>
-      <c r="G8" s="14" t="inlineStr">
-        <is>
-          <t>19,94 TRY - 39,88 TRY - 398,84 TRY</t>
-        </is>
-      </c>
+      <c r="G8" s="14" t="inlineStr"/>
       <c r="H8" s="14" t="inlineStr"/>
       <c r="I8" s="14" t="inlineStr"/>
       <c r="J8" s="14" t="inlineStr"/>
@@ -831,11 +807,7 @@
       <c r="D9" s="14" t="inlineStr"/>
       <c r="E9" s="14" t="inlineStr"/>
       <c r="F9" s="14" t="inlineStr"/>
-      <c r="G9" s="14" t="inlineStr">
-        <is>
-          <t>13,92 TRY - 27,85 TRY - 199,42 TRY</t>
-        </is>
-      </c>
+      <c r="G9" s="14" t="inlineStr"/>
       <c r="H9" s="14" t="inlineStr"/>
       <c r="I9" s="14" t="inlineStr"/>
       <c r="J9" s="14" t="inlineStr"/>
@@ -851,11 +823,7 @@
       <c r="D10" s="14" t="inlineStr"/>
       <c r="E10" s="14" t="inlineStr"/>
       <c r="F10" s="14" t="inlineStr"/>
-      <c r="G10" s="14" t="inlineStr">
-        <is>
-          <t>3,99 TRY - 7,98 TRY - 99,71 TRY</t>
-        </is>
-      </c>
+      <c r="G10" s="14" t="inlineStr"/>
       <c r="H10" s="14" t="inlineStr"/>
       <c r="I10" s="14" t="inlineStr"/>
       <c r="J10" s="14" t="inlineStr"/>
@@ -871,11 +839,7 @@
       <c r="D11" s="14" t="inlineStr"/>
       <c r="E11" s="14" t="inlineStr"/>
       <c r="F11" s="14" t="inlineStr"/>
-      <c r="G11" s="14" t="inlineStr">
-        <is>
-          <t>3,99 TRY - 7,98 TRY - 99,71 TRY</t>
-        </is>
-      </c>
+      <c r="G11" s="14" t="inlineStr"/>
       <c r="H11" s="14" t="inlineStr"/>
       <c r="I11" s="14" t="inlineStr"/>
       <c r="J11" s="14" t="inlineStr"/>
@@ -892,19 +856,11 @@
           <t>GİDEN SWIFT</t>
         </is>
       </c>
-      <c r="C12" s="14" t="inlineStr">
-        <is>
-          <t>WU: 1.000,01 USD–9,51 USD</t>
-        </is>
-      </c>
+      <c r="C12" s="14" t="inlineStr"/>
       <c r="D12" s="14" t="inlineStr"/>
       <c r="E12" s="14" t="inlineStr"/>
       <c r="F12" s="14" t="inlineStr"/>
-      <c r="G12" s="14" t="inlineStr">
-        <is>
-          <t>Şube (Kasadan): %0,5; Şube (Hesaptan): %0,75; İnternet: 15 USD</t>
-        </is>
-      </c>
+      <c r="G12" s="14" t="inlineStr"/>
       <c r="H12" s="14" t="inlineStr"/>
       <c r="I12" s="14" t="inlineStr"/>
       <c r="J12" s="14" t="inlineStr"/>
@@ -920,11 +876,7 @@
           <t>GELEN SWIFT</t>
         </is>
       </c>
-      <c r="C13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 0 TL | Azami 0,94 TL</t>
-        </is>
-      </c>
+      <c r="C13" s="14" t="inlineStr"/>
       <c r="D13" s="14" t="inlineStr"/>
       <c r="E13" s="14" t="inlineStr">
         <is>
@@ -960,23 +912,19 @@
           <t>GİDEN SWIFT - Mobil</t>
         </is>
       </c>
-      <c r="C14" s="14" t="inlineStr">
-        <is>
-          <t>40.000 TL - 2.485,72 TL</t>
-        </is>
-      </c>
+      <c r="C14" s="14" t="inlineStr"/>
       <c r="D14" s="14" t="inlineStr"/>
       <c r="E14" s="14" t="inlineStr">
         <is>
           <t>2.170 TL - 2.170 TL</t>
         </is>
       </c>
-      <c r="F14" s="14" t="inlineStr"/>
-      <c r="G14" s="14" t="inlineStr">
-        <is>
-          <t>8.300 TL - 7,97 TL</t>
-        </is>
-      </c>
+      <c r="F14" s="14" t="inlineStr">
+        <is>
+          <t>2.785,72 TL - 12.380,95 TL</t>
+        </is>
+      </c>
+      <c r="G14" s="14" t="inlineStr"/>
       <c r="H14" s="14" t="inlineStr">
         <is>
           <t>3.000 TL - 6.000 TL</t>

</xml_diff>

<commit_message>
Update benchmark: 2026-04-23 08:01:07 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -662,7 +662,11 @@
       <c r="D3" s="14" t="inlineStr"/>
       <c r="E3" s="14" t="inlineStr"/>
       <c r="F3" s="14" t="inlineStr"/>
-      <c r="G3" s="14" t="inlineStr"/>
+      <c r="G3" s="14" t="inlineStr">
+        <is>
+          <t>39,87 TRY - 79,76 TRY - 797,68 TRY</t>
+        </is>
+      </c>
       <c r="H3" s="14" t="inlineStr"/>
       <c r="I3" s="14" t="inlineStr"/>
       <c r="J3" s="14" t="inlineStr"/>
@@ -678,7 +682,11 @@
       <c r="D4" s="14" t="inlineStr"/>
       <c r="E4" s="14" t="inlineStr"/>
       <c r="F4" s="14" t="inlineStr"/>
-      <c r="G4" s="14" t="inlineStr"/>
+      <c r="G4" s="14" t="inlineStr">
+        <is>
+          <t>27,84 TRY - 55,69 TRY - 398,83 TRY</t>
+        </is>
+      </c>
       <c r="H4" s="14" t="inlineStr"/>
       <c r="I4" s="14" t="inlineStr"/>
       <c r="J4" s="14" t="inlineStr"/>
@@ -694,7 +702,11 @@
       <c r="D5" s="14" t="inlineStr"/>
       <c r="E5" s="14" t="inlineStr"/>
       <c r="F5" s="14" t="inlineStr"/>
-      <c r="G5" s="14" t="inlineStr"/>
+      <c r="G5" s="14" t="inlineStr">
+        <is>
+          <t>7,97 TRY - 15,96 TRY - 199,41 TRY</t>
+        </is>
+      </c>
       <c r="H5" s="14" t="inlineStr"/>
       <c r="I5" s="14" t="inlineStr"/>
       <c r="J5" s="14" t="inlineStr"/>
@@ -706,15 +718,27 @@
           <t>DÜZENLİ EFT</t>
         </is>
       </c>
-      <c r="C6" s="14" t="inlineStr"/>
-      <c r="D6" s="14" t="inlineStr"/>
+      <c r="C6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 199,41 TL</t>
+        </is>
+      </c>
+      <c r="D6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 199,41 TL</t>
+        </is>
+      </c>
       <c r="E6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
       <c r="F6" s="14" t="inlineStr"/>
-      <c r="G6" s="14" t="inlineStr"/>
+      <c r="G6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 99,71 TL</t>
+        </is>
+      </c>
       <c r="H6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
@@ -730,11 +754,7 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="K6" s="14" t="inlineStr">
-        <is>
-          <t>7,97 TL - 15,96 TL - 199,41 TL</t>
-        </is>
-      </c>
+      <c r="K6" s="14" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="B7" s="13" t="inlineStr">
@@ -791,7 +811,11 @@
       <c r="D8" s="14" t="inlineStr"/>
       <c r="E8" s="14" t="inlineStr"/>
       <c r="F8" s="14" t="inlineStr"/>
-      <c r="G8" s="14" t="inlineStr"/>
+      <c r="G8" s="14" t="inlineStr">
+        <is>
+          <t>19,94 TRY - 39,88 TRY - 398,84 TRY</t>
+        </is>
+      </c>
       <c r="H8" s="14" t="inlineStr"/>
       <c r="I8" s="14" t="inlineStr"/>
       <c r="J8" s="14" t="inlineStr"/>
@@ -807,7 +831,11 @@
       <c r="D9" s="14" t="inlineStr"/>
       <c r="E9" s="14" t="inlineStr"/>
       <c r="F9" s="14" t="inlineStr"/>
-      <c r="G9" s="14" t="inlineStr"/>
+      <c r="G9" s="14" t="inlineStr">
+        <is>
+          <t>13,92 TRY - 27,85 TRY - 199,42 TRY</t>
+        </is>
+      </c>
       <c r="H9" s="14" t="inlineStr"/>
       <c r="I9" s="14" t="inlineStr"/>
       <c r="J9" s="14" t="inlineStr"/>
@@ -823,7 +851,11 @@
       <c r="D10" s="14" t="inlineStr"/>
       <c r="E10" s="14" t="inlineStr"/>
       <c r="F10" s="14" t="inlineStr"/>
-      <c r="G10" s="14" t="inlineStr"/>
+      <c r="G10" s="14" t="inlineStr">
+        <is>
+          <t>3,99 TRY - 7,98 TRY - 99,71 TRY</t>
+        </is>
+      </c>
       <c r="H10" s="14" t="inlineStr"/>
       <c r="I10" s="14" t="inlineStr"/>
       <c r="J10" s="14" t="inlineStr"/>
@@ -839,7 +871,11 @@
       <c r="D11" s="14" t="inlineStr"/>
       <c r="E11" s="14" t="inlineStr"/>
       <c r="F11" s="14" t="inlineStr"/>
-      <c r="G11" s="14" t="inlineStr"/>
+      <c r="G11" s="14" t="inlineStr">
+        <is>
+          <t>3,99 TRY - 7,98 TRY - 99,71 TRY</t>
+        </is>
+      </c>
       <c r="H11" s="14" t="inlineStr"/>
       <c r="I11" s="14" t="inlineStr"/>
       <c r="J11" s="14" t="inlineStr"/>
@@ -856,19 +892,27 @@
           <t>GİDEN SWIFT</t>
         </is>
       </c>
-      <c r="C12" s="14" t="inlineStr"/>
-      <c r="D12" s="14" t="inlineStr"/>
+      <c r="C12" s="14" t="inlineStr">
+        <is>
+          <t>WU: 1.000,01 USD–9,51 USD</t>
+        </is>
+      </c>
+      <c r="D12" s="14" t="inlineStr">
+        <is>
+          <t>WU: 0,75 USD–12 USD; Diğer: 700 TL–4.000 TL</t>
+        </is>
+      </c>
       <c r="E12" s="14" t="inlineStr"/>
       <c r="F12" s="14" t="inlineStr"/>
-      <c r="G12" s="14" t="inlineStr"/>
+      <c r="G12" s="14" t="inlineStr">
+        <is>
+          <t>Şube (Kasadan): %0,5; Şube (Hesaptan): %0,75; İnternet: 15 USD</t>
+        </is>
+      </c>
       <c r="H12" s="14" t="inlineStr"/>
       <c r="I12" s="14" t="inlineStr"/>
       <c r="J12" s="14" t="inlineStr"/>
-      <c r="K12" s="14" t="inlineStr">
-        <is>
-          <t>WU: ,USD–; Diğer: 529 TL–4.454,74 TL</t>
-        </is>
-      </c>
+      <c r="K12" s="14" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="B13" s="13" t="inlineStr">
@@ -876,8 +920,16 @@
           <t>GELEN SWIFT</t>
         </is>
       </c>
-      <c r="C13" s="14" t="inlineStr"/>
-      <c r="D13" s="14" t="inlineStr"/>
+      <c r="C13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 0 TL | Azami 0,94 TL</t>
+        </is>
+      </c>
+      <c r="D13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
+        </is>
+      </c>
       <c r="E13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
@@ -900,11 +952,7 @@
           <t>Hesaba: Asgari 1 TL | Azami 1.303 TL</t>
         </is>
       </c>
-      <c r="K13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 865,75 TL</t>
-        </is>
-      </c>
+      <c r="K13" s="14" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="B14" s="13" t="inlineStr">
@@ -912,8 +960,16 @@
           <t>GİDEN SWIFT - Mobil</t>
         </is>
       </c>
-      <c r="C14" s="14" t="inlineStr"/>
-      <c r="D14" s="14" t="inlineStr"/>
+      <c r="C14" s="14" t="inlineStr">
+        <is>
+          <t>40.000 TL - 2.485,72 TL</t>
+        </is>
+      </c>
+      <c r="D14" s="14" t="inlineStr">
+        <is>
+          <t>3.500 TL - 13.500 TL</t>
+        </is>
+      </c>
       <c r="E14" s="14" t="inlineStr">
         <is>
           <t>2.170 TL - 2.170 TL</t>
@@ -924,7 +980,11 @@
           <t>2.785,72 TL - 12.380,95 TL</t>
         </is>
       </c>
-      <c r="G14" s="14" t="inlineStr"/>
+      <c r="G14" s="14" t="inlineStr">
+        <is>
+          <t>8.300 TL - 7,97 TL</t>
+        </is>
+      </c>
       <c r="H14" s="14" t="inlineStr">
         <is>
           <t>3.000 TL - 6.000 TL</t>
@@ -936,11 +996,7 @@
           <t>1.554,97 TL - 7.784 TL</t>
         </is>
       </c>
-      <c r="K14" s="14" t="inlineStr">
-        <is>
-          <t>1.196,51 TL - 5.583,74 TL</t>
-        </is>
-      </c>
+      <c r="K14" s="14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="12" t="inlineStr">

</xml_diff>

<commit_message>
Update benchmark: 2026-04-24 08:12:08 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -754,7 +754,11 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="K6" s="14" t="inlineStr"/>
+      <c r="K6" s="14" t="inlineStr">
+        <is>
+          <t>7,97 TL - 15,96 TL - 199,41 TL</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="B7" s="13" t="inlineStr">
@@ -912,7 +916,11 @@
       <c r="H12" s="14" t="inlineStr"/>
       <c r="I12" s="14" t="inlineStr"/>
       <c r="J12" s="14" t="inlineStr"/>
-      <c r="K12" s="14" t="inlineStr"/>
+      <c r="K12" s="14" t="inlineStr">
+        <is>
+          <t>WU: ,USD–; Diğer: 529 TL–4.454,74 TL</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="B13" s="13" t="inlineStr">
@@ -952,7 +960,11 @@
           <t>Hesaba: Asgari 1 TL | Azami 1.303 TL</t>
         </is>
       </c>
-      <c r="K13" s="14" t="inlineStr"/>
+      <c r="K13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 865,75 TL</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="B14" s="13" t="inlineStr">
@@ -996,7 +1008,11 @@
           <t>1.554,97 TL - 7.784 TL</t>
         </is>
       </c>
-      <c r="K14" s="14" t="inlineStr"/>
+      <c r="K14" s="14" t="inlineStr">
+        <is>
+          <t>1.196,51 TL - 5.583,74 TL</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="12" t="inlineStr">

</xml_diff>

<commit_message>
Update benchmark: 2026-04-29 08:27:16 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -718,47 +718,27 @@
           <t>DÜZENLİ EFT</t>
         </is>
       </c>
-      <c r="C6" s="14" t="inlineStr">
+      <c r="C6" s="14" t="inlineStr"/>
+      <c r="D6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="D6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 199,41 TL</t>
-        </is>
-      </c>
-      <c r="E6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 199,41 TL</t>
-        </is>
-      </c>
+      <c r="E6" s="14" t="inlineStr"/>
       <c r="F6" s="14" t="inlineStr"/>
       <c r="G6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 99,71 TL</t>
         </is>
       </c>
-      <c r="H6" s="14" t="inlineStr">
+      <c r="H6" s="14" t="inlineStr"/>
+      <c r="I6" s="14" t="inlineStr"/>
+      <c r="J6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="I6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 199,41 TL</t>
-        </is>
-      </c>
-      <c r="J6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 199,41 TL</t>
-        </is>
-      </c>
-      <c r="K6" s="14" t="inlineStr">
-        <is>
-          <t>7,97 TL - 15,96 TL - 199,41 TL</t>
-        </is>
-      </c>
+      <c r="K6" s="14" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="B7" s="13" t="inlineStr">
@@ -896,11 +876,7 @@
           <t>GİDEN SWIFT</t>
         </is>
       </c>
-      <c r="C12" s="14" t="inlineStr">
-        <is>
-          <t>WU: 1.000,01 USD–9,51 USD</t>
-        </is>
-      </c>
+      <c r="C12" s="14" t="inlineStr"/>
       <c r="D12" s="14" t="inlineStr">
         <is>
           <t>WU: 0,75 USD–12 USD; Diğer: 700 TL–4.000 TL</t>
@@ -916,11 +892,7 @@
       <c r="H12" s="14" t="inlineStr"/>
       <c r="I12" s="14" t="inlineStr"/>
       <c r="J12" s="14" t="inlineStr"/>
-      <c r="K12" s="14" t="inlineStr">
-        <is>
-          <t>WU: ,USD–; Diğer: 529 TL–4.454,74 TL</t>
-        </is>
-      </c>
+      <c r="K12" s="14" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="B13" s="13" t="inlineStr">
@@ -928,43 +900,23 @@
           <t>GELEN SWIFT</t>
         </is>
       </c>
-      <c r="C13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 0 TL | Azami 0,94 TL</t>
-        </is>
-      </c>
+      <c r="C13" s="14" t="inlineStr"/>
       <c r="D13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
         </is>
       </c>
-      <c r="E13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
-        </is>
-      </c>
+      <c r="E13" s="14" t="inlineStr"/>
       <c r="F13" s="14" t="inlineStr"/>
       <c r="G13" s="14" t="inlineStr"/>
-      <c r="H13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
-        </is>
-      </c>
-      <c r="I13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
-        </is>
-      </c>
+      <c r="H13" s="14" t="inlineStr"/>
+      <c r="I13" s="14" t="inlineStr"/>
       <c r="J13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.303 TL</t>
         </is>
       </c>
-      <c r="K13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 865,75 TL</t>
-        </is>
-      </c>
+      <c r="K13" s="14" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="B14" s="13" t="inlineStr">
@@ -972,47 +924,27 @@
           <t>GİDEN SWIFT - Mobil</t>
         </is>
       </c>
-      <c r="C14" s="14" t="inlineStr">
-        <is>
-          <t>40.000 TL - 2.485,72 TL</t>
-        </is>
-      </c>
+      <c r="C14" s="14" t="inlineStr"/>
       <c r="D14" s="14" t="inlineStr">
         <is>
           <t>3.500 TL - 13.500 TL</t>
         </is>
       </c>
-      <c r="E14" s="14" t="inlineStr">
-        <is>
-          <t>2.170 TL - 2.170 TL</t>
-        </is>
-      </c>
-      <c r="F14" s="14" t="inlineStr">
-        <is>
-          <t>2.785,72 TL - 12.380,95 TL</t>
-        </is>
-      </c>
+      <c r="E14" s="14" t="inlineStr"/>
+      <c r="F14" s="14" t="inlineStr"/>
       <c r="G14" s="14" t="inlineStr">
         <is>
           <t>8.300 TL - 7,97 TL</t>
         </is>
       </c>
-      <c r="H14" s="14" t="inlineStr">
-        <is>
-          <t>3.000 TL - 6.000 TL</t>
-        </is>
-      </c>
+      <c r="H14" s="14" t="inlineStr"/>
       <c r="I14" s="14" t="inlineStr"/>
       <c r="J14" s="14" t="inlineStr">
         <is>
           <t>1.554,97 TL - 7.784 TL</t>
         </is>
       </c>
-      <c r="K14" s="14" t="inlineStr">
-        <is>
-          <t>1.196,51 TL - 5.583,74 TL</t>
-        </is>
-      </c>
+      <c r="K14" s="14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="12" t="inlineStr">
@@ -1057,7 +989,7 @@
       </c>
       <c r="I15" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Asgari Tutar: 170 TL Azami Tutar: 170 TL / 170 TL</t>
+          <t xml:space="preserve"> Asgari Tutar: 220 TL Azami Tutar: 220 TL / 220 TL</t>
         </is>
       </c>
       <c r="J15" s="14" t="inlineStr">
@@ -1125,7 +1057,7 @@
       </c>
       <c r="I17" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Asgari Tutar: 170 TL Azami Tutar: </t>
+          <t xml:space="preserve"> Asgari Tutar: 220 TL Azami Tutar: </t>
         </is>
       </c>
       <c r="J17" s="14" t="inlineStr">
@@ -1205,7 +1137,7 @@
       </c>
       <c r="I20" s="14" t="inlineStr">
         <is>
-          <t>25 TL</t>
+          <t>30 TL</t>
         </is>
       </c>
       <c r="J20" s="14" t="inlineStr">
@@ -1257,7 +1189,7 @@
       </c>
       <c r="I21" s="14" t="inlineStr">
         <is>
-          <t>%0,5 Asgari Tutar: 185 TL Azami Tutar: 185 TL / 1.780 TL</t>
+          <t>%0,5 Asgari Tutar: 240 TL Azami Tutar: 240 TL / 2.325 TL</t>
         </is>
       </c>
       <c r="J21" s="14" t="inlineStr">
@@ -1309,7 +1241,7 @@
       </c>
       <c r="I22" s="14" t="inlineStr">
         <is>
-          <t>%0,32 Asgari Tutar: 230 TL Azami Tutar: 230 TL / 230 TL</t>
+          <t>%0,32 Asgari Tutar: 300 TL Azami Tutar: 300 TL / 300 TL</t>
         </is>
       </c>
       <c r="J22" s="14" t="inlineStr">
@@ -1361,7 +1293,7 @@
       </c>
       <c r="I23" s="14" t="inlineStr">
         <is>
-          <t>350 TL</t>
+          <t>455 TL</t>
         </is>
       </c>
       <c r="J23" s="14" t="inlineStr">
@@ -1466,7 +1398,7 @@
       </c>
       <c r="I25" s="14" t="inlineStr">
         <is>
-          <t>230 TL</t>
+          <t>300 TL</t>
         </is>
       </c>
       <c r="J25" s="14" t="inlineStr">

</xml_diff>

<commit_message>
Update benchmark: 2026-04-30 08:30:35 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -606,11 +606,7 @@
           <t>30 TL - 30 TL</t>
         </is>
       </c>
-      <c r="D2" s="14" t="inlineStr">
-        <is>
-          <t>33,33 TL - 33,33 TL</t>
-        </is>
-      </c>
+      <c r="D2" s="14" t="inlineStr"/>
       <c r="E2" s="14" t="inlineStr">
         <is>
           <t>26 TL - 26 TL</t>
@@ -724,21 +720,37 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="E6" s="14" t="inlineStr"/>
+      <c r="E6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 199,41 TL</t>
+        </is>
+      </c>
       <c r="F6" s="14" t="inlineStr"/>
       <c r="G6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 99,71 TL</t>
         </is>
       </c>
-      <c r="H6" s="14" t="inlineStr"/>
-      <c r="I6" s="14" t="inlineStr"/>
+      <c r="H6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 199,41 TL</t>
+        </is>
+      </c>
+      <c r="I6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 199,41 TL</t>
+        </is>
+      </c>
       <c r="J6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="K6" s="14" t="inlineStr"/>
+      <c r="K6" s="14" t="inlineStr">
+        <is>
+          <t>7,97 TL - 15,96 TL - 199,41 TL</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="B7" s="13" t="inlineStr">
@@ -747,11 +759,7 @@
         </is>
       </c>
       <c r="C7" s="14" t="inlineStr"/>
-      <c r="D7" s="14" t="inlineStr">
-        <is>
-          <t>%1,6</t>
-        </is>
-      </c>
+      <c r="D7" s="14" t="inlineStr"/>
       <c r="E7" s="14" t="inlineStr"/>
       <c r="F7" s="14" t="inlineStr">
         <is>
@@ -892,7 +900,11 @@
       <c r="H12" s="14" t="inlineStr"/>
       <c r="I12" s="14" t="inlineStr"/>
       <c r="J12" s="14" t="inlineStr"/>
-      <c r="K12" s="14" t="inlineStr"/>
+      <c r="K12" s="14" t="inlineStr">
+        <is>
+          <t>WU: ,USD–; Diğer: 529 TL–4.454,74 TL</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="B13" s="13" t="inlineStr">
@@ -906,17 +918,33 @@
           <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
         </is>
       </c>
-      <c r="E13" s="14" t="inlineStr"/>
+      <c r="E13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
+        </is>
+      </c>
       <c r="F13" s="14" t="inlineStr"/>
       <c r="G13" s="14" t="inlineStr"/>
-      <c r="H13" s="14" t="inlineStr"/>
-      <c r="I13" s="14" t="inlineStr"/>
+      <c r="H13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
+        </is>
+      </c>
+      <c r="I13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
+        </is>
+      </c>
       <c r="J13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.303 TL</t>
         </is>
       </c>
-      <c r="K13" s="14" t="inlineStr"/>
+      <c r="K13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 865,75 TL</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="B14" s="13" t="inlineStr">
@@ -930,21 +958,37 @@
           <t>3.500 TL - 13.500 TL</t>
         </is>
       </c>
-      <c r="E14" s="14" t="inlineStr"/>
-      <c r="F14" s="14" t="inlineStr"/>
+      <c r="E14" s="14" t="inlineStr">
+        <is>
+          <t>2.170 TL - 2.170 TL</t>
+        </is>
+      </c>
+      <c r="F14" s="14" t="inlineStr">
+        <is>
+          <t>2.785,72 TL - 12.380,95 TL</t>
+        </is>
+      </c>
       <c r="G14" s="14" t="inlineStr">
         <is>
           <t>8.300 TL - 7,97 TL</t>
         </is>
       </c>
-      <c r="H14" s="14" t="inlineStr"/>
+      <c r="H14" s="14" t="inlineStr">
+        <is>
+          <t>3.000 TL - 6.000 TL</t>
+        </is>
+      </c>
       <c r="I14" s="14" t="inlineStr"/>
       <c r="J14" s="14" t="inlineStr">
         <is>
           <t>1.554,97 TL - 7.784 TL</t>
         </is>
       </c>
-      <c r="K14" s="14" t="inlineStr"/>
+      <c r="K14" s="14" t="inlineStr">
+        <is>
+          <t>1.196,51 TL - 5.583,74 TL</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="12" t="inlineStr">
@@ -1323,11 +1367,7 @@
           <t>600 TL</t>
         </is>
       </c>
-      <c r="D24" s="14" t="inlineStr">
-        <is>
-          <t>476,2 TL</t>
-        </is>
-      </c>
+      <c r="D24" s="14" t="inlineStr"/>
       <c r="E24" s="14" t="inlineStr">
         <is>
           <t>780 TL</t>
@@ -1375,11 +1415,7 @@
           <t>495,24 TL</t>
         </is>
       </c>
-      <c r="D25" s="14" t="inlineStr">
-        <is>
-          <t>428,58 TL</t>
-        </is>
-      </c>
+      <c r="D25" s="14" t="inlineStr"/>
       <c r="E25" s="14" t="inlineStr">
         <is>
           <t>780 TL</t>

</xml_diff>

<commit_message>
Update benchmark: 2026-05-01 08:20:02 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -606,7 +606,11 @@
           <t>30 TL - 30 TL</t>
         </is>
       </c>
-      <c r="D2" s="14" t="inlineStr"/>
+      <c r="D2" s="14" t="inlineStr">
+        <is>
+          <t>33,33 TL - 33,33 TL</t>
+        </is>
+      </c>
       <c r="E2" s="14" t="inlineStr">
         <is>
           <t>26 TL - 26 TL</t>
@@ -714,12 +718,12 @@
           <t>DÜZENLİ EFT</t>
         </is>
       </c>
-      <c r="C6" s="14" t="inlineStr"/>
-      <c r="D6" s="14" t="inlineStr">
+      <c r="C6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
+      <c r="D6" s="14" t="inlineStr"/>
       <c r="E6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
@@ -759,7 +763,11 @@
         </is>
       </c>
       <c r="C7" s="14" t="inlineStr"/>
-      <c r="D7" s="14" t="inlineStr"/>
+      <c r="D7" s="14" t="inlineStr">
+        <is>
+          <t>%1,6</t>
+        </is>
+      </c>
       <c r="E7" s="14" t="inlineStr"/>
       <c r="F7" s="14" t="inlineStr">
         <is>
@@ -884,12 +892,12 @@
           <t>GİDEN SWIFT</t>
         </is>
       </c>
-      <c r="C12" s="14" t="inlineStr"/>
-      <c r="D12" s="14" t="inlineStr">
-        <is>
-          <t>WU: 0,75 USD–12 USD; Diğer: 700 TL–4.000 TL</t>
-        </is>
-      </c>
+      <c r="C12" s="14" t="inlineStr">
+        <is>
+          <t>WU: 1.000,01 USD–9,51 USD</t>
+        </is>
+      </c>
+      <c r="D12" s="14" t="inlineStr"/>
       <c r="E12" s="14" t="inlineStr"/>
       <c r="F12" s="14" t="inlineStr"/>
       <c r="G12" s="14" t="inlineStr">
@@ -912,12 +920,12 @@
           <t>GELEN SWIFT</t>
         </is>
       </c>
-      <c r="C13" s="14" t="inlineStr"/>
-      <c r="D13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
-        </is>
-      </c>
+      <c r="C13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 0 TL | Azami 0,94 TL</t>
+        </is>
+      </c>
+      <c r="D13" s="14" t="inlineStr"/>
       <c r="E13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
@@ -952,22 +960,18 @@
           <t>GİDEN SWIFT - Mobil</t>
         </is>
       </c>
-      <c r="C14" s="14" t="inlineStr"/>
-      <c r="D14" s="14" t="inlineStr">
-        <is>
-          <t>3.500 TL - 13.500 TL</t>
-        </is>
-      </c>
+      <c r="C14" s="14" t="inlineStr">
+        <is>
+          <t>40.000 TL - 2.485,72 TL</t>
+        </is>
+      </c>
+      <c r="D14" s="14" t="inlineStr"/>
       <c r="E14" s="14" t="inlineStr">
         <is>
           <t>2.170 TL - 2.170 TL</t>
         </is>
       </c>
-      <c r="F14" s="14" t="inlineStr">
-        <is>
-          <t>2.785,72 TL - 12.380,95 TL</t>
-        </is>
-      </c>
+      <c r="F14" s="14" t="inlineStr"/>
       <c r="G14" s="14" t="inlineStr">
         <is>
           <t>8.300 TL - 7,97 TL</t>
@@ -1367,7 +1371,11 @@
           <t>600 TL</t>
         </is>
       </c>
-      <c r="D24" s="14" t="inlineStr"/>
+      <c r="D24" s="14" t="inlineStr">
+        <is>
+          <t>476,2 TL</t>
+        </is>
+      </c>
       <c r="E24" s="14" t="inlineStr">
         <is>
           <t>780 TL</t>
@@ -1415,7 +1423,11 @@
           <t>495,24 TL</t>
         </is>
       </c>
-      <c r="D25" s="14" t="inlineStr"/>
+      <c r="D25" s="14" t="inlineStr">
+        <is>
+          <t>428,58 TL</t>
+        </is>
+      </c>
       <c r="E25" s="14" t="inlineStr">
         <is>
           <t>780 TL</t>

</xml_diff>

<commit_message>
Update benchmark: 2026-05-02 07:53:19 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -723,7 +723,11 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="D6" s="14" t="inlineStr"/>
+      <c r="D6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 199,41 TL</t>
+        </is>
+      </c>
       <c r="E6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
@@ -740,11 +744,7 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="I6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 199,41 TL</t>
-        </is>
-      </c>
+      <c r="I6" s="14" t="inlineStr"/>
       <c r="J6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
@@ -897,7 +897,11 @@
           <t>WU: 1.000,01 USD–9,51 USD</t>
         </is>
       </c>
-      <c r="D12" s="14" t="inlineStr"/>
+      <c r="D12" s="14" t="inlineStr">
+        <is>
+          <t>WU: 0,75 USD–12 USD; Diğer: 700 TL–4.000 TL</t>
+        </is>
+      </c>
       <c r="E12" s="14" t="inlineStr"/>
       <c r="F12" s="14" t="inlineStr"/>
       <c r="G12" s="14" t="inlineStr">
@@ -925,7 +929,11 @@
           <t>Hesaba: Asgari 0 TL | Azami 0,94 TL</t>
         </is>
       </c>
-      <c r="D13" s="14" t="inlineStr"/>
+      <c r="D13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
+        </is>
+      </c>
       <c r="E13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
@@ -938,11 +946,7 @@
           <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
         </is>
       </c>
-      <c r="I13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
-        </is>
-      </c>
+      <c r="I13" s="14" t="inlineStr"/>
       <c r="J13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.303 TL</t>
@@ -965,13 +969,21 @@
           <t>40.000 TL - 2.485,72 TL</t>
         </is>
       </c>
-      <c r="D14" s="14" t="inlineStr"/>
+      <c r="D14" s="14" t="inlineStr">
+        <is>
+          <t>3.500 TL - 13.500 TL</t>
+        </is>
+      </c>
       <c r="E14" s="14" t="inlineStr">
         <is>
           <t>2.170 TL - 2.170 TL</t>
         </is>
       </c>
-      <c r="F14" s="14" t="inlineStr"/>
+      <c r="F14" s="14" t="inlineStr">
+        <is>
+          <t>2.785,72 TL - 12.380,95 TL</t>
+        </is>
+      </c>
       <c r="G14" s="14" t="inlineStr">
         <is>
           <t>8.300 TL - 7,97 TL</t>

</xml_diff>

<commit_message>
Update benchmark: 2026-05-03 08:10:00 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -739,12 +739,12 @@
           <t>8.300,01 TL - 99,71 TL</t>
         </is>
       </c>
-      <c r="H6" s="14" t="inlineStr">
+      <c r="H6" s="14" t="inlineStr"/>
+      <c r="I6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="I6" s="14" t="inlineStr"/>
       <c r="J6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
@@ -941,12 +941,12 @@
       </c>
       <c r="F13" s="14" t="inlineStr"/>
       <c r="G13" s="14" t="inlineStr"/>
-      <c r="H13" s="14" t="inlineStr">
+      <c r="H13" s="14" t="inlineStr"/>
+      <c r="I13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
         </is>
       </c>
-      <c r="I13" s="14" t="inlineStr"/>
       <c r="J13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.303 TL</t>
@@ -989,11 +989,7 @@
           <t>8.300 TL - 7,97 TL</t>
         </is>
       </c>
-      <c r="H14" s="14" t="inlineStr">
-        <is>
-          <t>3.000 TL - 6.000 TL</t>
-        </is>
-      </c>
+      <c r="H14" s="14" t="inlineStr"/>
       <c r="I14" s="14" t="inlineStr"/>
       <c r="J14" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update benchmark: 2026-05-04 08:37:36 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -723,11 +723,7 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="D6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 199,41 TL</t>
-        </is>
-      </c>
+      <c r="D6" s="14" t="inlineStr"/>
       <c r="E6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
@@ -739,7 +735,11 @@
           <t>8.300,01 TL - 99,71 TL</t>
         </is>
       </c>
-      <c r="H6" s="14" t="inlineStr"/>
+      <c r="H6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 199,41 TL</t>
+        </is>
+      </c>
       <c r="I6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
@@ -897,11 +897,7 @@
           <t>WU: 1.000,01 USD–9,51 USD</t>
         </is>
       </c>
-      <c r="D12" s="14" t="inlineStr">
-        <is>
-          <t>WU: 0,75 USD–12 USD; Diğer: 700 TL–4.000 TL</t>
-        </is>
-      </c>
+      <c r="D12" s="14" t="inlineStr"/>
       <c r="E12" s="14" t="inlineStr"/>
       <c r="F12" s="14" t="inlineStr"/>
       <c r="G12" s="14" t="inlineStr">
@@ -929,11 +925,7 @@
           <t>Hesaba: Asgari 0 TL | Azami 0,94 TL</t>
         </is>
       </c>
-      <c r="D13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
-        </is>
-      </c>
+      <c r="D13" s="14" t="inlineStr"/>
       <c r="E13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
@@ -941,7 +933,11 @@
       </c>
       <c r="F13" s="14" t="inlineStr"/>
       <c r="G13" s="14" t="inlineStr"/>
-      <c r="H13" s="14" t="inlineStr"/>
+      <c r="H13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
+        </is>
+      </c>
       <c r="I13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
@@ -969,11 +965,7 @@
           <t>40.000 TL - 2.485,72 TL</t>
         </is>
       </c>
-      <c r="D14" s="14" t="inlineStr">
-        <is>
-          <t>3.500 TL - 13.500 TL</t>
-        </is>
-      </c>
+      <c r="D14" s="14" t="inlineStr"/>
       <c r="E14" s="14" t="inlineStr">
         <is>
           <t>2.170 TL - 2.170 TL</t>
@@ -989,7 +981,11 @@
           <t>8.300 TL - 7,97 TL</t>
         </is>
       </c>
-      <c r="H14" s="14" t="inlineStr"/>
+      <c r="H14" s="14" t="inlineStr">
+        <is>
+          <t>3.000 TL - 6.000 TL</t>
+        </is>
+      </c>
       <c r="I14" s="14" t="inlineStr"/>
       <c r="J14" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update benchmark: 2026-05-05 08:18:12 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -601,11 +601,7 @@
         </is>
       </c>
       <c r="B2" s="13" t="inlineStr"/>
-      <c r="C2" s="14" t="inlineStr">
-        <is>
-          <t>30 TL - 30 TL</t>
-        </is>
-      </c>
+      <c r="C2" s="14" t="inlineStr"/>
       <c r="D2" s="14" t="inlineStr">
         <is>
           <t>33,33 TL - 33,33 TL</t>
@@ -616,31 +612,19 @@
           <t>26 TL - 26 TL</t>
         </is>
       </c>
-      <c r="F2" s="14" t="inlineStr">
-        <is>
-          <t>33,33 TL - 33,33 TL</t>
-        </is>
-      </c>
-      <c r="G2" s="14" t="inlineStr">
+      <c r="F2" s="14" t="inlineStr"/>
+      <c r="G2" s="14" t="inlineStr"/>
+      <c r="H2" s="14" t="inlineStr">
         <is>
           <t>15 TL - 15 TL</t>
         </is>
       </c>
-      <c r="H2" s="14" t="inlineStr">
-        <is>
-          <t>15 TL - 15 TL</t>
-        </is>
-      </c>
       <c r="I2" s="14" t="inlineStr">
         <is>
           <t>18 TL - 18 TL</t>
         </is>
       </c>
-      <c r="J2" s="14" t="inlineStr">
-        <is>
-          <t>65 TL - 65 TL</t>
-        </is>
-      </c>
+      <c r="J2" s="14" t="inlineStr"/>
       <c r="K2" s="14" t="inlineStr">
         <is>
           <t>32,62 TL - 32,62 TL</t>
@@ -723,7 +707,11 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="D6" s="14" t="inlineStr"/>
+      <c r="D6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 199,41 TL</t>
+        </is>
+      </c>
       <c r="E6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
@@ -769,27 +757,15 @@
         </is>
       </c>
       <c r="E7" s="14" t="inlineStr"/>
-      <c r="F7" s="14" t="inlineStr">
-        <is>
-          <t>%3</t>
-        </is>
-      </c>
-      <c r="G7" s="14" t="inlineStr">
-        <is>
-          <t>1 TRY (Kredi kartı ile ödemelerde ek olarak nakit avans faizi uygulanır.)</t>
-        </is>
-      </c>
+      <c r="F7" s="14" t="inlineStr"/>
+      <c r="G7" s="14" t="inlineStr"/>
       <c r="H7" s="14" t="inlineStr">
         <is>
           <t>%3,09</t>
         </is>
       </c>
       <c r="I7" s="14" t="inlineStr"/>
-      <c r="J7" s="14" t="inlineStr">
-        <is>
-          <t>%3,5</t>
-        </is>
-      </c>
+      <c r="J7" s="14" t="inlineStr"/>
       <c r="K7" s="14" t="inlineStr">
         <is>
           <t>%3,1</t>
@@ -894,10 +870,14 @@
       </c>
       <c r="C12" s="14" t="inlineStr">
         <is>
-          <t>WU: 1.000,01 USD–9,51 USD</t>
-        </is>
-      </c>
-      <c r="D12" s="14" t="inlineStr"/>
+          <t>WU: 1.000,01 USD–</t>
+        </is>
+      </c>
+      <c r="D12" s="14" t="inlineStr">
+        <is>
+          <t>WU: 0,75 USD–12 USD; Diğer: 700 TL–4.000 TL</t>
+        </is>
+      </c>
       <c r="E12" s="14" t="inlineStr"/>
       <c r="F12" s="14" t="inlineStr"/>
       <c r="G12" s="14" t="inlineStr">
@@ -922,13 +902,17 @@
       </c>
       <c r="C13" s="14" t="inlineStr">
         <is>
-          <t>Hesaba: Asgari 0 TL | Azami 0,94 TL</t>
-        </is>
-      </c>
-      <c r="D13" s="14" t="inlineStr"/>
+          <t>Hesaba: Asgari 0 TL | Azami 3.295,24 TL</t>
+        </is>
+      </c>
+      <c r="D13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
+        </is>
+      </c>
       <c r="E13" s="14" t="inlineStr">
         <is>
-          <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
+          <t>Hesaba: Asgari 1 TL | Azami 11.380 TL</t>
         </is>
       </c>
       <c r="F13" s="14" t="inlineStr"/>
@@ -950,7 +934,7 @@
       </c>
       <c r="K13" s="14" t="inlineStr">
         <is>
-          <t>Hesaba: Asgari 1 TL | Azami 865,75 TL</t>
+          <t>Hesaba: Asgari 1 TL | Azami 75 TL</t>
         </is>
       </c>
     </row>
@@ -965,7 +949,11 @@
           <t>40.000 TL - 2.485,72 TL</t>
         </is>
       </c>
-      <c r="D14" s="14" t="inlineStr"/>
+      <c r="D14" s="14" t="inlineStr">
+        <is>
+          <t>3.500 TL - 13.500 TL</t>
+        </is>
+      </c>
       <c r="E14" s="14" t="inlineStr">
         <is>
           <t>2.170 TL - 2.170 TL</t>
@@ -1051,7 +1039,7 @@
       </c>
       <c r="K15" s="14" t="inlineStr">
         <is>
-          <t>%0,3 Asgari Tutar: 237,26 TL Azami Tutar: 237,26 TL / 298,96 TL</t>
+          <t>%0,5 Asgari Tutar: 375 TL Azami Tutar: 375 TL / 6.500 TL</t>
         </is>
       </c>
     </row>
@@ -1119,7 +1107,7 @@
       </c>
       <c r="K17" s="14" t="inlineStr">
         <is>
-          <t>%0,6 Asgari Tutar: 237,26 TL Azami Tutar: 237,26 TL / 3.034,67 TL</t>
+          <t>%0,5 Asgari Tutar: 350 TL Azami Tutar: 350 TL / 5.500 TL</t>
         </is>
       </c>
     </row>
@@ -1199,7 +1187,7 @@
       </c>
       <c r="K20" s="14" t="inlineStr">
         <is>
-          <t>147,11 TL</t>
+          <t>200 TL</t>
         </is>
       </c>
     </row>
@@ -1251,7 +1239,7 @@
       </c>
       <c r="K21" s="14" t="inlineStr">
         <is>
-          <t>%0,9 Asgari Tutar: 446,06 TL Azami Tutar: 446,06 TL / 2.427,26 TL</t>
+          <t>%0,5 Asgari Tutar: 500 TL Azami Tutar: 500 TL / 5.000 TL</t>
         </is>
       </c>
     </row>
@@ -1303,7 +1291,7 @@
       </c>
       <c r="K22" s="14" t="inlineStr">
         <is>
-          <t>%0,3 Asgari Tutar: 73,56 TL Azami Tutar: 73,56 TL / 9.115,86 TL</t>
+          <t>%0,5 Asgari Tutar: 1.500 TL Azami Tutar: 1.500 TL / 9.000 TL</t>
         </is>
       </c>
     </row>
@@ -1355,7 +1343,7 @@
       </c>
       <c r="K23" s="14" t="inlineStr">
         <is>
-          <t>64,8 TL</t>
+          <t>75 TL</t>
         </is>
       </c>
     </row>
@@ -1405,14 +1393,10 @@
           <t>20 TL</t>
         </is>
       </c>
-      <c r="J24" s="14" t="inlineStr">
+      <c r="J24" s="14" t="inlineStr"/>
+      <c r="K24" s="14" t="inlineStr">
         <is>
           <t>500 TL</t>
-        </is>
-      </c>
-      <c r="K24" s="14" t="inlineStr">
-        <is>
-          <t>446,06 TL</t>
         </is>
       </c>
     </row>
@@ -1453,14 +1437,10 @@
           <t>300 TL</t>
         </is>
       </c>
-      <c r="J25" s="14" t="inlineStr">
+      <c r="J25" s="14" t="inlineStr"/>
+      <c r="K25" s="14" t="inlineStr">
         <is>
           <t>750 TL</t>
-        </is>
-      </c>
-      <c r="K25" s="14" t="inlineStr">
-        <is>
-          <t>374,4 TL</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update benchmark: 2026-05-07 08:44:13 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -601,7 +601,11 @@
         </is>
       </c>
       <c r="B2" s="13" t="inlineStr"/>
-      <c r="C2" s="14" t="inlineStr"/>
+      <c r="C2" s="14" t="inlineStr">
+        <is>
+          <t>30 TL - 30 TL</t>
+        </is>
+      </c>
       <c r="D2" s="14" t="inlineStr">
         <is>
           <t>33,33 TL - 33,33 TL</t>
@@ -612,8 +616,16 @@
           <t>26 TL - 26 TL</t>
         </is>
       </c>
-      <c r="F2" s="14" t="inlineStr"/>
-      <c r="G2" s="14" t="inlineStr"/>
+      <c r="F2" s="14" t="inlineStr">
+        <is>
+          <t>33,33 TL - 33,33 TL</t>
+        </is>
+      </c>
+      <c r="G2" s="14" t="inlineStr">
+        <is>
+          <t>15 TL - 15 TL</t>
+        </is>
+      </c>
       <c r="H2" s="14" t="inlineStr">
         <is>
           <t>15 TL - 15 TL</t>
@@ -624,7 +636,11 @@
           <t>18 TL - 18 TL</t>
         </is>
       </c>
-      <c r="J2" s="14" t="inlineStr"/>
+      <c r="J2" s="14" t="inlineStr">
+        <is>
+          <t>65 TL - 65 TL</t>
+        </is>
+      </c>
       <c r="K2" s="14" t="inlineStr">
         <is>
           <t>32,62 TL - 32,62 TL</t>
@@ -733,11 +749,7 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="J6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 199,41 TL</t>
-        </is>
-      </c>
+      <c r="J6" s="14" t="inlineStr"/>
       <c r="K6" s="14" t="inlineStr">
         <is>
           <t>7,97 TL - 15,96 TL - 199,41 TL</t>
@@ -757,15 +769,27 @@
         </is>
       </c>
       <c r="E7" s="14" t="inlineStr"/>
-      <c r="F7" s="14" t="inlineStr"/>
-      <c r="G7" s="14" t="inlineStr"/>
+      <c r="F7" s="14" t="inlineStr">
+        <is>
+          <t>%3</t>
+        </is>
+      </c>
+      <c r="G7" s="14" t="inlineStr">
+        <is>
+          <t>1 TRY (Kredi kartı ile ödemelerde ek olarak nakit avans faizi uygulanır.)</t>
+        </is>
+      </c>
       <c r="H7" s="14" t="inlineStr">
         <is>
           <t>%3,09</t>
         </is>
       </c>
       <c r="I7" s="14" t="inlineStr"/>
-      <c r="J7" s="14" t="inlineStr"/>
+      <c r="J7" s="14" t="inlineStr">
+        <is>
+          <t>%3,5</t>
+        </is>
+      </c>
       <c r="K7" s="14" t="inlineStr">
         <is>
           <t>%3,1</t>
@@ -870,7 +894,7 @@
       </c>
       <c r="C12" s="14" t="inlineStr">
         <is>
-          <t>WU: 1.000,01 USD–</t>
+          <t>WU: 1.000,01 USD–9,51 USD</t>
         </is>
       </c>
       <c r="D12" s="14" t="inlineStr">
@@ -902,7 +926,7 @@
       </c>
       <c r="C13" s="14" t="inlineStr">
         <is>
-          <t>Hesaba: Asgari 0 TL | Azami 3.295,24 TL</t>
+          <t>Hesaba: Asgari 0 TL | Azami 0,94 TL</t>
         </is>
       </c>
       <c r="D13" s="14" t="inlineStr">
@@ -912,7 +936,7 @@
       </c>
       <c r="E13" s="14" t="inlineStr">
         <is>
-          <t>Hesaba: Asgari 1 TL | Azami 11.380 TL</t>
+          <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
         </is>
       </c>
       <c r="F13" s="14" t="inlineStr"/>
@@ -927,14 +951,10 @@
           <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
         </is>
       </c>
-      <c r="J13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 1.303 TL</t>
-        </is>
-      </c>
+      <c r="J13" s="14" t="inlineStr"/>
       <c r="K13" s="14" t="inlineStr">
         <is>
-          <t>Hesaba: Asgari 1 TL | Azami 75 TL</t>
+          <t>Hesaba: Asgari 1 TL | Azami 865,75 TL</t>
         </is>
       </c>
     </row>
@@ -975,11 +995,7 @@
         </is>
       </c>
       <c r="I14" s="14" t="inlineStr"/>
-      <c r="J14" s="14" t="inlineStr">
-        <is>
-          <t>1.554,97 TL - 7.784 TL</t>
-        </is>
-      </c>
+      <c r="J14" s="14" t="inlineStr"/>
       <c r="K14" s="14" t="inlineStr">
         <is>
           <t>1.196,51 TL - 5.583,74 TL</t>
@@ -1039,7 +1055,7 @@
       </c>
       <c r="K15" s="14" t="inlineStr">
         <is>
-          <t>%0,5 Asgari Tutar: 375 TL Azami Tutar: 375 TL / 6.500 TL</t>
+          <t>%0,3 Asgari Tutar: 237,26 TL Azami Tutar: 237,26 TL / 298,96 TL</t>
         </is>
       </c>
     </row>
@@ -1107,7 +1123,7 @@
       </c>
       <c r="K17" s="14" t="inlineStr">
         <is>
-          <t>%0,5 Asgari Tutar: 350 TL Azami Tutar: 350 TL / 5.500 TL</t>
+          <t>%0,6 Asgari Tutar: 237,26 TL Azami Tutar: 237,26 TL / 3.034,67 TL</t>
         </is>
       </c>
     </row>
@@ -1187,7 +1203,7 @@
       </c>
       <c r="K20" s="14" t="inlineStr">
         <is>
-          <t>200 TL</t>
+          <t>147,11 TL</t>
         </is>
       </c>
     </row>
@@ -1239,7 +1255,7 @@
       </c>
       <c r="K21" s="14" t="inlineStr">
         <is>
-          <t>%0,5 Asgari Tutar: 500 TL Azami Tutar: 500 TL / 5.000 TL</t>
+          <t>%0,9 Asgari Tutar: 446,06 TL Azami Tutar: 446,06 TL / 2.427,26 TL</t>
         </is>
       </c>
     </row>
@@ -1291,7 +1307,7 @@
       </c>
       <c r="K22" s="14" t="inlineStr">
         <is>
-          <t>%0,5 Asgari Tutar: 1.500 TL Azami Tutar: 1.500 TL / 9.000 TL</t>
+          <t>%0,3 Asgari Tutar: 73,56 TL Azami Tutar: 73,56 TL / 9.115,86 TL</t>
         </is>
       </c>
     </row>
@@ -1343,7 +1359,7 @@
       </c>
       <c r="K23" s="14" t="inlineStr">
         <is>
-          <t>75 TL</t>
+          <t>64,8 TL</t>
         </is>
       </c>
     </row>
@@ -1393,10 +1409,14 @@
           <t>20 TL</t>
         </is>
       </c>
-      <c r="J24" s="14" t="inlineStr"/>
+      <c r="J24" s="14" t="inlineStr">
+        <is>
+          <t>500 TL</t>
+        </is>
+      </c>
       <c r="K24" s="14" t="inlineStr">
         <is>
-          <t>500 TL</t>
+          <t>446,06 TL</t>
         </is>
       </c>
     </row>
@@ -1437,10 +1457,14 @@
           <t>300 TL</t>
         </is>
       </c>
-      <c r="J25" s="14" t="inlineStr"/>
+      <c r="J25" s="14" t="inlineStr">
+        <is>
+          <t>750 TL</t>
+        </is>
+      </c>
       <c r="K25" s="14" t="inlineStr">
         <is>
-          <t>750 TL</t>
+          <t>374,4 TL</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update benchmark: 2026-05-08 07:50:26 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -749,7 +749,11 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="J6" s="14" t="inlineStr"/>
+      <c r="J6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 199,41 TL</t>
+        </is>
+      </c>
       <c r="K6" s="14" t="inlineStr">
         <is>
           <t>7,97 TL - 15,96 TL - 199,41 TL</t>
@@ -951,7 +955,11 @@
           <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
         </is>
       </c>
-      <c r="J13" s="14" t="inlineStr"/>
+      <c r="J13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 1.303 TL</t>
+        </is>
+      </c>
       <c r="K13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 865,75 TL</t>
@@ -995,7 +1003,11 @@
         </is>
       </c>
       <c r="I14" s="14" t="inlineStr"/>
-      <c r="J14" s="14" t="inlineStr"/>
+      <c r="J14" s="14" t="inlineStr">
+        <is>
+          <t>1.554,97 TL - 7.784 TL</t>
+        </is>
+      </c>
       <c r="K14" s="14" t="inlineStr">
         <is>
           <t>1.196,51 TL - 5.583,74 TL</t>

</xml_diff>

<commit_message>
Update benchmark: 2026-05-09 08:04:56 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -754,11 +754,7 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="K6" s="14" t="inlineStr">
-        <is>
-          <t>7,97 TL - 15,96 TL - 199,41 TL</t>
-        </is>
-      </c>
+      <c r="K6" s="14" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="B7" s="13" t="inlineStr">
@@ -916,11 +912,7 @@
       <c r="H12" s="14" t="inlineStr"/>
       <c r="I12" s="14" t="inlineStr"/>
       <c r="J12" s="14" t="inlineStr"/>
-      <c r="K12" s="14" t="inlineStr">
-        <is>
-          <t>WU: ,USD–; Diğer: 529 TL–4.454,74 TL</t>
-        </is>
-      </c>
+      <c r="K12" s="14" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="B13" s="13" t="inlineStr">
@@ -960,11 +952,7 @@
           <t>Hesaba: Asgari 1 TL | Azami 1.303 TL</t>
         </is>
       </c>
-      <c r="K13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 865,75 TL</t>
-        </is>
-      </c>
+      <c r="K13" s="14" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="B14" s="13" t="inlineStr">
@@ -1008,11 +996,7 @@
           <t>1.554,97 TL - 7.784 TL</t>
         </is>
       </c>
-      <c r="K14" s="14" t="inlineStr">
-        <is>
-          <t>1.196,51 TL - 5.583,74 TL</t>
-        </is>
-      </c>
+      <c r="K14" s="14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="12" t="inlineStr">

</xml_diff>

<commit_message>
Update benchmark: 2026-05-10 08:15:51 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -754,7 +754,11 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="K6" s="14" t="inlineStr"/>
+      <c r="K6" s="14" t="inlineStr">
+        <is>
+          <t>7,97 TL - 15,96 TL - 199,41 TL</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="B7" s="13" t="inlineStr">
@@ -912,7 +916,11 @@
       <c r="H12" s="14" t="inlineStr"/>
       <c r="I12" s="14" t="inlineStr"/>
       <c r="J12" s="14" t="inlineStr"/>
-      <c r="K12" s="14" t="inlineStr"/>
+      <c r="K12" s="14" t="inlineStr">
+        <is>
+          <t>WU: ,USD–; Diğer: 529 TL–4.454,74 TL</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="B13" s="13" t="inlineStr">
@@ -952,7 +960,11 @@
           <t>Hesaba: Asgari 1 TL | Azami 1.303 TL</t>
         </is>
       </c>
-      <c r="K13" s="14" t="inlineStr"/>
+      <c r="K13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 865,75 TL</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="B14" s="13" t="inlineStr">
@@ -996,7 +1008,11 @@
           <t>1.554,97 TL - 7.784 TL</t>
         </is>
       </c>
-      <c r="K14" s="14" t="inlineStr"/>
+      <c r="K14" s="14" t="inlineStr">
+        <is>
+          <t>1.196,51 TL - 5.583,74 TL</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="12" t="inlineStr">

</xml_diff>

<commit_message>
Update benchmark: 2026-05-11 09:47:19 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -616,11 +616,7 @@
           <t>26 TL - 26 TL</t>
         </is>
       </c>
-      <c r="F2" s="14" t="inlineStr">
-        <is>
-          <t>33,33 TL - 33,33 TL</t>
-        </is>
-      </c>
+      <c r="F2" s="14" t="inlineStr"/>
       <c r="G2" s="14" t="inlineStr">
         <is>
           <t>15 TL - 15 TL</t>
@@ -773,11 +769,7 @@
         </is>
       </c>
       <c r="E7" s="14" t="inlineStr"/>
-      <c r="F7" s="14" t="inlineStr">
-        <is>
-          <t>%3</t>
-        </is>
-      </c>
+      <c r="F7" s="14" t="inlineStr"/>
       <c r="G7" s="14" t="inlineStr">
         <is>
           <t>1 TRY (Kredi kartı ile ödemelerde ek olarak nakit avans faizi uygulanır.)</t>

</xml_diff>

<commit_message>
Update benchmark: 2026-05-12 08:48:24 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -616,7 +616,11 @@
           <t>26 TL - 26 TL</t>
         </is>
       </c>
-      <c r="F2" s="14" t="inlineStr"/>
+      <c r="F2" s="14" t="inlineStr">
+        <is>
+          <t>33,33 TL - 33,33 TL</t>
+        </is>
+      </c>
       <c r="G2" s="14" t="inlineStr">
         <is>
           <t>15 TL - 15 TL</t>
@@ -769,7 +773,11 @@
         </is>
       </c>
       <c r="E7" s="14" t="inlineStr"/>
-      <c r="F7" s="14" t="inlineStr"/>
+      <c r="F7" s="14" t="inlineStr">
+        <is>
+          <t>%3</t>
+        </is>
+      </c>
       <c r="G7" s="14" t="inlineStr">
         <is>
           <t>1 TRY (Kredi kartı ile ödemelerde ek olarak nakit avans faizi uygulanır.)</t>

</xml_diff>

<commit_message>
Update benchmark: 2026-05-13 08:51:42 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -606,11 +606,7 @@
           <t>30 TL - 30 TL</t>
         </is>
       </c>
-      <c r="D2" s="14" t="inlineStr">
-        <is>
-          <t>33,33 TL - 33,33 TL</t>
-        </is>
-      </c>
+      <c r="D2" s="14" t="inlineStr"/>
       <c r="E2" s="14" t="inlineStr">
         <is>
           <t>26 TL - 26 TL</t>
@@ -662,11 +658,7 @@
       <c r="D3" s="14" t="inlineStr"/>
       <c r="E3" s="14" t="inlineStr"/>
       <c r="F3" s="14" t="inlineStr"/>
-      <c r="G3" s="14" t="inlineStr">
-        <is>
-          <t>39,87 TRY - 79,76 TRY - 797,68 TRY</t>
-        </is>
-      </c>
+      <c r="G3" s="14" t="inlineStr"/>
       <c r="H3" s="14" t="inlineStr"/>
       <c r="I3" s="14" t="inlineStr"/>
       <c r="J3" s="14" t="inlineStr"/>
@@ -682,11 +674,7 @@
       <c r="D4" s="14" t="inlineStr"/>
       <c r="E4" s="14" t="inlineStr"/>
       <c r="F4" s="14" t="inlineStr"/>
-      <c r="G4" s="14" t="inlineStr">
-        <is>
-          <t>27,84 TRY - 55,69 TRY - 398,83 TRY</t>
-        </is>
-      </c>
+      <c r="G4" s="14" t="inlineStr"/>
       <c r="H4" s="14" t="inlineStr"/>
       <c r="I4" s="14" t="inlineStr"/>
       <c r="J4" s="14" t="inlineStr"/>
@@ -702,11 +690,7 @@
       <c r="D5" s="14" t="inlineStr"/>
       <c r="E5" s="14" t="inlineStr"/>
       <c r="F5" s="14" t="inlineStr"/>
-      <c r="G5" s="14" t="inlineStr">
-        <is>
-          <t>7,97 TRY - 15,96 TRY - 199,41 TRY</t>
-        </is>
-      </c>
+      <c r="G5" s="14" t="inlineStr"/>
       <c r="H5" s="14" t="inlineStr"/>
       <c r="I5" s="14" t="inlineStr"/>
       <c r="J5" s="14" t="inlineStr"/>
@@ -718,47 +702,23 @@
           <t>DÜZENLİ EFT</t>
         </is>
       </c>
-      <c r="C6" s="14" t="inlineStr">
+      <c r="C6" s="14" t="inlineStr"/>
+      <c r="D6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="D6" s="14" t="inlineStr">
+      <c r="E6" s="14" t="inlineStr"/>
+      <c r="F6" s="14" t="inlineStr"/>
+      <c r="G6" s="14" t="inlineStr"/>
+      <c r="H6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="E6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 199,41 TL</t>
-        </is>
-      </c>
-      <c r="F6" s="14" t="inlineStr"/>
-      <c r="G6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 99,71 TL</t>
-        </is>
-      </c>
-      <c r="H6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 199,41 TL</t>
-        </is>
-      </c>
-      <c r="I6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 199,41 TL</t>
-        </is>
-      </c>
-      <c r="J6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 199,41 TL</t>
-        </is>
-      </c>
-      <c r="K6" s="14" t="inlineStr">
-        <is>
-          <t>7,97 TL - 15,96 TL - 199,41 TL</t>
-        </is>
-      </c>
+      <c r="I6" s="14" t="inlineStr"/>
+      <c r="J6" s="14" t="inlineStr"/>
+      <c r="K6" s="14" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="B7" s="13" t="inlineStr">
@@ -767,11 +727,7 @@
         </is>
       </c>
       <c r="C7" s="14" t="inlineStr"/>
-      <c r="D7" s="14" t="inlineStr">
-        <is>
-          <t>%1,6</t>
-        </is>
-      </c>
+      <c r="D7" s="14" t="inlineStr"/>
       <c r="E7" s="14" t="inlineStr"/>
       <c r="F7" s="14" t="inlineStr">
         <is>
@@ -785,7 +741,7 @@
       </c>
       <c r="H7" s="14" t="inlineStr">
         <is>
-          <t>%3,09</t>
+          <t>%3,5</t>
         </is>
       </c>
       <c r="I7" s="14" t="inlineStr"/>
@@ -815,11 +771,7 @@
       <c r="D8" s="14" t="inlineStr"/>
       <c r="E8" s="14" t="inlineStr"/>
       <c r="F8" s="14" t="inlineStr"/>
-      <c r="G8" s="14" t="inlineStr">
-        <is>
-          <t>19,94 TRY - 39,88 TRY - 398,84 TRY</t>
-        </is>
-      </c>
+      <c r="G8" s="14" t="inlineStr"/>
       <c r="H8" s="14" t="inlineStr"/>
       <c r="I8" s="14" t="inlineStr"/>
       <c r="J8" s="14" t="inlineStr"/>
@@ -835,11 +787,7 @@
       <c r="D9" s="14" t="inlineStr"/>
       <c r="E9" s="14" t="inlineStr"/>
       <c r="F9" s="14" t="inlineStr"/>
-      <c r="G9" s="14" t="inlineStr">
-        <is>
-          <t>13,92 TRY - 27,85 TRY - 199,42 TRY</t>
-        </is>
-      </c>
+      <c r="G9" s="14" t="inlineStr"/>
       <c r="H9" s="14" t="inlineStr"/>
       <c r="I9" s="14" t="inlineStr"/>
       <c r="J9" s="14" t="inlineStr"/>
@@ -855,11 +803,7 @@
       <c r="D10" s="14" t="inlineStr"/>
       <c r="E10" s="14" t="inlineStr"/>
       <c r="F10" s="14" t="inlineStr"/>
-      <c r="G10" s="14" t="inlineStr">
-        <is>
-          <t>3,99 TRY - 7,98 TRY - 99,71 TRY</t>
-        </is>
-      </c>
+      <c r="G10" s="14" t="inlineStr"/>
       <c r="H10" s="14" t="inlineStr"/>
       <c r="I10" s="14" t="inlineStr"/>
       <c r="J10" s="14" t="inlineStr"/>
@@ -875,11 +819,7 @@
       <c r="D11" s="14" t="inlineStr"/>
       <c r="E11" s="14" t="inlineStr"/>
       <c r="F11" s="14" t="inlineStr"/>
-      <c r="G11" s="14" t="inlineStr">
-        <is>
-          <t>3,99 TRY - 7,98 TRY - 99,71 TRY</t>
-        </is>
-      </c>
+      <c r="G11" s="14" t="inlineStr"/>
       <c r="H11" s="14" t="inlineStr"/>
       <c r="I11" s="14" t="inlineStr"/>
       <c r="J11" s="14" t="inlineStr"/>
@@ -896,11 +836,7 @@
           <t>GİDEN SWIFT</t>
         </is>
       </c>
-      <c r="C12" s="14" t="inlineStr">
-        <is>
-          <t>WU: 1.000,01 USD–9,51 USD</t>
-        </is>
-      </c>
+      <c r="C12" s="14" t="inlineStr"/>
       <c r="D12" s="14" t="inlineStr">
         <is>
           <t>WU: 0,75 USD–12 USD; Diğer: 700 TL–4.000 TL</t>
@@ -908,19 +844,11 @@
       </c>
       <c r="E12" s="14" t="inlineStr"/>
       <c r="F12" s="14" t="inlineStr"/>
-      <c r="G12" s="14" t="inlineStr">
-        <is>
-          <t>Şube (Kasadan): %0,5; Şube (Hesaptan): %0,75; İnternet: 15 USD</t>
-        </is>
-      </c>
+      <c r="G12" s="14" t="inlineStr"/>
       <c r="H12" s="14" t="inlineStr"/>
       <c r="I12" s="14" t="inlineStr"/>
       <c r="J12" s="14" t="inlineStr"/>
-      <c r="K12" s="14" t="inlineStr">
-        <is>
-          <t>WU: ,USD–; Diğer: 529 TL–4.454,74 TL</t>
-        </is>
-      </c>
+      <c r="K12" s="14" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="B13" s="13" t="inlineStr">
@@ -928,21 +856,13 @@
           <t>GELEN SWIFT</t>
         </is>
       </c>
-      <c r="C13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 0 TL | Azami 0,94 TL</t>
-        </is>
-      </c>
+      <c r="C13" s="14" t="inlineStr"/>
       <c r="D13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
         </is>
       </c>
-      <c r="E13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
-        </is>
-      </c>
+      <c r="E13" s="14" t="inlineStr"/>
       <c r="F13" s="14" t="inlineStr"/>
       <c r="G13" s="14" t="inlineStr"/>
       <c r="H13" s="14" t="inlineStr">
@@ -950,21 +870,9 @@
           <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
         </is>
       </c>
-      <c r="I13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
-        </is>
-      </c>
-      <c r="J13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 1.303 TL</t>
-        </is>
-      </c>
-      <c r="K13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 865,75 TL</t>
-        </is>
-      </c>
+      <c r="I13" s="14" t="inlineStr"/>
+      <c r="J13" s="14" t="inlineStr"/>
+      <c r="K13" s="14" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="B14" s="13" t="inlineStr">
@@ -972,47 +880,23 @@
           <t>GİDEN SWIFT - Mobil</t>
         </is>
       </c>
-      <c r="C14" s="14" t="inlineStr">
-        <is>
-          <t>40.000 TL - 2.485,72 TL</t>
-        </is>
-      </c>
+      <c r="C14" s="14" t="inlineStr"/>
       <c r="D14" s="14" t="inlineStr">
         <is>
           <t>3.500 TL - 13.500 TL</t>
         </is>
       </c>
-      <c r="E14" s="14" t="inlineStr">
-        <is>
-          <t>2.170 TL - 2.170 TL</t>
-        </is>
-      </c>
-      <c r="F14" s="14" t="inlineStr">
-        <is>
-          <t>2.785,72 TL - 12.380,95 TL</t>
-        </is>
-      </c>
-      <c r="G14" s="14" t="inlineStr">
-        <is>
-          <t>8.300 TL - 7,97 TL</t>
-        </is>
-      </c>
+      <c r="E14" s="14" t="inlineStr"/>
+      <c r="F14" s="14" t="inlineStr"/>
+      <c r="G14" s="14" t="inlineStr"/>
       <c r="H14" s="14" t="inlineStr">
         <is>
           <t>3.000 TL - 6.000 TL</t>
         </is>
       </c>
       <c r="I14" s="14" t="inlineStr"/>
-      <c r="J14" s="14" t="inlineStr">
-        <is>
-          <t>1.554,97 TL - 7.784 TL</t>
-        </is>
-      </c>
-      <c r="K14" s="14" t="inlineStr">
-        <is>
-          <t>1.196,51 TL - 5.583,74 TL</t>
-        </is>
-      </c>
+      <c r="J14" s="14" t="inlineStr"/>
+      <c r="K14" s="14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="12" t="inlineStr">

</xml_diff>

<commit_message>
Update benchmark: 2026-05-14 08:45:59 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -601,12 +601,12 @@
         </is>
       </c>
       <c r="B2" s="13" t="inlineStr"/>
-      <c r="C2" s="14" t="inlineStr">
-        <is>
-          <t>30 TL - 30 TL</t>
-        </is>
-      </c>
-      <c r="D2" s="14" t="inlineStr"/>
+      <c r="C2" s="14" t="inlineStr"/>
+      <c r="D2" s="14" t="inlineStr">
+        <is>
+          <t>33,33 TL - 33,33 TL</t>
+        </is>
+      </c>
       <c r="E2" s="14" t="inlineStr">
         <is>
           <t>26 TL - 26 TL</t>
@@ -658,7 +658,11 @@
       <c r="D3" s="14" t="inlineStr"/>
       <c r="E3" s="14" t="inlineStr"/>
       <c r="F3" s="14" t="inlineStr"/>
-      <c r="G3" s="14" t="inlineStr"/>
+      <c r="G3" s="14" t="inlineStr">
+        <is>
+          <t>39,87 TRY - 79,76 TRY - 797,68 TRY</t>
+        </is>
+      </c>
       <c r="H3" s="14" t="inlineStr"/>
       <c r="I3" s="14" t="inlineStr"/>
       <c r="J3" s="14" t="inlineStr"/>
@@ -674,7 +678,11 @@
       <c r="D4" s="14" t="inlineStr"/>
       <c r="E4" s="14" t="inlineStr"/>
       <c r="F4" s="14" t="inlineStr"/>
-      <c r="G4" s="14" t="inlineStr"/>
+      <c r="G4" s="14" t="inlineStr">
+        <is>
+          <t>27,84 TRY - 55,69 TRY - 398,83 TRY</t>
+        </is>
+      </c>
       <c r="H4" s="14" t="inlineStr"/>
       <c r="I4" s="14" t="inlineStr"/>
       <c r="J4" s="14" t="inlineStr"/>
@@ -690,7 +698,11 @@
       <c r="D5" s="14" t="inlineStr"/>
       <c r="E5" s="14" t="inlineStr"/>
       <c r="F5" s="14" t="inlineStr"/>
-      <c r="G5" s="14" t="inlineStr"/>
+      <c r="G5" s="14" t="inlineStr">
+        <is>
+          <t>7,97 TRY - 15,96 TRY - 199,41 TRY</t>
+        </is>
+      </c>
       <c r="H5" s="14" t="inlineStr"/>
       <c r="I5" s="14" t="inlineStr"/>
       <c r="J5" s="14" t="inlineStr"/>
@@ -702,23 +714,47 @@
           <t>DÜZENLİ EFT</t>
         </is>
       </c>
-      <c r="C6" s="14" t="inlineStr"/>
+      <c r="C6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 199,41 TL</t>
+        </is>
+      </c>
       <c r="D6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="E6" s="14" t="inlineStr"/>
+      <c r="E6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 199,41 TL</t>
+        </is>
+      </c>
       <c r="F6" s="14" t="inlineStr"/>
-      <c r="G6" s="14" t="inlineStr"/>
+      <c r="G6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 99,71 TL</t>
+        </is>
+      </c>
       <c r="H6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="I6" s="14" t="inlineStr"/>
-      <c r="J6" s="14" t="inlineStr"/>
-      <c r="K6" s="14" t="inlineStr"/>
+      <c r="I6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 199,41 TL</t>
+        </is>
+      </c>
+      <c r="J6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 199,41 TL</t>
+        </is>
+      </c>
+      <c r="K6" s="14" t="inlineStr">
+        <is>
+          <t>7,97 TL - 15,96 TL - 199,41 TL</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="B7" s="13" t="inlineStr">
@@ -727,7 +763,11 @@
         </is>
       </c>
       <c r="C7" s="14" t="inlineStr"/>
-      <c r="D7" s="14" t="inlineStr"/>
+      <c r="D7" s="14" t="inlineStr">
+        <is>
+          <t>%1,6</t>
+        </is>
+      </c>
       <c r="E7" s="14" t="inlineStr"/>
       <c r="F7" s="14" t="inlineStr">
         <is>
@@ -771,7 +811,11 @@
       <c r="D8" s="14" t="inlineStr"/>
       <c r="E8" s="14" t="inlineStr"/>
       <c r="F8" s="14" t="inlineStr"/>
-      <c r="G8" s="14" t="inlineStr"/>
+      <c r="G8" s="14" t="inlineStr">
+        <is>
+          <t>19,94 TRY - 39,88 TRY - 398,84 TRY</t>
+        </is>
+      </c>
       <c r="H8" s="14" t="inlineStr"/>
       <c r="I8" s="14" t="inlineStr"/>
       <c r="J8" s="14" t="inlineStr"/>
@@ -787,7 +831,11 @@
       <c r="D9" s="14" t="inlineStr"/>
       <c r="E9" s="14" t="inlineStr"/>
       <c r="F9" s="14" t="inlineStr"/>
-      <c r="G9" s="14" t="inlineStr"/>
+      <c r="G9" s="14" t="inlineStr">
+        <is>
+          <t>13,92 TRY - 27,85 TRY - 199,42 TRY</t>
+        </is>
+      </c>
       <c r="H9" s="14" t="inlineStr"/>
       <c r="I9" s="14" t="inlineStr"/>
       <c r="J9" s="14" t="inlineStr"/>
@@ -803,7 +851,11 @@
       <c r="D10" s="14" t="inlineStr"/>
       <c r="E10" s="14" t="inlineStr"/>
       <c r="F10" s="14" t="inlineStr"/>
-      <c r="G10" s="14" t="inlineStr"/>
+      <c r="G10" s="14" t="inlineStr">
+        <is>
+          <t>3,99 TRY - 7,98 TRY - 99,71 TRY</t>
+        </is>
+      </c>
       <c r="H10" s="14" t="inlineStr"/>
       <c r="I10" s="14" t="inlineStr"/>
       <c r="J10" s="14" t="inlineStr"/>
@@ -819,7 +871,11 @@
       <c r="D11" s="14" t="inlineStr"/>
       <c r="E11" s="14" t="inlineStr"/>
       <c r="F11" s="14" t="inlineStr"/>
-      <c r="G11" s="14" t="inlineStr"/>
+      <c r="G11" s="14" t="inlineStr">
+        <is>
+          <t>3,99 TRY - 7,98 TRY - 99,71 TRY</t>
+        </is>
+      </c>
       <c r="H11" s="14" t="inlineStr"/>
       <c r="I11" s="14" t="inlineStr"/>
       <c r="J11" s="14" t="inlineStr"/>
@@ -836,7 +892,11 @@
           <t>GİDEN SWIFT</t>
         </is>
       </c>
-      <c r="C12" s="14" t="inlineStr"/>
+      <c r="C12" s="14" t="inlineStr">
+        <is>
+          <t>WU: 1.000,01 USD–</t>
+        </is>
+      </c>
       <c r="D12" s="14" t="inlineStr">
         <is>
           <t>WU: 0,75 USD–12 USD; Diğer: 700 TL–4.000 TL</t>
@@ -844,11 +904,19 @@
       </c>
       <c r="E12" s="14" t="inlineStr"/>
       <c r="F12" s="14" t="inlineStr"/>
-      <c r="G12" s="14" t="inlineStr"/>
+      <c r="G12" s="14" t="inlineStr">
+        <is>
+          <t>Şube (Kasadan): %0,5; Şube (Hesaptan): %0,75; İnternet: 15 USD</t>
+        </is>
+      </c>
       <c r="H12" s="14" t="inlineStr"/>
       <c r="I12" s="14" t="inlineStr"/>
       <c r="J12" s="14" t="inlineStr"/>
-      <c r="K12" s="14" t="inlineStr"/>
+      <c r="K12" s="14" t="inlineStr">
+        <is>
+          <t>WU: ,USD–; Diğer: 529 TL–4.454,74 TL</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="B13" s="13" t="inlineStr">
@@ -856,13 +924,21 @@
           <t>GELEN SWIFT</t>
         </is>
       </c>
-      <c r="C13" s="14" t="inlineStr"/>
+      <c r="C13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 0 TL | Azami 3.295,24 TL</t>
+        </is>
+      </c>
       <c r="D13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
         </is>
       </c>
-      <c r="E13" s="14" t="inlineStr"/>
+      <c r="E13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
+        </is>
+      </c>
       <c r="F13" s="14" t="inlineStr"/>
       <c r="G13" s="14" t="inlineStr"/>
       <c r="H13" s="14" t="inlineStr">
@@ -870,9 +946,21 @@
           <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
         </is>
       </c>
-      <c r="I13" s="14" t="inlineStr"/>
-      <c r="J13" s="14" t="inlineStr"/>
-      <c r="K13" s="14" t="inlineStr"/>
+      <c r="I13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
+        </is>
+      </c>
+      <c r="J13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 1.303 TL</t>
+        </is>
+      </c>
+      <c r="K13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 865,75 TL</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="B14" s="13" t="inlineStr">
@@ -880,23 +968,47 @@
           <t>GİDEN SWIFT - Mobil</t>
         </is>
       </c>
-      <c r="C14" s="14" t="inlineStr"/>
+      <c r="C14" s="14" t="inlineStr">
+        <is>
+          <t>40.000 TL - 2.485,72 TL</t>
+        </is>
+      </c>
       <c r="D14" s="14" t="inlineStr">
         <is>
           <t>3.500 TL - 13.500 TL</t>
         </is>
       </c>
-      <c r="E14" s="14" t="inlineStr"/>
-      <c r="F14" s="14" t="inlineStr"/>
-      <c r="G14" s="14" t="inlineStr"/>
+      <c r="E14" s="14" t="inlineStr">
+        <is>
+          <t>2.170 TL - 2.170 TL</t>
+        </is>
+      </c>
+      <c r="F14" s="14" t="inlineStr">
+        <is>
+          <t>2.785,72 TL - 12.380,95 TL</t>
+        </is>
+      </c>
+      <c r="G14" s="14" t="inlineStr">
+        <is>
+          <t>8.300 TL - 7,97 TL</t>
+        </is>
+      </c>
       <c r="H14" s="14" t="inlineStr">
         <is>
           <t>3.000 TL - 6.000 TL</t>
         </is>
       </c>
       <c r="I14" s="14" t="inlineStr"/>
-      <c r="J14" s="14" t="inlineStr"/>
-      <c r="K14" s="14" t="inlineStr"/>
+      <c r="J14" s="14" t="inlineStr">
+        <is>
+          <t>1.554,97 TL - 7.784 TL</t>
+        </is>
+      </c>
+      <c r="K14" s="14" t="inlineStr">
+        <is>
+          <t>1.196,51 TL - 5.583,74 TL</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="12" t="inlineStr">

</xml_diff>

<commit_message>
Update benchmark: 2026-05-15 08:57:28 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -601,7 +601,11 @@
         </is>
       </c>
       <c r="B2" s="13" t="inlineStr"/>
-      <c r="C2" s="14" t="inlineStr"/>
+      <c r="C2" s="14" t="inlineStr">
+        <is>
+          <t>30 TL - 30 TL</t>
+        </is>
+      </c>
       <c r="D2" s="14" t="inlineStr">
         <is>
           <t>33,33 TL - 33,33 TL</t>
@@ -714,11 +718,7 @@
           <t>DÜZENLİ EFT</t>
         </is>
       </c>
-      <c r="C6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 199,41 TL</t>
-        </is>
-      </c>
+      <c r="C6" s="14" t="inlineStr"/>
       <c r="D6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
@@ -735,11 +735,7 @@
           <t>8.300,01 TL - 99,71 TL</t>
         </is>
       </c>
-      <c r="H6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 199,41 TL</t>
-        </is>
-      </c>
+      <c r="H6" s="14" t="inlineStr"/>
       <c r="I6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
@@ -892,11 +888,7 @@
           <t>GİDEN SWIFT</t>
         </is>
       </c>
-      <c r="C12" s="14" t="inlineStr">
-        <is>
-          <t>WU: 1.000,01 USD–</t>
-        </is>
-      </c>
+      <c r="C12" s="14" t="inlineStr"/>
       <c r="D12" s="14" t="inlineStr">
         <is>
           <t>WU: 0,75 USD–12 USD; Diğer: 700 TL–4.000 TL</t>
@@ -924,11 +916,7 @@
           <t>GELEN SWIFT</t>
         </is>
       </c>
-      <c r="C13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 0 TL | Azami 3.295,24 TL</t>
-        </is>
-      </c>
+      <c r="C13" s="14" t="inlineStr"/>
       <c r="D13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
@@ -941,11 +929,7 @@
       </c>
       <c r="F13" s="14" t="inlineStr"/>
       <c r="G13" s="14" t="inlineStr"/>
-      <c r="H13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
-        </is>
-      </c>
+      <c r="H13" s="14" t="inlineStr"/>
       <c r="I13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
@@ -968,11 +952,7 @@
           <t>GİDEN SWIFT - Mobil</t>
         </is>
       </c>
-      <c r="C14" s="14" t="inlineStr">
-        <is>
-          <t>40.000 TL - 2.485,72 TL</t>
-        </is>
-      </c>
+      <c r="C14" s="14" t="inlineStr"/>
       <c r="D14" s="14" t="inlineStr">
         <is>
           <t>3.500 TL - 13.500 TL</t>
@@ -993,11 +973,7 @@
           <t>8.300 TL - 7,97 TL</t>
         </is>
       </c>
-      <c r="H14" s="14" t="inlineStr">
-        <is>
-          <t>3.000 TL - 6.000 TL</t>
-        </is>
-      </c>
+      <c r="H14" s="14" t="inlineStr"/>
       <c r="I14" s="14" t="inlineStr"/>
       <c r="J14" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update benchmark: 2026-05-16 08:13:56 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -611,21 +611,13 @@
           <t>33,33 TL - 33,33 TL</t>
         </is>
       </c>
-      <c r="E2" s="14" t="inlineStr">
-        <is>
-          <t>26 TL - 26 TL</t>
-        </is>
-      </c>
+      <c r="E2" s="14" t="inlineStr"/>
       <c r="F2" s="14" t="inlineStr">
         <is>
           <t>33,33 TL - 33,33 TL</t>
         </is>
       </c>
-      <c r="G2" s="14" t="inlineStr">
-        <is>
-          <t>15 TL - 15 TL</t>
-        </is>
-      </c>
+      <c r="G2" s="14" t="inlineStr"/>
       <c r="H2" s="14" t="inlineStr">
         <is>
           <t>15 TL - 15 TL</t>
@@ -718,7 +710,11 @@
           <t>DÜZENLİ EFT</t>
         </is>
       </c>
-      <c r="C6" s="14" t="inlineStr"/>
+      <c r="C6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 199,41 TL</t>
+        </is>
+      </c>
       <c r="D6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
@@ -735,7 +731,11 @@
           <t>8.300,01 TL - 99,71 TL</t>
         </is>
       </c>
-      <c r="H6" s="14" t="inlineStr"/>
+      <c r="H6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 199,41 TL</t>
+        </is>
+      </c>
       <c r="I6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
@@ -770,11 +770,7 @@
           <t>%3</t>
         </is>
       </c>
-      <c r="G7" s="14" t="inlineStr">
-        <is>
-          <t>1 TRY (Kredi kartı ile ödemelerde ek olarak nakit avans faizi uygulanır.)</t>
-        </is>
-      </c>
+      <c r="G7" s="14" t="inlineStr"/>
       <c r="H7" s="14" t="inlineStr">
         <is>
           <t>%3,5</t>
@@ -888,7 +884,11 @@
           <t>GİDEN SWIFT</t>
         </is>
       </c>
-      <c r="C12" s="14" t="inlineStr"/>
+      <c r="C12" s="14" t="inlineStr">
+        <is>
+          <t>WU: 1.000,01 USD–9,51 USD</t>
+        </is>
+      </c>
       <c r="D12" s="14" t="inlineStr">
         <is>
           <t>WU: 0,75 USD–12 USD; Diğer: 700 TL–4.000 TL</t>
@@ -916,7 +916,11 @@
           <t>GELEN SWIFT</t>
         </is>
       </c>
-      <c r="C13" s="14" t="inlineStr"/>
+      <c r="C13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 0 TL | Azami 0,94 TL</t>
+        </is>
+      </c>
       <c r="D13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
@@ -929,7 +933,11 @@
       </c>
       <c r="F13" s="14" t="inlineStr"/>
       <c r="G13" s="14" t="inlineStr"/>
-      <c r="H13" s="14" t="inlineStr"/>
+      <c r="H13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
+        </is>
+      </c>
       <c r="I13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
@@ -942,7 +950,7 @@
       </c>
       <c r="K13" s="14" t="inlineStr">
         <is>
-          <t>Hesaba: Asgari 1 TL | Azami 865,75 TL</t>
+          <t>Hesaba: Asgari 1 TL | Azami 69,62 TL</t>
         </is>
       </c>
     </row>
@@ -952,7 +960,11 @@
           <t>GİDEN SWIFT - Mobil</t>
         </is>
       </c>
-      <c r="C14" s="14" t="inlineStr"/>
+      <c r="C14" s="14" t="inlineStr">
+        <is>
+          <t>40.000 TL - 2.485,72 TL</t>
+        </is>
+      </c>
       <c r="D14" s="14" t="inlineStr">
         <is>
           <t>3.500 TL - 13.500 TL</t>
@@ -973,7 +985,11 @@
           <t>8.300 TL - 7,97 TL</t>
         </is>
       </c>
-      <c r="H14" s="14" t="inlineStr"/>
+      <c r="H14" s="14" t="inlineStr">
+        <is>
+          <t>3.000 TL - 6.000 TL</t>
+        </is>
+      </c>
       <c r="I14" s="14" t="inlineStr"/>
       <c r="J14" s="14" t="inlineStr">
         <is>
@@ -1019,7 +1035,7 @@
       </c>
       <c r="G15" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Asgari Tutar: 150 TL Azami Tutar: 150 TL</t>
+          <t xml:space="preserve"> Asgari Tutar:  Azami Tutar: </t>
         </is>
       </c>
       <c r="H15" s="14" t="inlineStr">
@@ -1087,7 +1103,7 @@
       </c>
       <c r="G17" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Asgari Tutar: 300 TL Azami Tutar: 300 TL</t>
+          <t xml:space="preserve"> Asgari Tutar:  Azami Tutar: </t>
         </is>
       </c>
       <c r="H17" s="14" t="inlineStr">
@@ -1219,7 +1235,7 @@
       </c>
       <c r="G21" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">%0,16 Asgari Tutar: 300 TL Azami Tutar: </t>
+          <t xml:space="preserve"> Asgari Tutar:  Azami Tutar: </t>
         </is>
       </c>
       <c r="H21" s="14" t="inlineStr">
@@ -1321,11 +1337,7 @@
           <t>86,67 TL</t>
         </is>
       </c>
-      <c r="G23" s="14" t="inlineStr">
-        <is>
-          <t>600 TL</t>
-        </is>
-      </c>
+      <c r="G23" s="14" t="inlineStr"/>
       <c r="H23" s="14" t="inlineStr">
         <is>
           <t>57,5 TL</t>
@@ -1378,11 +1390,7 @@
           <t>600 TL</t>
         </is>
       </c>
-      <c r="G24" s="14" t="inlineStr">
-        <is>
-          <t>160 TL</t>
-        </is>
-      </c>
+      <c r="G24" s="14" t="inlineStr"/>
       <c r="H24" s="14" t="inlineStr">
         <is>
           <t>350 TL</t>

</xml_diff>

<commit_message>
Update benchmark: 2026-05-17 08:29:54 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -611,13 +611,21 @@
           <t>33,33 TL - 33,33 TL</t>
         </is>
       </c>
-      <c r="E2" s="14" t="inlineStr"/>
+      <c r="E2" s="14" t="inlineStr">
+        <is>
+          <t>26 TL - 26 TL</t>
+        </is>
+      </c>
       <c r="F2" s="14" t="inlineStr">
         <is>
           <t>33,33 TL - 33,33 TL</t>
         </is>
       </c>
-      <c r="G2" s="14" t="inlineStr"/>
+      <c r="G2" s="14" t="inlineStr">
+        <is>
+          <t>15 TL - 15 TL</t>
+        </is>
+      </c>
       <c r="H2" s="14" t="inlineStr">
         <is>
           <t>15 TL - 15 TL</t>
@@ -770,7 +778,11 @@
           <t>%3</t>
         </is>
       </c>
-      <c r="G7" s="14" t="inlineStr"/>
+      <c r="G7" s="14" t="inlineStr">
+        <is>
+          <t>1 TRY (Kredi kartı ile ödemelerde ek olarak nakit avans faizi uygulanır.)</t>
+        </is>
+      </c>
       <c r="H7" s="14" t="inlineStr">
         <is>
           <t>%3,5</t>
@@ -950,7 +962,7 @@
       </c>
       <c r="K13" s="14" t="inlineStr">
         <is>
-          <t>Hesaba: Asgari 1 TL | Azami 69,62 TL</t>
+          <t>Hesaba: Asgari 1 TL | Azami 865,75 TL</t>
         </is>
       </c>
     </row>
@@ -1035,7 +1047,7 @@
       </c>
       <c r="G15" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Asgari Tutar:  Azami Tutar: </t>
+          <t xml:space="preserve"> Asgari Tutar: 150 TL Azami Tutar: 150 TL</t>
         </is>
       </c>
       <c r="H15" s="14" t="inlineStr">
@@ -1103,7 +1115,7 @@
       </c>
       <c r="G17" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Asgari Tutar:  Azami Tutar: </t>
+          <t xml:space="preserve"> Asgari Tutar: 300 TL Azami Tutar: 300 TL</t>
         </is>
       </c>
       <c r="H17" s="14" t="inlineStr">
@@ -1235,7 +1247,7 @@
       </c>
       <c r="G21" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Asgari Tutar:  Azami Tutar: </t>
+          <t xml:space="preserve">%0,16 Asgari Tutar: 300 TL Azami Tutar: </t>
         </is>
       </c>
       <c r="H21" s="14" t="inlineStr">
@@ -1337,7 +1349,11 @@
           <t>86,67 TL</t>
         </is>
       </c>
-      <c r="G23" s="14" t="inlineStr"/>
+      <c r="G23" s="14" t="inlineStr">
+        <is>
+          <t>600 TL</t>
+        </is>
+      </c>
       <c r="H23" s="14" t="inlineStr">
         <is>
           <t>57,5 TL</t>
@@ -1390,7 +1406,11 @@
           <t>600 TL</t>
         </is>
       </c>
-      <c r="G24" s="14" t="inlineStr"/>
+      <c r="G24" s="14" t="inlineStr">
+        <is>
+          <t>160 TL</t>
+        </is>
+      </c>
       <c r="H24" s="14" t="inlineStr">
         <is>
           <t>350 TL</t>

</xml_diff>

<commit_message>
Update benchmark: 2026-05-20 09:36:15 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -611,11 +611,7 @@
           <t>33,33 TL - 33,33 TL</t>
         </is>
       </c>
-      <c r="E2" s="14" t="inlineStr">
-        <is>
-          <t>26 TL - 26 TL</t>
-        </is>
-      </c>
+      <c r="E2" s="14" t="inlineStr"/>
       <c r="F2" s="14" t="inlineStr">
         <is>
           <t>33,33 TL - 33,33 TL</t>
@@ -723,11 +719,7 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="D6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 199,41 TL</t>
-        </is>
-      </c>
+      <c r="D6" s="14" t="inlineStr"/>
       <c r="E6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
@@ -901,11 +893,7 @@
           <t>WU: 1.000,01 USD–9,51 USD</t>
         </is>
       </c>
-      <c r="D12" s="14" t="inlineStr">
-        <is>
-          <t>WU: 0,75 USD–12 USD; Diğer: 700 TL–4.000 TL</t>
-        </is>
-      </c>
+      <c r="D12" s="14" t="inlineStr"/>
       <c r="E12" s="14" t="inlineStr"/>
       <c r="F12" s="14" t="inlineStr"/>
       <c r="G12" s="14" t="inlineStr">
@@ -933,11 +921,7 @@
           <t>Hesaba: Asgari 0 TL | Azami 0,94 TL</t>
         </is>
       </c>
-      <c r="D13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
-        </is>
-      </c>
+      <c r="D13" s="14" t="inlineStr"/>
       <c r="E13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
@@ -977,11 +961,7 @@
           <t>40.000 TL - 2.485,72 TL</t>
         </is>
       </c>
-      <c r="D14" s="14" t="inlineStr">
-        <is>
-          <t>3.500 TL - 13.500 TL</t>
-        </is>
-      </c>
+      <c r="D14" s="14" t="inlineStr"/>
       <c r="E14" s="14" t="inlineStr">
         <is>
           <t>2.170 TL - 2.170 TL</t>

</xml_diff>

<commit_message>
Update benchmark: 2026-05-21 09:42:29 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -611,7 +611,11 @@
           <t>33,33 TL - 33,33 TL</t>
         </is>
       </c>
-      <c r="E2" s="14" t="inlineStr"/>
+      <c r="E2" s="14" t="inlineStr">
+        <is>
+          <t>26 TL - 26 TL</t>
+        </is>
+      </c>
       <c r="F2" s="14" t="inlineStr">
         <is>
           <t>33,33 TL - 33,33 TL</t>
@@ -719,7 +723,11 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="D6" s="14" t="inlineStr"/>
+      <c r="D6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 199,41 TL</t>
+        </is>
+      </c>
       <c r="E6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
@@ -893,7 +901,11 @@
           <t>WU: 1.000,01 USD–9,51 USD</t>
         </is>
       </c>
-      <c r="D12" s="14" t="inlineStr"/>
+      <c r="D12" s="14" t="inlineStr">
+        <is>
+          <t>WU: 0,75 USD–12 USD; Diğer: 700 TL–4.000 TL</t>
+        </is>
+      </c>
       <c r="E12" s="14" t="inlineStr"/>
       <c r="F12" s="14" t="inlineStr"/>
       <c r="G12" s="14" t="inlineStr">
@@ -921,7 +933,11 @@
           <t>Hesaba: Asgari 0 TL | Azami 0,94 TL</t>
         </is>
       </c>
-      <c r="D13" s="14" t="inlineStr"/>
+      <c r="D13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
+        </is>
+      </c>
       <c r="E13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
@@ -961,7 +977,11 @@
           <t>40.000 TL - 2.485,72 TL</t>
         </is>
       </c>
-      <c r="D14" s="14" t="inlineStr"/>
+      <c r="D14" s="14" t="inlineStr">
+        <is>
+          <t>3.500 TL - 13.500 TL</t>
+        </is>
+      </c>
       <c r="E14" s="14" t="inlineStr">
         <is>
           <t>2.170 TL - 2.170 TL</t>

</xml_diff>

<commit_message>
Update benchmark: 2026-05-22 09:24:18 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -723,11 +723,7 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="D6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 199,41 TL</t>
-        </is>
-      </c>
+      <c r="D6" s="14" t="inlineStr"/>
       <c r="E6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
@@ -901,11 +897,7 @@
           <t>WU: 1.000,01 USD–9,51 USD</t>
         </is>
       </c>
-      <c r="D12" s="14" t="inlineStr">
-        <is>
-          <t>WU: 0,75 USD–12 USD; Diğer: 700 TL–4.000 TL</t>
-        </is>
-      </c>
+      <c r="D12" s="14" t="inlineStr"/>
       <c r="E12" s="14" t="inlineStr"/>
       <c r="F12" s="14" t="inlineStr"/>
       <c r="G12" s="14" t="inlineStr">
@@ -933,11 +925,7 @@
           <t>Hesaba: Asgari 0 TL | Azami 0,94 TL</t>
         </is>
       </c>
-      <c r="D13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
-        </is>
-      </c>
+      <c r="D13" s="14" t="inlineStr"/>
       <c r="E13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
@@ -977,21 +965,13 @@
           <t>40.000 TL - 2.485,72 TL</t>
         </is>
       </c>
-      <c r="D14" s="14" t="inlineStr">
-        <is>
-          <t>3.500 TL - 13.500 TL</t>
-        </is>
-      </c>
+      <c r="D14" s="14" t="inlineStr"/>
       <c r="E14" s="14" t="inlineStr">
         <is>
           <t>2.170 TL - 2.170 TL</t>
         </is>
       </c>
-      <c r="F14" s="14" t="inlineStr">
-        <is>
-          <t>2.785,72 TL - 12.380,95 TL</t>
-        </is>
-      </c>
+      <c r="F14" s="14" t="inlineStr"/>
       <c r="G14" s="14" t="inlineStr">
         <is>
           <t>8.300 TL - 7,97 TL</t>

</xml_diff>

<commit_message>
Update benchmark: 2026-05-23 08:21:43 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -662,11 +662,7 @@
       <c r="D3" s="14" t="inlineStr"/>
       <c r="E3" s="14" t="inlineStr"/>
       <c r="F3" s="14" t="inlineStr"/>
-      <c r="G3" s="14" t="inlineStr">
-        <is>
-          <t>39,87 TRY - 79,76 TRY - 797,68 TRY</t>
-        </is>
-      </c>
+      <c r="G3" s="14" t="inlineStr"/>
       <c r="H3" s="14" t="inlineStr"/>
       <c r="I3" s="14" t="inlineStr"/>
       <c r="J3" s="14" t="inlineStr"/>
@@ -682,11 +678,7 @@
       <c r="D4" s="14" t="inlineStr"/>
       <c r="E4" s="14" t="inlineStr"/>
       <c r="F4" s="14" t="inlineStr"/>
-      <c r="G4" s="14" t="inlineStr">
-        <is>
-          <t>27,84 TRY - 55,69 TRY - 398,83 TRY</t>
-        </is>
-      </c>
+      <c r="G4" s="14" t="inlineStr"/>
       <c r="H4" s="14" t="inlineStr"/>
       <c r="I4" s="14" t="inlineStr"/>
       <c r="J4" s="14" t="inlineStr"/>
@@ -702,11 +694,7 @@
       <c r="D5" s="14" t="inlineStr"/>
       <c r="E5" s="14" t="inlineStr"/>
       <c r="F5" s="14" t="inlineStr"/>
-      <c r="G5" s="14" t="inlineStr">
-        <is>
-          <t>7,97 TRY - 15,96 TRY - 199,41 TRY</t>
-        </is>
-      </c>
+      <c r="G5" s="14" t="inlineStr"/>
       <c r="H5" s="14" t="inlineStr"/>
       <c r="I5" s="14" t="inlineStr"/>
       <c r="J5" s="14" t="inlineStr"/>
@@ -723,18 +711,18 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="D6" s="14" t="inlineStr"/>
+      <c r="D6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 199,41 TL</t>
+        </is>
+      </c>
       <c r="E6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
       <c r="F6" s="14" t="inlineStr"/>
-      <c r="G6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 99,71 TL</t>
-        </is>
-      </c>
+      <c r="G6" s="14" t="inlineStr"/>
       <c r="H6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
@@ -811,11 +799,7 @@
       <c r="D8" s="14" t="inlineStr"/>
       <c r="E8" s="14" t="inlineStr"/>
       <c r="F8" s="14" t="inlineStr"/>
-      <c r="G8" s="14" t="inlineStr">
-        <is>
-          <t>19,94 TRY - 39,88 TRY - 398,84 TRY</t>
-        </is>
-      </c>
+      <c r="G8" s="14" t="inlineStr"/>
       <c r="H8" s="14" t="inlineStr"/>
       <c r="I8" s="14" t="inlineStr"/>
       <c r="J8" s="14" t="inlineStr"/>
@@ -831,11 +815,7 @@
       <c r="D9" s="14" t="inlineStr"/>
       <c r="E9" s="14" t="inlineStr"/>
       <c r="F9" s="14" t="inlineStr"/>
-      <c r="G9" s="14" t="inlineStr">
-        <is>
-          <t>13,92 TRY - 27,85 TRY - 199,42 TRY</t>
-        </is>
-      </c>
+      <c r="G9" s="14" t="inlineStr"/>
       <c r="H9" s="14" t="inlineStr"/>
       <c r="I9" s="14" t="inlineStr"/>
       <c r="J9" s="14" t="inlineStr"/>
@@ -851,11 +831,7 @@
       <c r="D10" s="14" t="inlineStr"/>
       <c r="E10" s="14" t="inlineStr"/>
       <c r="F10" s="14" t="inlineStr"/>
-      <c r="G10" s="14" t="inlineStr">
-        <is>
-          <t>3,99 TRY - 7,98 TRY - 99,71 TRY</t>
-        </is>
-      </c>
+      <c r="G10" s="14" t="inlineStr"/>
       <c r="H10" s="14" t="inlineStr"/>
       <c r="I10" s="14" t="inlineStr"/>
       <c r="J10" s="14" t="inlineStr"/>
@@ -871,11 +847,7 @@
       <c r="D11" s="14" t="inlineStr"/>
       <c r="E11" s="14" t="inlineStr"/>
       <c r="F11" s="14" t="inlineStr"/>
-      <c r="G11" s="14" t="inlineStr">
-        <is>
-          <t>3,99 TRY - 7,98 TRY - 99,71 TRY</t>
-        </is>
-      </c>
+      <c r="G11" s="14" t="inlineStr"/>
       <c r="H11" s="14" t="inlineStr"/>
       <c r="I11" s="14" t="inlineStr"/>
       <c r="J11" s="14" t="inlineStr"/>
@@ -897,14 +869,14 @@
           <t>WU: 1.000,01 USD–9,51 USD</t>
         </is>
       </c>
-      <c r="D12" s="14" t="inlineStr"/>
+      <c r="D12" s="14" t="inlineStr">
+        <is>
+          <t>WU: 0,75 USD–12 USD; Diğer: 700 TL–4.000 TL</t>
+        </is>
+      </c>
       <c r="E12" s="14" t="inlineStr"/>
       <c r="F12" s="14" t="inlineStr"/>
-      <c r="G12" s="14" t="inlineStr">
-        <is>
-          <t>Şube (Kasadan): %0,5; Şube (Hesaptan): %0,75; İnternet: 15 USD</t>
-        </is>
-      </c>
+      <c r="G12" s="14" t="inlineStr"/>
       <c r="H12" s="14" t="inlineStr"/>
       <c r="I12" s="14" t="inlineStr"/>
       <c r="J12" s="14" t="inlineStr"/>
@@ -925,7 +897,11 @@
           <t>Hesaba: Asgari 0 TL | Azami 0,94 TL</t>
         </is>
       </c>
-      <c r="D13" s="14" t="inlineStr"/>
+      <c r="D13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
+        </is>
+      </c>
       <c r="E13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
@@ -965,18 +941,22 @@
           <t>40.000 TL - 2.485,72 TL</t>
         </is>
       </c>
-      <c r="D14" s="14" t="inlineStr"/>
+      <c r="D14" s="14" t="inlineStr">
+        <is>
+          <t>3.500 TL - 13.500 TL</t>
+        </is>
+      </c>
       <c r="E14" s="14" t="inlineStr">
         <is>
           <t>2.170 TL - 2.170 TL</t>
         </is>
       </c>
-      <c r="F14" s="14" t="inlineStr"/>
-      <c r="G14" s="14" t="inlineStr">
-        <is>
-          <t>8.300 TL - 7,97 TL</t>
-        </is>
-      </c>
+      <c r="F14" s="14" t="inlineStr">
+        <is>
+          <t>2.785,72 TL - 12.380,95 TL</t>
+        </is>
+      </c>
+      <c r="G14" s="14" t="inlineStr"/>
       <c r="H14" s="14" t="inlineStr">
         <is>
           <t>3.000 TL - 6.000 TL</t>

</xml_diff>

<commit_message>
Update benchmark: 2026-05-24 08:30:39 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -662,7 +662,11 @@
       <c r="D3" s="14" t="inlineStr"/>
       <c r="E3" s="14" t="inlineStr"/>
       <c r="F3" s="14" t="inlineStr"/>
-      <c r="G3" s="14" t="inlineStr"/>
+      <c r="G3" s="14" t="inlineStr">
+        <is>
+          <t>39,87 TRY - 79,76 TRY - 797,68 TRY</t>
+        </is>
+      </c>
       <c r="H3" s="14" t="inlineStr"/>
       <c r="I3" s="14" t="inlineStr"/>
       <c r="J3" s="14" t="inlineStr"/>
@@ -678,7 +682,11 @@
       <c r="D4" s="14" t="inlineStr"/>
       <c r="E4" s="14" t="inlineStr"/>
       <c r="F4" s="14" t="inlineStr"/>
-      <c r="G4" s="14" t="inlineStr"/>
+      <c r="G4" s="14" t="inlineStr">
+        <is>
+          <t>27,84 TRY - 55,69 TRY - 398,83 TRY</t>
+        </is>
+      </c>
       <c r="H4" s="14" t="inlineStr"/>
       <c r="I4" s="14" t="inlineStr"/>
       <c r="J4" s="14" t="inlineStr"/>
@@ -694,7 +702,11 @@
       <c r="D5" s="14" t="inlineStr"/>
       <c r="E5" s="14" t="inlineStr"/>
       <c r="F5" s="14" t="inlineStr"/>
-      <c r="G5" s="14" t="inlineStr"/>
+      <c r="G5" s="14" t="inlineStr">
+        <is>
+          <t>7,97 TRY - 15,96 TRY - 199,41 TRY</t>
+        </is>
+      </c>
       <c r="H5" s="14" t="inlineStr"/>
       <c r="I5" s="14" t="inlineStr"/>
       <c r="J5" s="14" t="inlineStr"/>
@@ -722,17 +734,17 @@
         </is>
       </c>
       <c r="F6" s="14" t="inlineStr"/>
-      <c r="G6" s="14" t="inlineStr"/>
+      <c r="G6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 99,71 TL</t>
+        </is>
+      </c>
       <c r="H6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="I6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 199,41 TL</t>
-        </is>
-      </c>
+      <c r="I6" s="14" t="inlineStr"/>
       <c r="J6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
@@ -799,7 +811,11 @@
       <c r="D8" s="14" t="inlineStr"/>
       <c r="E8" s="14" t="inlineStr"/>
       <c r="F8" s="14" t="inlineStr"/>
-      <c r="G8" s="14" t="inlineStr"/>
+      <c r="G8" s="14" t="inlineStr">
+        <is>
+          <t>19,94 TRY - 39,88 TRY - 398,84 TRY</t>
+        </is>
+      </c>
       <c r="H8" s="14" t="inlineStr"/>
       <c r="I8" s="14" t="inlineStr"/>
       <c r="J8" s="14" t="inlineStr"/>
@@ -815,7 +831,11 @@
       <c r="D9" s="14" t="inlineStr"/>
       <c r="E9" s="14" t="inlineStr"/>
       <c r="F9" s="14" t="inlineStr"/>
-      <c r="G9" s="14" t="inlineStr"/>
+      <c r="G9" s="14" t="inlineStr">
+        <is>
+          <t>13,92 TRY - 27,85 TRY - 199,42 TRY</t>
+        </is>
+      </c>
       <c r="H9" s="14" t="inlineStr"/>
       <c r="I9" s="14" t="inlineStr"/>
       <c r="J9" s="14" t="inlineStr"/>
@@ -831,7 +851,11 @@
       <c r="D10" s="14" t="inlineStr"/>
       <c r="E10" s="14" t="inlineStr"/>
       <c r="F10" s="14" t="inlineStr"/>
-      <c r="G10" s="14" t="inlineStr"/>
+      <c r="G10" s="14" t="inlineStr">
+        <is>
+          <t>3,99 TRY - 7,98 TRY - 99,71 TRY</t>
+        </is>
+      </c>
       <c r="H10" s="14" t="inlineStr"/>
       <c r="I10" s="14" t="inlineStr"/>
       <c r="J10" s="14" t="inlineStr"/>
@@ -847,7 +871,11 @@
       <c r="D11" s="14" t="inlineStr"/>
       <c r="E11" s="14" t="inlineStr"/>
       <c r="F11" s="14" t="inlineStr"/>
-      <c r="G11" s="14" t="inlineStr"/>
+      <c r="G11" s="14" t="inlineStr">
+        <is>
+          <t>3,99 TRY - 7,98 TRY - 99,71 TRY</t>
+        </is>
+      </c>
       <c r="H11" s="14" t="inlineStr"/>
       <c r="I11" s="14" t="inlineStr"/>
       <c r="J11" s="14" t="inlineStr"/>
@@ -871,12 +899,16 @@
       </c>
       <c r="D12" s="14" t="inlineStr">
         <is>
-          <t>WU: 0,75 USD–12 USD; Diğer: 700 TL–4.000 TL</t>
+          <t>Diğer: 700 TL–4.000 TL</t>
         </is>
       </c>
       <c r="E12" s="14" t="inlineStr"/>
       <c r="F12" s="14" t="inlineStr"/>
-      <c r="G12" s="14" t="inlineStr"/>
+      <c r="G12" s="14" t="inlineStr">
+        <is>
+          <t>Şube (Kasadan): %0,5; Şube (Hesaptan): %0,75; İnternet: 15 USD</t>
+        </is>
+      </c>
       <c r="H12" s="14" t="inlineStr"/>
       <c r="I12" s="14" t="inlineStr"/>
       <c r="J12" s="14" t="inlineStr"/>
@@ -914,11 +946,7 @@
           <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
         </is>
       </c>
-      <c r="I13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
-        </is>
-      </c>
+      <c r="I13" s="14" t="inlineStr"/>
       <c r="J13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.303 TL</t>
@@ -951,12 +979,12 @@
           <t>2.170 TL - 2.170 TL</t>
         </is>
       </c>
-      <c r="F14" s="14" t="inlineStr">
-        <is>
-          <t>2.785,72 TL - 12.380,95 TL</t>
-        </is>
-      </c>
-      <c r="G14" s="14" t="inlineStr"/>
+      <c r="F14" s="14" t="inlineStr"/>
+      <c r="G14" s="14" t="inlineStr">
+        <is>
+          <t>8.300 TL - 7,97 TL</t>
+        </is>
+      </c>
       <c r="H14" s="14" t="inlineStr">
         <is>
           <t>3.000 TL - 6.000 TL</t>

</xml_diff>

<commit_message>
Update benchmark: 2026-05-25 10:07:32 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -744,7 +744,11 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="I6" s="14" t="inlineStr"/>
+      <c r="I6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 199,41 TL</t>
+        </is>
+      </c>
       <c r="J6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
@@ -899,7 +903,7 @@
       </c>
       <c r="D12" s="14" t="inlineStr">
         <is>
-          <t>Diğer: 700 TL–4.000 TL</t>
+          <t>WU: 0,75 USD–12 USD; Diğer: 700 TL–4.000 TL</t>
         </is>
       </c>
       <c r="E12" s="14" t="inlineStr"/>
@@ -936,7 +940,7 @@
       </c>
       <c r="E13" s="14" t="inlineStr">
         <is>
-          <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
+          <t>Hesaba: Asgari 1 TL | Azami 11.380 TL</t>
         </is>
       </c>
       <c r="F13" s="14" t="inlineStr"/>
@@ -946,7 +950,11 @@
           <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
         </is>
       </c>
-      <c r="I13" s="14" t="inlineStr"/>
+      <c r="I13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
+        </is>
+      </c>
       <c r="J13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.303 TL</t>
@@ -979,7 +987,11 @@
           <t>2.170 TL - 2.170 TL</t>
         </is>
       </c>
-      <c r="F14" s="14" t="inlineStr"/>
+      <c r="F14" s="14" t="inlineStr">
+        <is>
+          <t>2.785,72 TL - 12.380,95 TL</t>
+        </is>
+      </c>
       <c r="G14" s="14" t="inlineStr">
         <is>
           <t>8.300 TL - 7,97 TL</t>

</xml_diff>

<commit_message>
Update benchmark: 2026-05-26 09:57:48 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -749,11 +749,7 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="J6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 199,41 TL</t>
-        </is>
-      </c>
+      <c r="J6" s="14" t="inlineStr"/>
       <c r="K6" s="14" t="inlineStr">
         <is>
           <t>7,97 TL - 15,96 TL - 199,41 TL</t>
@@ -940,7 +936,7 @@
       </c>
       <c r="E13" s="14" t="inlineStr">
         <is>
-          <t>Hesaba: Asgari 1 TL | Azami 11.380 TL</t>
+          <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
         </is>
       </c>
       <c r="F13" s="14" t="inlineStr"/>
@@ -955,11 +951,7 @@
           <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
         </is>
       </c>
-      <c r="J13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 1.303 TL</t>
-        </is>
-      </c>
+      <c r="J13" s="14" t="inlineStr"/>
       <c r="K13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 865,75 TL</t>
@@ -987,11 +979,7 @@
           <t>2.170 TL - 2.170 TL</t>
         </is>
       </c>
-      <c r="F14" s="14" t="inlineStr">
-        <is>
-          <t>2.785,72 TL - 12.380,95 TL</t>
-        </is>
-      </c>
+      <c r="F14" s="14" t="inlineStr"/>
       <c r="G14" s="14" t="inlineStr">
         <is>
           <t>8.300 TL - 7,97 TL</t>
@@ -1003,11 +991,7 @@
         </is>
       </c>
       <c r="I14" s="14" t="inlineStr"/>
-      <c r="J14" s="14" t="inlineStr">
-        <is>
-          <t>1.554,97 TL - 7.784 TL</t>
-        </is>
-      </c>
+      <c r="J14" s="14" t="inlineStr"/>
       <c r="K14" s="14" t="inlineStr">
         <is>
           <t>1.196,51 TL - 5.583,74 TL</t>

</xml_diff>

<commit_message>
Update benchmark: 2026-05-27 09:50:35 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -736,7 +736,7 @@
       <c r="F6" s="14" t="inlineStr"/>
       <c r="G6" s="14" t="inlineStr">
         <is>
-          <t>8.300,01 TL - 99,71 TL</t>
+          <t>8.300,01 TL - 57,5 TL - 115 TL</t>
         </is>
       </c>
       <c r="H6" s="14" t="inlineStr">
@@ -749,7 +749,11 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="J6" s="14" t="inlineStr"/>
+      <c r="J6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 199,41 TL</t>
+        </is>
+      </c>
       <c r="K6" s="14" t="inlineStr">
         <is>
           <t>7,97 TL - 15,96 TL - 199,41 TL</t>
@@ -811,11 +815,7 @@
       <c r="D8" s="14" t="inlineStr"/>
       <c r="E8" s="14" t="inlineStr"/>
       <c r="F8" s="14" t="inlineStr"/>
-      <c r="G8" s="14" t="inlineStr">
-        <is>
-          <t>19,94 TRY - 39,88 TRY - 398,84 TRY</t>
-        </is>
-      </c>
+      <c r="G8" s="14" t="inlineStr"/>
       <c r="H8" s="14" t="inlineStr"/>
       <c r="I8" s="14" t="inlineStr"/>
       <c r="J8" s="14" t="inlineStr"/>
@@ -831,11 +831,7 @@
       <c r="D9" s="14" t="inlineStr"/>
       <c r="E9" s="14" t="inlineStr"/>
       <c r="F9" s="14" t="inlineStr"/>
-      <c r="G9" s="14" t="inlineStr">
-        <is>
-          <t>13,92 TRY - 27,85 TRY - 199,42 TRY</t>
-        </is>
-      </c>
+      <c r="G9" s="14" t="inlineStr"/>
       <c r="H9" s="14" t="inlineStr"/>
       <c r="I9" s="14" t="inlineStr"/>
       <c r="J9" s="14" t="inlineStr"/>
@@ -851,11 +847,7 @@
       <c r="D10" s="14" t="inlineStr"/>
       <c r="E10" s="14" t="inlineStr"/>
       <c r="F10" s="14" t="inlineStr"/>
-      <c r="G10" s="14" t="inlineStr">
-        <is>
-          <t>3,99 TRY - 7,98 TRY - 99,71 TRY</t>
-        </is>
-      </c>
+      <c r="G10" s="14" t="inlineStr"/>
       <c r="H10" s="14" t="inlineStr"/>
       <c r="I10" s="14" t="inlineStr"/>
       <c r="J10" s="14" t="inlineStr"/>
@@ -871,11 +863,7 @@
       <c r="D11" s="14" t="inlineStr"/>
       <c r="E11" s="14" t="inlineStr"/>
       <c r="F11" s="14" t="inlineStr"/>
-      <c r="G11" s="14" t="inlineStr">
-        <is>
-          <t>3,99 TRY - 7,98 TRY - 99,71 TRY</t>
-        </is>
-      </c>
+      <c r="G11" s="14" t="inlineStr"/>
       <c r="H11" s="14" t="inlineStr"/>
       <c r="I11" s="14" t="inlineStr"/>
       <c r="J11" s="14" t="inlineStr"/>
@@ -904,11 +892,7 @@
       </c>
       <c r="E12" s="14" t="inlineStr"/>
       <c r="F12" s="14" t="inlineStr"/>
-      <c r="G12" s="14" t="inlineStr">
-        <is>
-          <t>Şube (Kasadan): %0,5; Şube (Hesaptan): %0,75; İnternet: 15 USD</t>
-        </is>
-      </c>
+      <c r="G12" s="14" t="inlineStr"/>
       <c r="H12" s="14" t="inlineStr"/>
       <c r="I12" s="14" t="inlineStr"/>
       <c r="J12" s="14" t="inlineStr"/>
@@ -979,12 +963,12 @@
           <t>2.170 TL - 2.170 TL</t>
         </is>
       </c>
-      <c r="F14" s="14" t="inlineStr"/>
-      <c r="G14" s="14" t="inlineStr">
-        <is>
-          <t>8.300 TL - 7,97 TL</t>
-        </is>
-      </c>
+      <c r="F14" s="14" t="inlineStr">
+        <is>
+          <t>2.785,72 TL - 12.380,95 TL</t>
+        </is>
+      </c>
+      <c r="G14" s="14" t="inlineStr"/>
       <c r="H14" s="14" t="inlineStr">
         <is>
           <t>3.000 TL - 6.000 TL</t>

</xml_diff>

<commit_message>
Update benchmark: 2026-05-28 10:02:06 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -736,7 +736,7 @@
       <c r="F6" s="14" t="inlineStr"/>
       <c r="G6" s="14" t="inlineStr">
         <is>
-          <t>8.300,01 TL - 57,5 TL - 115 TL</t>
+          <t>8.300,01 TL - 99,71 TL</t>
         </is>
       </c>
       <c r="H6" s="14" t="inlineStr">
@@ -815,7 +815,11 @@
       <c r="D8" s="14" t="inlineStr"/>
       <c r="E8" s="14" t="inlineStr"/>
       <c r="F8" s="14" t="inlineStr"/>
-      <c r="G8" s="14" t="inlineStr"/>
+      <c r="G8" s="14" t="inlineStr">
+        <is>
+          <t>19,94 TRY - 39,88 TRY - 398,84 TRY</t>
+        </is>
+      </c>
       <c r="H8" s="14" t="inlineStr"/>
       <c r="I8" s="14" t="inlineStr"/>
       <c r="J8" s="14" t="inlineStr"/>
@@ -831,7 +835,11 @@
       <c r="D9" s="14" t="inlineStr"/>
       <c r="E9" s="14" t="inlineStr"/>
       <c r="F9" s="14" t="inlineStr"/>
-      <c r="G9" s="14" t="inlineStr"/>
+      <c r="G9" s="14" t="inlineStr">
+        <is>
+          <t>13,92 TRY - 27,85 TRY - 199,42 TRY</t>
+        </is>
+      </c>
       <c r="H9" s="14" t="inlineStr"/>
       <c r="I9" s="14" t="inlineStr"/>
       <c r="J9" s="14" t="inlineStr"/>
@@ -847,7 +855,11 @@
       <c r="D10" s="14" t="inlineStr"/>
       <c r="E10" s="14" t="inlineStr"/>
       <c r="F10" s="14" t="inlineStr"/>
-      <c r="G10" s="14" t="inlineStr"/>
+      <c r="G10" s="14" t="inlineStr">
+        <is>
+          <t>3,99 TRY - 7,98 TRY - 99,71 TRY</t>
+        </is>
+      </c>
       <c r="H10" s="14" t="inlineStr"/>
       <c r="I10" s="14" t="inlineStr"/>
       <c r="J10" s="14" t="inlineStr"/>
@@ -863,7 +875,11 @@
       <c r="D11" s="14" t="inlineStr"/>
       <c r="E11" s="14" t="inlineStr"/>
       <c r="F11" s="14" t="inlineStr"/>
-      <c r="G11" s="14" t="inlineStr"/>
+      <c r="G11" s="14" t="inlineStr">
+        <is>
+          <t>3,99 TRY - 7,98 TRY - 99,71 TRY</t>
+        </is>
+      </c>
       <c r="H11" s="14" t="inlineStr"/>
       <c r="I11" s="14" t="inlineStr"/>
       <c r="J11" s="14" t="inlineStr"/>
@@ -892,7 +908,11 @@
       </c>
       <c r="E12" s="14" t="inlineStr"/>
       <c r="F12" s="14" t="inlineStr"/>
-      <c r="G12" s="14" t="inlineStr"/>
+      <c r="G12" s="14" t="inlineStr">
+        <is>
+          <t>Şube (Kasadan): %0,5; Şube (Hesaptan): %0,75; İnternet: 15 USD</t>
+        </is>
+      </c>
       <c r="H12" s="14" t="inlineStr"/>
       <c r="I12" s="14" t="inlineStr"/>
       <c r="J12" s="14" t="inlineStr"/>
@@ -935,7 +955,11 @@
           <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
         </is>
       </c>
-      <c r="J13" s="14" t="inlineStr"/>
+      <c r="J13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 1.303 TL</t>
+        </is>
+      </c>
       <c r="K13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 865,75 TL</t>
@@ -968,14 +992,22 @@
           <t>2.785,72 TL - 12.380,95 TL</t>
         </is>
       </c>
-      <c r="G14" s="14" t="inlineStr"/>
+      <c r="G14" s="14" t="inlineStr">
+        <is>
+          <t>8.300 TL - 7,97 TL</t>
+        </is>
+      </c>
       <c r="H14" s="14" t="inlineStr">
         <is>
           <t>3.000 TL - 6.000 TL</t>
         </is>
       </c>
       <c r="I14" s="14" t="inlineStr"/>
-      <c r="J14" s="14" t="inlineStr"/>
+      <c r="J14" s="14" t="inlineStr">
+        <is>
+          <t>1.554,97 TL - 7.784 TL</t>
+        </is>
+      </c>
       <c r="K14" s="14" t="inlineStr">
         <is>
           <t>1.196,51 TL - 5.583,74 TL</t>

</xml_diff>

<commit_message>
Update benchmark: 2026-05-30 08:29:37 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -744,11 +744,7 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="I6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 199,41 TL</t>
-        </is>
-      </c>
+      <c r="I6" s="14" t="inlineStr"/>
       <c r="J6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
@@ -903,7 +899,7 @@
       </c>
       <c r="D12" s="14" t="inlineStr">
         <is>
-          <t>WU: 0,75 USD–12 USD; Diğer: 700 TL–4.000 TL</t>
+          <t>Diğer: 700 TL–4.000 TL</t>
         </is>
       </c>
       <c r="E12" s="14" t="inlineStr"/>
@@ -950,11 +946,7 @@
           <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
         </is>
       </c>
-      <c r="I13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
-        </is>
-      </c>
+      <c r="I13" s="14" t="inlineStr"/>
       <c r="J13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.303 TL</t>

</xml_diff>

<commit_message>
Update benchmark: 2026-06-01 11:34:57 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -736,7 +736,7 @@
       <c r="F6" s="14" t="inlineStr"/>
       <c r="G6" s="14" t="inlineStr">
         <is>
-          <t>8.300,01 TL - 99,71 TL</t>
+          <t>8.300,01 TL - 57,5 TL - 115 TL</t>
         </is>
       </c>
       <c r="H6" s="14" t="inlineStr">
@@ -744,7 +744,11 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="I6" s="14" t="inlineStr"/>
+      <c r="I6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 199,41 TL</t>
+        </is>
+      </c>
       <c r="J6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
@@ -811,11 +815,7 @@
       <c r="D8" s="14" t="inlineStr"/>
       <c r="E8" s="14" t="inlineStr"/>
       <c r="F8" s="14" t="inlineStr"/>
-      <c r="G8" s="14" t="inlineStr">
-        <is>
-          <t>19,94 TRY - 39,88 TRY - 398,84 TRY</t>
-        </is>
-      </c>
+      <c r="G8" s="14" t="inlineStr"/>
       <c r="H8" s="14" t="inlineStr"/>
       <c r="I8" s="14" t="inlineStr"/>
       <c r="J8" s="14" t="inlineStr"/>
@@ -831,11 +831,7 @@
       <c r="D9" s="14" t="inlineStr"/>
       <c r="E9" s="14" t="inlineStr"/>
       <c r="F9" s="14" t="inlineStr"/>
-      <c r="G9" s="14" t="inlineStr">
-        <is>
-          <t>13,92 TRY - 27,85 TRY - 199,42 TRY</t>
-        </is>
-      </c>
+      <c r="G9" s="14" t="inlineStr"/>
       <c r="H9" s="14" t="inlineStr"/>
       <c r="I9" s="14" t="inlineStr"/>
       <c r="J9" s="14" t="inlineStr"/>
@@ -851,11 +847,7 @@
       <c r="D10" s="14" t="inlineStr"/>
       <c r="E10" s="14" t="inlineStr"/>
       <c r="F10" s="14" t="inlineStr"/>
-      <c r="G10" s="14" t="inlineStr">
-        <is>
-          <t>3,99 TRY - 7,98 TRY - 99,71 TRY</t>
-        </is>
-      </c>
+      <c r="G10" s="14" t="inlineStr"/>
       <c r="H10" s="14" t="inlineStr"/>
       <c r="I10" s="14" t="inlineStr"/>
       <c r="J10" s="14" t="inlineStr"/>
@@ -871,11 +863,7 @@
       <c r="D11" s="14" t="inlineStr"/>
       <c r="E11" s="14" t="inlineStr"/>
       <c r="F11" s="14" t="inlineStr"/>
-      <c r="G11" s="14" t="inlineStr">
-        <is>
-          <t>3,99 TRY - 7,98 TRY - 99,71 TRY</t>
-        </is>
-      </c>
+      <c r="G11" s="14" t="inlineStr"/>
       <c r="H11" s="14" t="inlineStr"/>
       <c r="I11" s="14" t="inlineStr"/>
       <c r="J11" s="14" t="inlineStr"/>
@@ -899,16 +887,12 @@
       </c>
       <c r="D12" s="14" t="inlineStr">
         <is>
-          <t>Diğer: 700 TL–4.000 TL</t>
+          <t>WU: 0,75 USD–12 USD; Diğer: 700 TL–4.000 TL</t>
         </is>
       </c>
       <c r="E12" s="14" t="inlineStr"/>
       <c r="F12" s="14" t="inlineStr"/>
-      <c r="G12" s="14" t="inlineStr">
-        <is>
-          <t>Şube (Kasadan): %0,5; Şube (Hesaptan): %0,75; İnternet: 15 USD</t>
-        </is>
-      </c>
+      <c r="G12" s="14" t="inlineStr"/>
       <c r="H12" s="14" t="inlineStr"/>
       <c r="I12" s="14" t="inlineStr"/>
       <c r="J12" s="14" t="inlineStr"/>
@@ -946,7 +930,11 @@
           <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
         </is>
       </c>
-      <c r="I13" s="14" t="inlineStr"/>
+      <c r="I13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
+        </is>
+      </c>
       <c r="J13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.303 TL</t>
@@ -984,11 +972,7 @@
           <t>2.785,72 TL - 12.380,95 TL</t>
         </is>
       </c>
-      <c r="G14" s="14" t="inlineStr">
-        <is>
-          <t>8.300 TL - 7,97 TL</t>
-        </is>
-      </c>
+      <c r="G14" s="14" t="inlineStr"/>
       <c r="H14" s="14" t="inlineStr">
         <is>
           <t>3.000 TL - 6.000 TL</t>

</xml_diff>

<commit_message>
Update benchmark: 2026-06-02 10:25:24 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -736,7 +736,7 @@
       <c r="F6" s="14" t="inlineStr"/>
       <c r="G6" s="14" t="inlineStr">
         <is>
-          <t>8.300,01 TL - 57,5 TL - 115 TL</t>
+          <t>8.300,01 TL - 99,71 TL</t>
         </is>
       </c>
       <c r="H6" s="14" t="inlineStr">
@@ -815,7 +815,11 @@
       <c r="D8" s="14" t="inlineStr"/>
       <c r="E8" s="14" t="inlineStr"/>
       <c r="F8" s="14" t="inlineStr"/>
-      <c r="G8" s="14" t="inlineStr"/>
+      <c r="G8" s="14" t="inlineStr">
+        <is>
+          <t>19,94 TRY - 39,88 TRY - 398,84 TRY</t>
+        </is>
+      </c>
       <c r="H8" s="14" t="inlineStr"/>
       <c r="I8" s="14" t="inlineStr"/>
       <c r="J8" s="14" t="inlineStr"/>
@@ -831,7 +835,11 @@
       <c r="D9" s="14" t="inlineStr"/>
       <c r="E9" s="14" t="inlineStr"/>
       <c r="F9" s="14" t="inlineStr"/>
-      <c r="G9" s="14" t="inlineStr"/>
+      <c r="G9" s="14" t="inlineStr">
+        <is>
+          <t>13,92 TRY - 27,85 TRY - 199,42 TRY</t>
+        </is>
+      </c>
       <c r="H9" s="14" t="inlineStr"/>
       <c r="I9" s="14" t="inlineStr"/>
       <c r="J9" s="14" t="inlineStr"/>
@@ -847,7 +855,11 @@
       <c r="D10" s="14" t="inlineStr"/>
       <c r="E10" s="14" t="inlineStr"/>
       <c r="F10" s="14" t="inlineStr"/>
-      <c r="G10" s="14" t="inlineStr"/>
+      <c r="G10" s="14" t="inlineStr">
+        <is>
+          <t>3,99 TRY - 7,98 TRY - 99,71 TRY</t>
+        </is>
+      </c>
       <c r="H10" s="14" t="inlineStr"/>
       <c r="I10" s="14" t="inlineStr"/>
       <c r="J10" s="14" t="inlineStr"/>
@@ -863,7 +875,11 @@
       <c r="D11" s="14" t="inlineStr"/>
       <c r="E11" s="14" t="inlineStr"/>
       <c r="F11" s="14" t="inlineStr"/>
-      <c r="G11" s="14" t="inlineStr"/>
+      <c r="G11" s="14" t="inlineStr">
+        <is>
+          <t>3,99 TRY - 7,98 TRY - 99,71 TRY</t>
+        </is>
+      </c>
       <c r="H11" s="14" t="inlineStr"/>
       <c r="I11" s="14" t="inlineStr"/>
       <c r="J11" s="14" t="inlineStr"/>
@@ -892,7 +908,11 @@
       </c>
       <c r="E12" s="14" t="inlineStr"/>
       <c r="F12" s="14" t="inlineStr"/>
-      <c r="G12" s="14" t="inlineStr"/>
+      <c r="G12" s="14" t="inlineStr">
+        <is>
+          <t>Şube (Kasadan): %0,5; Şube (Hesaptan): %0,75; İnternet: 15 USD</t>
+        </is>
+      </c>
       <c r="H12" s="14" t="inlineStr"/>
       <c r="I12" s="14" t="inlineStr"/>
       <c r="J12" s="14" t="inlineStr"/>
@@ -972,7 +992,11 @@
           <t>2.785,72 TL - 12.380,95 TL</t>
         </is>
       </c>
-      <c r="G14" s="14" t="inlineStr"/>
+      <c r="G14" s="14" t="inlineStr">
+        <is>
+          <t>8.300 TL - 7,97 TL</t>
+        </is>
+      </c>
       <c r="H14" s="14" t="inlineStr">
         <is>
           <t>3.000 TL - 6.000 TL</t>

</xml_diff>

<commit_message>
Update benchmark: 2026-06-03 11:01:10 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -601,11 +601,7 @@
         </is>
       </c>
       <c r="B2" s="13" t="inlineStr"/>
-      <c r="C2" s="14" t="inlineStr">
-        <is>
-          <t>30 TL - 30 TL</t>
-        </is>
-      </c>
+      <c r="C2" s="14" t="inlineStr"/>
       <c r="D2" s="14" t="inlineStr">
         <is>
           <t>33,33 TL - 33,33 TL</t>
@@ -898,7 +894,7 @@
       </c>
       <c r="C12" s="14" t="inlineStr">
         <is>
-          <t>WU: 1.000,01 USD–9,51 USD</t>
+          <t>WU: 1.000,01 USD–</t>
         </is>
       </c>
       <c r="D12" s="14" t="inlineStr">
@@ -930,7 +926,7 @@
       </c>
       <c r="C13" s="14" t="inlineStr">
         <is>
-          <t>Hesaba: Asgari 0 TL | Azami 0,94 TL</t>
+          <t>Hesaba: Asgari 0 TL | Azami 3.295,24 TL</t>
         </is>
       </c>
       <c r="D13" s="14" t="inlineStr">

</xml_diff>

<commit_message>
Update benchmark: 2026-06-04 09:57:17 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -601,7 +601,11 @@
         </is>
       </c>
       <c r="B2" s="13" t="inlineStr"/>
-      <c r="C2" s="14" t="inlineStr"/>
+      <c r="C2" s="14" t="inlineStr">
+        <is>
+          <t>30 TL - 30 TL</t>
+        </is>
+      </c>
       <c r="D2" s="14" t="inlineStr">
         <is>
           <t>33,33 TL - 33,33 TL</t>
@@ -714,11 +718,7 @@
           <t>DÜZENLİ EFT</t>
         </is>
       </c>
-      <c r="C6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 199,41 TL</t>
-        </is>
-      </c>
+      <c r="C6" s="14" t="inlineStr"/>
       <c r="D6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
@@ -732,7 +732,7 @@
       <c r="F6" s="14" t="inlineStr"/>
       <c r="G6" s="14" t="inlineStr">
         <is>
-          <t>8.300,01 TL - 99,71 TL</t>
+          <t>8.300,01 TL - 57,5 TL - 115 TL</t>
         </is>
       </c>
       <c r="H6" s="14" t="inlineStr">
@@ -811,11 +811,7 @@
       <c r="D8" s="14" t="inlineStr"/>
       <c r="E8" s="14" t="inlineStr"/>
       <c r="F8" s="14" t="inlineStr"/>
-      <c r="G8" s="14" t="inlineStr">
-        <is>
-          <t>19,94 TRY - 39,88 TRY - 398,84 TRY</t>
-        </is>
-      </c>
+      <c r="G8" s="14" t="inlineStr"/>
       <c r="H8" s="14" t="inlineStr"/>
       <c r="I8" s="14" t="inlineStr"/>
       <c r="J8" s="14" t="inlineStr"/>
@@ -831,11 +827,7 @@
       <c r="D9" s="14" t="inlineStr"/>
       <c r="E9" s="14" t="inlineStr"/>
       <c r="F9" s="14" t="inlineStr"/>
-      <c r="G9" s="14" t="inlineStr">
-        <is>
-          <t>13,92 TRY - 27,85 TRY - 199,42 TRY</t>
-        </is>
-      </c>
+      <c r="G9" s="14" t="inlineStr"/>
       <c r="H9" s="14" t="inlineStr"/>
       <c r="I9" s="14" t="inlineStr"/>
       <c r="J9" s="14" t="inlineStr"/>
@@ -851,11 +843,7 @@
       <c r="D10" s="14" t="inlineStr"/>
       <c r="E10" s="14" t="inlineStr"/>
       <c r="F10" s="14" t="inlineStr"/>
-      <c r="G10" s="14" t="inlineStr">
-        <is>
-          <t>3,99 TRY - 7,98 TRY - 99,71 TRY</t>
-        </is>
-      </c>
+      <c r="G10" s="14" t="inlineStr"/>
       <c r="H10" s="14" t="inlineStr"/>
       <c r="I10" s="14" t="inlineStr"/>
       <c r="J10" s="14" t="inlineStr"/>
@@ -871,11 +859,7 @@
       <c r="D11" s="14" t="inlineStr"/>
       <c r="E11" s="14" t="inlineStr"/>
       <c r="F11" s="14" t="inlineStr"/>
-      <c r="G11" s="14" t="inlineStr">
-        <is>
-          <t>3,99 TRY - 7,98 TRY - 99,71 TRY</t>
-        </is>
-      </c>
+      <c r="G11" s="14" t="inlineStr"/>
       <c r="H11" s="14" t="inlineStr"/>
       <c r="I11" s="14" t="inlineStr"/>
       <c r="J11" s="14" t="inlineStr"/>
@@ -892,23 +876,15 @@
           <t>GİDEN SWIFT</t>
         </is>
       </c>
-      <c r="C12" s="14" t="inlineStr">
-        <is>
-          <t>WU: 1.000,01 USD–</t>
-        </is>
-      </c>
+      <c r="C12" s="14" t="inlineStr"/>
       <c r="D12" s="14" t="inlineStr">
         <is>
-          <t>WU: 0,75 USD–12 USD; Diğer: 700 TL–4.000 TL</t>
+          <t>Diğer: 700 TL–4.000 TL</t>
         </is>
       </c>
       <c r="E12" s="14" t="inlineStr"/>
       <c r="F12" s="14" t="inlineStr"/>
-      <c r="G12" s="14" t="inlineStr">
-        <is>
-          <t>Şube (Kasadan): %0,5; Şube (Hesaptan): %0,75; İnternet: 15 USD</t>
-        </is>
-      </c>
+      <c r="G12" s="14" t="inlineStr"/>
       <c r="H12" s="14" t="inlineStr"/>
       <c r="I12" s="14" t="inlineStr"/>
       <c r="J12" s="14" t="inlineStr"/>
@@ -924,11 +900,7 @@
           <t>GELEN SWIFT</t>
         </is>
       </c>
-      <c r="C13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 0 TL | Azami 3.295,24 TL</t>
-        </is>
-      </c>
+      <c r="C13" s="14" t="inlineStr"/>
       <c r="D13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
@@ -941,11 +913,7 @@
       </c>
       <c r="F13" s="14" t="inlineStr"/>
       <c r="G13" s="14" t="inlineStr"/>
-      <c r="H13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
-        </is>
-      </c>
+      <c r="H13" s="14" t="inlineStr"/>
       <c r="I13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
@@ -968,11 +936,7 @@
           <t>GİDEN SWIFT - Mobil</t>
         </is>
       </c>
-      <c r="C14" s="14" t="inlineStr">
-        <is>
-          <t>40.000 TL - 2.485,72 TL</t>
-        </is>
-      </c>
+      <c r="C14" s="14" t="inlineStr"/>
       <c r="D14" s="14" t="inlineStr">
         <is>
           <t>3.500 TL - 13.500 TL</t>
@@ -988,16 +952,8 @@
           <t>2.785,72 TL - 12.380,95 TL</t>
         </is>
       </c>
-      <c r="G14" s="14" t="inlineStr">
-        <is>
-          <t>8.300 TL - 7,97 TL</t>
-        </is>
-      </c>
-      <c r="H14" s="14" t="inlineStr">
-        <is>
-          <t>3.000 TL - 6.000 TL</t>
-        </is>
-      </c>
+      <c r="G14" s="14" t="inlineStr"/>
+      <c r="H14" s="14" t="inlineStr"/>
       <c r="I14" s="14" t="inlineStr"/>
       <c r="J14" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update benchmark: 2026-06-05 09:52:04 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -601,11 +601,7 @@
         </is>
       </c>
       <c r="B2" s="13" t="inlineStr"/>
-      <c r="C2" s="14" t="inlineStr">
-        <is>
-          <t>30 TL - 30 TL</t>
-        </is>
-      </c>
+      <c r="C2" s="14" t="inlineStr"/>
       <c r="D2" s="14" t="inlineStr">
         <is>
           <t>33,33 TL - 33,33 TL</t>
@@ -718,12 +714,12 @@
           <t>DÜZENLİ EFT</t>
         </is>
       </c>
-      <c r="C6" s="14" t="inlineStr"/>
-      <c r="D6" s="14" t="inlineStr">
+      <c r="C6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
+      <c r="D6" s="14" t="inlineStr"/>
       <c r="E6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
@@ -732,7 +728,7 @@
       <c r="F6" s="14" t="inlineStr"/>
       <c r="G6" s="14" t="inlineStr">
         <is>
-          <t>8.300,01 TL - 57,5 TL - 115 TL</t>
+          <t>8.300,01 TL - 99,71 TL</t>
         </is>
       </c>
       <c r="H6" s="14" t="inlineStr">
@@ -811,7 +807,11 @@
       <c r="D8" s="14" t="inlineStr"/>
       <c r="E8" s="14" t="inlineStr"/>
       <c r="F8" s="14" t="inlineStr"/>
-      <c r="G8" s="14" t="inlineStr"/>
+      <c r="G8" s="14" t="inlineStr">
+        <is>
+          <t>19,94 TRY - 39,88 TRY - 398,84 TRY</t>
+        </is>
+      </c>
       <c r="H8" s="14" t="inlineStr"/>
       <c r="I8" s="14" t="inlineStr"/>
       <c r="J8" s="14" t="inlineStr"/>
@@ -827,7 +827,11 @@
       <c r="D9" s="14" t="inlineStr"/>
       <c r="E9" s="14" t="inlineStr"/>
       <c r="F9" s="14" t="inlineStr"/>
-      <c r="G9" s="14" t="inlineStr"/>
+      <c r="G9" s="14" t="inlineStr">
+        <is>
+          <t>13,92 TRY - 27,85 TRY - 199,42 TRY</t>
+        </is>
+      </c>
       <c r="H9" s="14" t="inlineStr"/>
       <c r="I9" s="14" t="inlineStr"/>
       <c r="J9" s="14" t="inlineStr"/>
@@ -843,7 +847,11 @@
       <c r="D10" s="14" t="inlineStr"/>
       <c r="E10" s="14" t="inlineStr"/>
       <c r="F10" s="14" t="inlineStr"/>
-      <c r="G10" s="14" t="inlineStr"/>
+      <c r="G10" s="14" t="inlineStr">
+        <is>
+          <t>3,99 TRY - 7,98 TRY - 99,71 TRY</t>
+        </is>
+      </c>
       <c r="H10" s="14" t="inlineStr"/>
       <c r="I10" s="14" t="inlineStr"/>
       <c r="J10" s="14" t="inlineStr"/>
@@ -859,7 +867,11 @@
       <c r="D11" s="14" t="inlineStr"/>
       <c r="E11" s="14" t="inlineStr"/>
       <c r="F11" s="14" t="inlineStr"/>
-      <c r="G11" s="14" t="inlineStr"/>
+      <c r="G11" s="14" t="inlineStr">
+        <is>
+          <t>3,99 TRY - 7,98 TRY - 99,71 TRY</t>
+        </is>
+      </c>
       <c r="H11" s="14" t="inlineStr"/>
       <c r="I11" s="14" t="inlineStr"/>
       <c r="J11" s="14" t="inlineStr"/>
@@ -876,15 +888,19 @@
           <t>GİDEN SWIFT</t>
         </is>
       </c>
-      <c r="C12" s="14" t="inlineStr"/>
-      <c r="D12" s="14" t="inlineStr">
-        <is>
-          <t>Diğer: 700 TL–4.000 TL</t>
-        </is>
-      </c>
+      <c r="C12" s="14" t="inlineStr">
+        <is>
+          <t>WU: 1.000,01 USD–</t>
+        </is>
+      </c>
+      <c r="D12" s="14" t="inlineStr"/>
       <c r="E12" s="14" t="inlineStr"/>
       <c r="F12" s="14" t="inlineStr"/>
-      <c r="G12" s="14" t="inlineStr"/>
+      <c r="G12" s="14" t="inlineStr">
+        <is>
+          <t>Şube (Kasadan): %0,5; Şube (Hesaptan): %0,75; İnternet: 15 USD</t>
+        </is>
+      </c>
       <c r="H12" s="14" t="inlineStr"/>
       <c r="I12" s="14" t="inlineStr"/>
       <c r="J12" s="14" t="inlineStr"/>
@@ -900,12 +916,12 @@
           <t>GELEN SWIFT</t>
         </is>
       </c>
-      <c r="C13" s="14" t="inlineStr"/>
-      <c r="D13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
-        </is>
-      </c>
+      <c r="C13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 0 TL | Azami 3.295,24 TL</t>
+        </is>
+      </c>
+      <c r="D13" s="14" t="inlineStr"/>
       <c r="E13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
@@ -913,7 +929,11 @@
       </c>
       <c r="F13" s="14" t="inlineStr"/>
       <c r="G13" s="14" t="inlineStr"/>
-      <c r="H13" s="14" t="inlineStr"/>
+      <c r="H13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
+        </is>
+      </c>
       <c r="I13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
@@ -936,12 +956,12 @@
           <t>GİDEN SWIFT - Mobil</t>
         </is>
       </c>
-      <c r="C14" s="14" t="inlineStr"/>
-      <c r="D14" s="14" t="inlineStr">
-        <is>
-          <t>3.500 TL - 13.500 TL</t>
-        </is>
-      </c>
+      <c r="C14" s="14" t="inlineStr">
+        <is>
+          <t>40.000 TL - 2.485,72 TL</t>
+        </is>
+      </c>
+      <c r="D14" s="14" t="inlineStr"/>
       <c r="E14" s="14" t="inlineStr">
         <is>
           <t>2.170 TL - 2.170 TL</t>
@@ -952,8 +972,16 @@
           <t>2.785,72 TL - 12.380,95 TL</t>
         </is>
       </c>
-      <c r="G14" s="14" t="inlineStr"/>
-      <c r="H14" s="14" t="inlineStr"/>
+      <c r="G14" s="14" t="inlineStr">
+        <is>
+          <t>8.300 TL - 7,97 TL</t>
+        </is>
+      </c>
+      <c r="H14" s="14" t="inlineStr">
+        <is>
+          <t>3.000 TL - 6.000 TL</t>
+        </is>
+      </c>
       <c r="I14" s="14" t="inlineStr"/>
       <c r="J14" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update benchmark: 2026-06-06 08:34:41 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -601,7 +601,11 @@
         </is>
       </c>
       <c r="B2" s="13" t="inlineStr"/>
-      <c r="C2" s="14" t="inlineStr"/>
+      <c r="C2" s="14" t="inlineStr">
+        <is>
+          <t>30 TL - 30 TL</t>
+        </is>
+      </c>
       <c r="D2" s="14" t="inlineStr">
         <is>
           <t>33,33 TL - 33,33 TL</t>
@@ -714,12 +718,12 @@
           <t>DÜZENLİ EFT</t>
         </is>
       </c>
-      <c r="C6" s="14" t="inlineStr">
+      <c r="C6" s="14" t="inlineStr"/>
+      <c r="D6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="D6" s="14" t="inlineStr"/>
       <c r="E6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
@@ -746,11 +750,7 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="K6" s="14" t="inlineStr">
-        <is>
-          <t>7,97 TL - 15,96 TL - 199,41 TL</t>
-        </is>
-      </c>
+      <c r="K6" s="14" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="B7" s="13" t="inlineStr">
@@ -888,11 +888,7 @@
           <t>GİDEN SWIFT</t>
         </is>
       </c>
-      <c r="C12" s="14" t="inlineStr">
-        <is>
-          <t>WU: 1.000,01 USD–</t>
-        </is>
-      </c>
+      <c r="C12" s="14" t="inlineStr"/>
       <c r="D12" s="14" t="inlineStr"/>
       <c r="E12" s="14" t="inlineStr"/>
       <c r="F12" s="14" t="inlineStr"/>
@@ -904,11 +900,7 @@
       <c r="H12" s="14" t="inlineStr"/>
       <c r="I12" s="14" t="inlineStr"/>
       <c r="J12" s="14" t="inlineStr"/>
-      <c r="K12" s="14" t="inlineStr">
-        <is>
-          <t>WU: ,USD–; Diğer: 529 TL–4.454,74 TL</t>
-        </is>
-      </c>
+      <c r="K12" s="14" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="B13" s="13" t="inlineStr">
@@ -916,39 +908,23 @@
           <t>GELEN SWIFT</t>
         </is>
       </c>
-      <c r="C13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 0 TL | Azami 3.295,24 TL</t>
-        </is>
-      </c>
+      <c r="C13" s="14" t="inlineStr"/>
       <c r="D13" s="14" t="inlineStr"/>
-      <c r="E13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
-        </is>
-      </c>
+      <c r="E13" s="14" t="inlineStr"/>
       <c r="F13" s="14" t="inlineStr"/>
       <c r="G13" s="14" t="inlineStr"/>
-      <c r="H13" s="14" t="inlineStr">
+      <c r="H13" s="14" t="inlineStr"/>
+      <c r="I13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
         </is>
       </c>
-      <c r="I13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
-        </is>
-      </c>
       <c r="J13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.303 TL</t>
         </is>
       </c>
-      <c r="K13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 865,75 TL</t>
-        </is>
-      </c>
+      <c r="K13" s="14" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="B14" s="13" t="inlineStr">
@@ -956,17 +932,9 @@
           <t>GİDEN SWIFT - Mobil</t>
         </is>
       </c>
-      <c r="C14" s="14" t="inlineStr">
-        <is>
-          <t>40.000 TL - 2.485,72 TL</t>
-        </is>
-      </c>
+      <c r="C14" s="14" t="inlineStr"/>
       <c r="D14" s="14" t="inlineStr"/>
-      <c r="E14" s="14" t="inlineStr">
-        <is>
-          <t>2.170 TL - 2.170 TL</t>
-        </is>
-      </c>
+      <c r="E14" s="14" t="inlineStr"/>
       <c r="F14" s="14" t="inlineStr">
         <is>
           <t>2.785,72 TL - 12.380,95 TL</t>
@@ -977,22 +945,14 @@
           <t>8.300 TL - 7,97 TL</t>
         </is>
       </c>
-      <c r="H14" s="14" t="inlineStr">
-        <is>
-          <t>3.000 TL - 6.000 TL</t>
-        </is>
-      </c>
+      <c r="H14" s="14" t="inlineStr"/>
       <c r="I14" s="14" t="inlineStr"/>
       <c r="J14" s="14" t="inlineStr">
         <is>
           <t>1.554,97 TL - 7.784 TL</t>
         </is>
       </c>
-      <c r="K14" s="14" t="inlineStr">
-        <is>
-          <t>1.196,51 TL - 5.583,74 TL</t>
-        </is>
-      </c>
+      <c r="K14" s="14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="12" t="inlineStr">

</xml_diff>

<commit_message>
Update benchmark: 2026-06-07 08:57:31 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -718,12 +718,12 @@
           <t>DÜZENLİ EFT</t>
         </is>
       </c>
-      <c r="C6" s="14" t="inlineStr"/>
-      <c r="D6" s="14" t="inlineStr">
+      <c r="C6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
+      <c r="D6" s="14" t="inlineStr"/>
       <c r="E6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
@@ -750,7 +750,11 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="K6" s="14" t="inlineStr"/>
+      <c r="K6" s="14" t="inlineStr">
+        <is>
+          <t>7,97 TL - 15,96 TL - 199,41 TL</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="B7" s="13" t="inlineStr">
@@ -888,7 +892,11 @@
           <t>GİDEN SWIFT</t>
         </is>
       </c>
-      <c r="C12" s="14" t="inlineStr"/>
+      <c r="C12" s="14" t="inlineStr">
+        <is>
+          <t>WU: 1.000,01 USD–9,51 USD</t>
+        </is>
+      </c>
       <c r="D12" s="14" t="inlineStr"/>
       <c r="E12" s="14" t="inlineStr"/>
       <c r="F12" s="14" t="inlineStr"/>
@@ -900,7 +908,11 @@
       <c r="H12" s="14" t="inlineStr"/>
       <c r="I12" s="14" t="inlineStr"/>
       <c r="J12" s="14" t="inlineStr"/>
-      <c r="K12" s="14" t="inlineStr"/>
+      <c r="K12" s="14" t="inlineStr">
+        <is>
+          <t>WU: ,USD–; Diğer: 529 TL–4.454,74 TL</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="B13" s="13" t="inlineStr">
@@ -908,23 +920,35 @@
           <t>GELEN SWIFT</t>
         </is>
       </c>
-      <c r="C13" s="14" t="inlineStr"/>
+      <c r="C13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 0 TL | Azami 0,94 TL</t>
+        </is>
+      </c>
       <c r="D13" s="14" t="inlineStr"/>
-      <c r="E13" s="14" t="inlineStr"/>
+      <c r="E13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
+        </is>
+      </c>
       <c r="F13" s="14" t="inlineStr"/>
       <c r="G13" s="14" t="inlineStr"/>
-      <c r="H13" s="14" t="inlineStr"/>
-      <c r="I13" s="14" t="inlineStr">
+      <c r="H13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
         </is>
       </c>
+      <c r="I13" s="14" t="inlineStr"/>
       <c r="J13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.303 TL</t>
         </is>
       </c>
-      <c r="K13" s="14" t="inlineStr"/>
+      <c r="K13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 865,75 TL</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="B14" s="13" t="inlineStr">
@@ -932,27 +956,39 @@
           <t>GİDEN SWIFT - Mobil</t>
         </is>
       </c>
-      <c r="C14" s="14" t="inlineStr"/>
+      <c r="C14" s="14" t="inlineStr">
+        <is>
+          <t>40.000 TL - 2.485,72 TL</t>
+        </is>
+      </c>
       <c r="D14" s="14" t="inlineStr"/>
-      <c r="E14" s="14" t="inlineStr"/>
-      <c r="F14" s="14" t="inlineStr">
-        <is>
-          <t>2.785,72 TL - 12.380,95 TL</t>
-        </is>
-      </c>
+      <c r="E14" s="14" t="inlineStr">
+        <is>
+          <t>2.170 TL - 2.170 TL</t>
+        </is>
+      </c>
+      <c r="F14" s="14" t="inlineStr"/>
       <c r="G14" s="14" t="inlineStr">
         <is>
           <t>8.300 TL - 7,97 TL</t>
         </is>
       </c>
-      <c r="H14" s="14" t="inlineStr"/>
+      <c r="H14" s="14" t="inlineStr">
+        <is>
+          <t>3.000 TL - 6.000 TL</t>
+        </is>
+      </c>
       <c r="I14" s="14" t="inlineStr"/>
       <c r="J14" s="14" t="inlineStr">
         <is>
           <t>1.554,97 TL - 7.784 TL</t>
         </is>
       </c>
-      <c r="K14" s="14" t="inlineStr"/>
+      <c r="K14" s="14" t="inlineStr">
+        <is>
+          <t>1.196,51 TL - 5.583,74 TL</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="12" t="inlineStr">

</xml_diff>

<commit_message>
Update benchmark: 2026-06-08 10:56:28 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -723,7 +723,11 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="D6" s="14" t="inlineStr"/>
+      <c r="D6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 199,41 TL</t>
+        </is>
+      </c>
       <c r="E6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
@@ -897,7 +901,11 @@
           <t>WU: 1.000,01 USD–9,51 USD</t>
         </is>
       </c>
-      <c r="D12" s="14" t="inlineStr"/>
+      <c r="D12" s="14" t="inlineStr">
+        <is>
+          <t>WU: 0,75 USD–12 USD; Diğer: 700 TL–4.000 TL</t>
+        </is>
+      </c>
       <c r="E12" s="14" t="inlineStr"/>
       <c r="F12" s="14" t="inlineStr"/>
       <c r="G12" s="14" t="inlineStr">
@@ -925,7 +933,11 @@
           <t>Hesaba: Asgari 0 TL | Azami 0,94 TL</t>
         </is>
       </c>
-      <c r="D13" s="14" t="inlineStr"/>
+      <c r="D13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
+        </is>
+      </c>
       <c r="E13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
@@ -938,7 +950,11 @@
           <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
         </is>
       </c>
-      <c r="I13" s="14" t="inlineStr"/>
+      <c r="I13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
+        </is>
+      </c>
       <c r="J13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.303 TL</t>
@@ -961,13 +977,21 @@
           <t>40.000 TL - 2.485,72 TL</t>
         </is>
       </c>
-      <c r="D14" s="14" t="inlineStr"/>
+      <c r="D14" s="14" t="inlineStr">
+        <is>
+          <t>3.500 TL - 13.500 TL</t>
+        </is>
+      </c>
       <c r="E14" s="14" t="inlineStr">
         <is>
           <t>2.170 TL - 2.170 TL</t>
         </is>
       </c>
-      <c r="F14" s="14" t="inlineStr"/>
+      <c r="F14" s="14" t="inlineStr">
+        <is>
+          <t>2.785,72 TL - 12.380,95 TL</t>
+        </is>
+      </c>
       <c r="G14" s="14" t="inlineStr">
         <is>
           <t>8.300 TL - 7,97 TL</t>

</xml_diff>

<commit_message>
Update benchmark: 2026-06-10 10:01:29 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -723,11 +723,7 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="D6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 199,41 TL</t>
-        </is>
-      </c>
+      <c r="D6" s="14" t="inlineStr"/>
       <c r="E6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
@@ -901,11 +897,7 @@
           <t>WU: 1.000,01 USD–9,51 USD</t>
         </is>
       </c>
-      <c r="D12" s="14" t="inlineStr">
-        <is>
-          <t>WU: 0,75 USD–12 USD; Diğer: 700 TL–4.000 TL</t>
-        </is>
-      </c>
+      <c r="D12" s="14" t="inlineStr"/>
       <c r="E12" s="14" t="inlineStr"/>
       <c r="F12" s="14" t="inlineStr"/>
       <c r="G12" s="14" t="inlineStr">
@@ -933,11 +925,7 @@
           <t>Hesaba: Asgari 0 TL | Azami 0,94 TL</t>
         </is>
       </c>
-      <c r="D13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
-        </is>
-      </c>
+      <c r="D13" s="14" t="inlineStr"/>
       <c r="E13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
@@ -977,11 +965,7 @@
           <t>40.000 TL - 2.485,72 TL</t>
         </is>
       </c>
-      <c r="D14" s="14" t="inlineStr">
-        <is>
-          <t>3.500 TL - 13.500 TL</t>
-        </is>
-      </c>
+      <c r="D14" s="14" t="inlineStr"/>
       <c r="E14" s="14" t="inlineStr">
         <is>
           <t>2.170 TL - 2.170 TL</t>

</xml_diff>

<commit_message>
Update benchmark: 2026-06-11 10:25:44 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -723,7 +723,11 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="D6" s="14" t="inlineStr"/>
+      <c r="D6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 199,41 TL</t>
+        </is>
+      </c>
       <c r="E6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
@@ -897,7 +901,11 @@
           <t>WU: 1.000,01 USD–9,51 USD</t>
         </is>
       </c>
-      <c r="D12" s="14" t="inlineStr"/>
+      <c r="D12" s="14" t="inlineStr">
+        <is>
+          <t>WU: 0,75 USD–12 USD; Diğer: 700 TL–4.000 TL</t>
+        </is>
+      </c>
       <c r="E12" s="14" t="inlineStr"/>
       <c r="F12" s="14" t="inlineStr"/>
       <c r="G12" s="14" t="inlineStr">
@@ -925,7 +933,11 @@
           <t>Hesaba: Asgari 0 TL | Azami 0,94 TL</t>
         </is>
       </c>
-      <c r="D13" s="14" t="inlineStr"/>
+      <c r="D13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
+        </is>
+      </c>
       <c r="E13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
@@ -965,7 +977,11 @@
           <t>40.000 TL - 2.485,72 TL</t>
         </is>
       </c>
-      <c r="D14" s="14" t="inlineStr"/>
+      <c r="D14" s="14" t="inlineStr">
+        <is>
+          <t>3.500 TL - 13.500 TL</t>
+        </is>
+      </c>
       <c r="E14" s="14" t="inlineStr">
         <is>
           <t>2.170 TL - 2.170 TL</t>

</xml_diff>

<commit_message>
Update benchmark: 2026-06-14 09:35:18 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -736,7 +736,7 @@
       <c r="F6" s="14" t="inlineStr"/>
       <c r="G6" s="14" t="inlineStr">
         <is>
-          <t>8.300,01 TL - 99,71 TL</t>
+          <t>8.300,01 TL - 57,5 TL - 115 TL</t>
         </is>
       </c>
       <c r="H6" s="14" t="inlineStr">
@@ -744,11 +744,7 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="I6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 199,41 TL</t>
-        </is>
-      </c>
+      <c r="I6" s="14" t="inlineStr"/>
       <c r="J6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
@@ -815,11 +811,7 @@
       <c r="D8" s="14" t="inlineStr"/>
       <c r="E8" s="14" t="inlineStr"/>
       <c r="F8" s="14" t="inlineStr"/>
-      <c r="G8" s="14" t="inlineStr">
-        <is>
-          <t>19,94 TRY - 39,88 TRY - 398,84 TRY</t>
-        </is>
-      </c>
+      <c r="G8" s="14" t="inlineStr"/>
       <c r="H8" s="14" t="inlineStr"/>
       <c r="I8" s="14" t="inlineStr"/>
       <c r="J8" s="14" t="inlineStr"/>
@@ -835,11 +827,7 @@
       <c r="D9" s="14" t="inlineStr"/>
       <c r="E9" s="14" t="inlineStr"/>
       <c r="F9" s="14" t="inlineStr"/>
-      <c r="G9" s="14" t="inlineStr">
-        <is>
-          <t>13,92 TRY - 27,85 TRY - 199,42 TRY</t>
-        </is>
-      </c>
+      <c r="G9" s="14" t="inlineStr"/>
       <c r="H9" s="14" t="inlineStr"/>
       <c r="I9" s="14" t="inlineStr"/>
       <c r="J9" s="14" t="inlineStr"/>
@@ -855,11 +843,7 @@
       <c r="D10" s="14" t="inlineStr"/>
       <c r="E10" s="14" t="inlineStr"/>
       <c r="F10" s="14" t="inlineStr"/>
-      <c r="G10" s="14" t="inlineStr">
-        <is>
-          <t>3,99 TRY - 7,98 TRY - 99,71 TRY</t>
-        </is>
-      </c>
+      <c r="G10" s="14" t="inlineStr"/>
       <c r="H10" s="14" t="inlineStr"/>
       <c r="I10" s="14" t="inlineStr"/>
       <c r="J10" s="14" t="inlineStr"/>
@@ -875,11 +859,7 @@
       <c r="D11" s="14" t="inlineStr"/>
       <c r="E11" s="14" t="inlineStr"/>
       <c r="F11" s="14" t="inlineStr"/>
-      <c r="G11" s="14" t="inlineStr">
-        <is>
-          <t>3,99 TRY - 7,98 TRY - 99,71 TRY</t>
-        </is>
-      </c>
+      <c r="G11" s="14" t="inlineStr"/>
       <c r="H11" s="14" t="inlineStr"/>
       <c r="I11" s="14" t="inlineStr"/>
       <c r="J11" s="14" t="inlineStr"/>
@@ -908,11 +888,7 @@
       </c>
       <c r="E12" s="14" t="inlineStr"/>
       <c r="F12" s="14" t="inlineStr"/>
-      <c r="G12" s="14" t="inlineStr">
-        <is>
-          <t>Şube (Kasadan): %0,5; Şube (Hesaptan): %0,75; İnternet: 15 USD</t>
-        </is>
-      </c>
+      <c r="G12" s="14" t="inlineStr"/>
       <c r="H12" s="14" t="inlineStr"/>
       <c r="I12" s="14" t="inlineStr"/>
       <c r="J12" s="14" t="inlineStr"/>
@@ -938,11 +914,7 @@
           <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
         </is>
       </c>
-      <c r="E13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
-        </is>
-      </c>
+      <c r="E13" s="14" t="inlineStr"/>
       <c r="F13" s="14" t="inlineStr"/>
       <c r="G13" s="14" t="inlineStr"/>
       <c r="H13" s="14" t="inlineStr">
@@ -950,11 +922,7 @@
           <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
         </is>
       </c>
-      <c r="I13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
-        </is>
-      </c>
+      <c r="I13" s="14" t="inlineStr"/>
       <c r="J13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.303 TL</t>
@@ -982,21 +950,9 @@
           <t>3.500 TL - 13.500 TL</t>
         </is>
       </c>
-      <c r="E14" s="14" t="inlineStr">
-        <is>
-          <t>2.170 TL - 2.170 TL</t>
-        </is>
-      </c>
-      <c r="F14" s="14" t="inlineStr">
-        <is>
-          <t>2.785,72 TL - 12.380,95 TL</t>
-        </is>
-      </c>
-      <c r="G14" s="14" t="inlineStr">
-        <is>
-          <t>8.300 TL - 7,97 TL</t>
-        </is>
-      </c>
+      <c r="E14" s="14" t="inlineStr"/>
+      <c r="F14" s="14" t="inlineStr"/>
+      <c r="G14" s="14" t="inlineStr"/>
       <c r="H14" s="14" t="inlineStr">
         <is>
           <t>3.000 TL - 6.000 TL</t>

</xml_diff>

<commit_message>
Update benchmark: 2026-06-16 11:12:04 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -736,7 +736,7 @@
       <c r="F6" s="14" t="inlineStr"/>
       <c r="G6" s="14" t="inlineStr">
         <is>
-          <t>8.300,01 TL - 57,5 TL - 115 TL</t>
+          <t>8.300,01 TL - 99,71 TL</t>
         </is>
       </c>
       <c r="H6" s="14" t="inlineStr">
@@ -744,7 +744,11 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="I6" s="14" t="inlineStr"/>
+      <c r="I6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 199,41 TL</t>
+        </is>
+      </c>
       <c r="J6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
@@ -811,7 +815,11 @@
       <c r="D8" s="14" t="inlineStr"/>
       <c r="E8" s="14" t="inlineStr"/>
       <c r="F8" s="14" t="inlineStr"/>
-      <c r="G8" s="14" t="inlineStr"/>
+      <c r="G8" s="14" t="inlineStr">
+        <is>
+          <t>19,94 TRY - 39,88 TRY - 398,84 TRY</t>
+        </is>
+      </c>
       <c r="H8" s="14" t="inlineStr"/>
       <c r="I8" s="14" t="inlineStr"/>
       <c r="J8" s="14" t="inlineStr"/>
@@ -827,7 +835,11 @@
       <c r="D9" s="14" t="inlineStr"/>
       <c r="E9" s="14" t="inlineStr"/>
       <c r="F9" s="14" t="inlineStr"/>
-      <c r="G9" s="14" t="inlineStr"/>
+      <c r="G9" s="14" t="inlineStr">
+        <is>
+          <t>13,92 TRY - 27,85 TRY - 199,42 TRY</t>
+        </is>
+      </c>
       <c r="H9" s="14" t="inlineStr"/>
       <c r="I9" s="14" t="inlineStr"/>
       <c r="J9" s="14" t="inlineStr"/>
@@ -843,7 +855,11 @@
       <c r="D10" s="14" t="inlineStr"/>
       <c r="E10" s="14" t="inlineStr"/>
       <c r="F10" s="14" t="inlineStr"/>
-      <c r="G10" s="14" t="inlineStr"/>
+      <c r="G10" s="14" t="inlineStr">
+        <is>
+          <t>3,99 TRY - 7,98 TRY - 99,71 TRY</t>
+        </is>
+      </c>
       <c r="H10" s="14" t="inlineStr"/>
       <c r="I10" s="14" t="inlineStr"/>
       <c r="J10" s="14" t="inlineStr"/>
@@ -859,7 +875,11 @@
       <c r="D11" s="14" t="inlineStr"/>
       <c r="E11" s="14" t="inlineStr"/>
       <c r="F11" s="14" t="inlineStr"/>
-      <c r="G11" s="14" t="inlineStr"/>
+      <c r="G11" s="14" t="inlineStr">
+        <is>
+          <t>3,99 TRY - 7,98 TRY - 99,71 TRY</t>
+        </is>
+      </c>
       <c r="H11" s="14" t="inlineStr"/>
       <c r="I11" s="14" t="inlineStr"/>
       <c r="J11" s="14" t="inlineStr"/>
@@ -888,7 +908,11 @@
       </c>
       <c r="E12" s="14" t="inlineStr"/>
       <c r="F12" s="14" t="inlineStr"/>
-      <c r="G12" s="14" t="inlineStr"/>
+      <c r="G12" s="14" t="inlineStr">
+        <is>
+          <t>Şube (Kasadan): %0,5; Şube (Hesaptan): %0,75; İnternet: 15 USD</t>
+        </is>
+      </c>
       <c r="H12" s="14" t="inlineStr"/>
       <c r="I12" s="14" t="inlineStr"/>
       <c r="J12" s="14" t="inlineStr"/>
@@ -914,7 +938,11 @@
           <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
         </is>
       </c>
-      <c r="E13" s="14" t="inlineStr"/>
+      <c r="E13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
+        </is>
+      </c>
       <c r="F13" s="14" t="inlineStr"/>
       <c r="G13" s="14" t="inlineStr"/>
       <c r="H13" s="14" t="inlineStr">
@@ -922,7 +950,11 @@
           <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
         </is>
       </c>
-      <c r="I13" s="14" t="inlineStr"/>
+      <c r="I13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
+        </is>
+      </c>
       <c r="J13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.303 TL</t>
@@ -950,9 +982,21 @@
           <t>3.500 TL - 13.500 TL</t>
         </is>
       </c>
-      <c r="E14" s="14" t="inlineStr"/>
-      <c r="F14" s="14" t="inlineStr"/>
-      <c r="G14" s="14" t="inlineStr"/>
+      <c r="E14" s="14" t="inlineStr">
+        <is>
+          <t>2.170 TL - 2.170 TL</t>
+        </is>
+      </c>
+      <c r="F14" s="14" t="inlineStr">
+        <is>
+          <t>2.785,72 TL - 12.380,95 TL</t>
+        </is>
+      </c>
+      <c r="G14" s="14" t="inlineStr">
+        <is>
+          <t>8.300 TL - 7,97 TL</t>
+        </is>
+      </c>
       <c r="H14" s="14" t="inlineStr">
         <is>
           <t>3.000 TL - 6.000 TL</t>

</xml_diff>

<commit_message>
Update benchmark: 2026-06-18 10:22:03 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -718,11 +718,7 @@
           <t>DÜZENLİ EFT</t>
         </is>
       </c>
-      <c r="C6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 199,41 TL</t>
-        </is>
-      </c>
+      <c r="C6" s="14" t="inlineStr"/>
       <c r="D6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
@@ -896,11 +892,7 @@
           <t>GİDEN SWIFT</t>
         </is>
       </c>
-      <c r="C12" s="14" t="inlineStr">
-        <is>
-          <t>WU: 1.000,01 USD–9,51 USD</t>
-        </is>
-      </c>
+      <c r="C12" s="14" t="inlineStr"/>
       <c r="D12" s="14" t="inlineStr">
         <is>
           <t>WU: 0,75 USD–12 USD; Diğer: 700 TL–4.000 TL</t>
@@ -928,11 +920,7 @@
           <t>GELEN SWIFT</t>
         </is>
       </c>
-      <c r="C13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 0 TL | Azami 0,94 TL</t>
-        </is>
-      </c>
+      <c r="C13" s="14" t="inlineStr"/>
       <c r="D13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
@@ -972,11 +960,7 @@
           <t>GİDEN SWIFT - Mobil</t>
         </is>
       </c>
-      <c r="C14" s="14" t="inlineStr">
-        <is>
-          <t>40.000 TL - 2.485,72 TL</t>
-        </is>
-      </c>
+      <c r="C14" s="14" t="inlineStr"/>
       <c r="D14" s="14" t="inlineStr">
         <is>
           <t>3.500 TL - 13.500 TL</t>

</xml_diff>

<commit_message>
Update benchmark: 2026-06-19 10:27:31 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -718,7 +718,11 @@
           <t>DÜZENLİ EFT</t>
         </is>
       </c>
-      <c r="C6" s="14" t="inlineStr"/>
+      <c r="C6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 199,41 TL</t>
+        </is>
+      </c>
       <c r="D6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
@@ -892,7 +896,11 @@
           <t>GİDEN SWIFT</t>
         </is>
       </c>
-      <c r="C12" s="14" t="inlineStr"/>
+      <c r="C12" s="14" t="inlineStr">
+        <is>
+          <t>WU: 1.000,01 USD–9,51 USD</t>
+        </is>
+      </c>
       <c r="D12" s="14" t="inlineStr">
         <is>
           <t>WU: 0,75 USD–12 USD; Diğer: 700 TL–4.000 TL</t>
@@ -920,7 +928,11 @@
           <t>GELEN SWIFT</t>
         </is>
       </c>
-      <c r="C13" s="14" t="inlineStr"/>
+      <c r="C13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 0 TL | Azami 0,94 TL</t>
+        </is>
+      </c>
       <c r="D13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
@@ -960,7 +972,11 @@
           <t>GİDEN SWIFT - Mobil</t>
         </is>
       </c>
-      <c r="C14" s="14" t="inlineStr"/>
+      <c r="C14" s="14" t="inlineStr">
+        <is>
+          <t>40.000 TL - 2.485,72 TL</t>
+        </is>
+      </c>
       <c r="D14" s="14" t="inlineStr">
         <is>
           <t>3.500 TL - 13.500 TL</t>

</xml_diff>

<commit_message>
Update benchmark: 2026-06-21 09:52:16 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -723,11 +723,7 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="D6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 199,41 TL</t>
-        </is>
-      </c>
+      <c r="D6" s="14" t="inlineStr"/>
       <c r="E6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
@@ -739,16 +735,8 @@
           <t>8.300,01 TL - 99,71 TL</t>
         </is>
       </c>
-      <c r="H6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 199,41 TL</t>
-        </is>
-      </c>
-      <c r="I6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 199,41 TL</t>
-        </is>
-      </c>
+      <c r="H6" s="14" t="inlineStr"/>
+      <c r="I6" s="14" t="inlineStr"/>
       <c r="J6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
@@ -896,16 +884,8 @@
           <t>GİDEN SWIFT</t>
         </is>
       </c>
-      <c r="C12" s="14" t="inlineStr">
-        <is>
-          <t>WU: 1.000,01 USD–9,51 USD</t>
-        </is>
-      </c>
-      <c r="D12" s="14" t="inlineStr">
-        <is>
-          <t>WU: 0,75 USD–12 USD; Diğer: 700 TL–4.000 TL</t>
-        </is>
-      </c>
+      <c r="C12" s="14" t="inlineStr"/>
+      <c r="D12" s="14" t="inlineStr"/>
       <c r="E12" s="14" t="inlineStr"/>
       <c r="F12" s="14" t="inlineStr"/>
       <c r="G12" s="14" t="inlineStr">
@@ -928,33 +908,13 @@
           <t>GELEN SWIFT</t>
         </is>
       </c>
-      <c r="C13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 0 TL | Azami 0,94 TL</t>
-        </is>
-      </c>
-      <c r="D13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
-        </is>
-      </c>
-      <c r="E13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
-        </is>
-      </c>
+      <c r="C13" s="14" t="inlineStr"/>
+      <c r="D13" s="14" t="inlineStr"/>
+      <c r="E13" s="14" t="inlineStr"/>
       <c r="F13" s="14" t="inlineStr"/>
       <c r="G13" s="14" t="inlineStr"/>
-      <c r="H13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
-        </is>
-      </c>
-      <c r="I13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
-        </is>
-      </c>
+      <c r="H13" s="14" t="inlineStr"/>
+      <c r="I13" s="14" t="inlineStr"/>
       <c r="J13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.303 TL</t>
@@ -972,36 +932,16 @@
           <t>GİDEN SWIFT - Mobil</t>
         </is>
       </c>
-      <c r="C14" s="14" t="inlineStr">
-        <is>
-          <t>40.000 TL - 2.485,72 TL</t>
-        </is>
-      </c>
-      <c r="D14" s="14" t="inlineStr">
-        <is>
-          <t>3.500 TL - 13.500 TL</t>
-        </is>
-      </c>
-      <c r="E14" s="14" t="inlineStr">
-        <is>
-          <t>2.170 TL - 2.170 TL</t>
-        </is>
-      </c>
-      <c r="F14" s="14" t="inlineStr">
-        <is>
-          <t>2.785,72 TL - 12.380,95 TL</t>
-        </is>
-      </c>
+      <c r="C14" s="14" t="inlineStr"/>
+      <c r="D14" s="14" t="inlineStr"/>
+      <c r="E14" s="14" t="inlineStr"/>
+      <c r="F14" s="14" t="inlineStr"/>
       <c r="G14" s="14" t="inlineStr">
         <is>
           <t>8.300 TL - 7,97 TL</t>
         </is>
       </c>
-      <c r="H14" s="14" t="inlineStr">
-        <is>
-          <t>3.000 TL - 6.000 TL</t>
-        </is>
-      </c>
+      <c r="H14" s="14" t="inlineStr"/>
       <c r="I14" s="14" t="inlineStr"/>
       <c r="J14" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update benchmark: 2026-06-22 11:55:25 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -723,7 +723,11 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="D6" s="14" t="inlineStr"/>
+      <c r="D6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 199,41 TL</t>
+        </is>
+      </c>
       <c r="E6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
@@ -735,8 +739,16 @@
           <t>8.300,01 TL - 99,71 TL</t>
         </is>
       </c>
-      <c r="H6" s="14" t="inlineStr"/>
-      <c r="I6" s="14" t="inlineStr"/>
+      <c r="H6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 199,41 TL</t>
+        </is>
+      </c>
+      <c r="I6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 199,41 TL</t>
+        </is>
+      </c>
       <c r="J6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
@@ -884,8 +896,16 @@
           <t>GİDEN SWIFT</t>
         </is>
       </c>
-      <c r="C12" s="14" t="inlineStr"/>
-      <c r="D12" s="14" t="inlineStr"/>
+      <c r="C12" s="14" t="inlineStr">
+        <is>
+          <t>WU: 1.000,01 USD–9,51 USD</t>
+        </is>
+      </c>
+      <c r="D12" s="14" t="inlineStr">
+        <is>
+          <t>WU: 0,75 USD–12 USD; Diğer: 700 TL–4.000 TL</t>
+        </is>
+      </c>
       <c r="E12" s="14" t="inlineStr"/>
       <c r="F12" s="14" t="inlineStr"/>
       <c r="G12" s="14" t="inlineStr">
@@ -908,13 +928,33 @@
           <t>GELEN SWIFT</t>
         </is>
       </c>
-      <c r="C13" s="14" t="inlineStr"/>
-      <c r="D13" s="14" t="inlineStr"/>
-      <c r="E13" s="14" t="inlineStr"/>
+      <c r="C13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 0 TL | Azami 0,94 TL</t>
+        </is>
+      </c>
+      <c r="D13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
+        </is>
+      </c>
+      <c r="E13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
+        </is>
+      </c>
       <c r="F13" s="14" t="inlineStr"/>
       <c r="G13" s="14" t="inlineStr"/>
-      <c r="H13" s="14" t="inlineStr"/>
-      <c r="I13" s="14" t="inlineStr"/>
+      <c r="H13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
+        </is>
+      </c>
+      <c r="I13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
+        </is>
+      </c>
       <c r="J13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.303 TL</t>
@@ -932,16 +972,36 @@
           <t>GİDEN SWIFT - Mobil</t>
         </is>
       </c>
-      <c r="C14" s="14" t="inlineStr"/>
-      <c r="D14" s="14" t="inlineStr"/>
-      <c r="E14" s="14" t="inlineStr"/>
-      <c r="F14" s="14" t="inlineStr"/>
+      <c r="C14" s="14" t="inlineStr">
+        <is>
+          <t>40.000 TL - 2.485,72 TL</t>
+        </is>
+      </c>
+      <c r="D14" s="14" t="inlineStr">
+        <is>
+          <t>3.500 TL - 13.500 TL</t>
+        </is>
+      </c>
+      <c r="E14" s="14" t="inlineStr">
+        <is>
+          <t>2.170 TL - 2.170 TL</t>
+        </is>
+      </c>
+      <c r="F14" s="14" t="inlineStr">
+        <is>
+          <t>2.785,72 TL - 12.380,95 TL</t>
+        </is>
+      </c>
       <c r="G14" s="14" t="inlineStr">
         <is>
           <t>8.300 TL - 7,97 TL</t>
         </is>
       </c>
-      <c r="H14" s="14" t="inlineStr"/>
+      <c r="H14" s="14" t="inlineStr">
+        <is>
+          <t>3.000 TL - 6.000 TL</t>
+        </is>
+      </c>
       <c r="I14" s="14" t="inlineStr"/>
       <c r="J14" s="14" t="inlineStr">
         <is>
@@ -1219,7 +1279,7 @@
       </c>
       <c r="C22" s="14" t="inlineStr">
         <is>
-          <t>%0,57 Asgari Tutar: 1.243,81 TL Azami Tutar: 1.243,81 TL</t>
+          <t>%0,57 Asgari Tutar: 1.469,52 TL Azami Tutar: 1.469,52 TL</t>
         </is>
       </c>
       <c r="D22" s="14" t="inlineStr">

</xml_diff>

<commit_message>
Update benchmark: 2026-06-25 09:22:48 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -754,11 +754,7 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="K6" s="14" t="inlineStr">
-        <is>
-          <t>7,97 TL - 15,96 TL - 199,41 TL</t>
-        </is>
-      </c>
+      <c r="K6" s="14" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="B7" s="13" t="inlineStr">
@@ -916,11 +912,7 @@
       <c r="H12" s="14" t="inlineStr"/>
       <c r="I12" s="14" t="inlineStr"/>
       <c r="J12" s="14" t="inlineStr"/>
-      <c r="K12" s="14" t="inlineStr">
-        <is>
-          <t>WU: ,USD–; Diğer: 529 TL–4.454,74 TL</t>
-        </is>
-      </c>
+      <c r="K12" s="14" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="B13" s="13" t="inlineStr">
@@ -960,11 +952,7 @@
           <t>Hesaba: Asgari 1 TL | Azami 1.303 TL</t>
         </is>
       </c>
-      <c r="K13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 865,75 TL</t>
-        </is>
-      </c>
+      <c r="K13" s="14" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="B14" s="13" t="inlineStr">
@@ -1008,11 +996,7 @@
           <t>1.554,97 TL - 7.784 TL</t>
         </is>
       </c>
-      <c r="K14" s="14" t="inlineStr">
-        <is>
-          <t>1.196,51 TL - 5.583,74 TL</t>
-        </is>
-      </c>
+      <c r="K14" s="14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="12" t="inlineStr">

</xml_diff>

<commit_message>
Update benchmark: 2026-06-26 09:28:10 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -754,7 +754,11 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="K6" s="14" t="inlineStr"/>
+      <c r="K6" s="14" t="inlineStr">
+        <is>
+          <t>7,97 TL - 15,96 TL - 199,41 TL</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="B7" s="13" t="inlineStr">
@@ -912,7 +916,11 @@
       <c r="H12" s="14" t="inlineStr"/>
       <c r="I12" s="14" t="inlineStr"/>
       <c r="J12" s="14" t="inlineStr"/>
-      <c r="K12" s="14" t="inlineStr"/>
+      <c r="K12" s="14" t="inlineStr">
+        <is>
+          <t>WU: ,USD–; Diğer: 529 TL–4.454,74 TL</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="B13" s="13" t="inlineStr">
@@ -952,7 +960,11 @@
           <t>Hesaba: Asgari 1 TL | Azami 1.303 TL</t>
         </is>
       </c>
-      <c r="K13" s="14" t="inlineStr"/>
+      <c r="K13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 865,75 TL</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="B14" s="13" t="inlineStr">
@@ -996,7 +1008,11 @@
           <t>1.554,97 TL - 7.784 TL</t>
         </is>
       </c>
-      <c r="K14" s="14" t="inlineStr"/>
+      <c r="K14" s="14" t="inlineStr">
+        <is>
+          <t>1.196,51 TL - 5.583,74 TL</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="12" t="inlineStr">

</xml_diff>

<commit_message>
Update benchmark: 2026-06-29 11:01:56 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -945,11 +945,7 @@
       </c>
       <c r="F13" s="14" t="inlineStr"/>
       <c r="G13" s="14" t="inlineStr"/>
-      <c r="H13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
-        </is>
-      </c>
+      <c r="H13" s="14" t="inlineStr"/>
       <c r="I13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
@@ -997,11 +993,7 @@
           <t>8.300 TL - 7,97 TL</t>
         </is>
       </c>
-      <c r="H14" s="14" t="inlineStr">
-        <is>
-          <t>3.000 TL - 6.000 TL</t>
-        </is>
-      </c>
+      <c r="H14" s="14" t="inlineStr"/>
       <c r="I14" s="14" t="inlineStr"/>
       <c r="J14" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update benchmark: 2026-06-30 09:36:51 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -901,11 +901,7 @@
           <t>WU: 1.000,01 USD–9,51 USD</t>
         </is>
       </c>
-      <c r="D12" s="14" t="inlineStr">
-        <is>
-          <t>WU: 0,75 USD–12 USD; Diğer: 700 TL–4.000 TL</t>
-        </is>
-      </c>
+      <c r="D12" s="14" t="inlineStr"/>
       <c r="E12" s="14" t="inlineStr"/>
       <c r="F12" s="14" t="inlineStr"/>
       <c r="G12" s="14" t="inlineStr">
@@ -933,11 +929,7 @@
           <t>Hesaba: Asgari 0 TL | Azami 0,94 TL</t>
         </is>
       </c>
-      <c r="D13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
-        </is>
-      </c>
+      <c r="D13" s="14" t="inlineStr"/>
       <c r="E13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
@@ -945,7 +937,11 @@
       </c>
       <c r="F13" s="14" t="inlineStr"/>
       <c r="G13" s="14" t="inlineStr"/>
-      <c r="H13" s="14" t="inlineStr"/>
+      <c r="H13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
+        </is>
+      </c>
       <c r="I13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
@@ -973,27 +969,23 @@
           <t>40.000 TL - 2.485,72 TL</t>
         </is>
       </c>
-      <c r="D14" s="14" t="inlineStr">
-        <is>
-          <t>3.500 TL - 13.500 TL</t>
-        </is>
-      </c>
+      <c r="D14" s="14" t="inlineStr"/>
       <c r="E14" s="14" t="inlineStr">
         <is>
           <t>2.170 TL - 2.170 TL</t>
         </is>
       </c>
-      <c r="F14" s="14" t="inlineStr">
-        <is>
-          <t>2.785,72 TL - 12.380,95 TL</t>
-        </is>
-      </c>
+      <c r="F14" s="14" t="inlineStr"/>
       <c r="G14" s="14" t="inlineStr">
         <is>
           <t>8.300 TL - 7,97 TL</t>
         </is>
       </c>
-      <c r="H14" s="14" t="inlineStr"/>
+      <c r="H14" s="14" t="inlineStr">
+        <is>
+          <t>3.000 TL - 6.000 TL</t>
+        </is>
+      </c>
       <c r="I14" s="14" t="inlineStr"/>
       <c r="J14" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update benchmark: 2026-07-01 09:47:57 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -901,7 +901,11 @@
           <t>WU: 1.000,01 USD–9,51 USD</t>
         </is>
       </c>
-      <c r="D12" s="14" t="inlineStr"/>
+      <c r="D12" s="14" t="inlineStr">
+        <is>
+          <t>WU: 0,75 USD–12 USD; Diğer: 700 TL–4.000 TL</t>
+        </is>
+      </c>
       <c r="E12" s="14" t="inlineStr"/>
       <c r="F12" s="14" t="inlineStr"/>
       <c r="G12" s="14" t="inlineStr">
@@ -929,7 +933,11 @@
           <t>Hesaba: Asgari 0 TL | Azami 0,94 TL</t>
         </is>
       </c>
-      <c r="D13" s="14" t="inlineStr"/>
+      <c r="D13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
+        </is>
+      </c>
       <c r="E13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
@@ -969,13 +977,21 @@
           <t>40.000 TL - 2.485,72 TL</t>
         </is>
       </c>
-      <c r="D14" s="14" t="inlineStr"/>
+      <c r="D14" s="14" t="inlineStr">
+        <is>
+          <t>3.500 TL - 13.500 TL</t>
+        </is>
+      </c>
       <c r="E14" s="14" t="inlineStr">
         <is>
           <t>2.170 TL - 2.170 TL</t>
         </is>
       </c>
-      <c r="F14" s="14" t="inlineStr"/>
+      <c r="F14" s="14" t="inlineStr">
+        <is>
+          <t>2.785,72 TL - 12.380,95 TL</t>
+        </is>
+      </c>
       <c r="G14" s="14" t="inlineStr">
         <is>
           <t>8.300 TL - 7,97 TL</t>

</xml_diff>

<commit_message>
Update benchmark: 2026-07-02 08:57:29 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -749,11 +749,7 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="J6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 199,41 TL</t>
-        </is>
-      </c>
+      <c r="J6" s="14" t="inlineStr"/>
       <c r="K6" s="14" t="inlineStr">
         <is>
           <t>7,97 TL - 15,96 TL - 199,41 TL</t>
@@ -901,11 +897,7 @@
           <t>WU: 1.000,01 USD–9,51 USD</t>
         </is>
       </c>
-      <c r="D12" s="14" t="inlineStr">
-        <is>
-          <t>WU: 0,75 USD–12 USD; Diğer: 700 TL–4.000 TL</t>
-        </is>
-      </c>
+      <c r="D12" s="14" t="inlineStr"/>
       <c r="E12" s="14" t="inlineStr"/>
       <c r="F12" s="14" t="inlineStr"/>
       <c r="G12" s="14" t="inlineStr">
@@ -933,11 +925,7 @@
           <t>Hesaba: Asgari 0 TL | Azami 0,94 TL</t>
         </is>
       </c>
-      <c r="D13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
-        </is>
-      </c>
+      <c r="D13" s="14" t="inlineStr"/>
       <c r="E13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
@@ -955,11 +943,7 @@
           <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
         </is>
       </c>
-      <c r="J13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 1.303 TL</t>
-        </is>
-      </c>
+      <c r="J13" s="14" t="inlineStr"/>
       <c r="K13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 865,75 TL</t>
@@ -977,11 +961,7 @@
           <t>40.000 TL - 2.485,72 TL</t>
         </is>
       </c>
-      <c r="D14" s="14" t="inlineStr">
-        <is>
-          <t>3.500 TL - 13.500 TL</t>
-        </is>
-      </c>
+      <c r="D14" s="14" t="inlineStr"/>
       <c r="E14" s="14" t="inlineStr">
         <is>
           <t>2.170 TL - 2.170 TL</t>
@@ -1003,11 +983,7 @@
         </is>
       </c>
       <c r="I14" s="14" t="inlineStr"/>
-      <c r="J14" s="14" t="inlineStr">
-        <is>
-          <t>1.554,97 TL - 7.784 TL</t>
-        </is>
-      </c>
+      <c r="J14" s="14" t="inlineStr"/>
       <c r="K14" s="14" t="inlineStr">
         <is>
           <t>1.196,51 TL - 5.583,74 TL</t>

</xml_diff>

<commit_message>
Update benchmark: 2026-07-03 09:19:01 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -749,7 +749,11 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="J6" s="14" t="inlineStr"/>
+      <c r="J6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 199,41 TL</t>
+        </is>
+      </c>
       <c r="K6" s="14" t="inlineStr">
         <is>
           <t>7,97 TL - 15,96 TL - 199,41 TL</t>
@@ -897,7 +901,11 @@
           <t>WU: 1.000,01 USD–9,51 USD</t>
         </is>
       </c>
-      <c r="D12" s="14" t="inlineStr"/>
+      <c r="D12" s="14" t="inlineStr">
+        <is>
+          <t>Diğer: 700 TL–4.000 TL</t>
+        </is>
+      </c>
       <c r="E12" s="14" t="inlineStr"/>
       <c r="F12" s="14" t="inlineStr"/>
       <c r="G12" s="14" t="inlineStr">
@@ -925,7 +933,11 @@
           <t>Hesaba: Asgari 0 TL | Azami 0,94 TL</t>
         </is>
       </c>
-      <c r="D13" s="14" t="inlineStr"/>
+      <c r="D13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
+        </is>
+      </c>
       <c r="E13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
@@ -943,7 +955,11 @@
           <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
         </is>
       </c>
-      <c r="J13" s="14" t="inlineStr"/>
+      <c r="J13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 1.303 TL</t>
+        </is>
+      </c>
       <c r="K13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 865,75 TL</t>
@@ -961,7 +977,11 @@
           <t>40.000 TL - 2.485,72 TL</t>
         </is>
       </c>
-      <c r="D14" s="14" t="inlineStr"/>
+      <c r="D14" s="14" t="inlineStr">
+        <is>
+          <t>3.500 TL - 13.500 TL</t>
+        </is>
+      </c>
       <c r="E14" s="14" t="inlineStr">
         <is>
           <t>2.170 TL - 2.170 TL</t>
@@ -983,7 +1003,11 @@
         </is>
       </c>
       <c r="I14" s="14" t="inlineStr"/>
-      <c r="J14" s="14" t="inlineStr"/>
+      <c r="J14" s="14" t="inlineStr">
+        <is>
+          <t>1.554,97 TL - 7.784 TL</t>
+        </is>
+      </c>
       <c r="K14" s="14" t="inlineStr">
         <is>
           <t>1.196,51 TL - 5.583,74 TL</t>

</xml_diff>

<commit_message>
Update benchmark: 2026-07-04 08:38:38 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -903,7 +903,7 @@
       </c>
       <c r="D12" s="14" t="inlineStr">
         <is>
-          <t>Diğer: 700 TL–4.000 TL</t>
+          <t>WU: 0,75 USD–12 USD; Diğer: 700 TL–4.000 TL</t>
         </is>
       </c>
       <c r="E12" s="14" t="inlineStr"/>
@@ -940,7 +940,7 @@
       </c>
       <c r="E13" s="14" t="inlineStr">
         <is>
-          <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
+          <t>Hesaba: Asgari 1 TL | Azami 11.380 TL</t>
         </is>
       </c>
       <c r="F13" s="14" t="inlineStr"/>

</xml_diff>

<commit_message>
Update benchmark: 2026-07-09 09:40:47 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -938,11 +938,7 @@
           <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
         </is>
       </c>
-      <c r="E13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
-        </is>
-      </c>
+      <c r="E13" s="14" t="inlineStr"/>
       <c r="F13" s="14" t="inlineStr"/>
       <c r="G13" s="14" t="inlineStr"/>
       <c r="H13" s="14" t="inlineStr">
@@ -982,11 +978,7 @@
           <t>3.500 TL - 13.500 TL</t>
         </is>
       </c>
-      <c r="E14" s="14" t="inlineStr">
-        <is>
-          <t>2.170 TL - 2.170 TL</t>
-        </is>
-      </c>
+      <c r="E14" s="14" t="inlineStr"/>
       <c r="F14" s="14" t="inlineStr">
         <is>
           <t>2.785,72 TL - 12.380,95 TL</t>

</xml_diff>

<commit_message>
Update benchmark: 2026-07-10 09:35:48 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -728,11 +728,7 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="E6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 199,41 TL</t>
-        </is>
-      </c>
+      <c r="E6" s="14" t="inlineStr"/>
       <c r="F6" s="14" t="inlineStr"/>
       <c r="G6" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update benchmark: 2026-07-11 07:57:43 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -616,11 +616,7 @@
           <t>26 TL - 26 TL</t>
         </is>
       </c>
-      <c r="F2" s="14" t="inlineStr">
-        <is>
-          <t>33,33 TL - 33,33 TL</t>
-        </is>
-      </c>
+      <c r="F2" s="14" t="inlineStr"/>
       <c r="G2" s="14" t="inlineStr">
         <is>
           <t>15 TL - 15 TL</t>
@@ -728,7 +724,11 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="E6" s="14" t="inlineStr"/>
+      <c r="E6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 199,41 TL</t>
+        </is>
+      </c>
       <c r="F6" s="14" t="inlineStr"/>
       <c r="G6" s="14" t="inlineStr">
         <is>
@@ -745,11 +745,7 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="J6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 199,41 TL</t>
-        </is>
-      </c>
+      <c r="J6" s="14" t="inlineStr"/>
       <c r="K6" s="14" t="inlineStr">
         <is>
           <t>7,97 TL - 15,96 TL - 199,41 TL</t>
@@ -769,11 +765,7 @@
         </is>
       </c>
       <c r="E7" s="14" t="inlineStr"/>
-      <c r="F7" s="14" t="inlineStr">
-        <is>
-          <t>%3</t>
-        </is>
-      </c>
+      <c r="F7" s="14" t="inlineStr"/>
       <c r="G7" s="14" t="inlineStr">
         <is>
           <t>1 TRY (Kredi kartı ile ödemelerde ek olarak nakit avans faizi uygulanır.)</t>
@@ -934,7 +926,11 @@
           <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
         </is>
       </c>
-      <c r="E13" s="14" t="inlineStr"/>
+      <c r="E13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
+        </is>
+      </c>
       <c r="F13" s="14" t="inlineStr"/>
       <c r="G13" s="14" t="inlineStr"/>
       <c r="H13" s="14" t="inlineStr">
@@ -947,11 +943,7 @@
           <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
         </is>
       </c>
-      <c r="J13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 1.303 TL</t>
-        </is>
-      </c>
+      <c r="J13" s="14" t="inlineStr"/>
       <c r="K13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 865,75 TL</t>
@@ -974,7 +966,11 @@
           <t>3.500 TL - 13.500 TL</t>
         </is>
       </c>
-      <c r="E14" s="14" t="inlineStr"/>
+      <c r="E14" s="14" t="inlineStr">
+        <is>
+          <t>2.170 TL - 2.170 TL</t>
+        </is>
+      </c>
       <c r="F14" s="14" t="inlineStr">
         <is>
           <t>2.785,72 TL - 12.380,95 TL</t>
@@ -991,11 +987,7 @@
         </is>
       </c>
       <c r="I14" s="14" t="inlineStr"/>
-      <c r="J14" s="14" t="inlineStr">
-        <is>
-          <t>1.554,97 TL - 7.784 TL</t>
-        </is>
-      </c>
+      <c r="J14" s="14" t="inlineStr"/>
       <c r="K14" s="14" t="inlineStr">
         <is>
           <t>1.196,51 TL - 5.583,74 TL</t>

</xml_diff>

<commit_message>
Update benchmark: 2026-07-12 08:18:19 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -616,7 +616,11 @@
           <t>26 TL - 26 TL</t>
         </is>
       </c>
-      <c r="F2" s="14" t="inlineStr"/>
+      <c r="F2" s="14" t="inlineStr">
+        <is>
+          <t>33,33 TL - 33,33 TL</t>
+        </is>
+      </c>
       <c r="G2" s="14" t="inlineStr">
         <is>
           <t>15 TL - 15 TL</t>
@@ -714,11 +718,7 @@
           <t>DÜZENLİ EFT</t>
         </is>
       </c>
-      <c r="C6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 199,41 TL</t>
-        </is>
-      </c>
+      <c r="C6" s="14" t="inlineStr"/>
       <c r="D6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
@@ -745,7 +745,11 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="J6" s="14" t="inlineStr"/>
+      <c r="J6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 199,41 TL</t>
+        </is>
+      </c>
       <c r="K6" s="14" t="inlineStr">
         <is>
           <t>7,97 TL - 15,96 TL - 199,41 TL</t>
@@ -765,7 +769,11 @@
         </is>
       </c>
       <c r="E7" s="14" t="inlineStr"/>
-      <c r="F7" s="14" t="inlineStr"/>
+      <c r="F7" s="14" t="inlineStr">
+        <is>
+          <t>%3</t>
+        </is>
+      </c>
       <c r="G7" s="14" t="inlineStr">
         <is>
           <t>1 TRY (Kredi kartı ile ödemelerde ek olarak nakit avans faizi uygulanır.)</t>
@@ -884,16 +892,8 @@
           <t>GİDEN SWIFT</t>
         </is>
       </c>
-      <c r="C12" s="14" t="inlineStr">
-        <is>
-          <t>WU: 1.000,01 USD–9,51 USD</t>
-        </is>
-      </c>
-      <c r="D12" s="14" t="inlineStr">
-        <is>
-          <t>WU: 0,75 USD–12 USD; Diğer: 700 TL–4.000 TL</t>
-        </is>
-      </c>
+      <c r="C12" s="14" t="inlineStr"/>
+      <c r="D12" s="14" t="inlineStr"/>
       <c r="E12" s="14" t="inlineStr"/>
       <c r="F12" s="14" t="inlineStr"/>
       <c r="G12" s="14" t="inlineStr">
@@ -916,16 +916,8 @@
           <t>GELEN SWIFT</t>
         </is>
       </c>
-      <c r="C13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 0 TL | Azami 0,94 TL</t>
-        </is>
-      </c>
-      <c r="D13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
-        </is>
-      </c>
+      <c r="C13" s="14" t="inlineStr"/>
+      <c r="D13" s="14" t="inlineStr"/>
       <c r="E13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
@@ -943,7 +935,11 @@
           <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
         </is>
       </c>
-      <c r="J13" s="14" t="inlineStr"/>
+      <c r="J13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 1.303 TL</t>
+        </is>
+      </c>
       <c r="K13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 865,75 TL</t>
@@ -956,26 +952,14 @@
           <t>GİDEN SWIFT - Mobil</t>
         </is>
       </c>
-      <c r="C14" s="14" t="inlineStr">
-        <is>
-          <t>40.000 TL - 2.485,72 TL</t>
-        </is>
-      </c>
-      <c r="D14" s="14" t="inlineStr">
-        <is>
-          <t>3.500 TL - 13.500 TL</t>
-        </is>
-      </c>
+      <c r="C14" s="14" t="inlineStr"/>
+      <c r="D14" s="14" t="inlineStr"/>
       <c r="E14" s="14" t="inlineStr">
         <is>
           <t>2.170 TL - 2.170 TL</t>
         </is>
       </c>
-      <c r="F14" s="14" t="inlineStr">
-        <is>
-          <t>2.785,72 TL - 12.380,95 TL</t>
-        </is>
-      </c>
+      <c r="F14" s="14" t="inlineStr"/>
       <c r="G14" s="14" t="inlineStr">
         <is>
           <t>8.300 TL - 7,97 TL</t>
@@ -987,7 +971,11 @@
         </is>
       </c>
       <c r="I14" s="14" t="inlineStr"/>
-      <c r="J14" s="14" t="inlineStr"/>
+      <c r="J14" s="14" t="inlineStr">
+        <is>
+          <t>1.554,97 TL - 7.784 TL</t>
+        </is>
+      </c>
       <c r="K14" s="14" t="inlineStr">
         <is>
           <t>1.196,51 TL - 5.583,74 TL</t>
@@ -1386,11 +1374,7 @@
           <t>600 TL</t>
         </is>
       </c>
-      <c r="G24" s="14" t="inlineStr">
-        <is>
-          <t>160 TL</t>
-        </is>
-      </c>
+      <c r="G24" s="14" t="inlineStr"/>
       <c r="H24" s="14" t="inlineStr">
         <is>
           <t>350 TL</t>

</xml_diff>

<commit_message>
Update benchmark: 2026-07-13 09:27:40 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -718,7 +718,11 @@
           <t>DÜZENLİ EFT</t>
         </is>
       </c>
-      <c r="C6" s="14" t="inlineStr"/>
+      <c r="C6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 199,41 TL</t>
+        </is>
+      </c>
       <c r="D6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
@@ -892,8 +896,16 @@
           <t>GİDEN SWIFT</t>
         </is>
       </c>
-      <c r="C12" s="14" t="inlineStr"/>
-      <c r="D12" s="14" t="inlineStr"/>
+      <c r="C12" s="14" t="inlineStr">
+        <is>
+          <t>WU: 3.000,01 USD–9,51 USD</t>
+        </is>
+      </c>
+      <c r="D12" s="14" t="inlineStr">
+        <is>
+          <t>WU: 0,75 USD–12 USD; Diğer: 700 TL–4.000 TL</t>
+        </is>
+      </c>
       <c r="E12" s="14" t="inlineStr"/>
       <c r="F12" s="14" t="inlineStr"/>
       <c r="G12" s="14" t="inlineStr">
@@ -916,8 +928,16 @@
           <t>GELEN SWIFT</t>
         </is>
       </c>
-      <c r="C13" s="14" t="inlineStr"/>
-      <c r="D13" s="14" t="inlineStr"/>
+      <c r="C13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 0 TL | Azami 0,94 TL</t>
+        </is>
+      </c>
+      <c r="D13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
+        </is>
+      </c>
       <c r="E13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
@@ -952,14 +972,26 @@
           <t>GİDEN SWIFT - Mobil</t>
         </is>
       </c>
-      <c r="C14" s="14" t="inlineStr"/>
-      <c r="D14" s="14" t="inlineStr"/>
+      <c r="C14" s="14" t="inlineStr">
+        <is>
+          <t>40.000 TL - 2.485,72 TL</t>
+        </is>
+      </c>
+      <c r="D14" s="14" t="inlineStr">
+        <is>
+          <t>3.500 TL - 13.500 TL</t>
+        </is>
+      </c>
       <c r="E14" s="14" t="inlineStr">
         <is>
           <t>2.170 TL - 2.170 TL</t>
         </is>
       </c>
-      <c r="F14" s="14" t="inlineStr"/>
+      <c r="F14" s="14" t="inlineStr">
+        <is>
+          <t>2.785,72 TL - 12.380,95 TL</t>
+        </is>
+      </c>
       <c r="G14" s="14" t="inlineStr">
         <is>
           <t>8.300 TL - 7,97 TL</t>
@@ -1374,7 +1406,11 @@
           <t>600 TL</t>
         </is>
       </c>
-      <c r="G24" s="14" t="inlineStr"/>
+      <c r="G24" s="14" t="inlineStr">
+        <is>
+          <t>160 TL</t>
+        </is>
+      </c>
       <c r="H24" s="14" t="inlineStr">
         <is>
           <t>350 TL</t>

</xml_diff>

<commit_message>
Update benchmark: 2026-07-16 08:13:47 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -718,11 +718,7 @@
           <t>DÜZENLİ EFT</t>
         </is>
       </c>
-      <c r="C6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 199,41 TL</t>
-        </is>
-      </c>
+      <c r="C6" s="14" t="inlineStr"/>
       <c r="D6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
@@ -896,16 +892,8 @@
           <t>GİDEN SWIFT</t>
         </is>
       </c>
-      <c r="C12" s="14" t="inlineStr">
-        <is>
-          <t>WU: 0,1 USD–9,51 USD</t>
-        </is>
-      </c>
-      <c r="D12" s="14" t="inlineStr">
-        <is>
-          <t>WU: 0,75 USD–12 USD; Diğer: 700 TL–4.000 TL</t>
-        </is>
-      </c>
+      <c r="C12" s="14" t="inlineStr"/>
+      <c r="D12" s="14" t="inlineStr"/>
       <c r="E12" s="14" t="inlineStr"/>
       <c r="F12" s="14" t="inlineStr"/>
       <c r="G12" s="14" t="inlineStr">
@@ -928,16 +916,8 @@
           <t>GELEN SWIFT</t>
         </is>
       </c>
-      <c r="C13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 0 TL | Azami 0,94 TL</t>
-        </is>
-      </c>
-      <c r="D13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
-        </is>
-      </c>
+      <c r="C13" s="14" t="inlineStr"/>
+      <c r="D13" s="14" t="inlineStr"/>
       <c r="E13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
@@ -972,16 +952,8 @@
           <t>GİDEN SWIFT - Mobil</t>
         </is>
       </c>
-      <c r="C14" s="14" t="inlineStr">
-        <is>
-          <t>40.000 TL - 2.485,72 TL</t>
-        </is>
-      </c>
-      <c r="D14" s="14" t="inlineStr">
-        <is>
-          <t>3.500 TL - 13.500 TL</t>
-        </is>
-      </c>
+      <c r="C14" s="14" t="inlineStr"/>
+      <c r="D14" s="14" t="inlineStr"/>
       <c r="E14" s="14" t="inlineStr">
         <is>
           <t>2.170 TL - 2.170 TL</t>

</xml_diff>

<commit_message>
Update benchmark: 2026-07-17 08:11:08 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -718,7 +718,11 @@
           <t>DÜZENLİ EFT</t>
         </is>
       </c>
-      <c r="C6" s="14" t="inlineStr"/>
+      <c r="C6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 199,41 TL</t>
+        </is>
+      </c>
       <c r="D6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
@@ -892,8 +896,16 @@
           <t>GİDEN SWIFT</t>
         </is>
       </c>
-      <c r="C12" s="14" t="inlineStr"/>
-      <c r="D12" s="14" t="inlineStr"/>
+      <c r="C12" s="14" t="inlineStr">
+        <is>
+          <t>WU: 3.000,01 USD–9,51 USD</t>
+        </is>
+      </c>
+      <c r="D12" s="14" t="inlineStr">
+        <is>
+          <t>WU: 0,75 USD–12 USD; Diğer: 700 TL–4.000 TL</t>
+        </is>
+      </c>
       <c r="E12" s="14" t="inlineStr"/>
       <c r="F12" s="14" t="inlineStr"/>
       <c r="G12" s="14" t="inlineStr">
@@ -916,8 +928,16 @@
           <t>GELEN SWIFT</t>
         </is>
       </c>
-      <c r="C13" s="14" t="inlineStr"/>
-      <c r="D13" s="14" t="inlineStr"/>
+      <c r="C13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 0 TL | Azami 0,94 TL</t>
+        </is>
+      </c>
+      <c r="D13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
+        </is>
+      </c>
       <c r="E13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
@@ -952,8 +972,16 @@
           <t>GİDEN SWIFT - Mobil</t>
         </is>
       </c>
-      <c r="C14" s="14" t="inlineStr"/>
-      <c r="D14" s="14" t="inlineStr"/>
+      <c r="C14" s="14" t="inlineStr">
+        <is>
+          <t>40.000 TL - 2.485,72 TL</t>
+        </is>
+      </c>
+      <c r="D14" s="14" t="inlineStr">
+        <is>
+          <t>3.500 TL - 13.500 TL</t>
+        </is>
+      </c>
       <c r="E14" s="14" t="inlineStr">
         <is>
           <t>2.170 TL - 2.170 TL</t>

</xml_diff>

<commit_message>
Update benchmark: 2026-07-19 08:20:02 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -916,11 +916,7 @@
       <c r="H12" s="14" t="inlineStr"/>
       <c r="I12" s="14" t="inlineStr"/>
       <c r="J12" s="14" t="inlineStr"/>
-      <c r="K12" s="14" t="inlineStr">
-        <is>
-          <t>WU: ,USD–; Diğer: 529 TL–4.454,74 TL</t>
-        </is>
-      </c>
+      <c r="K12" s="14" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="B13" s="13" t="inlineStr">
@@ -960,11 +956,7 @@
           <t>Hesaba: Asgari 1 TL | Azami 1.303 TL</t>
         </is>
       </c>
-      <c r="K13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 865,75 TL</t>
-        </is>
-      </c>
+      <c r="K13" s="14" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="B14" s="13" t="inlineStr">
@@ -1008,11 +1000,7 @@
           <t>1.554,97 TL - 7.784 TL</t>
         </is>
       </c>
-      <c r="K14" s="14" t="inlineStr">
-        <is>
-          <t>1.196,51 TL - 5.583,74 TL</t>
-        </is>
-      </c>
+      <c r="K14" s="14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="12" t="inlineStr">

</xml_diff>

<commit_message>
Update benchmark: 2026-07-20 08:59:22 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -916,7 +916,11 @@
       <c r="H12" s="14" t="inlineStr"/>
       <c r="I12" s="14" t="inlineStr"/>
       <c r="J12" s="14" t="inlineStr"/>
-      <c r="K12" s="14" t="inlineStr"/>
+      <c r="K12" s="14" t="inlineStr">
+        <is>
+          <t>WU: ,USD–; Diğer: 529 TL–4.454,74 TL</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="B13" s="13" t="inlineStr">
@@ -956,7 +960,11 @@
           <t>Hesaba: Asgari 1 TL | Azami 1.303 TL</t>
         </is>
       </c>
-      <c r="K13" s="14" t="inlineStr"/>
+      <c r="K13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 865,75 TL</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="B14" s="13" t="inlineStr">
@@ -1000,7 +1008,11 @@
           <t>1.554,97 TL - 7.784 TL</t>
         </is>
       </c>
-      <c r="K14" s="14" t="inlineStr"/>
+      <c r="K14" s="14" t="inlineStr">
+        <is>
+          <t>1.196,51 TL - 5.583,74 TL</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="12" t="inlineStr">

</xml_diff>

<commit_message>
Update benchmark: 2026-07-21 08:30:09 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -896,11 +896,7 @@
           <t>GİDEN SWIFT</t>
         </is>
       </c>
-      <c r="C12" s="14" t="inlineStr">
-        <is>
-          <t>WU: 3.000,01 USD–9,51 USD</t>
-        </is>
-      </c>
+      <c r="C12" s="14" t="inlineStr"/>
       <c r="D12" s="14" t="inlineStr">
         <is>
           <t>WU: 0,75 USD–12 USD; Diğer: 700 TL–4.000 TL</t>
@@ -928,11 +924,7 @@
           <t>GELEN SWIFT</t>
         </is>
       </c>
-      <c r="C13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 0 TL | Azami 0,94 TL</t>
-        </is>
-      </c>
+      <c r="C13" s="14" t="inlineStr"/>
       <c r="D13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
@@ -950,11 +942,7 @@
           <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
         </is>
       </c>
-      <c r="I13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
-        </is>
-      </c>
+      <c r="I13" s="14" t="inlineStr"/>
       <c r="J13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.303 TL</t>
@@ -972,11 +960,7 @@
           <t>GİDEN SWIFT - Mobil</t>
         </is>
       </c>
-      <c r="C14" s="14" t="inlineStr">
-        <is>
-          <t>40.000 TL - 2.485,72 TL</t>
-        </is>
-      </c>
+      <c r="C14" s="14" t="inlineStr"/>
       <c r="D14" s="14" t="inlineStr">
         <is>
           <t>3.500 TL - 13.500 TL</t>

</xml_diff>

<commit_message>
Update benchmark: 2026-07-22 08:30:53 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -626,16 +626,8 @@
           <t>15 TL - 15 TL</t>
         </is>
       </c>
-      <c r="H2" s="14" t="inlineStr">
-        <is>
-          <t>15 TL - 15 TL</t>
-        </is>
-      </c>
-      <c r="I2" s="14" t="inlineStr">
-        <is>
-          <t>18 TL - 18 TL</t>
-        </is>
-      </c>
+      <c r="H2" s="14" t="inlineStr"/>
+      <c r="I2" s="14" t="inlineStr"/>
       <c r="J2" s="14" t="inlineStr">
         <is>
           <t>65 TL - 65 TL</t>
@@ -783,11 +775,7 @@
           <t>1 TRY (Kredi kartı ile ödemelerde ek olarak nakit avans faizi uygulanır.)</t>
         </is>
       </c>
-      <c r="H7" s="14" t="inlineStr">
-        <is>
-          <t>%3,5</t>
-        </is>
-      </c>
+      <c r="H7" s="14" t="inlineStr"/>
       <c r="I7" s="14" t="inlineStr"/>
       <c r="J7" s="14" t="inlineStr">
         <is>
@@ -896,7 +884,11 @@
           <t>GİDEN SWIFT</t>
         </is>
       </c>
-      <c r="C12" s="14" t="inlineStr"/>
+      <c r="C12" s="14" t="inlineStr">
+        <is>
+          <t>WU: 0,1 USD–9,51 USD</t>
+        </is>
+      </c>
       <c r="D12" s="14" t="inlineStr">
         <is>
           <t>WU: 0,75 USD–12 USD; Diğer: 700 TL–4.000 TL</t>
@@ -924,7 +916,11 @@
           <t>GELEN SWIFT</t>
         </is>
       </c>
-      <c r="C13" s="14" t="inlineStr"/>
+      <c r="C13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 0 TL | Azami 0,94 TL</t>
+        </is>
+      </c>
       <c r="D13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
@@ -942,7 +938,11 @@
           <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
         </is>
       </c>
-      <c r="I13" s="14" t="inlineStr"/>
+      <c r="I13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
+        </is>
+      </c>
       <c r="J13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.303 TL</t>
@@ -960,7 +960,11 @@
           <t>GİDEN SWIFT - Mobil</t>
         </is>
       </c>
-      <c r="C14" s="14" t="inlineStr"/>
+      <c r="C14" s="14" t="inlineStr">
+        <is>
+          <t>40.000 TL - 2.485,72 TL</t>
+        </is>
+      </c>
       <c r="D14" s="14" t="inlineStr">
         <is>
           <t>3.500 TL - 13.500 TL</t>

</xml_diff>

<commit_message>
Update benchmark: 2026-07-23 08:30:57 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -626,8 +626,16 @@
           <t>15 TL - 15 TL</t>
         </is>
       </c>
-      <c r="H2" s="14" t="inlineStr"/>
-      <c r="I2" s="14" t="inlineStr"/>
+      <c r="H2" s="14" t="inlineStr">
+        <is>
+          <t>15 TL - 15 TL</t>
+        </is>
+      </c>
+      <c r="I2" s="14" t="inlineStr">
+        <is>
+          <t>18 TL - 18 TL</t>
+        </is>
+      </c>
       <c r="J2" s="14" t="inlineStr">
         <is>
           <t>65 TL - 65 TL</t>
@@ -710,11 +718,7 @@
           <t>DÜZENLİ EFT</t>
         </is>
       </c>
-      <c r="C6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 199,41 TL</t>
-        </is>
-      </c>
+      <c r="C6" s="14" t="inlineStr"/>
       <c r="D6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
@@ -775,7 +779,11 @@
           <t>1 TRY (Kredi kartı ile ödemelerde ek olarak nakit avans faizi uygulanır.)</t>
         </is>
       </c>
-      <c r="H7" s="14" t="inlineStr"/>
+      <c r="H7" s="14" t="inlineStr">
+        <is>
+          <t>%3,5</t>
+        </is>
+      </c>
       <c r="I7" s="14" t="inlineStr"/>
       <c r="J7" s="14" t="inlineStr">
         <is>
@@ -884,11 +892,7 @@
           <t>GİDEN SWIFT</t>
         </is>
       </c>
-      <c r="C12" s="14" t="inlineStr">
-        <is>
-          <t>WU: 0,1 USD–9,51 USD</t>
-        </is>
-      </c>
+      <c r="C12" s="14" t="inlineStr"/>
       <c r="D12" s="14" t="inlineStr">
         <is>
           <t>WU: 0,75 USD–12 USD; Diğer: 700 TL–4.000 TL</t>
@@ -916,11 +920,7 @@
           <t>GELEN SWIFT</t>
         </is>
       </c>
-      <c r="C13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 0 TL | Azami 0,94 TL</t>
-        </is>
-      </c>
+      <c r="C13" s="14" t="inlineStr"/>
       <c r="D13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
@@ -960,11 +960,7 @@
           <t>GİDEN SWIFT - Mobil</t>
         </is>
       </c>
-      <c r="C14" s="14" t="inlineStr">
-        <is>
-          <t>40.000 TL - 2.485,72 TL</t>
-        </is>
-      </c>
+      <c r="C14" s="14" t="inlineStr"/>
       <c r="D14" s="14" t="inlineStr">
         <is>
           <t>3.500 TL - 13.500 TL</t>

</xml_diff>

<commit_message>
Update benchmark: 2026-07-24 08:28:11 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -718,12 +718,12 @@
           <t>DÜZENLİ EFT</t>
         </is>
       </c>
-      <c r="C6" s="14" t="inlineStr"/>
-      <c r="D6" s="14" t="inlineStr">
+      <c r="C6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
+      <c r="D6" s="14" t="inlineStr"/>
       <c r="E6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
@@ -740,21 +740,9 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="I6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 199,41 TL</t>
-        </is>
-      </c>
-      <c r="J6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 199,41 TL</t>
-        </is>
-      </c>
-      <c r="K6" s="14" t="inlineStr">
-        <is>
-          <t>7,97 TL - 15,96 TL - 199,41 TL</t>
-        </is>
-      </c>
+      <c r="I6" s="14" t="inlineStr"/>
+      <c r="J6" s="14" t="inlineStr"/>
+      <c r="K6" s="14" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="B7" s="13" t="inlineStr">
@@ -893,11 +881,7 @@
         </is>
       </c>
       <c r="C12" s="14" t="inlineStr"/>
-      <c r="D12" s="14" t="inlineStr">
-        <is>
-          <t>WU: 0,75 USD–12 USD; Diğer: 700 TL–4.000 TL</t>
-        </is>
-      </c>
+      <c r="D12" s="14" t="inlineStr"/>
       <c r="E12" s="14" t="inlineStr"/>
       <c r="F12" s="14" t="inlineStr"/>
       <c r="G12" s="14" t="inlineStr">
@@ -908,11 +892,7 @@
       <c r="H12" s="14" t="inlineStr"/>
       <c r="I12" s="14" t="inlineStr"/>
       <c r="J12" s="14" t="inlineStr"/>
-      <c r="K12" s="14" t="inlineStr">
-        <is>
-          <t>WU: ,USD–; Diğer: 529 TL–4.454,74 TL</t>
-        </is>
-      </c>
+      <c r="K12" s="14" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="B13" s="13" t="inlineStr">
@@ -921,11 +901,7 @@
         </is>
       </c>
       <c r="C13" s="14" t="inlineStr"/>
-      <c r="D13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
-        </is>
-      </c>
+      <c r="D13" s="14" t="inlineStr"/>
       <c r="E13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
@@ -938,21 +914,9 @@
           <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
         </is>
       </c>
-      <c r="I13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
-        </is>
-      </c>
-      <c r="J13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 1.303 TL</t>
-        </is>
-      </c>
-      <c r="K13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 865,75 TL</t>
-        </is>
-      </c>
+      <c r="I13" s="14" t="inlineStr"/>
+      <c r="J13" s="14" t="inlineStr"/>
+      <c r="K13" s="14" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="B14" s="13" t="inlineStr">
@@ -961,21 +925,13 @@
         </is>
       </c>
       <c r="C14" s="14" t="inlineStr"/>
-      <c r="D14" s="14" t="inlineStr">
-        <is>
-          <t>3.500 TL - 13.500 TL</t>
-        </is>
-      </c>
+      <c r="D14" s="14" t="inlineStr"/>
       <c r="E14" s="14" t="inlineStr">
         <is>
           <t>2.170 TL - 2.170 TL</t>
         </is>
       </c>
-      <c r="F14" s="14" t="inlineStr">
-        <is>
-          <t>2.785,72 TL - 12.380,95 TL</t>
-        </is>
-      </c>
+      <c r="F14" s="14" t="inlineStr"/>
       <c r="G14" s="14" t="inlineStr">
         <is>
           <t>8.300 TL - 7,97 TL</t>
@@ -987,16 +943,8 @@
         </is>
       </c>
       <c r="I14" s="14" t="inlineStr"/>
-      <c r="J14" s="14" t="inlineStr">
-        <is>
-          <t>1.554,97 TL - 7.784 TL</t>
-        </is>
-      </c>
-      <c r="K14" s="14" t="inlineStr">
-        <is>
-          <t>1.196,51 TL - 5.583,74 TL</t>
-        </is>
-      </c>
+      <c r="J14" s="14" t="inlineStr"/>
+      <c r="K14" s="14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="12" t="inlineStr">

</xml_diff>

<commit_message>
Update benchmark: 2026-07-25 08:07:43 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -606,11 +606,7 @@
           <t>30 TL - 30 TL</t>
         </is>
       </c>
-      <c r="D2" s="14" t="inlineStr">
-        <is>
-          <t>33,33 TL - 33,33 TL</t>
-        </is>
-      </c>
+      <c r="D2" s="14" t="inlineStr"/>
       <c r="E2" s="14" t="inlineStr">
         <is>
           <t>26 TL - 26 TL</t>
@@ -723,7 +719,11 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="D6" s="14" t="inlineStr"/>
+      <c r="D6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 199,41 TL</t>
+        </is>
+      </c>
       <c r="E6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
@@ -740,8 +740,16 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="I6" s="14" t="inlineStr"/>
-      <c r="J6" s="14" t="inlineStr"/>
+      <c r="I6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 199,41 TL</t>
+        </is>
+      </c>
+      <c r="J6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 199,41 TL</t>
+        </is>
+      </c>
       <c r="K6" s="14" t="inlineStr"/>
     </row>
     <row r="7">
@@ -751,11 +759,7 @@
         </is>
       </c>
       <c r="C7" s="14" t="inlineStr"/>
-      <c r="D7" s="14" t="inlineStr">
-        <is>
-          <t>%1,6</t>
-        </is>
-      </c>
+      <c r="D7" s="14" t="inlineStr"/>
       <c r="E7" s="14" t="inlineStr"/>
       <c r="F7" s="14" t="inlineStr">
         <is>
@@ -880,8 +884,16 @@
           <t>GİDEN SWIFT</t>
         </is>
       </c>
-      <c r="C12" s="14" t="inlineStr"/>
-      <c r="D12" s="14" t="inlineStr"/>
+      <c r="C12" s="14" t="inlineStr">
+        <is>
+          <t>WU: 1.000,01 USD–9,51 USD</t>
+        </is>
+      </c>
+      <c r="D12" s="14" t="inlineStr">
+        <is>
+          <t>WU: 0,75 USD–12 USD; Diğer: 700 TL–4.000 TL</t>
+        </is>
+      </c>
       <c r="E12" s="14" t="inlineStr"/>
       <c r="F12" s="14" t="inlineStr"/>
       <c r="G12" s="14" t="inlineStr">
@@ -900,8 +912,16 @@
           <t>GELEN SWIFT</t>
         </is>
       </c>
-      <c r="C13" s="14" t="inlineStr"/>
-      <c r="D13" s="14" t="inlineStr"/>
+      <c r="C13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 0 TL | Azami 0,94 TL</t>
+        </is>
+      </c>
+      <c r="D13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
+        </is>
+      </c>
       <c r="E13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
@@ -914,8 +934,16 @@
           <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
         </is>
       </c>
-      <c r="I13" s="14" t="inlineStr"/>
-      <c r="J13" s="14" t="inlineStr"/>
+      <c r="I13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
+        </is>
+      </c>
+      <c r="J13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 1.303 TL</t>
+        </is>
+      </c>
       <c r="K13" s="14" t="inlineStr"/>
     </row>
     <row r="14">
@@ -924,14 +952,26 @@
           <t>GİDEN SWIFT - Mobil</t>
         </is>
       </c>
-      <c r="C14" s="14" t="inlineStr"/>
-      <c r="D14" s="14" t="inlineStr"/>
+      <c r="C14" s="14" t="inlineStr">
+        <is>
+          <t>40.000 TL - 2.485,72 TL</t>
+        </is>
+      </c>
+      <c r="D14" s="14" t="inlineStr">
+        <is>
+          <t>3.500 TL - 13.500 TL</t>
+        </is>
+      </c>
       <c r="E14" s="14" t="inlineStr">
         <is>
           <t>2.170 TL - 2.170 TL</t>
         </is>
       </c>
-      <c r="F14" s="14" t="inlineStr"/>
+      <c r="F14" s="14" t="inlineStr">
+        <is>
+          <t>2.785,72 TL - 12.380,95 TL</t>
+        </is>
+      </c>
       <c r="G14" s="14" t="inlineStr">
         <is>
           <t>8.300 TL - 7,97 TL</t>
@@ -943,7 +983,11 @@
         </is>
       </c>
       <c r="I14" s="14" t="inlineStr"/>
-      <c r="J14" s="14" t="inlineStr"/>
+      <c r="J14" s="14" t="inlineStr">
+        <is>
+          <t>1.554,97 TL - 7.784 TL</t>
+        </is>
+      </c>
       <c r="K14" s="14" t="inlineStr"/>
     </row>
     <row r="15">

</xml_diff>

<commit_message>
Update benchmark: 2026-07-26 08:27:50 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -606,7 +606,11 @@
           <t>30 TL - 30 TL</t>
         </is>
       </c>
-      <c r="D2" s="14" t="inlineStr"/>
+      <c r="D2" s="14" t="inlineStr">
+        <is>
+          <t>33,33 TL - 33,33 TL</t>
+        </is>
+      </c>
       <c r="E2" s="14" t="inlineStr">
         <is>
           <t>26 TL - 26 TL</t>
@@ -750,7 +754,11 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="K6" s="14" t="inlineStr"/>
+      <c r="K6" s="14" t="inlineStr">
+        <is>
+          <t>7,97 TL - 15,96 TL - 199,41 TL</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="B7" s="13" t="inlineStr">
@@ -759,7 +767,11 @@
         </is>
       </c>
       <c r="C7" s="14" t="inlineStr"/>
-      <c r="D7" s="14" t="inlineStr"/>
+      <c r="D7" s="14" t="inlineStr">
+        <is>
+          <t>%1,6</t>
+        </is>
+      </c>
       <c r="E7" s="14" t="inlineStr"/>
       <c r="F7" s="14" t="inlineStr">
         <is>
@@ -884,11 +896,7 @@
           <t>GİDEN SWIFT</t>
         </is>
       </c>
-      <c r="C12" s="14" t="inlineStr">
-        <is>
-          <t>WU: 1.000,01 USD–9,51 USD</t>
-        </is>
-      </c>
+      <c r="C12" s="14" t="inlineStr"/>
       <c r="D12" s="14" t="inlineStr">
         <is>
           <t>WU: 0,75 USD–12 USD; Diğer: 700 TL–4.000 TL</t>
@@ -904,7 +912,11 @@
       <c r="H12" s="14" t="inlineStr"/>
       <c r="I12" s="14" t="inlineStr"/>
       <c r="J12" s="14" t="inlineStr"/>
-      <c r="K12" s="14" t="inlineStr"/>
+      <c r="K12" s="14" t="inlineStr">
+        <is>
+          <t>WU: ,USD–; Diğer: 529 TL–4.454,74 TL</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="B13" s="13" t="inlineStr">
@@ -912,11 +924,7 @@
           <t>GELEN SWIFT</t>
         </is>
       </c>
-      <c r="C13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 0 TL | Azami 0,94 TL</t>
-        </is>
-      </c>
+      <c r="C13" s="14" t="inlineStr"/>
       <c r="D13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
@@ -944,7 +952,11 @@
           <t>Hesaba: Asgari 1 TL | Azami 1.303 TL</t>
         </is>
       </c>
-      <c r="K13" s="14" t="inlineStr"/>
+      <c r="K13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 865,75 TL</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="B14" s="13" t="inlineStr">
@@ -952,11 +964,7 @@
           <t>GİDEN SWIFT - Mobil</t>
         </is>
       </c>
-      <c r="C14" s="14" t="inlineStr">
-        <is>
-          <t>40.000 TL - 2.485,72 TL</t>
-        </is>
-      </c>
+      <c r="C14" s="14" t="inlineStr"/>
       <c r="D14" s="14" t="inlineStr">
         <is>
           <t>3.500 TL - 13.500 TL</t>
@@ -988,7 +996,11 @@
           <t>1.554,97 TL - 7.784 TL</t>
         </is>
       </c>
-      <c r="K14" s="14" t="inlineStr"/>
+      <c r="K14" s="14" t="inlineStr">
+        <is>
+          <t>1.196,51 TL - 5.583,74 TL</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="12" t="inlineStr">

</xml_diff>

<commit_message>
Update benchmark: 2026-07-27 09:52:52 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -896,7 +896,11 @@
           <t>GİDEN SWIFT</t>
         </is>
       </c>
-      <c r="C12" s="14" t="inlineStr"/>
+      <c r="C12" s="14" t="inlineStr">
+        <is>
+          <t>WU: 3.000,01 USD–9,51 USD</t>
+        </is>
+      </c>
       <c r="D12" s="14" t="inlineStr">
         <is>
           <t>WU: 0,75 USD–12 USD; Diğer: 700 TL–4.000 TL</t>
@@ -924,7 +928,11 @@
           <t>GELEN SWIFT</t>
         </is>
       </c>
-      <c r="C13" s="14" t="inlineStr"/>
+      <c r="C13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 0 TL | Azami 0,94 TL</t>
+        </is>
+      </c>
       <c r="D13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
@@ -964,7 +972,11 @@
           <t>GİDEN SWIFT - Mobil</t>
         </is>
       </c>
-      <c r="C14" s="14" t="inlineStr"/>
+      <c r="C14" s="14" t="inlineStr">
+        <is>
+          <t>40.000 TL - 2.485,72 TL</t>
+        </is>
+      </c>
       <c r="D14" s="14" t="inlineStr">
         <is>
           <t>3.500 TL - 13.500 TL</t>

</xml_diff>

<commit_message>
Update benchmark: 2026-07-28 08:34:41 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -631,11 +631,7 @@
           <t>15 TL - 15 TL</t>
         </is>
       </c>
-      <c r="I2" s="14" t="inlineStr">
-        <is>
-          <t>18 TL - 18 TL</t>
-        </is>
-      </c>
+      <c r="I2" s="14" t="inlineStr"/>
       <c r="J2" s="14" t="inlineStr">
         <is>
           <t>65 TL - 65 TL</t>

</xml_diff>

<commit_message>
Update benchmark: 2026-07-29 08:41:42 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -631,7 +631,11 @@
           <t>15 TL - 15 TL</t>
         </is>
       </c>
-      <c r="I2" s="14" t="inlineStr"/>
+      <c r="I2" s="14" t="inlineStr">
+        <is>
+          <t>18 TL - 18 TL</t>
+        </is>
+      </c>
       <c r="J2" s="14" t="inlineStr">
         <is>
           <t>65 TL - 65 TL</t>
@@ -750,11 +754,7 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="K6" s="14" t="inlineStr">
-        <is>
-          <t>7,97 TL - 15,96 TL - 199,41 TL</t>
-        </is>
-      </c>
+      <c r="K6" s="14" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="B7" s="13" t="inlineStr">
@@ -912,11 +912,7 @@
       <c r="H12" s="14" t="inlineStr"/>
       <c r="I12" s="14" t="inlineStr"/>
       <c r="J12" s="14" t="inlineStr"/>
-      <c r="K12" s="14" t="inlineStr">
-        <is>
-          <t>WU: ,USD–; Diğer: 529 TL–4.454,74 TL</t>
-        </is>
-      </c>
+      <c r="K12" s="14" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="B13" s="13" t="inlineStr">
@@ -956,11 +952,7 @@
           <t>Hesaba: Asgari 1 TL | Azami 1.303 TL</t>
         </is>
       </c>
-      <c r="K13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 865,75 TL</t>
-        </is>
-      </c>
+      <c r="K13" s="14" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="B14" s="13" t="inlineStr">
@@ -983,11 +975,7 @@
           <t>2.170 TL - 2.170 TL</t>
         </is>
       </c>
-      <c r="F14" s="14" t="inlineStr">
-        <is>
-          <t>2.785,72 TL - 12.380,95 TL</t>
-        </is>
-      </c>
+      <c r="F14" s="14" t="inlineStr"/>
       <c r="G14" s="14" t="inlineStr">
         <is>
           <t>8.300 TL - 7,97 TL</t>
@@ -1004,11 +992,7 @@
           <t>1.554,97 TL - 7.784 TL</t>
         </is>
       </c>
-      <c r="K14" s="14" t="inlineStr">
-        <is>
-          <t>1.196,51 TL - 5.583,74 TL</t>
-        </is>
-      </c>
+      <c r="K14" s="14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="12" t="inlineStr">

</xml_diff>

<commit_message>
Update benchmark: 2026-07-30 08:27:37 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -754,7 +754,11 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="K6" s="14" t="inlineStr"/>
+      <c r="K6" s="14" t="inlineStr">
+        <is>
+          <t>7,97 TL - 15,96 TL - 199,41 TL</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="B7" s="13" t="inlineStr">
@@ -894,7 +898,7 @@
       </c>
       <c r="C12" s="14" t="inlineStr">
         <is>
-          <t>WU: 3.000,01 USD–9,51 USD</t>
+          <t>WU: 0,1 USD–9,51 USD</t>
         </is>
       </c>
       <c r="D12" s="14" t="inlineStr">
@@ -912,7 +916,11 @@
       <c r="H12" s="14" t="inlineStr"/>
       <c r="I12" s="14" t="inlineStr"/>
       <c r="J12" s="14" t="inlineStr"/>
-      <c r="K12" s="14" t="inlineStr"/>
+      <c r="K12" s="14" t="inlineStr">
+        <is>
+          <t>WU: ,USD–; Diğer: 529 TL–4.454,74 TL</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="B13" s="13" t="inlineStr">
@@ -952,7 +960,11 @@
           <t>Hesaba: Asgari 1 TL | Azami 1.303 TL</t>
         </is>
       </c>
-      <c r="K13" s="14" t="inlineStr"/>
+      <c r="K13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 865,75 TL</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="B14" s="13" t="inlineStr">
@@ -975,7 +987,11 @@
           <t>2.170 TL - 2.170 TL</t>
         </is>
       </c>
-      <c r="F14" s="14" t="inlineStr"/>
+      <c r="F14" s="14" t="inlineStr">
+        <is>
+          <t>2.785,72 TL - 12.380,95 TL</t>
+        </is>
+      </c>
       <c r="G14" s="14" t="inlineStr">
         <is>
           <t>8.300 TL - 7,97 TL</t>
@@ -992,7 +1008,11 @@
           <t>1.554,97 TL - 7.784 TL</t>
         </is>
       </c>
-      <c r="K14" s="14" t="inlineStr"/>
+      <c r="K14" s="14" t="inlineStr">
+        <is>
+          <t>1.196,51 TL - 5.583,74 TL</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="12" t="inlineStr">

</xml_diff>

<commit_message>
Update benchmark: 2026-07-31 08:50:38 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -898,7 +898,7 @@
       </c>
       <c r="C12" s="14" t="inlineStr">
         <is>
-          <t>WU: 0,1 USD–9,51 USD</t>
+          <t>WU: 3.000,01 USD–9,51 USD</t>
         </is>
       </c>
       <c r="D12" s="14" t="inlineStr">
@@ -938,11 +938,7 @@
           <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
         </is>
       </c>
-      <c r="E13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
-        </is>
-      </c>
+      <c r="E13" s="14" t="inlineStr"/>
       <c r="F13" s="14" t="inlineStr"/>
       <c r="G13" s="14" t="inlineStr"/>
       <c r="H13" s="14" t="inlineStr">
@@ -982,11 +978,7 @@
           <t>3.500 TL - 13.500 TL</t>
         </is>
       </c>
-      <c r="E14" s="14" t="inlineStr">
-        <is>
-          <t>2.170 TL - 2.170 TL</t>
-        </is>
-      </c>
+      <c r="E14" s="14" t="inlineStr"/>
       <c r="F14" s="14" t="inlineStr">
         <is>
           <t>2.785,72 TL - 12.380,95 TL</t>

</xml_diff>

<commit_message>
Update benchmark: 2026-08-01 08:22:24 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -938,7 +938,11 @@
           <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
         </is>
       </c>
-      <c r="E13" s="14" t="inlineStr"/>
+      <c r="E13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
+        </is>
+      </c>
       <c r="F13" s="14" t="inlineStr"/>
       <c r="G13" s="14" t="inlineStr"/>
       <c r="H13" s="14" t="inlineStr">
@@ -978,7 +982,11 @@
           <t>3.500 TL - 13.500 TL</t>
         </is>
       </c>
-      <c r="E14" s="14" t="inlineStr"/>
+      <c r="E14" s="14" t="inlineStr">
+        <is>
+          <t>2.170 TL - 2.170 TL</t>
+        </is>
+      </c>
       <c r="F14" s="14" t="inlineStr">
         <is>
           <t>2.785,72 TL - 12.380,95 TL</t>

</xml_diff>

<commit_message>
Update benchmark: 2026-08-02 08:24:48 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -901,11 +901,7 @@
           <t>WU: 3.000,01 USD–9,51 USD</t>
         </is>
       </c>
-      <c r="D12" s="14" t="inlineStr">
-        <is>
-          <t>WU: 0,75 USD–12 USD; Diğer: 700 TL–4.000 TL</t>
-        </is>
-      </c>
+      <c r="D12" s="14" t="inlineStr"/>
       <c r="E12" s="14" t="inlineStr"/>
       <c r="F12" s="14" t="inlineStr"/>
       <c r="G12" s="14" t="inlineStr">
@@ -933,11 +929,7 @@
           <t>Hesaba: Asgari 0 TL | Azami 0,94 TL</t>
         </is>
       </c>
-      <c r="D13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
-        </is>
-      </c>
+      <c r="D13" s="14" t="inlineStr"/>
       <c r="E13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
@@ -977,11 +969,7 @@
           <t>40.000 TL - 2.485,72 TL</t>
         </is>
       </c>
-      <c r="D14" s="14" t="inlineStr">
-        <is>
-          <t>3.500 TL - 13.500 TL</t>
-        </is>
-      </c>
+      <c r="D14" s="14" t="inlineStr"/>
       <c r="E14" s="14" t="inlineStr">
         <is>
           <t>2.170 TL - 2.170 TL</t>

</xml_diff>

<commit_message>
Update benchmark: 2026-08-03 09:44:28 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -603,7 +603,7 @@
       <c r="B2" s="13" t="inlineStr"/>
       <c r="C2" s="14" t="inlineStr">
         <is>
-          <t>30 TL - 30 TL</t>
+          <t>35,71 TL - 35,71 TL</t>
         </is>
       </c>
       <c r="D2" s="14" t="inlineStr">
@@ -901,7 +901,11 @@
           <t>WU: 3.000,01 USD–9,51 USD</t>
         </is>
       </c>
-      <c r="D12" s="14" t="inlineStr"/>
+      <c r="D12" s="14" t="inlineStr">
+        <is>
+          <t>WU: 0,75 USD–12 USD; Diğer: 700 TL–4.000 TL</t>
+        </is>
+      </c>
       <c r="E12" s="14" t="inlineStr"/>
       <c r="F12" s="14" t="inlineStr"/>
       <c r="G12" s="14" t="inlineStr">
@@ -929,7 +933,11 @@
           <t>Hesaba: Asgari 0 TL | Azami 0,94 TL</t>
         </is>
       </c>
-      <c r="D13" s="14" t="inlineStr"/>
+      <c r="D13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
+        </is>
+      </c>
       <c r="E13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
@@ -969,7 +977,11 @@
           <t>40.000 TL - 2.485,72 TL</t>
         </is>
       </c>
-      <c r="D14" s="14" t="inlineStr"/>
+      <c r="D14" s="14" t="inlineStr">
+        <is>
+          <t>3.500 TL - 13.500 TL</t>
+        </is>
+      </c>
       <c r="E14" s="14" t="inlineStr">
         <is>
           <t>2.170 TL - 2.170 TL</t>

</xml_diff>

<commit_message>
Update benchmark: 2026-08-04 08:36:53 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -744,16 +744,8 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="I6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 199,41 TL</t>
-        </is>
-      </c>
-      <c r="J6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 199,41 TL</t>
-        </is>
-      </c>
+      <c r="I6" s="14" t="inlineStr"/>
+      <c r="J6" s="14" t="inlineStr"/>
       <c r="K6" s="14" t="inlineStr">
         <is>
           <t>7,97 TL - 15,96 TL - 199,41 TL</t>
@@ -950,16 +942,8 @@
           <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
         </is>
       </c>
-      <c r="I13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
-        </is>
-      </c>
-      <c r="J13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 1.303 TL</t>
-        </is>
-      </c>
+      <c r="I13" s="14" t="inlineStr"/>
+      <c r="J13" s="14" t="inlineStr"/>
       <c r="K13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 865,75 TL</t>
@@ -1003,11 +987,7 @@
         </is>
       </c>
       <c r="I14" s="14" t="inlineStr"/>
-      <c r="J14" s="14" t="inlineStr">
-        <is>
-          <t>1.554,97 TL - 7.784 TL</t>
-        </is>
-      </c>
+      <c r="J14" s="14" t="inlineStr"/>
       <c r="K14" s="14" t="inlineStr">
         <is>
           <t>1.196,51 TL - 5.583,74 TL</t>

</xml_diff>

<commit_message>
Update benchmark: 2026-08-05 08:36:29 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -744,8 +744,16 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="I6" s="14" t="inlineStr"/>
-      <c r="J6" s="14" t="inlineStr"/>
+      <c r="I6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 199,41 TL</t>
+        </is>
+      </c>
+      <c r="J6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 199,41 TL</t>
+        </is>
+      </c>
       <c r="K6" s="14" t="inlineStr">
         <is>
           <t>7,97 TL - 15,96 TL - 199,41 TL</t>
@@ -942,8 +950,16 @@
           <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
         </is>
       </c>
-      <c r="I13" s="14" t="inlineStr"/>
-      <c r="J13" s="14" t="inlineStr"/>
+      <c r="I13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
+        </is>
+      </c>
+      <c r="J13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 1.303 TL</t>
+        </is>
+      </c>
       <c r="K13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 865,75 TL</t>
@@ -987,7 +1003,11 @@
         </is>
       </c>
       <c r="I14" s="14" t="inlineStr"/>
-      <c r="J14" s="14" t="inlineStr"/>
+      <c r="J14" s="14" t="inlineStr">
+        <is>
+          <t>1.554,97 TL - 7.784 TL</t>
+        </is>
+      </c>
       <c r="K14" s="14" t="inlineStr">
         <is>
           <t>1.196,51 TL - 5.583,74 TL</t>

</xml_diff>

<commit_message>
Update benchmark: 2026-08-07 07:16:18 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -898,7 +898,7 @@
       </c>
       <c r="C12" s="14" t="inlineStr">
         <is>
-          <t>WU: 3.000,01 USD–9,51 USD</t>
+          <t>WU: 1.000,01 USD–9,51 USD</t>
         </is>
       </c>
       <c r="D12" s="14" t="inlineStr">
@@ -962,7 +962,7 @@
       </c>
       <c r="K13" s="14" t="inlineStr">
         <is>
-          <t>Hesaba: Asgari 1 TL | Azami 69,62 TL</t>
+          <t>Hesaba: Asgari 1 TL | Azami 865,75 TL</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update benchmark: 2026-08-08 06:53:48 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -744,11 +744,7 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="I6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 199,41 TL</t>
-        </is>
-      </c>
+      <c r="I6" s="14" t="inlineStr"/>
       <c r="J6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
@@ -898,7 +894,7 @@
       </c>
       <c r="C12" s="14" t="inlineStr">
         <is>
-          <t>WU: 1.000,01 USD–9,51 USD</t>
+          <t>WU: 3.000,01 USD–9,51 USD</t>
         </is>
       </c>
       <c r="D12" s="14" t="inlineStr">
@@ -938,11 +934,7 @@
           <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
         </is>
       </c>
-      <c r="E13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
-        </is>
-      </c>
+      <c r="E13" s="14" t="inlineStr"/>
       <c r="F13" s="14" t="inlineStr"/>
       <c r="G13" s="14" t="inlineStr"/>
       <c r="H13" s="14" t="inlineStr">
@@ -950,11 +942,7 @@
           <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
         </is>
       </c>
-      <c r="I13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
-        </is>
-      </c>
+      <c r="I13" s="14" t="inlineStr"/>
       <c r="J13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.303 TL</t>
@@ -982,11 +970,7 @@
           <t>3.500 TL - 13.500 TL</t>
         </is>
       </c>
-      <c r="E14" s="14" t="inlineStr">
-        <is>
-          <t>2.170 TL - 2.170 TL</t>
-        </is>
-      </c>
+      <c r="E14" s="14" t="inlineStr"/>
       <c r="F14" s="14" t="inlineStr">
         <is>
           <t>2.785,72 TL - 12.380,95 TL</t>

</xml_diff>

<commit_message>
Update benchmark: 2026-08-09 06:56:47 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -718,11 +718,7 @@
           <t>DÜZENLİ EFT</t>
         </is>
       </c>
-      <c r="C6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 199,41 TL</t>
-        </is>
-      </c>
+      <c r="C6" s="14" t="inlineStr"/>
       <c r="D6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
@@ -744,7 +740,11 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="I6" s="14" t="inlineStr"/>
+      <c r="I6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 199,41 TL</t>
+        </is>
+      </c>
       <c r="J6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
@@ -892,11 +892,7 @@
           <t>GİDEN SWIFT</t>
         </is>
       </c>
-      <c r="C12" s="14" t="inlineStr">
-        <is>
-          <t>WU: 3.000,01 USD–9,51 USD</t>
-        </is>
-      </c>
+      <c r="C12" s="14" t="inlineStr"/>
       <c r="D12" s="14" t="inlineStr">
         <is>
           <t>WU: 0,75 USD–12 USD; Diğer: 700 TL–4.000 TL</t>
@@ -924,11 +920,7 @@
           <t>GELEN SWIFT</t>
         </is>
       </c>
-      <c r="C13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 0 TL | Azami 0,94 TL</t>
-        </is>
-      </c>
+      <c r="C13" s="14" t="inlineStr"/>
       <c r="D13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
@@ -942,7 +934,11 @@
           <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
         </is>
       </c>
-      <c r="I13" s="14" t="inlineStr"/>
+      <c r="I13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
+        </is>
+      </c>
       <c r="J13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.303 TL</t>
@@ -960,11 +956,7 @@
           <t>GİDEN SWIFT - Mobil</t>
         </is>
       </c>
-      <c r="C14" s="14" t="inlineStr">
-        <is>
-          <t>40.000 TL - 2.485,72 TL</t>
-        </is>
-      </c>
+      <c r="C14" s="14" t="inlineStr"/>
       <c r="D14" s="14" t="inlineStr">
         <is>
           <t>3.500 TL - 13.500 TL</t>

</xml_diff>

<commit_message>
Update benchmark: 2026-08-10 07:41:26 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -718,7 +718,11 @@
           <t>DÜZENLİ EFT</t>
         </is>
       </c>
-      <c r="C6" s="14" t="inlineStr"/>
+      <c r="C6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 199,41 TL</t>
+        </is>
+      </c>
       <c r="D6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
@@ -892,7 +896,11 @@
           <t>GİDEN SWIFT</t>
         </is>
       </c>
-      <c r="C12" s="14" t="inlineStr"/>
+      <c r="C12" s="14" t="inlineStr">
+        <is>
+          <t>WU: 3.000,01 USD–9,51 USD</t>
+        </is>
+      </c>
       <c r="D12" s="14" t="inlineStr">
         <is>
           <t>WU: 0,75 USD–12 USD; Diğer: 700 TL–4.000 TL</t>
@@ -920,13 +928,21 @@
           <t>GELEN SWIFT</t>
         </is>
       </c>
-      <c r="C13" s="14" t="inlineStr"/>
+      <c r="C13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 0 TL | Azami 0,94 TL</t>
+        </is>
+      </c>
       <c r="D13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
         </is>
       </c>
-      <c r="E13" s="14" t="inlineStr"/>
+      <c r="E13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
+        </is>
+      </c>
       <c r="F13" s="14" t="inlineStr"/>
       <c r="G13" s="14" t="inlineStr"/>
       <c r="H13" s="14" t="inlineStr">
@@ -956,13 +972,21 @@
           <t>GİDEN SWIFT - Mobil</t>
         </is>
       </c>
-      <c r="C14" s="14" t="inlineStr"/>
+      <c r="C14" s="14" t="inlineStr">
+        <is>
+          <t>40.000 TL - 2.485,72 TL</t>
+        </is>
+      </c>
       <c r="D14" s="14" t="inlineStr">
         <is>
           <t>3.500 TL - 13.500 TL</t>
         </is>
       </c>
-      <c r="E14" s="14" t="inlineStr"/>
+      <c r="E14" s="14" t="inlineStr">
+        <is>
+          <t>2.170 TL - 2.170 TL</t>
+        </is>
+      </c>
       <c r="F14" s="14" t="inlineStr">
         <is>
           <t>2.785,72 TL - 12.380,95 TL</t>

</xml_diff>

<commit_message>
Update benchmark: 2026-08-11 07:07:43 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -754,11 +754,7 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="K6" s="14" t="inlineStr">
-        <is>
-          <t>7,97 TL - 15,96 TL - 199,41 TL</t>
-        </is>
-      </c>
+      <c r="K6" s="14" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="B7" s="13" t="inlineStr">
@@ -903,7 +899,7 @@
       </c>
       <c r="D12" s="14" t="inlineStr">
         <is>
-          <t>WU: 0,75 USD–12 USD; Diğer: 700 TL–4.000 TL</t>
+          <t>WU: 6 USD–12 USD; Diğer: 700 TL–4.000 TL</t>
         </is>
       </c>
       <c r="E12" s="14" t="inlineStr"/>
@@ -916,11 +912,7 @@
       <c r="H12" s="14" t="inlineStr"/>
       <c r="I12" s="14" t="inlineStr"/>
       <c r="J12" s="14" t="inlineStr"/>
-      <c r="K12" s="14" t="inlineStr">
-        <is>
-          <t>WU: ,USD–; Diğer: 529 TL–4.454,74 TL</t>
-        </is>
-      </c>
+      <c r="K12" s="14" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="B13" s="13" t="inlineStr">
@@ -960,11 +952,7 @@
           <t>Hesaba: Asgari 1 TL | Azami 1.303 TL</t>
         </is>
       </c>
-      <c r="K13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 865,75 TL</t>
-        </is>
-      </c>
+      <c r="K13" s="14" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="B14" s="13" t="inlineStr">
@@ -1008,11 +996,7 @@
           <t>1.554,97 TL - 7.784 TL</t>
         </is>
       </c>
-      <c r="K14" s="14" t="inlineStr">
-        <is>
-          <t>1.196,51 TL - 5.583,74 TL</t>
-        </is>
-      </c>
+      <c r="K14" s="14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="12" t="inlineStr">

</xml_diff>

<commit_message>
Update benchmark: 2026-08-12 07:24:54 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -754,7 +754,11 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="K6" s="14" t="inlineStr"/>
+      <c r="K6" s="14" t="inlineStr">
+        <is>
+          <t>7,97 TL - 15,96 TL - 199,41 TL</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="B7" s="13" t="inlineStr">
@@ -894,7 +898,7 @@
       </c>
       <c r="C12" s="14" t="inlineStr">
         <is>
-          <t>WU: 3.000,01 USD–9,51 USD</t>
+          <t>WU: 1.000,01 USD–9,51 USD</t>
         </is>
       </c>
       <c r="D12" s="14" t="inlineStr">
@@ -912,7 +916,11 @@
       <c r="H12" s="14" t="inlineStr"/>
       <c r="I12" s="14" t="inlineStr"/>
       <c r="J12" s="14" t="inlineStr"/>
-      <c r="K12" s="14" t="inlineStr"/>
+      <c r="K12" s="14" t="inlineStr">
+        <is>
+          <t>WU: ,USD–; Diğer: 529 TL–4.454,74 TL</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="B13" s="13" t="inlineStr">
@@ -952,7 +960,11 @@
           <t>Hesaba: Asgari 1 TL | Azami 1.303 TL</t>
         </is>
       </c>
-      <c r="K13" s="14" t="inlineStr"/>
+      <c r="K13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 865,75 TL</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="B14" s="13" t="inlineStr">
@@ -996,7 +1008,11 @@
           <t>1.554,97 TL - 7.784 TL</t>
         </is>
       </c>
-      <c r="K14" s="14" t="inlineStr"/>
+      <c r="K14" s="14" t="inlineStr">
+        <is>
+          <t>1.196,51 TL - 5.583,74 TL</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="12" t="inlineStr">
@@ -1410,11 +1426,7 @@
           <t>500 TL</t>
         </is>
       </c>
-      <c r="K24" s="14" t="inlineStr">
-        <is>
-          <t>446,06 TL</t>
-        </is>
-      </c>
+      <c r="K24" s="14" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="B25" s="13" t="inlineStr">
@@ -1458,11 +1470,7 @@
           <t>750 TL</t>
         </is>
       </c>
-      <c r="K25" s="14" t="inlineStr">
-        <is>
-          <t>374,4 TL</t>
-        </is>
-      </c>
+      <c r="K25" s="14" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="6">

</xml_diff>

<commit_message>
Update benchmark: 2026-08-13 07:27:28 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -898,7 +898,7 @@
       </c>
       <c r="C12" s="14" t="inlineStr">
         <is>
-          <t>WU: 1.000,01 USD–9,51 USD</t>
+          <t>WU: 0,1 USD–9,51 USD</t>
         </is>
       </c>
       <c r="D12" s="14" t="inlineStr">
@@ -1426,7 +1426,11 @@
           <t>500 TL</t>
         </is>
       </c>
-      <c r="K24" s="14" t="inlineStr"/>
+      <c r="K24" s="14" t="inlineStr">
+        <is>
+          <t>446,06 TL</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="B25" s="13" t="inlineStr">
@@ -1470,7 +1474,11 @@
           <t>750 TL</t>
         </is>
       </c>
-      <c r="K25" s="14" t="inlineStr"/>
+      <c r="K25" s="14" t="inlineStr">
+        <is>
+          <t>374,4 TL</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="6">

</xml_diff>

<commit_message>
Update benchmark: 2026-08-14 07:25:32 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -728,11 +728,7 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="E6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 199,41 TL</t>
-        </is>
-      </c>
+      <c r="E6" s="14" t="inlineStr"/>
       <c r="F6" s="14" t="inlineStr"/>
       <c r="G6" s="14" t="inlineStr">
         <is>
@@ -896,11 +892,7 @@
           <t>GİDEN SWIFT</t>
         </is>
       </c>
-      <c r="C12" s="14" t="inlineStr">
-        <is>
-          <t>WU: 0,1 USD–9,51 USD</t>
-        </is>
-      </c>
+      <c r="C12" s="14" t="inlineStr"/>
       <c r="D12" s="14" t="inlineStr">
         <is>
           <t>WU: 6 USD–12 USD; Diğer: 700 TL–4.000 TL</t>
@@ -928,21 +920,13 @@
           <t>GELEN SWIFT</t>
         </is>
       </c>
-      <c r="C13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 0 TL | Azami 0,94 TL</t>
-        </is>
-      </c>
+      <c r="C13" s="14" t="inlineStr"/>
       <c r="D13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
         </is>
       </c>
-      <c r="E13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
-        </is>
-      </c>
+      <c r="E13" s="14" t="inlineStr"/>
       <c r="F13" s="14" t="inlineStr"/>
       <c r="G13" s="14" t="inlineStr"/>
       <c r="H13" s="14" t="inlineStr">
@@ -972,26 +956,14 @@
           <t>GİDEN SWIFT - Mobil</t>
         </is>
       </c>
-      <c r="C14" s="14" t="inlineStr">
-        <is>
-          <t>40.000 TL - 2.485,72 TL</t>
-        </is>
-      </c>
+      <c r="C14" s="14" t="inlineStr"/>
       <c r="D14" s="14" t="inlineStr">
         <is>
           <t>3.500 TL - 13.500 TL</t>
         </is>
       </c>
-      <c r="E14" s="14" t="inlineStr">
-        <is>
-          <t>2.170 TL - 2.170 TL</t>
-        </is>
-      </c>
-      <c r="F14" s="14" t="inlineStr">
-        <is>
-          <t>2.785,72 TL - 12.380,95 TL</t>
-        </is>
-      </c>
+      <c r="E14" s="14" t="inlineStr"/>
+      <c r="F14" s="14" t="inlineStr"/>
       <c r="G14" s="14" t="inlineStr">
         <is>
           <t>8.300 TL - 7,97 TL</t>

</xml_diff>

<commit_message>
Update benchmark: 2026-08-15 06:38:04 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -728,7 +728,11 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="E6" s="14" t="inlineStr"/>
+      <c r="E6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 199,41 TL</t>
+        </is>
+      </c>
       <c r="F6" s="14" t="inlineStr"/>
       <c r="G6" s="14" t="inlineStr">
         <is>
@@ -892,7 +896,11 @@
           <t>GİDEN SWIFT</t>
         </is>
       </c>
-      <c r="C12" s="14" t="inlineStr"/>
+      <c r="C12" s="14" t="inlineStr">
+        <is>
+          <t>WU: 0,1 USD–9,51 USD</t>
+        </is>
+      </c>
       <c r="D12" s="14" t="inlineStr">
         <is>
           <t>WU: 6 USD–12 USD; Diğer: 700 TL–4.000 TL</t>
@@ -920,13 +928,21 @@
           <t>GELEN SWIFT</t>
         </is>
       </c>
-      <c r="C13" s="14" t="inlineStr"/>
+      <c r="C13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 0 TL | Azami 0,94 TL</t>
+        </is>
+      </c>
       <c r="D13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
         </is>
       </c>
-      <c r="E13" s="14" t="inlineStr"/>
+      <c r="E13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
+        </is>
+      </c>
       <c r="F13" s="14" t="inlineStr"/>
       <c r="G13" s="14" t="inlineStr"/>
       <c r="H13" s="14" t="inlineStr">
@@ -946,7 +962,7 @@
       </c>
       <c r="K13" s="14" t="inlineStr">
         <is>
-          <t>Hesaba: Asgari 1 TL | Azami 865,75 TL</t>
+          <t>Hesaba: Asgari 1 TL | Azami 1.133 TL</t>
         </is>
       </c>
     </row>
@@ -956,14 +972,26 @@
           <t>GİDEN SWIFT - Mobil</t>
         </is>
       </c>
-      <c r="C14" s="14" t="inlineStr"/>
+      <c r="C14" s="14" t="inlineStr">
+        <is>
+          <t>40.000 TL - 2.485,72 TL</t>
+        </is>
+      </c>
       <c r="D14" s="14" t="inlineStr">
         <is>
           <t>3.500 TL - 13.500 TL</t>
         </is>
       </c>
-      <c r="E14" s="14" t="inlineStr"/>
-      <c r="F14" s="14" t="inlineStr"/>
+      <c r="E14" s="14" t="inlineStr">
+        <is>
+          <t>2.170 TL - 2.170 TL</t>
+        </is>
+      </c>
+      <c r="F14" s="14" t="inlineStr">
+        <is>
+          <t>2.785,72 TL - 12.380,95 TL</t>
+        </is>
+      </c>
       <c r="G14" s="14" t="inlineStr">
         <is>
           <t>8.300 TL - 7,97 TL</t>

</xml_diff>

<commit_message>
Update benchmark: 2026-08-20 06:45:14 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -898,7 +898,7 @@
       </c>
       <c r="C12" s="14" t="inlineStr">
         <is>
-          <t>WU: 0,1 USD–9,51 USD</t>
+          <t>WU: 1.000,01 USD–9,51 USD</t>
         </is>
       </c>
       <c r="D12" s="14" t="inlineStr">
@@ -987,11 +987,7 @@
           <t>2.170 TL - 2.170 TL</t>
         </is>
       </c>
-      <c r="F14" s="14" t="inlineStr">
-        <is>
-          <t>2.785,72 TL - 12.380,95 TL</t>
-        </is>
-      </c>
+      <c r="F14" s="14" t="inlineStr"/>
       <c r="G14" s="14" t="inlineStr">
         <is>
           <t>8.300 TL - 7,97 TL</t>

</xml_diff>

<commit_message>
Update benchmark: 2026-08-21 06:45:44 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -744,11 +744,7 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="I6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 199,41 TL</t>
-        </is>
-      </c>
+      <c r="I6" s="14" t="inlineStr"/>
       <c r="J6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
@@ -940,7 +936,7 @@
       </c>
       <c r="E13" s="14" t="inlineStr">
         <is>
-          <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
+          <t>Hesaba: Asgari 1 TL | Azami 11.380 TL</t>
         </is>
       </c>
       <c r="F13" s="14" t="inlineStr"/>
@@ -950,11 +946,7 @@
           <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
         </is>
       </c>
-      <c r="I13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
-        </is>
-      </c>
+      <c r="I13" s="14" t="inlineStr"/>
       <c r="J13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.303 TL</t>
@@ -987,7 +979,11 @@
           <t>2.170 TL - 2.170 TL</t>
         </is>
       </c>
-      <c r="F14" s="14" t="inlineStr"/>
+      <c r="F14" s="14" t="inlineStr">
+        <is>
+          <t>2.785,72 TL - 12.380,95 TL</t>
+        </is>
+      </c>
       <c r="G14" s="14" t="inlineStr">
         <is>
           <t>8.300 TL - 7,97 TL</t>

</xml_diff>

<commit_message>
Update benchmark: 2026-08-22 06:39:45 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -618,7 +618,7 @@
       </c>
       <c r="F2" s="14" t="inlineStr">
         <is>
-          <t>33,33 TL - 33,33 TL</t>
+          <t>37,86 TL - 37,86 TL</t>
         </is>
       </c>
       <c r="G2" s="14" t="inlineStr">
@@ -744,7 +744,11 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="I6" s="14" t="inlineStr"/>
+      <c r="I6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 199,41 TL</t>
+        </is>
+      </c>
       <c r="J6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
@@ -894,7 +898,7 @@
       </c>
       <c r="C12" s="14" t="inlineStr">
         <is>
-          <t>WU: 1.000,01 USD–9,51 USD</t>
+          <t>WU: 3.000,01 USD–9,51 USD</t>
         </is>
       </c>
       <c r="D12" s="14" t="inlineStr">
@@ -936,7 +940,7 @@
       </c>
       <c r="E13" s="14" t="inlineStr">
         <is>
-          <t>Hesaba: Asgari 1 TL | Azami 11.380 TL</t>
+          <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
         </is>
       </c>
       <c r="F13" s="14" t="inlineStr"/>
@@ -946,7 +950,11 @@
           <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
         </is>
       </c>
-      <c r="I13" s="14" t="inlineStr"/>
+      <c r="I13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
+        </is>
+      </c>
       <c r="J13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.303 TL</t>

</xml_diff>